<commit_message>
Comparatif : « Montant total prévu » et colonnes FCFA jumelles
- Renommage « Budget prévu » en « Montant total prévu »
- Colonnes FCFA à côté de chaque colonne en euros (PU prévu, montant
  prévu, dépense réelle, écart) avec conversion automatique en euros
  dès qu'un montant est saisi en FCFA

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/budget-par-don-les-petits-enfants-de-marie.xlsx
+++ b/budget-par-don-les-petits-enfants-de-marie.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t xml:space="preserve">BUDGET PAR DON — LISTE D'ACHATS</t>
   </si>
@@ -119,28 +119,34 @@
     <t xml:space="preserve">TOTAL — ENVELOPPE À ENVOYER</t>
   </si>
   <si>
-    <t xml:space="preserve">COMPARATIF BUDGET PRÉVU / DÉPENSES RÉELLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La partie « Prévu » se remplit toute seule depuis l'onglet Budget du don. Après les achats, saisissez la quantité et le prix réellement payés (en € OU en FCFA) : les écarts se calculent automatiquement. Écart en vert = économie, en rouge = dépassement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUDGET PRÉVU (€)</t>
+    <t xml:space="preserve">COMPARATIF MONTANT TOTAL PRÉVU / DÉPENSES RÉELLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La partie « Prévu » se remplit toute seule depuis l'onglet Budget du don. Après les achats, saisissez la quantité et le prix réellement payés — en € OU en FCFA : dès qu'un montant est saisi en FCFA, il est converti en euros automatiquement. Chaque colonne en euros a sa jumelle en FCFA. Écart en vert = économie, en rouge = dépassement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTANT TOTAL PRÉVU (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTANT TOTAL PRÉVU (FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">DÉPENSES RÉELLES (€)</t>
   </si>
   <si>
+    <t xml:space="preserve">DÉPENSES RÉELLES (FCFA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ÉCART GLOBAL (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">% DU BUDGET DÉPENSÉ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUDGET PRÉVU (automatique)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DÉPENSES RÉELLES (à saisir)</t>
+    <t xml:space="preserve">% DU MONTANT PRÉVU DÉPENSÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTANT TOTAL PRÉVU (automatique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÉPENSES RÉELLES (à saisir : € ou FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">ANALYSE (automatique)</t>
@@ -155,7 +161,13 @@
     <t xml:space="preserve">PU prévu (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Budget prévu (€)</t>
+    <t xml:space="preserve">PU prévu (FCFA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montant total prévu (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montant total prévu (FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">Qté réelle</t>
@@ -170,7 +182,13 @@
     <t xml:space="preserve">Dépense réelle (€)</t>
   </si>
   <si>
+    <t xml:space="preserve">Dépense réelle (FCFA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Écart (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart (FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">Écart de prix unitaire</t>
@@ -405,7 +423,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -502,6 +520,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -551,6 +573,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1625,21 +1651,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1657,6 +1685,10 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -1673,6 +1705,10 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
@@ -1691,1658 +1727,2349 @@
         <v>37</v>
       </c>
       <c r="H4" s="8"/>
+      <c r="I4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="n">
-        <f aca="false">SUM(E9:E48)</f>
+        <f aca="false">SUM(F9:F48)</f>
         <v>182.938820684892</v>
       </c>
       <c r="B5" s="23"/>
       <c r="C5" s="24" t="n">
-        <f aca="false">SUM(I9:I48)</f>
+        <f aca="false">SUM(F9:F48)*'Budget du don'!$G$4</f>
+        <v>120000</v>
+      </c>
+      <c r="D5" s="24"/>
+      <c r="E5" s="25" t="n">
+        <f aca="false">SUM(K9:K48)</f>
         <v>195.134742063885</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="9" t="n">
-        <f aca="false">SUM(E9:E48)-SUM(I9:I48)</f>
+      <c r="F5" s="25"/>
+      <c r="G5" s="10" t="n">
+        <f aca="false">SUM(K9:K48)*'Budget du don'!$G$4</f>
+        <v>128000</v>
+      </c>
+      <c r="H5" s="10"/>
+      <c r="I5" s="9" t="n">
+        <f aca="false">SUM(F9:F48)-SUM(K9:K48)</f>
         <v>-12.1959213789929</v>
       </c>
-      <c r="F5" s="9"/>
-      <c r="G5" s="25" t="n">
-        <f aca="false">IF(SUM(E9:E48)=0,"",SUM(I9:I48)/SUM(E9:E48))</f>
+      <c r="J5" s="9"/>
+      <c r="K5" s="26" t="n">
+        <f aca="false">IF(SUM(F9:F48)=0,"",SUM(K9:K48)/SUM(F9:F48))</f>
         <v>1.06666666666667</v>
       </c>
-      <c r="H5" s="25"/>
+      <c r="L5" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="27" t="s">
-        <v>39</v>
-      </c>
+      <c r="A7" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
       <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28" t="s">
-        <v>40</v>
-      </c>
+      <c r="H7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
       <c r="K7" s="28"/>
       <c r="L7" s="28"/>
+      <c r="M7" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" s="29"/>
+      <c r="O7" s="29"/>
+      <c r="P7" s="29"/>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="P8" s="12" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="str">
+      <c r="A9" s="30" t="str">
         <f aca="false">IF('Budget du don'!A9="","",'Budget du don'!A9)</f>
         <v>Sac de riz 25 kg</v>
       </c>
-      <c r="B9" s="30" t="str">
+      <c r="B9" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A9="",'Budget du don'!B9=""),"",'Budget du don'!B9)</f>
         <v>sac</v>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="32" t="n">
         <f aca="false">IF(OR('Budget du don'!A9="",'Budget du don'!C9=""),"",'Budget du don'!C9)</f>
         <v>10</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="33" t="n">
         <f aca="false">IF('Budget du don'!A9="","",IF('Budget du don'!D9&lt;&gt;"",'Budget du don'!D9,IF('Budget du don'!E9&lt;&gt;"",'Budget du don'!E9/'Budget du don'!$G$4,"")))</f>
         <v>18.2938820684892</v>
       </c>
-      <c r="E9" s="32" t="n">
+      <c r="E9" s="18" t="n">
+        <f aca="false">IF(D9="","",D9*'Budget du don'!$G$4)</f>
+        <v>12000</v>
+      </c>
+      <c r="F9" s="33" t="n">
         <f aca="false">IF('Budget du don'!F9="","",'Budget du don'!F9)</f>
         <v>182.938820684892</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="G9" s="18" t="n">
+        <f aca="false">IF(F9="","",F9*'Budget du don'!$G$4)</f>
+        <v>120000</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16" t="n">
+      <c r="I9" s="15"/>
+      <c r="J9" s="16" t="n">
         <v>12800</v>
       </c>
-      <c r="I9" s="17" t="n">
-        <f aca="false">IF(OR(F9="",AND(G9="",H9="")),"",F9*IF(G9&lt;&gt;"",G9,H9/'Budget du don'!$G$4))</f>
+      <c r="K9" s="17" t="n">
+        <f aca="false">IF(OR(H9="",AND(I9="",J9="")),"",H9*IF(I9&lt;&gt;"",I9,J9/'Budget du don'!$G$4))</f>
         <v>195.134742063885</v>
       </c>
-      <c r="J9" s="32" t="n">
-        <f aca="false">IF(OR(E9="",I9=""),"",E9-I9)</f>
+      <c r="L9" s="18" t="n">
+        <f aca="false">IF(K9="","",K9*'Budget du don'!$G$4)</f>
+        <v>128000</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <f aca="false">IF(OR(F9="",K9=""),"",F9-K9)</f>
         <v>-12.1959213789929</v>
       </c>
-      <c r="K9" s="33" t="n">
-        <f aca="false">IF(OR(D9="",D9=0,F9="",AND(G9="",H9="")),"",(IF(G9&lt;&gt;"",G9,H9/'Budget du don'!$G$4)-D9)/D9)</f>
+      <c r="N9" s="18" t="n">
+        <f aca="false">IF(M9="","",M9*'Budget du don'!$G$4)</f>
+        <v>-8000.00000000002</v>
+      </c>
+      <c r="O9" s="34" t="n">
+        <f aca="false">IF(OR(D9="",D9=0,H9="",AND(I9="",J9="")),"",(IF(I9&lt;&gt;"",I9,J9/'Budget du don'!$G$4)-D9)/D9)</f>
         <v>0.0666666666666667</v>
       </c>
-      <c r="L9" s="4" t="s">
-        <v>52</v>
+      <c r="P9" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="str">
+      <c r="A10" s="30" t="str">
         <f aca="false">IF('Budget du don'!A10="","",'Budget du don'!A10)</f>
         <v>Cahier 96 pages</v>
       </c>
-      <c r="B10" s="30" t="str">
+      <c r="B10" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A10="",'Budget du don'!B10=""),"",'Budget du don'!B10)</f>
         <v>pièce</v>
       </c>
-      <c r="C10" s="31" t="str">
+      <c r="C10" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A10="",'Budget du don'!C10=""),"",'Budget du don'!C10)</f>
         <v/>
       </c>
-      <c r="D10" s="32" t="str">
+      <c r="D10" s="33" t="str">
         <f aca="false">IF('Budget du don'!A10="","",IF('Budget du don'!D10&lt;&gt;"",'Budget du don'!D10,IF('Budget du don'!E10&lt;&gt;"",'Budget du don'!E10/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E10" s="32" t="str">
+      <c r="E10" s="18" t="str">
+        <f aca="false">IF(D10="","",D10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F10" s="33" t="str">
         <f aca="false">IF('Budget du don'!F10="","",'Budget du don'!F10)</f>
         <v/>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="17" t="str">
-        <f aca="false">IF(OR(F10="",AND(G10="",H10="")),"",F10*IF(G10&lt;&gt;"",G10,H10/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J10" s="32" t="str">
-        <f aca="false">IF(OR(E10="",I10=""),"",E10-I10)</f>
-        <v/>
-      </c>
-      <c r="K10" s="33" t="str">
-        <f aca="false">IF(OR(D10="",D10=0,F10="",AND(G10="",H10="")),"",(IF(G10&lt;&gt;"",G10,H10/'Budget du don'!$G$4)-D10)/D10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="4"/>
+      <c r="G10" s="18" t="str">
+        <f aca="false">IF(F10="","",F10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="17" t="str">
+        <f aca="false">IF(OR(H10="",AND(I10="",J10="")),"",H10*IF(I10&lt;&gt;"",I10,J10/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L10" s="18" t="str">
+        <f aca="false">IF(K10="","",K10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M10" s="33" t="str">
+        <f aca="false">IF(OR(F10="",K10=""),"",F10-K10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="18" t="str">
+        <f aca="false">IF(M10="","",M10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O10" s="34" t="str">
+        <f aca="false">IF(OR(D10="",D10=0,H10="",AND(I10="",J10="")),"",(IF(I10&lt;&gt;"",I10,J10/'Budget du don'!$G$4)-D10)/D10)</f>
+        <v/>
+      </c>
+      <c r="P10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="str">
+      <c r="A11" s="30" t="str">
         <f aca="false">IF('Budget du don'!A11="","",'Budget du don'!A11)</f>
         <v>Stylo bleu</v>
       </c>
-      <c r="B11" s="30" t="str">
+      <c r="B11" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A11="",'Budget du don'!B11=""),"",'Budget du don'!B11)</f>
         <v>pièce</v>
       </c>
-      <c r="C11" s="31" t="str">
+      <c r="C11" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A11="",'Budget du don'!C11=""),"",'Budget du don'!C11)</f>
         <v/>
       </c>
-      <c r="D11" s="32" t="str">
+      <c r="D11" s="33" t="str">
         <f aca="false">IF('Budget du don'!A11="","",IF('Budget du don'!D11&lt;&gt;"",'Budget du don'!D11,IF('Budget du don'!E11&lt;&gt;"",'Budget du don'!E11/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E11" s="32" t="str">
+      <c r="E11" s="18" t="str">
+        <f aca="false">IF(D11="","",D11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F11" s="33" t="str">
         <f aca="false">IF('Budget du don'!F11="","",'Budget du don'!F11)</f>
         <v/>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="17" t="str">
-        <f aca="false">IF(OR(F11="",AND(G11="",H11="")),"",F11*IF(G11&lt;&gt;"",G11,H11/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J11" s="32" t="str">
-        <f aca="false">IF(OR(E11="",I11=""),"",E11-I11)</f>
-        <v/>
-      </c>
-      <c r="K11" s="33" t="str">
-        <f aca="false">IF(OR(D11="",D11=0,F11="",AND(G11="",H11="")),"",(IF(G11&lt;&gt;"",G11,H11/'Budget du don'!$G$4)-D11)/D11)</f>
-        <v/>
-      </c>
-      <c r="L11" s="4"/>
+      <c r="G11" s="18" t="str">
+        <f aca="false">IF(F11="","",F11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H11" s="14"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="17" t="str">
+        <f aca="false">IF(OR(H11="",AND(I11="",J11="")),"",H11*IF(I11&lt;&gt;"",I11,J11/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L11" s="18" t="str">
+        <f aca="false">IF(K11="","",K11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M11" s="33" t="str">
+        <f aca="false">IF(OR(F11="",K11=""),"",F11-K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="18" t="str">
+        <f aca="false">IF(M11="","",M11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O11" s="34" t="str">
+        <f aca="false">IF(OR(D11="",D11=0,H11="",AND(I11="",J11="")),"",(IF(I11&lt;&gt;"",I11,J11/'Budget du don'!$G$4)-D11)/D11)</f>
+        <v/>
+      </c>
+      <c r="P11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="str">
+      <c r="A12" s="30" t="str">
         <f aca="false">IF('Budget du don'!A12="","",'Budget du don'!A12)</f>
         <v>Cartable</v>
       </c>
-      <c r="B12" s="30" t="str">
+      <c r="B12" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A12="",'Budget du don'!B12=""),"",'Budget du don'!B12)</f>
         <v>pièce</v>
       </c>
-      <c r="C12" s="31" t="str">
+      <c r="C12" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A12="",'Budget du don'!C12=""),"",'Budget du don'!C12)</f>
         <v/>
       </c>
-      <c r="D12" s="32" t="str">
+      <c r="D12" s="33" t="str">
         <f aca="false">IF('Budget du don'!A12="","",IF('Budget du don'!D12&lt;&gt;"",'Budget du don'!D12,IF('Budget du don'!E12&lt;&gt;"",'Budget du don'!E12/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E12" s="32" t="str">
+      <c r="E12" s="18" t="str">
+        <f aca="false">IF(D12="","",D12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F12" s="33" t="str">
         <f aca="false">IF('Budget du don'!F12="","",'Budget du don'!F12)</f>
         <v/>
       </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="17" t="str">
-        <f aca="false">IF(OR(F12="",AND(G12="",H12="")),"",F12*IF(G12&lt;&gt;"",G12,H12/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J12" s="32" t="str">
-        <f aca="false">IF(OR(E12="",I12=""),"",E12-I12)</f>
-        <v/>
-      </c>
-      <c r="K12" s="33" t="str">
-        <f aca="false">IF(OR(D12="",D12=0,F12="",AND(G12="",H12="")),"",(IF(G12&lt;&gt;"",G12,H12/'Budget du don'!$G$4)-D12)/D12)</f>
-        <v/>
-      </c>
-      <c r="L12" s="4"/>
+      <c r="G12" s="18" t="str">
+        <f aca="false">IF(F12="","",F12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="17" t="str">
+        <f aca="false">IF(OR(H12="",AND(I12="",J12="")),"",H12*IF(I12&lt;&gt;"",I12,J12/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L12" s="18" t="str">
+        <f aca="false">IF(K12="","",K12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M12" s="33" t="str">
+        <f aca="false">IF(OR(F12="",K12=""),"",F12-K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="18" t="str">
+        <f aca="false">IF(M12="","",M12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O12" s="34" t="str">
+        <f aca="false">IF(OR(D12="",D12=0,H12="",AND(I12="",J12="")),"",(IF(I12&lt;&gt;"",I12,J12/'Budget du don'!$G$4)-D12)/D12)</f>
+        <v/>
+      </c>
+      <c r="P12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="str">
+      <c r="A13" s="30" t="str">
         <f aca="false">IF('Budget du don'!A13="","",'Budget du don'!A13)</f>
         <v>Craie blanche</v>
       </c>
-      <c r="B13" s="30" t="str">
+      <c r="B13" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A13="",'Budget du don'!B13=""),"",'Budget du don'!B13)</f>
         <v>boîte de 100</v>
       </c>
-      <c r="C13" s="31" t="str">
+      <c r="C13" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A13="",'Budget du don'!C13=""),"",'Budget du don'!C13)</f>
         <v/>
       </c>
-      <c r="D13" s="32" t="str">
+      <c r="D13" s="33" t="str">
         <f aca="false">IF('Budget du don'!A13="","",IF('Budget du don'!D13&lt;&gt;"",'Budget du don'!D13,IF('Budget du don'!E13&lt;&gt;"",'Budget du don'!E13/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E13" s="32" t="str">
+      <c r="E13" s="18" t="str">
+        <f aca="false">IF(D13="","",D13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F13" s="33" t="str">
         <f aca="false">IF('Budget du don'!F13="","",'Budget du don'!F13)</f>
         <v/>
       </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="17" t="str">
-        <f aca="false">IF(OR(F13="",AND(G13="",H13="")),"",F13*IF(G13&lt;&gt;"",G13,H13/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J13" s="32" t="str">
-        <f aca="false">IF(OR(E13="",I13=""),"",E13-I13)</f>
-        <v/>
-      </c>
-      <c r="K13" s="33" t="str">
-        <f aca="false">IF(OR(D13="",D13=0,F13="",AND(G13="",H13="")),"",(IF(G13&lt;&gt;"",G13,H13/'Budget du don'!$G$4)-D13)/D13)</f>
-        <v/>
-      </c>
-      <c r="L13" s="4"/>
+      <c r="G13" s="18" t="str">
+        <f aca="false">IF(F13="","",F13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H13" s="14"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="17" t="str">
+        <f aca="false">IF(OR(H13="",AND(I13="",J13="")),"",H13*IF(I13&lt;&gt;"",I13,J13/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L13" s="18" t="str">
+        <f aca="false">IF(K13="","",K13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M13" s="33" t="str">
+        <f aca="false">IF(OR(F13="",K13=""),"",F13-K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="18" t="str">
+        <f aca="false">IF(M13="","",M13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O13" s="34" t="str">
+        <f aca="false">IF(OR(D13="",D13=0,H13="",AND(I13="",J13="")),"",(IF(I13&lt;&gt;"",I13,J13/'Budget du don'!$G$4)-D13)/D13)</f>
+        <v/>
+      </c>
+      <c r="P13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="str">
+      <c r="A14" s="30" t="str">
         <f aca="false">IF('Budget du don'!A14="","",'Budget du don'!A14)</f>
         <v>Huile végétale</v>
       </c>
-      <c r="B14" s="30" t="str">
+      <c r="B14" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A14="",'Budget du don'!B14=""),"",'Budget du don'!B14)</f>
         <v>bidon 1 L</v>
       </c>
-      <c r="C14" s="31" t="str">
+      <c r="C14" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A14="",'Budget du don'!C14=""),"",'Budget du don'!C14)</f>
         <v/>
       </c>
-      <c r="D14" s="32" t="str">
+      <c r="D14" s="33" t="str">
         <f aca="false">IF('Budget du don'!A14="","",IF('Budget du don'!D14&lt;&gt;"",'Budget du don'!D14,IF('Budget du don'!E14&lt;&gt;"",'Budget du don'!E14/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E14" s="32" t="str">
+      <c r="E14" s="18" t="str">
+        <f aca="false">IF(D14="","",D14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F14" s="33" t="str">
         <f aca="false">IF('Budget du don'!F14="","",'Budget du don'!F14)</f>
         <v/>
       </c>
-      <c r="F14" s="14"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="17" t="str">
-        <f aca="false">IF(OR(F14="",AND(G14="",H14="")),"",F14*IF(G14&lt;&gt;"",G14,H14/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J14" s="32" t="str">
-        <f aca="false">IF(OR(E14="",I14=""),"",E14-I14)</f>
-        <v/>
-      </c>
-      <c r="K14" s="33" t="str">
-        <f aca="false">IF(OR(D14="",D14=0,F14="",AND(G14="",H14="")),"",(IF(G14&lt;&gt;"",G14,H14/'Budget du don'!$G$4)-D14)/D14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="4"/>
+      <c r="G14" s="18" t="str">
+        <f aca="false">IF(F14="","",F14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H14" s="14"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="17" t="str">
+        <f aca="false">IF(OR(H14="",AND(I14="",J14="")),"",H14*IF(I14&lt;&gt;"",I14,J14/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L14" s="18" t="str">
+        <f aca="false">IF(K14="","",K14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M14" s="33" t="str">
+        <f aca="false">IF(OR(F14="",K14=""),"",F14-K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="18" t="str">
+        <f aca="false">IF(M14="","",M14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O14" s="34" t="str">
+        <f aca="false">IF(OR(D14="",D14=0,H14="",AND(I14="",J14="")),"",(IF(I14&lt;&gt;"",I14,J14/'Budget du don'!$G$4)-D14)/D14)</f>
+        <v/>
+      </c>
+      <c r="P14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="str">
+      <c r="A15" s="30" t="str">
         <f aca="false">IF('Budget du don'!A15="","",'Budget du don'!A15)</f>
         <v>Savon</v>
       </c>
-      <c r="B15" s="30" t="str">
+      <c r="B15" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A15="",'Budget du don'!B15=""),"",'Budget du don'!B15)</f>
         <v>pièce</v>
       </c>
-      <c r="C15" s="31" t="str">
+      <c r="C15" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A15="",'Budget du don'!C15=""),"",'Budget du don'!C15)</f>
         <v/>
       </c>
-      <c r="D15" s="32" t="str">
+      <c r="D15" s="33" t="str">
         <f aca="false">IF('Budget du don'!A15="","",IF('Budget du don'!D15&lt;&gt;"",'Budget du don'!D15,IF('Budget du don'!E15&lt;&gt;"",'Budget du don'!E15/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E15" s="32" t="str">
+      <c r="E15" s="18" t="str">
+        <f aca="false">IF(D15="","",D15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F15" s="33" t="str">
         <f aca="false">IF('Budget du don'!F15="","",'Budget du don'!F15)</f>
         <v/>
       </c>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="17" t="str">
-        <f aca="false">IF(OR(F15="",AND(G15="",H15="")),"",F15*IF(G15&lt;&gt;"",G15,H15/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J15" s="32" t="str">
-        <f aca="false">IF(OR(E15="",I15=""),"",E15-I15)</f>
-        <v/>
-      </c>
-      <c r="K15" s="33" t="str">
-        <f aca="false">IF(OR(D15="",D15=0,F15="",AND(G15="",H15="")),"",(IF(G15&lt;&gt;"",G15,H15/'Budget du don'!$G$4)-D15)/D15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="4"/>
+      <c r="G15" s="18" t="str">
+        <f aca="false">IF(F15="","",F15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H15" s="14"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="17" t="str">
+        <f aca="false">IF(OR(H15="",AND(I15="",J15="")),"",H15*IF(I15&lt;&gt;"",I15,J15/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L15" s="18" t="str">
+        <f aca="false">IF(K15="","",K15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M15" s="33" t="str">
+        <f aca="false">IF(OR(F15="",K15=""),"",F15-K15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="18" t="str">
+        <f aca="false">IF(M15="","",M15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O15" s="34" t="str">
+        <f aca="false">IF(OR(D15="",D15=0,H15="",AND(I15="",J15="")),"",(IF(I15&lt;&gt;"",I15,J15/'Budget du don'!$G$4)-D15)/D15)</f>
+        <v/>
+      </c>
+      <c r="P15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="str">
+      <c r="A16" s="30" t="str">
         <f aca="false">IF('Budget du don'!A16="","",'Budget du don'!A16)</f>
         <v>Vêtements enfant</v>
       </c>
-      <c r="B16" s="30" t="str">
+      <c r="B16" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A16="",'Budget du don'!B16=""),"",'Budget du don'!B16)</f>
         <v>lot</v>
       </c>
-      <c r="C16" s="31" t="str">
+      <c r="C16" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A16="",'Budget du don'!C16=""),"",'Budget du don'!C16)</f>
         <v/>
       </c>
-      <c r="D16" s="32" t="str">
+      <c r="D16" s="33" t="str">
         <f aca="false">IF('Budget du don'!A16="","",IF('Budget du don'!D16&lt;&gt;"",'Budget du don'!D16,IF('Budget du don'!E16&lt;&gt;"",'Budget du don'!E16/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E16" s="32" t="str">
+      <c r="E16" s="18" t="str">
+        <f aca="false">IF(D16="","",D16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F16" s="33" t="str">
         <f aca="false">IF('Budget du don'!F16="","",'Budget du don'!F16)</f>
         <v/>
       </c>
-      <c r="F16" s="14"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="17" t="str">
-        <f aca="false">IF(OR(F16="",AND(G16="",H16="")),"",F16*IF(G16&lt;&gt;"",G16,H16/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J16" s="32" t="str">
-        <f aca="false">IF(OR(E16="",I16=""),"",E16-I16)</f>
-        <v/>
-      </c>
-      <c r="K16" s="33" t="str">
-        <f aca="false">IF(OR(D16="",D16=0,F16="",AND(G16="",H16="")),"",(IF(G16&lt;&gt;"",G16,H16/'Budget du don'!$G$4)-D16)/D16)</f>
-        <v/>
-      </c>
-      <c r="L16" s="4"/>
+      <c r="G16" s="18" t="str">
+        <f aca="false">IF(F16="","",F16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H16" s="14"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="17" t="str">
+        <f aca="false">IF(OR(H16="",AND(I16="",J16="")),"",H16*IF(I16&lt;&gt;"",I16,J16/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L16" s="18" t="str">
+        <f aca="false">IF(K16="","",K16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M16" s="33" t="str">
+        <f aca="false">IF(OR(F16="",K16=""),"",F16-K16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="18" t="str">
+        <f aca="false">IF(M16="","",M16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O16" s="34" t="str">
+        <f aca="false">IF(OR(D16="",D16=0,H16="",AND(I16="",J16="")),"",(IF(I16&lt;&gt;"",I16,J16/'Budget du don'!$G$4)-D16)/D16)</f>
+        <v/>
+      </c>
+      <c r="P16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="str">
+      <c r="A17" s="30" t="str">
         <f aca="false">IF('Budget du don'!A17="","",'Budget du don'!A17)</f>
         <v/>
       </c>
-      <c r="B17" s="30" t="str">
+      <c r="B17" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A17="",'Budget du don'!B17=""),"",'Budget du don'!B17)</f>
         <v/>
       </c>
-      <c r="C17" s="31" t="str">
+      <c r="C17" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A17="",'Budget du don'!C17=""),"",'Budget du don'!C17)</f>
         <v/>
       </c>
-      <c r="D17" s="32" t="str">
+      <c r="D17" s="33" t="str">
         <f aca="false">IF('Budget du don'!A17="","",IF('Budget du don'!D17&lt;&gt;"",'Budget du don'!D17,IF('Budget du don'!E17&lt;&gt;"",'Budget du don'!E17/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E17" s="32" t="str">
+      <c r="E17" s="18" t="str">
+        <f aca="false">IF(D17="","",D17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F17" s="33" t="str">
         <f aca="false">IF('Budget du don'!F17="","",'Budget du don'!F17)</f>
         <v/>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="17" t="str">
-        <f aca="false">IF(OR(F17="",AND(G17="",H17="")),"",F17*IF(G17&lt;&gt;"",G17,H17/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J17" s="32" t="str">
-        <f aca="false">IF(OR(E17="",I17=""),"",E17-I17)</f>
-        <v/>
-      </c>
-      <c r="K17" s="33" t="str">
-        <f aca="false">IF(OR(D17="",D17=0,F17="",AND(G17="",H17="")),"",(IF(G17&lt;&gt;"",G17,H17/'Budget du don'!$G$4)-D17)/D17)</f>
-        <v/>
-      </c>
-      <c r="L17" s="4"/>
+      <c r="G17" s="18" t="str">
+        <f aca="false">IF(F17="","",F17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H17" s="14"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="17" t="str">
+        <f aca="false">IF(OR(H17="",AND(I17="",J17="")),"",H17*IF(I17&lt;&gt;"",I17,J17/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L17" s="18" t="str">
+        <f aca="false">IF(K17="","",K17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M17" s="33" t="str">
+        <f aca="false">IF(OR(F17="",K17=""),"",F17-K17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="18" t="str">
+        <f aca="false">IF(M17="","",M17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O17" s="34" t="str">
+        <f aca="false">IF(OR(D17="",D17=0,H17="",AND(I17="",J17="")),"",(IF(I17&lt;&gt;"",I17,J17/'Budget du don'!$G$4)-D17)/D17)</f>
+        <v/>
+      </c>
+      <c r="P17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="str">
+      <c r="A18" s="30" t="str">
         <f aca="false">IF('Budget du don'!A18="","",'Budget du don'!A18)</f>
         <v/>
       </c>
-      <c r="B18" s="30" t="str">
+      <c r="B18" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A18="",'Budget du don'!B18=""),"",'Budget du don'!B18)</f>
         <v/>
       </c>
-      <c r="C18" s="31" t="str">
+      <c r="C18" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A18="",'Budget du don'!C18=""),"",'Budget du don'!C18)</f>
         <v/>
       </c>
-      <c r="D18" s="32" t="str">
+      <c r="D18" s="33" t="str">
         <f aca="false">IF('Budget du don'!A18="","",IF('Budget du don'!D18&lt;&gt;"",'Budget du don'!D18,IF('Budget du don'!E18&lt;&gt;"",'Budget du don'!E18/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E18" s="32" t="str">
+      <c r="E18" s="18" t="str">
+        <f aca="false">IF(D18="","",D18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F18" s="33" t="str">
         <f aca="false">IF('Budget du don'!F18="","",'Budget du don'!F18)</f>
         <v/>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="17" t="str">
-        <f aca="false">IF(OR(F18="",AND(G18="",H18="")),"",F18*IF(G18&lt;&gt;"",G18,H18/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J18" s="32" t="str">
-        <f aca="false">IF(OR(E18="",I18=""),"",E18-I18)</f>
-        <v/>
-      </c>
-      <c r="K18" s="33" t="str">
-        <f aca="false">IF(OR(D18="",D18=0,F18="",AND(G18="",H18="")),"",(IF(G18&lt;&gt;"",G18,H18/'Budget du don'!$G$4)-D18)/D18)</f>
-        <v/>
-      </c>
-      <c r="L18" s="4"/>
+      <c r="G18" s="18" t="str">
+        <f aca="false">IF(F18="","",F18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="17" t="str">
+        <f aca="false">IF(OR(H18="",AND(I18="",J18="")),"",H18*IF(I18&lt;&gt;"",I18,J18/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L18" s="18" t="str">
+        <f aca="false">IF(K18="","",K18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M18" s="33" t="str">
+        <f aca="false">IF(OR(F18="",K18=""),"",F18-K18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="18" t="str">
+        <f aca="false">IF(M18="","",M18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O18" s="34" t="str">
+        <f aca="false">IF(OR(D18="",D18=0,H18="",AND(I18="",J18="")),"",(IF(I18&lt;&gt;"",I18,J18/'Budget du don'!$G$4)-D18)/D18)</f>
+        <v/>
+      </c>
+      <c r="P18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="str">
+      <c r="A19" s="30" t="str">
         <f aca="false">IF('Budget du don'!A19="","",'Budget du don'!A19)</f>
         <v/>
       </c>
-      <c r="B19" s="30" t="str">
+      <c r="B19" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A19="",'Budget du don'!B19=""),"",'Budget du don'!B19)</f>
         <v/>
       </c>
-      <c r="C19" s="31" t="str">
+      <c r="C19" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A19="",'Budget du don'!C19=""),"",'Budget du don'!C19)</f>
         <v/>
       </c>
-      <c r="D19" s="32" t="str">
+      <c r="D19" s="33" t="str">
         <f aca="false">IF('Budget du don'!A19="","",IF('Budget du don'!D19&lt;&gt;"",'Budget du don'!D19,IF('Budget du don'!E19&lt;&gt;"",'Budget du don'!E19/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E19" s="32" t="str">
+      <c r="E19" s="18" t="str">
+        <f aca="false">IF(D19="","",D19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F19" s="33" t="str">
         <f aca="false">IF('Budget du don'!F19="","",'Budget du don'!F19)</f>
         <v/>
       </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="17" t="str">
-        <f aca="false">IF(OR(F19="",AND(G19="",H19="")),"",F19*IF(G19&lt;&gt;"",G19,H19/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J19" s="32" t="str">
-        <f aca="false">IF(OR(E19="",I19=""),"",E19-I19)</f>
-        <v/>
-      </c>
-      <c r="K19" s="33" t="str">
-        <f aca="false">IF(OR(D19="",D19=0,F19="",AND(G19="",H19="")),"",(IF(G19&lt;&gt;"",G19,H19/'Budget du don'!$G$4)-D19)/D19)</f>
-        <v/>
-      </c>
-      <c r="L19" s="4"/>
+      <c r="G19" s="18" t="str">
+        <f aca="false">IF(F19="","",F19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="17" t="str">
+        <f aca="false">IF(OR(H19="",AND(I19="",J19="")),"",H19*IF(I19&lt;&gt;"",I19,J19/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L19" s="18" t="str">
+        <f aca="false">IF(K19="","",K19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M19" s="33" t="str">
+        <f aca="false">IF(OR(F19="",K19=""),"",F19-K19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="18" t="str">
+        <f aca="false">IF(M19="","",M19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O19" s="34" t="str">
+        <f aca="false">IF(OR(D19="",D19=0,H19="",AND(I19="",J19="")),"",(IF(I19&lt;&gt;"",I19,J19/'Budget du don'!$G$4)-D19)/D19)</f>
+        <v/>
+      </c>
+      <c r="P19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="str">
+      <c r="A20" s="30" t="str">
         <f aca="false">IF('Budget du don'!A20="","",'Budget du don'!A20)</f>
         <v/>
       </c>
-      <c r="B20" s="30" t="str">
+      <c r="B20" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A20="",'Budget du don'!B20=""),"",'Budget du don'!B20)</f>
         <v/>
       </c>
-      <c r="C20" s="31" t="str">
+      <c r="C20" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A20="",'Budget du don'!C20=""),"",'Budget du don'!C20)</f>
         <v/>
       </c>
-      <c r="D20" s="32" t="str">
+      <c r="D20" s="33" t="str">
         <f aca="false">IF('Budget du don'!A20="","",IF('Budget du don'!D20&lt;&gt;"",'Budget du don'!D20,IF('Budget du don'!E20&lt;&gt;"",'Budget du don'!E20/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E20" s="32" t="str">
+      <c r="E20" s="18" t="str">
+        <f aca="false">IF(D20="","",D20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F20" s="33" t="str">
         <f aca="false">IF('Budget du don'!F20="","",'Budget du don'!F20)</f>
         <v/>
       </c>
-      <c r="F20" s="14"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="17" t="str">
-        <f aca="false">IF(OR(F20="",AND(G20="",H20="")),"",F20*IF(G20&lt;&gt;"",G20,H20/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J20" s="32" t="str">
-        <f aca="false">IF(OR(E20="",I20=""),"",E20-I20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="33" t="str">
-        <f aca="false">IF(OR(D20="",D20=0,F20="",AND(G20="",H20="")),"",(IF(G20&lt;&gt;"",G20,H20/'Budget du don'!$G$4)-D20)/D20)</f>
-        <v/>
-      </c>
-      <c r="L20" s="4"/>
+      <c r="G20" s="18" t="str">
+        <f aca="false">IF(F20="","",F20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H20" s="14"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="17" t="str">
+        <f aca="false">IF(OR(H20="",AND(I20="",J20="")),"",H20*IF(I20&lt;&gt;"",I20,J20/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L20" s="18" t="str">
+        <f aca="false">IF(K20="","",K20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M20" s="33" t="str">
+        <f aca="false">IF(OR(F20="",K20=""),"",F20-K20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="18" t="str">
+        <f aca="false">IF(M20="","",M20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O20" s="34" t="str">
+        <f aca="false">IF(OR(D20="",D20=0,H20="",AND(I20="",J20="")),"",(IF(I20&lt;&gt;"",I20,J20/'Budget du don'!$G$4)-D20)/D20)</f>
+        <v/>
+      </c>
+      <c r="P20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="str">
+      <c r="A21" s="30" t="str">
         <f aca="false">IF('Budget du don'!A21="","",'Budget du don'!A21)</f>
         <v/>
       </c>
-      <c r="B21" s="30" t="str">
+      <c r="B21" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A21="",'Budget du don'!B21=""),"",'Budget du don'!B21)</f>
         <v/>
       </c>
-      <c r="C21" s="31" t="str">
+      <c r="C21" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A21="",'Budget du don'!C21=""),"",'Budget du don'!C21)</f>
         <v/>
       </c>
-      <c r="D21" s="32" t="str">
+      <c r="D21" s="33" t="str">
         <f aca="false">IF('Budget du don'!A21="","",IF('Budget du don'!D21&lt;&gt;"",'Budget du don'!D21,IF('Budget du don'!E21&lt;&gt;"",'Budget du don'!E21/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E21" s="32" t="str">
+      <c r="E21" s="18" t="str">
+        <f aca="false">IF(D21="","",D21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F21" s="33" t="str">
         <f aca="false">IF('Budget du don'!F21="","",'Budget du don'!F21)</f>
         <v/>
       </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="17" t="str">
-        <f aca="false">IF(OR(F21="",AND(G21="",H21="")),"",F21*IF(G21&lt;&gt;"",G21,H21/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J21" s="32" t="str">
-        <f aca="false">IF(OR(E21="",I21=""),"",E21-I21)</f>
-        <v/>
-      </c>
-      <c r="K21" s="33" t="str">
-        <f aca="false">IF(OR(D21="",D21=0,F21="",AND(G21="",H21="")),"",(IF(G21&lt;&gt;"",G21,H21/'Budget du don'!$G$4)-D21)/D21)</f>
-        <v/>
-      </c>
-      <c r="L21" s="4"/>
+      <c r="G21" s="18" t="str">
+        <f aca="false">IF(F21="","",F21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H21" s="14"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="17" t="str">
+        <f aca="false">IF(OR(H21="",AND(I21="",J21="")),"",H21*IF(I21&lt;&gt;"",I21,J21/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L21" s="18" t="str">
+        <f aca="false">IF(K21="","",K21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M21" s="33" t="str">
+        <f aca="false">IF(OR(F21="",K21=""),"",F21-K21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="18" t="str">
+        <f aca="false">IF(M21="","",M21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O21" s="34" t="str">
+        <f aca="false">IF(OR(D21="",D21=0,H21="",AND(I21="",J21="")),"",(IF(I21&lt;&gt;"",I21,J21/'Budget du don'!$G$4)-D21)/D21)</f>
+        <v/>
+      </c>
+      <c r="P21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="str">
+      <c r="A22" s="30" t="str">
         <f aca="false">IF('Budget du don'!A22="","",'Budget du don'!A22)</f>
         <v/>
       </c>
-      <c r="B22" s="30" t="str">
+      <c r="B22" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A22="",'Budget du don'!B22=""),"",'Budget du don'!B22)</f>
         <v/>
       </c>
-      <c r="C22" s="31" t="str">
+      <c r="C22" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A22="",'Budget du don'!C22=""),"",'Budget du don'!C22)</f>
         <v/>
       </c>
-      <c r="D22" s="32" t="str">
+      <c r="D22" s="33" t="str">
         <f aca="false">IF('Budget du don'!A22="","",IF('Budget du don'!D22&lt;&gt;"",'Budget du don'!D22,IF('Budget du don'!E22&lt;&gt;"",'Budget du don'!E22/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E22" s="32" t="str">
+      <c r="E22" s="18" t="str">
+        <f aca="false">IF(D22="","",D22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F22" s="33" t="str">
         <f aca="false">IF('Budget du don'!F22="","",'Budget du don'!F22)</f>
         <v/>
       </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="17" t="str">
-        <f aca="false">IF(OR(F22="",AND(G22="",H22="")),"",F22*IF(G22&lt;&gt;"",G22,H22/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J22" s="32" t="str">
-        <f aca="false">IF(OR(E22="",I22=""),"",E22-I22)</f>
-        <v/>
-      </c>
-      <c r="K22" s="33" t="str">
-        <f aca="false">IF(OR(D22="",D22=0,F22="",AND(G22="",H22="")),"",(IF(G22&lt;&gt;"",G22,H22/'Budget du don'!$G$4)-D22)/D22)</f>
-        <v/>
-      </c>
-      <c r="L22" s="4"/>
+      <c r="G22" s="18" t="str">
+        <f aca="false">IF(F22="","",F22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H22" s="14"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="17" t="str">
+        <f aca="false">IF(OR(H22="",AND(I22="",J22="")),"",H22*IF(I22&lt;&gt;"",I22,J22/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L22" s="18" t="str">
+        <f aca="false">IF(K22="","",K22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M22" s="33" t="str">
+        <f aca="false">IF(OR(F22="",K22=""),"",F22-K22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="18" t="str">
+        <f aca="false">IF(M22="","",M22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O22" s="34" t="str">
+        <f aca="false">IF(OR(D22="",D22=0,H22="",AND(I22="",J22="")),"",(IF(I22&lt;&gt;"",I22,J22/'Budget du don'!$G$4)-D22)/D22)</f>
+        <v/>
+      </c>
+      <c r="P22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="str">
+      <c r="A23" s="30" t="str">
         <f aca="false">IF('Budget du don'!A23="","",'Budget du don'!A23)</f>
         <v/>
       </c>
-      <c r="B23" s="30" t="str">
+      <c r="B23" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A23="",'Budget du don'!B23=""),"",'Budget du don'!B23)</f>
         <v/>
       </c>
-      <c r="C23" s="31" t="str">
+      <c r="C23" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A23="",'Budget du don'!C23=""),"",'Budget du don'!C23)</f>
         <v/>
       </c>
-      <c r="D23" s="32" t="str">
+      <c r="D23" s="33" t="str">
         <f aca="false">IF('Budget du don'!A23="","",IF('Budget du don'!D23&lt;&gt;"",'Budget du don'!D23,IF('Budget du don'!E23&lt;&gt;"",'Budget du don'!E23/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E23" s="32" t="str">
+      <c r="E23" s="18" t="str">
+        <f aca="false">IF(D23="","",D23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F23" s="33" t="str">
         <f aca="false">IF('Budget du don'!F23="","",'Budget du don'!F23)</f>
         <v/>
       </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="17" t="str">
-        <f aca="false">IF(OR(F23="",AND(G23="",H23="")),"",F23*IF(G23&lt;&gt;"",G23,H23/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J23" s="32" t="str">
-        <f aca="false">IF(OR(E23="",I23=""),"",E23-I23)</f>
-        <v/>
-      </c>
-      <c r="K23" s="33" t="str">
-        <f aca="false">IF(OR(D23="",D23=0,F23="",AND(G23="",H23="")),"",(IF(G23&lt;&gt;"",G23,H23/'Budget du don'!$G$4)-D23)/D23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="4"/>
+      <c r="G23" s="18" t="str">
+        <f aca="false">IF(F23="","",F23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="17" t="str">
+        <f aca="false">IF(OR(H23="",AND(I23="",J23="")),"",H23*IF(I23&lt;&gt;"",I23,J23/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L23" s="18" t="str">
+        <f aca="false">IF(K23="","",K23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M23" s="33" t="str">
+        <f aca="false">IF(OR(F23="",K23=""),"",F23-K23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="18" t="str">
+        <f aca="false">IF(M23="","",M23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O23" s="34" t="str">
+        <f aca="false">IF(OR(D23="",D23=0,H23="",AND(I23="",J23="")),"",(IF(I23&lt;&gt;"",I23,J23/'Budget du don'!$G$4)-D23)/D23)</f>
+        <v/>
+      </c>
+      <c r="P23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="str">
+      <c r="A24" s="30" t="str">
         <f aca="false">IF('Budget du don'!A24="","",'Budget du don'!A24)</f>
         <v/>
       </c>
-      <c r="B24" s="30" t="str">
+      <c r="B24" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A24="",'Budget du don'!B24=""),"",'Budget du don'!B24)</f>
         <v/>
       </c>
-      <c r="C24" s="31" t="str">
+      <c r="C24" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A24="",'Budget du don'!C24=""),"",'Budget du don'!C24)</f>
         <v/>
       </c>
-      <c r="D24" s="32" t="str">
+      <c r="D24" s="33" t="str">
         <f aca="false">IF('Budget du don'!A24="","",IF('Budget du don'!D24&lt;&gt;"",'Budget du don'!D24,IF('Budget du don'!E24&lt;&gt;"",'Budget du don'!E24/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E24" s="32" t="str">
+      <c r="E24" s="18" t="str">
+        <f aca="false">IF(D24="","",D24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F24" s="33" t="str">
         <f aca="false">IF('Budget du don'!F24="","",'Budget du don'!F24)</f>
         <v/>
       </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="17" t="str">
-        <f aca="false">IF(OR(F24="",AND(G24="",H24="")),"",F24*IF(G24&lt;&gt;"",G24,H24/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J24" s="32" t="str">
-        <f aca="false">IF(OR(E24="",I24=""),"",E24-I24)</f>
-        <v/>
-      </c>
-      <c r="K24" s="33" t="str">
-        <f aca="false">IF(OR(D24="",D24=0,F24="",AND(G24="",H24="")),"",(IF(G24&lt;&gt;"",G24,H24/'Budget du don'!$G$4)-D24)/D24)</f>
-        <v/>
-      </c>
-      <c r="L24" s="4"/>
+      <c r="G24" s="18" t="str">
+        <f aca="false">IF(F24="","",F24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="17" t="str">
+        <f aca="false">IF(OR(H24="",AND(I24="",J24="")),"",H24*IF(I24&lt;&gt;"",I24,J24/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L24" s="18" t="str">
+        <f aca="false">IF(K24="","",K24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M24" s="33" t="str">
+        <f aca="false">IF(OR(F24="",K24=""),"",F24-K24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="18" t="str">
+        <f aca="false">IF(M24="","",M24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O24" s="34" t="str">
+        <f aca="false">IF(OR(D24="",D24=0,H24="",AND(I24="",J24="")),"",(IF(I24&lt;&gt;"",I24,J24/'Budget du don'!$G$4)-D24)/D24)</f>
+        <v/>
+      </c>
+      <c r="P24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="str">
+      <c r="A25" s="30" t="str">
         <f aca="false">IF('Budget du don'!A25="","",'Budget du don'!A25)</f>
         <v/>
       </c>
-      <c r="B25" s="30" t="str">
+      <c r="B25" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A25="",'Budget du don'!B25=""),"",'Budget du don'!B25)</f>
         <v/>
       </c>
-      <c r="C25" s="31" t="str">
+      <c r="C25" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A25="",'Budget du don'!C25=""),"",'Budget du don'!C25)</f>
         <v/>
       </c>
-      <c r="D25" s="32" t="str">
+      <c r="D25" s="33" t="str">
         <f aca="false">IF('Budget du don'!A25="","",IF('Budget du don'!D25&lt;&gt;"",'Budget du don'!D25,IF('Budget du don'!E25&lt;&gt;"",'Budget du don'!E25/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E25" s="32" t="str">
+      <c r="E25" s="18" t="str">
+        <f aca="false">IF(D25="","",D25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F25" s="33" t="str">
         <f aca="false">IF('Budget du don'!F25="","",'Budget du don'!F25)</f>
         <v/>
       </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="17" t="str">
-        <f aca="false">IF(OR(F25="",AND(G25="",H25="")),"",F25*IF(G25&lt;&gt;"",G25,H25/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J25" s="32" t="str">
-        <f aca="false">IF(OR(E25="",I25=""),"",E25-I25)</f>
-        <v/>
-      </c>
-      <c r="K25" s="33" t="str">
-        <f aca="false">IF(OR(D25="",D25=0,F25="",AND(G25="",H25="")),"",(IF(G25&lt;&gt;"",G25,H25/'Budget du don'!$G$4)-D25)/D25)</f>
-        <v/>
-      </c>
-      <c r="L25" s="4"/>
+      <c r="G25" s="18" t="str">
+        <f aca="false">IF(F25="","",F25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H25" s="14"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="17" t="str">
+        <f aca="false">IF(OR(H25="",AND(I25="",J25="")),"",H25*IF(I25&lt;&gt;"",I25,J25/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L25" s="18" t="str">
+        <f aca="false">IF(K25="","",K25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M25" s="33" t="str">
+        <f aca="false">IF(OR(F25="",K25=""),"",F25-K25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="18" t="str">
+        <f aca="false">IF(M25="","",M25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O25" s="34" t="str">
+        <f aca="false">IF(OR(D25="",D25=0,H25="",AND(I25="",J25="")),"",(IF(I25&lt;&gt;"",I25,J25/'Budget du don'!$G$4)-D25)/D25)</f>
+        <v/>
+      </c>
+      <c r="P25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="str">
+      <c r="A26" s="30" t="str">
         <f aca="false">IF('Budget du don'!A26="","",'Budget du don'!A26)</f>
         <v/>
       </c>
-      <c r="B26" s="30" t="str">
+      <c r="B26" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A26="",'Budget du don'!B26=""),"",'Budget du don'!B26)</f>
         <v/>
       </c>
-      <c r="C26" s="31" t="str">
+      <c r="C26" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A26="",'Budget du don'!C26=""),"",'Budget du don'!C26)</f>
         <v/>
       </c>
-      <c r="D26" s="32" t="str">
+      <c r="D26" s="33" t="str">
         <f aca="false">IF('Budget du don'!A26="","",IF('Budget du don'!D26&lt;&gt;"",'Budget du don'!D26,IF('Budget du don'!E26&lt;&gt;"",'Budget du don'!E26/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E26" s="32" t="str">
+      <c r="E26" s="18" t="str">
+        <f aca="false">IF(D26="","",D26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F26" s="33" t="str">
         <f aca="false">IF('Budget du don'!F26="","",'Budget du don'!F26)</f>
         <v/>
       </c>
-      <c r="F26" s="14"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="17" t="str">
-        <f aca="false">IF(OR(F26="",AND(G26="",H26="")),"",F26*IF(G26&lt;&gt;"",G26,H26/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J26" s="32" t="str">
-        <f aca="false">IF(OR(E26="",I26=""),"",E26-I26)</f>
-        <v/>
-      </c>
-      <c r="K26" s="33" t="str">
-        <f aca="false">IF(OR(D26="",D26=0,F26="",AND(G26="",H26="")),"",(IF(G26&lt;&gt;"",G26,H26/'Budget du don'!$G$4)-D26)/D26)</f>
-        <v/>
-      </c>
-      <c r="L26" s="4"/>
+      <c r="G26" s="18" t="str">
+        <f aca="false">IF(F26="","",F26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H26" s="14"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="17" t="str">
+        <f aca="false">IF(OR(H26="",AND(I26="",J26="")),"",H26*IF(I26&lt;&gt;"",I26,J26/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L26" s="18" t="str">
+        <f aca="false">IF(K26="","",K26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M26" s="33" t="str">
+        <f aca="false">IF(OR(F26="",K26=""),"",F26-K26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="18" t="str">
+        <f aca="false">IF(M26="","",M26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O26" s="34" t="str">
+        <f aca="false">IF(OR(D26="",D26=0,H26="",AND(I26="",J26="")),"",(IF(I26&lt;&gt;"",I26,J26/'Budget du don'!$G$4)-D26)/D26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="str">
+      <c r="A27" s="30" t="str">
         <f aca="false">IF('Budget du don'!A27="","",'Budget du don'!A27)</f>
         <v/>
       </c>
-      <c r="B27" s="30" t="str">
+      <c r="B27" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A27="",'Budget du don'!B27=""),"",'Budget du don'!B27)</f>
         <v/>
       </c>
-      <c r="C27" s="31" t="str">
+      <c r="C27" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A27="",'Budget du don'!C27=""),"",'Budget du don'!C27)</f>
         <v/>
       </c>
-      <c r="D27" s="32" t="str">
+      <c r="D27" s="33" t="str">
         <f aca="false">IF('Budget du don'!A27="","",IF('Budget du don'!D27&lt;&gt;"",'Budget du don'!D27,IF('Budget du don'!E27&lt;&gt;"",'Budget du don'!E27/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E27" s="32" t="str">
+      <c r="E27" s="18" t="str">
+        <f aca="false">IF(D27="","",D27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F27" s="33" t="str">
         <f aca="false">IF('Budget du don'!F27="","",'Budget du don'!F27)</f>
         <v/>
       </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="17" t="str">
-        <f aca="false">IF(OR(F27="",AND(G27="",H27="")),"",F27*IF(G27&lt;&gt;"",G27,H27/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J27" s="32" t="str">
-        <f aca="false">IF(OR(E27="",I27=""),"",E27-I27)</f>
-        <v/>
-      </c>
-      <c r="K27" s="33" t="str">
-        <f aca="false">IF(OR(D27="",D27=0,F27="",AND(G27="",H27="")),"",(IF(G27&lt;&gt;"",G27,H27/'Budget du don'!$G$4)-D27)/D27)</f>
-        <v/>
-      </c>
-      <c r="L27" s="4"/>
+      <c r="G27" s="18" t="str">
+        <f aca="false">IF(F27="","",F27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H27" s="14"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="17" t="str">
+        <f aca="false">IF(OR(H27="",AND(I27="",J27="")),"",H27*IF(I27&lt;&gt;"",I27,J27/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L27" s="18" t="str">
+        <f aca="false">IF(K27="","",K27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M27" s="33" t="str">
+        <f aca="false">IF(OR(F27="",K27=""),"",F27-K27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="18" t="str">
+        <f aca="false">IF(M27="","",M27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O27" s="34" t="str">
+        <f aca="false">IF(OR(D27="",D27=0,H27="",AND(I27="",J27="")),"",(IF(I27&lt;&gt;"",I27,J27/'Budget du don'!$G$4)-D27)/D27)</f>
+        <v/>
+      </c>
+      <c r="P27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="str">
+      <c r="A28" s="30" t="str">
         <f aca="false">IF('Budget du don'!A28="","",'Budget du don'!A28)</f>
         <v/>
       </c>
-      <c r="B28" s="30" t="str">
+      <c r="B28" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A28="",'Budget du don'!B28=""),"",'Budget du don'!B28)</f>
         <v/>
       </c>
-      <c r="C28" s="31" t="str">
+      <c r="C28" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A28="",'Budget du don'!C28=""),"",'Budget du don'!C28)</f>
         <v/>
       </c>
-      <c r="D28" s="32" t="str">
+      <c r="D28" s="33" t="str">
         <f aca="false">IF('Budget du don'!A28="","",IF('Budget du don'!D28&lt;&gt;"",'Budget du don'!D28,IF('Budget du don'!E28&lt;&gt;"",'Budget du don'!E28/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E28" s="32" t="str">
+      <c r="E28" s="18" t="str">
+        <f aca="false">IF(D28="","",D28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F28" s="33" t="str">
         <f aca="false">IF('Budget du don'!F28="","",'Budget du don'!F28)</f>
         <v/>
       </c>
-      <c r="F28" s="14"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="17" t="str">
-        <f aca="false">IF(OR(F28="",AND(G28="",H28="")),"",F28*IF(G28&lt;&gt;"",G28,H28/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J28" s="32" t="str">
-        <f aca="false">IF(OR(E28="",I28=""),"",E28-I28)</f>
-        <v/>
-      </c>
-      <c r="K28" s="33" t="str">
-        <f aca="false">IF(OR(D28="",D28=0,F28="",AND(G28="",H28="")),"",(IF(G28&lt;&gt;"",G28,H28/'Budget du don'!$G$4)-D28)/D28)</f>
-        <v/>
-      </c>
-      <c r="L28" s="4"/>
+      <c r="G28" s="18" t="str">
+        <f aca="false">IF(F28="","",F28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H28" s="14"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="17" t="str">
+        <f aca="false">IF(OR(H28="",AND(I28="",J28="")),"",H28*IF(I28&lt;&gt;"",I28,J28/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L28" s="18" t="str">
+        <f aca="false">IF(K28="","",K28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M28" s="33" t="str">
+        <f aca="false">IF(OR(F28="",K28=""),"",F28-K28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="18" t="str">
+        <f aca="false">IF(M28="","",M28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O28" s="34" t="str">
+        <f aca="false">IF(OR(D28="",D28=0,H28="",AND(I28="",J28="")),"",(IF(I28&lt;&gt;"",I28,J28/'Budget du don'!$G$4)-D28)/D28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="str">
+      <c r="A29" s="30" t="str">
         <f aca="false">IF('Budget du don'!A29="","",'Budget du don'!A29)</f>
         <v/>
       </c>
-      <c r="B29" s="30" t="str">
+      <c r="B29" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A29="",'Budget du don'!B29=""),"",'Budget du don'!B29)</f>
         <v/>
       </c>
-      <c r="C29" s="31" t="str">
+      <c r="C29" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A29="",'Budget du don'!C29=""),"",'Budget du don'!C29)</f>
         <v/>
       </c>
-      <c r="D29" s="32" t="str">
+      <c r="D29" s="33" t="str">
         <f aca="false">IF('Budget du don'!A29="","",IF('Budget du don'!D29&lt;&gt;"",'Budget du don'!D29,IF('Budget du don'!E29&lt;&gt;"",'Budget du don'!E29/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E29" s="32" t="str">
+      <c r="E29" s="18" t="str">
+        <f aca="false">IF(D29="","",D29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F29" s="33" t="str">
         <f aca="false">IF('Budget du don'!F29="","",'Budget du don'!F29)</f>
         <v/>
       </c>
-      <c r="F29" s="14"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="17" t="str">
-        <f aca="false">IF(OR(F29="",AND(G29="",H29="")),"",F29*IF(G29&lt;&gt;"",G29,H29/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J29" s="32" t="str">
-        <f aca="false">IF(OR(E29="",I29=""),"",E29-I29)</f>
-        <v/>
-      </c>
-      <c r="K29" s="33" t="str">
-        <f aca="false">IF(OR(D29="",D29=0,F29="",AND(G29="",H29="")),"",(IF(G29&lt;&gt;"",G29,H29/'Budget du don'!$G$4)-D29)/D29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="4"/>
+      <c r="G29" s="18" t="str">
+        <f aca="false">IF(F29="","",F29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H29" s="14"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="17" t="str">
+        <f aca="false">IF(OR(H29="",AND(I29="",J29="")),"",H29*IF(I29&lt;&gt;"",I29,J29/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L29" s="18" t="str">
+        <f aca="false">IF(K29="","",K29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M29" s="33" t="str">
+        <f aca="false">IF(OR(F29="",K29=""),"",F29-K29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="18" t="str">
+        <f aca="false">IF(M29="","",M29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O29" s="34" t="str">
+        <f aca="false">IF(OR(D29="",D29=0,H29="",AND(I29="",J29="")),"",(IF(I29&lt;&gt;"",I29,J29/'Budget du don'!$G$4)-D29)/D29)</f>
+        <v/>
+      </c>
+      <c r="P29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="str">
+      <c r="A30" s="30" t="str">
         <f aca="false">IF('Budget du don'!A30="","",'Budget du don'!A30)</f>
         <v/>
       </c>
-      <c r="B30" s="30" t="str">
+      <c r="B30" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A30="",'Budget du don'!B30=""),"",'Budget du don'!B30)</f>
         <v/>
       </c>
-      <c r="C30" s="31" t="str">
+      <c r="C30" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A30="",'Budget du don'!C30=""),"",'Budget du don'!C30)</f>
         <v/>
       </c>
-      <c r="D30" s="32" t="str">
+      <c r="D30" s="33" t="str">
         <f aca="false">IF('Budget du don'!A30="","",IF('Budget du don'!D30&lt;&gt;"",'Budget du don'!D30,IF('Budget du don'!E30&lt;&gt;"",'Budget du don'!E30/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E30" s="32" t="str">
+      <c r="E30" s="18" t="str">
+        <f aca="false">IF(D30="","",D30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F30" s="33" t="str">
         <f aca="false">IF('Budget du don'!F30="","",'Budget du don'!F30)</f>
         <v/>
       </c>
-      <c r="F30" s="14"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="17" t="str">
-        <f aca="false">IF(OR(F30="",AND(G30="",H30="")),"",F30*IF(G30&lt;&gt;"",G30,H30/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J30" s="32" t="str">
-        <f aca="false">IF(OR(E30="",I30=""),"",E30-I30)</f>
-        <v/>
-      </c>
-      <c r="K30" s="33" t="str">
-        <f aca="false">IF(OR(D30="",D30=0,F30="",AND(G30="",H30="")),"",(IF(G30&lt;&gt;"",G30,H30/'Budget du don'!$G$4)-D30)/D30)</f>
-        <v/>
-      </c>
-      <c r="L30" s="4"/>
+      <c r="G30" s="18" t="str">
+        <f aca="false">IF(F30="","",F30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H30" s="14"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="17" t="str">
+        <f aca="false">IF(OR(H30="",AND(I30="",J30="")),"",H30*IF(I30&lt;&gt;"",I30,J30/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L30" s="18" t="str">
+        <f aca="false">IF(K30="","",K30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M30" s="33" t="str">
+        <f aca="false">IF(OR(F30="",K30=""),"",F30-K30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="18" t="str">
+        <f aca="false">IF(M30="","",M30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O30" s="34" t="str">
+        <f aca="false">IF(OR(D30="",D30=0,H30="",AND(I30="",J30="")),"",(IF(I30&lt;&gt;"",I30,J30/'Budget du don'!$G$4)-D30)/D30)</f>
+        <v/>
+      </c>
+      <c r="P30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="str">
+      <c r="A31" s="30" t="str">
         <f aca="false">IF('Budget du don'!A31="","",'Budget du don'!A31)</f>
         <v/>
       </c>
-      <c r="B31" s="30" t="str">
+      <c r="B31" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A31="",'Budget du don'!B31=""),"",'Budget du don'!B31)</f>
         <v/>
       </c>
-      <c r="C31" s="31" t="str">
+      <c r="C31" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A31="",'Budget du don'!C31=""),"",'Budget du don'!C31)</f>
         <v/>
       </c>
-      <c r="D31" s="32" t="str">
+      <c r="D31" s="33" t="str">
         <f aca="false">IF('Budget du don'!A31="","",IF('Budget du don'!D31&lt;&gt;"",'Budget du don'!D31,IF('Budget du don'!E31&lt;&gt;"",'Budget du don'!E31/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E31" s="32" t="str">
+      <c r="E31" s="18" t="str">
+        <f aca="false">IF(D31="","",D31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F31" s="33" t="str">
         <f aca="false">IF('Budget du don'!F31="","",'Budget du don'!F31)</f>
         <v/>
       </c>
-      <c r="F31" s="14"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="17" t="str">
-        <f aca="false">IF(OR(F31="",AND(G31="",H31="")),"",F31*IF(G31&lt;&gt;"",G31,H31/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J31" s="32" t="str">
-        <f aca="false">IF(OR(E31="",I31=""),"",E31-I31)</f>
-        <v/>
-      </c>
-      <c r="K31" s="33" t="str">
-        <f aca="false">IF(OR(D31="",D31=0,F31="",AND(G31="",H31="")),"",(IF(G31&lt;&gt;"",G31,H31/'Budget du don'!$G$4)-D31)/D31)</f>
-        <v/>
-      </c>
-      <c r="L31" s="4"/>
+      <c r="G31" s="18" t="str">
+        <f aca="false">IF(F31="","",F31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H31" s="14"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="17" t="str">
+        <f aca="false">IF(OR(H31="",AND(I31="",J31="")),"",H31*IF(I31&lt;&gt;"",I31,J31/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L31" s="18" t="str">
+        <f aca="false">IF(K31="","",K31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M31" s="33" t="str">
+        <f aca="false">IF(OR(F31="",K31=""),"",F31-K31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="18" t="str">
+        <f aca="false">IF(M31="","",M31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O31" s="34" t="str">
+        <f aca="false">IF(OR(D31="",D31=0,H31="",AND(I31="",J31="")),"",(IF(I31&lt;&gt;"",I31,J31/'Budget du don'!$G$4)-D31)/D31)</f>
+        <v/>
+      </c>
+      <c r="P31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="str">
+      <c r="A32" s="30" t="str">
         <f aca="false">IF('Budget du don'!A32="","",'Budget du don'!A32)</f>
         <v/>
       </c>
-      <c r="B32" s="30" t="str">
+      <c r="B32" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A32="",'Budget du don'!B32=""),"",'Budget du don'!B32)</f>
         <v/>
       </c>
-      <c r="C32" s="31" t="str">
+      <c r="C32" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A32="",'Budget du don'!C32=""),"",'Budget du don'!C32)</f>
         <v/>
       </c>
-      <c r="D32" s="32" t="str">
+      <c r="D32" s="33" t="str">
         <f aca="false">IF('Budget du don'!A32="","",IF('Budget du don'!D32&lt;&gt;"",'Budget du don'!D32,IF('Budget du don'!E32&lt;&gt;"",'Budget du don'!E32/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E32" s="32" t="str">
+      <c r="E32" s="18" t="str">
+        <f aca="false">IF(D32="","",D32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F32" s="33" t="str">
         <f aca="false">IF('Budget du don'!F32="","",'Budget du don'!F32)</f>
         <v/>
       </c>
-      <c r="F32" s="14"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="17" t="str">
-        <f aca="false">IF(OR(F32="",AND(G32="",H32="")),"",F32*IF(G32&lt;&gt;"",G32,H32/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J32" s="32" t="str">
-        <f aca="false">IF(OR(E32="",I32=""),"",E32-I32)</f>
-        <v/>
-      </c>
-      <c r="K32" s="33" t="str">
-        <f aca="false">IF(OR(D32="",D32=0,F32="",AND(G32="",H32="")),"",(IF(G32&lt;&gt;"",G32,H32/'Budget du don'!$G$4)-D32)/D32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="4"/>
+      <c r="G32" s="18" t="str">
+        <f aca="false">IF(F32="","",F32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H32" s="14"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="17" t="str">
+        <f aca="false">IF(OR(H32="",AND(I32="",J32="")),"",H32*IF(I32&lt;&gt;"",I32,J32/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L32" s="18" t="str">
+        <f aca="false">IF(K32="","",K32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M32" s="33" t="str">
+        <f aca="false">IF(OR(F32="",K32=""),"",F32-K32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="18" t="str">
+        <f aca="false">IF(M32="","",M32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O32" s="34" t="str">
+        <f aca="false">IF(OR(D32="",D32=0,H32="",AND(I32="",J32="")),"",(IF(I32&lt;&gt;"",I32,J32/'Budget du don'!$G$4)-D32)/D32)</f>
+        <v/>
+      </c>
+      <c r="P32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29" t="str">
+      <c r="A33" s="30" t="str">
         <f aca="false">IF('Budget du don'!A33="","",'Budget du don'!A33)</f>
         <v/>
       </c>
-      <c r="B33" s="30" t="str">
+      <c r="B33" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A33="",'Budget du don'!B33=""),"",'Budget du don'!B33)</f>
         <v/>
       </c>
-      <c r="C33" s="31" t="str">
+      <c r="C33" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A33="",'Budget du don'!C33=""),"",'Budget du don'!C33)</f>
         <v/>
       </c>
-      <c r="D33" s="32" t="str">
+      <c r="D33" s="33" t="str">
         <f aca="false">IF('Budget du don'!A33="","",IF('Budget du don'!D33&lt;&gt;"",'Budget du don'!D33,IF('Budget du don'!E33&lt;&gt;"",'Budget du don'!E33/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E33" s="32" t="str">
+      <c r="E33" s="18" t="str">
+        <f aca="false">IF(D33="","",D33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F33" s="33" t="str">
         <f aca="false">IF('Budget du don'!F33="","",'Budget du don'!F33)</f>
         <v/>
       </c>
-      <c r="F33" s="14"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="17" t="str">
-        <f aca="false">IF(OR(F33="",AND(G33="",H33="")),"",F33*IF(G33&lt;&gt;"",G33,H33/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J33" s="32" t="str">
-        <f aca="false">IF(OR(E33="",I33=""),"",E33-I33)</f>
-        <v/>
-      </c>
-      <c r="K33" s="33" t="str">
-        <f aca="false">IF(OR(D33="",D33=0,F33="",AND(G33="",H33="")),"",(IF(G33&lt;&gt;"",G33,H33/'Budget du don'!$G$4)-D33)/D33)</f>
-        <v/>
-      </c>
-      <c r="L33" s="4"/>
+      <c r="G33" s="18" t="str">
+        <f aca="false">IF(F33="","",F33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H33" s="14"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="17" t="str">
+        <f aca="false">IF(OR(H33="",AND(I33="",J33="")),"",H33*IF(I33&lt;&gt;"",I33,J33/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L33" s="18" t="str">
+        <f aca="false">IF(K33="","",K33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M33" s="33" t="str">
+        <f aca="false">IF(OR(F33="",K33=""),"",F33-K33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="18" t="str">
+        <f aca="false">IF(M33="","",M33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O33" s="34" t="str">
+        <f aca="false">IF(OR(D33="",D33=0,H33="",AND(I33="",J33="")),"",(IF(I33&lt;&gt;"",I33,J33/'Budget du don'!$G$4)-D33)/D33)</f>
+        <v/>
+      </c>
+      <c r="P33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29" t="str">
+      <c r="A34" s="30" t="str">
         <f aca="false">IF('Budget du don'!A34="","",'Budget du don'!A34)</f>
         <v/>
       </c>
-      <c r="B34" s="30" t="str">
+      <c r="B34" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A34="",'Budget du don'!B34=""),"",'Budget du don'!B34)</f>
         <v/>
       </c>
-      <c r="C34" s="31" t="str">
+      <c r="C34" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A34="",'Budget du don'!C34=""),"",'Budget du don'!C34)</f>
         <v/>
       </c>
-      <c r="D34" s="32" t="str">
+      <c r="D34" s="33" t="str">
         <f aca="false">IF('Budget du don'!A34="","",IF('Budget du don'!D34&lt;&gt;"",'Budget du don'!D34,IF('Budget du don'!E34&lt;&gt;"",'Budget du don'!E34/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E34" s="32" t="str">
+      <c r="E34" s="18" t="str">
+        <f aca="false">IF(D34="","",D34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F34" s="33" t="str">
         <f aca="false">IF('Budget du don'!F34="","",'Budget du don'!F34)</f>
         <v/>
       </c>
-      <c r="F34" s="14"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="17" t="str">
-        <f aca="false">IF(OR(F34="",AND(G34="",H34="")),"",F34*IF(G34&lt;&gt;"",G34,H34/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J34" s="32" t="str">
-        <f aca="false">IF(OR(E34="",I34=""),"",E34-I34)</f>
-        <v/>
-      </c>
-      <c r="K34" s="33" t="str">
-        <f aca="false">IF(OR(D34="",D34=0,F34="",AND(G34="",H34="")),"",(IF(G34&lt;&gt;"",G34,H34/'Budget du don'!$G$4)-D34)/D34)</f>
-        <v/>
-      </c>
-      <c r="L34" s="4"/>
+      <c r="G34" s="18" t="str">
+        <f aca="false">IF(F34="","",F34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H34" s="14"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="16"/>
+      <c r="K34" s="17" t="str">
+        <f aca="false">IF(OR(H34="",AND(I34="",J34="")),"",H34*IF(I34&lt;&gt;"",I34,J34/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L34" s="18" t="str">
+        <f aca="false">IF(K34="","",K34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M34" s="33" t="str">
+        <f aca="false">IF(OR(F34="",K34=""),"",F34-K34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="18" t="str">
+        <f aca="false">IF(M34="","",M34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O34" s="34" t="str">
+        <f aca="false">IF(OR(D34="",D34=0,H34="",AND(I34="",J34="")),"",(IF(I34&lt;&gt;"",I34,J34/'Budget du don'!$G$4)-D34)/D34)</f>
+        <v/>
+      </c>
+      <c r="P34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29" t="str">
+      <c r="A35" s="30" t="str">
         <f aca="false">IF('Budget du don'!A35="","",'Budget du don'!A35)</f>
         <v/>
       </c>
-      <c r="B35" s="30" t="str">
+      <c r="B35" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A35="",'Budget du don'!B35=""),"",'Budget du don'!B35)</f>
         <v/>
       </c>
-      <c r="C35" s="31" t="str">
+      <c r="C35" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A35="",'Budget du don'!C35=""),"",'Budget du don'!C35)</f>
         <v/>
       </c>
-      <c r="D35" s="32" t="str">
+      <c r="D35" s="33" t="str">
         <f aca="false">IF('Budget du don'!A35="","",IF('Budget du don'!D35&lt;&gt;"",'Budget du don'!D35,IF('Budget du don'!E35&lt;&gt;"",'Budget du don'!E35/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E35" s="32" t="str">
+      <c r="E35" s="18" t="str">
+        <f aca="false">IF(D35="","",D35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F35" s="33" t="str">
         <f aca="false">IF('Budget du don'!F35="","",'Budget du don'!F35)</f>
         <v/>
       </c>
-      <c r="F35" s="14"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="17" t="str">
-        <f aca="false">IF(OR(F35="",AND(G35="",H35="")),"",F35*IF(G35&lt;&gt;"",G35,H35/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J35" s="32" t="str">
-        <f aca="false">IF(OR(E35="",I35=""),"",E35-I35)</f>
-        <v/>
-      </c>
-      <c r="K35" s="33" t="str">
-        <f aca="false">IF(OR(D35="",D35=0,F35="",AND(G35="",H35="")),"",(IF(G35&lt;&gt;"",G35,H35/'Budget du don'!$G$4)-D35)/D35)</f>
-        <v/>
-      </c>
-      <c r="L35" s="4"/>
+      <c r="G35" s="18" t="str">
+        <f aca="false">IF(F35="","",F35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H35" s="14"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="17" t="str">
+        <f aca="false">IF(OR(H35="",AND(I35="",J35="")),"",H35*IF(I35&lt;&gt;"",I35,J35/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L35" s="18" t="str">
+        <f aca="false">IF(K35="","",K35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M35" s="33" t="str">
+        <f aca="false">IF(OR(F35="",K35=""),"",F35-K35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="18" t="str">
+        <f aca="false">IF(M35="","",M35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O35" s="34" t="str">
+        <f aca="false">IF(OR(D35="",D35=0,H35="",AND(I35="",J35="")),"",(IF(I35&lt;&gt;"",I35,J35/'Budget du don'!$G$4)-D35)/D35)</f>
+        <v/>
+      </c>
+      <c r="P35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="29" t="str">
+      <c r="A36" s="30" t="str">
         <f aca="false">IF('Budget du don'!A36="","",'Budget du don'!A36)</f>
         <v/>
       </c>
-      <c r="B36" s="30" t="str">
+      <c r="B36" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A36="",'Budget du don'!B36=""),"",'Budget du don'!B36)</f>
         <v/>
       </c>
-      <c r="C36" s="31" t="str">
+      <c r="C36" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A36="",'Budget du don'!C36=""),"",'Budget du don'!C36)</f>
         <v/>
       </c>
-      <c r="D36" s="32" t="str">
+      <c r="D36" s="33" t="str">
         <f aca="false">IF('Budget du don'!A36="","",IF('Budget du don'!D36&lt;&gt;"",'Budget du don'!D36,IF('Budget du don'!E36&lt;&gt;"",'Budget du don'!E36/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E36" s="32" t="str">
+      <c r="E36" s="18" t="str">
+        <f aca="false">IF(D36="","",D36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F36" s="33" t="str">
         <f aca="false">IF('Budget du don'!F36="","",'Budget du don'!F36)</f>
         <v/>
       </c>
-      <c r="F36" s="14"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="17" t="str">
-        <f aca="false">IF(OR(F36="",AND(G36="",H36="")),"",F36*IF(G36&lt;&gt;"",G36,H36/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J36" s="32" t="str">
-        <f aca="false">IF(OR(E36="",I36=""),"",E36-I36)</f>
-        <v/>
-      </c>
-      <c r="K36" s="33" t="str">
-        <f aca="false">IF(OR(D36="",D36=0,F36="",AND(G36="",H36="")),"",(IF(G36&lt;&gt;"",G36,H36/'Budget du don'!$G$4)-D36)/D36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="4"/>
+      <c r="G36" s="18" t="str">
+        <f aca="false">IF(F36="","",F36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H36" s="14"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="17" t="str">
+        <f aca="false">IF(OR(H36="",AND(I36="",J36="")),"",H36*IF(I36&lt;&gt;"",I36,J36/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L36" s="18" t="str">
+        <f aca="false">IF(K36="","",K36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M36" s="33" t="str">
+        <f aca="false">IF(OR(F36="",K36=""),"",F36-K36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="18" t="str">
+        <f aca="false">IF(M36="","",M36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O36" s="34" t="str">
+        <f aca="false">IF(OR(D36="",D36=0,H36="",AND(I36="",J36="")),"",(IF(I36&lt;&gt;"",I36,J36/'Budget du don'!$G$4)-D36)/D36)</f>
+        <v/>
+      </c>
+      <c r="P36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29" t="str">
+      <c r="A37" s="30" t="str">
         <f aca="false">IF('Budget du don'!A37="","",'Budget du don'!A37)</f>
         <v/>
       </c>
-      <c r="B37" s="30" t="str">
+      <c r="B37" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A37="",'Budget du don'!B37=""),"",'Budget du don'!B37)</f>
         <v/>
       </c>
-      <c r="C37" s="31" t="str">
+      <c r="C37" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A37="",'Budget du don'!C37=""),"",'Budget du don'!C37)</f>
         <v/>
       </c>
-      <c r="D37" s="32" t="str">
+      <c r="D37" s="33" t="str">
         <f aca="false">IF('Budget du don'!A37="","",IF('Budget du don'!D37&lt;&gt;"",'Budget du don'!D37,IF('Budget du don'!E37&lt;&gt;"",'Budget du don'!E37/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E37" s="32" t="str">
+      <c r="E37" s="18" t="str">
+        <f aca="false">IF(D37="","",D37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F37" s="33" t="str">
         <f aca="false">IF('Budget du don'!F37="","",'Budget du don'!F37)</f>
         <v/>
       </c>
-      <c r="F37" s="14"/>
-      <c r="G37" s="15"/>
-      <c r="H37" s="16"/>
-      <c r="I37" s="17" t="str">
-        <f aca="false">IF(OR(F37="",AND(G37="",H37="")),"",F37*IF(G37&lt;&gt;"",G37,H37/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J37" s="32" t="str">
-        <f aca="false">IF(OR(E37="",I37=""),"",E37-I37)</f>
-        <v/>
-      </c>
-      <c r="K37" s="33" t="str">
-        <f aca="false">IF(OR(D37="",D37=0,F37="",AND(G37="",H37="")),"",(IF(G37&lt;&gt;"",G37,H37/'Budget du don'!$G$4)-D37)/D37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="4"/>
+      <c r="G37" s="18" t="str">
+        <f aca="false">IF(F37="","",F37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H37" s="14"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="17" t="str">
+        <f aca="false">IF(OR(H37="",AND(I37="",J37="")),"",H37*IF(I37&lt;&gt;"",I37,J37/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L37" s="18" t="str">
+        <f aca="false">IF(K37="","",K37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M37" s="33" t="str">
+        <f aca="false">IF(OR(F37="",K37=""),"",F37-K37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="18" t="str">
+        <f aca="false">IF(M37="","",M37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O37" s="34" t="str">
+        <f aca="false">IF(OR(D37="",D37=0,H37="",AND(I37="",J37="")),"",(IF(I37&lt;&gt;"",I37,J37/'Budget du don'!$G$4)-D37)/D37)</f>
+        <v/>
+      </c>
+      <c r="P37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="str">
+      <c r="A38" s="30" t="str">
         <f aca="false">IF('Budget du don'!A38="","",'Budget du don'!A38)</f>
         <v/>
       </c>
-      <c r="B38" s="30" t="str">
+      <c r="B38" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A38="",'Budget du don'!B38=""),"",'Budget du don'!B38)</f>
         <v/>
       </c>
-      <c r="C38" s="31" t="str">
+      <c r="C38" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A38="",'Budget du don'!C38=""),"",'Budget du don'!C38)</f>
         <v/>
       </c>
-      <c r="D38" s="32" t="str">
+      <c r="D38" s="33" t="str">
         <f aca="false">IF('Budget du don'!A38="","",IF('Budget du don'!D38&lt;&gt;"",'Budget du don'!D38,IF('Budget du don'!E38&lt;&gt;"",'Budget du don'!E38/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E38" s="32" t="str">
+      <c r="E38" s="18" t="str">
+        <f aca="false">IF(D38="","",D38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F38" s="33" t="str">
         <f aca="false">IF('Budget du don'!F38="","",'Budget du don'!F38)</f>
         <v/>
       </c>
-      <c r="F38" s="14"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="16"/>
-      <c r="I38" s="17" t="str">
-        <f aca="false">IF(OR(F38="",AND(G38="",H38="")),"",F38*IF(G38&lt;&gt;"",G38,H38/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J38" s="32" t="str">
-        <f aca="false">IF(OR(E38="",I38=""),"",E38-I38)</f>
-        <v/>
-      </c>
-      <c r="K38" s="33" t="str">
-        <f aca="false">IF(OR(D38="",D38=0,F38="",AND(G38="",H38="")),"",(IF(G38&lt;&gt;"",G38,H38/'Budget du don'!$G$4)-D38)/D38)</f>
-        <v/>
-      </c>
-      <c r="L38" s="4"/>
+      <c r="G38" s="18" t="str">
+        <f aca="false">IF(F38="","",F38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H38" s="14"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="17" t="str">
+        <f aca="false">IF(OR(H38="",AND(I38="",J38="")),"",H38*IF(I38&lt;&gt;"",I38,J38/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L38" s="18" t="str">
+        <f aca="false">IF(K38="","",K38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M38" s="33" t="str">
+        <f aca="false">IF(OR(F38="",K38=""),"",F38-K38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="18" t="str">
+        <f aca="false">IF(M38="","",M38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O38" s="34" t="str">
+        <f aca="false">IF(OR(D38="",D38=0,H38="",AND(I38="",J38="")),"",(IF(I38&lt;&gt;"",I38,J38/'Budget du don'!$G$4)-D38)/D38)</f>
+        <v/>
+      </c>
+      <c r="P38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29" t="str">
+      <c r="A39" s="30" t="str">
         <f aca="false">IF('Budget du don'!A39="","",'Budget du don'!A39)</f>
         <v/>
       </c>
-      <c r="B39" s="30" t="str">
+      <c r="B39" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A39="",'Budget du don'!B39=""),"",'Budget du don'!B39)</f>
         <v/>
       </c>
-      <c r="C39" s="31" t="str">
+      <c r="C39" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A39="",'Budget du don'!C39=""),"",'Budget du don'!C39)</f>
         <v/>
       </c>
-      <c r="D39" s="32" t="str">
+      <c r="D39" s="33" t="str">
         <f aca="false">IF('Budget du don'!A39="","",IF('Budget du don'!D39&lt;&gt;"",'Budget du don'!D39,IF('Budget du don'!E39&lt;&gt;"",'Budget du don'!E39/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E39" s="32" t="str">
+      <c r="E39" s="18" t="str">
+        <f aca="false">IF(D39="","",D39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F39" s="33" t="str">
         <f aca="false">IF('Budget du don'!F39="","",'Budget du don'!F39)</f>
         <v/>
       </c>
-      <c r="F39" s="14"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="17" t="str">
-        <f aca="false">IF(OR(F39="",AND(G39="",H39="")),"",F39*IF(G39&lt;&gt;"",G39,H39/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J39" s="32" t="str">
-        <f aca="false">IF(OR(E39="",I39=""),"",E39-I39)</f>
-        <v/>
-      </c>
-      <c r="K39" s="33" t="str">
-        <f aca="false">IF(OR(D39="",D39=0,F39="",AND(G39="",H39="")),"",(IF(G39&lt;&gt;"",G39,H39/'Budget du don'!$G$4)-D39)/D39)</f>
-        <v/>
-      </c>
-      <c r="L39" s="4"/>
+      <c r="G39" s="18" t="str">
+        <f aca="false">IF(F39="","",F39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H39" s="14"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="17" t="str">
+        <f aca="false">IF(OR(H39="",AND(I39="",J39="")),"",H39*IF(I39&lt;&gt;"",I39,J39/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L39" s="18" t="str">
+        <f aca="false">IF(K39="","",K39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M39" s="33" t="str">
+        <f aca="false">IF(OR(F39="",K39=""),"",F39-K39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="18" t="str">
+        <f aca="false">IF(M39="","",M39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O39" s="34" t="str">
+        <f aca="false">IF(OR(D39="",D39=0,H39="",AND(I39="",J39="")),"",(IF(I39&lt;&gt;"",I39,J39/'Budget du don'!$G$4)-D39)/D39)</f>
+        <v/>
+      </c>
+      <c r="P39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="str">
+      <c r="A40" s="30" t="str">
         <f aca="false">IF('Budget du don'!A40="","",'Budget du don'!A40)</f>
         <v/>
       </c>
-      <c r="B40" s="30" t="str">
+      <c r="B40" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A40="",'Budget du don'!B40=""),"",'Budget du don'!B40)</f>
         <v/>
       </c>
-      <c r="C40" s="31" t="str">
+      <c r="C40" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A40="",'Budget du don'!C40=""),"",'Budget du don'!C40)</f>
         <v/>
       </c>
-      <c r="D40" s="32" t="str">
+      <c r="D40" s="33" t="str">
         <f aca="false">IF('Budget du don'!A40="","",IF('Budget du don'!D40&lt;&gt;"",'Budget du don'!D40,IF('Budget du don'!E40&lt;&gt;"",'Budget du don'!E40/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E40" s="32" t="str">
+      <c r="E40" s="18" t="str">
+        <f aca="false">IF(D40="","",D40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F40" s="33" t="str">
         <f aca="false">IF('Budget du don'!F40="","",'Budget du don'!F40)</f>
         <v/>
       </c>
-      <c r="F40" s="14"/>
-      <c r="G40" s="15"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="17" t="str">
-        <f aca="false">IF(OR(F40="",AND(G40="",H40="")),"",F40*IF(G40&lt;&gt;"",G40,H40/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J40" s="32" t="str">
-        <f aca="false">IF(OR(E40="",I40=""),"",E40-I40)</f>
-        <v/>
-      </c>
-      <c r="K40" s="33" t="str">
-        <f aca="false">IF(OR(D40="",D40=0,F40="",AND(G40="",H40="")),"",(IF(G40&lt;&gt;"",G40,H40/'Budget du don'!$G$4)-D40)/D40)</f>
-        <v/>
-      </c>
-      <c r="L40" s="4"/>
+      <c r="G40" s="18" t="str">
+        <f aca="false">IF(F40="","",F40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H40" s="14"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="17" t="str">
+        <f aca="false">IF(OR(H40="",AND(I40="",J40="")),"",H40*IF(I40&lt;&gt;"",I40,J40/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L40" s="18" t="str">
+        <f aca="false">IF(K40="","",K40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M40" s="33" t="str">
+        <f aca="false">IF(OR(F40="",K40=""),"",F40-K40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="18" t="str">
+        <f aca="false">IF(M40="","",M40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O40" s="34" t="str">
+        <f aca="false">IF(OR(D40="",D40=0,H40="",AND(I40="",J40="")),"",(IF(I40&lt;&gt;"",I40,J40/'Budget du don'!$G$4)-D40)/D40)</f>
+        <v/>
+      </c>
+      <c r="P40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="str">
+      <c r="A41" s="30" t="str">
         <f aca="false">IF('Budget du don'!A41="","",'Budget du don'!A41)</f>
         <v/>
       </c>
-      <c r="B41" s="30" t="str">
+      <c r="B41" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A41="",'Budget du don'!B41=""),"",'Budget du don'!B41)</f>
         <v/>
       </c>
-      <c r="C41" s="31" t="str">
+      <c r="C41" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A41="",'Budget du don'!C41=""),"",'Budget du don'!C41)</f>
         <v/>
       </c>
-      <c r="D41" s="32" t="str">
+      <c r="D41" s="33" t="str">
         <f aca="false">IF('Budget du don'!A41="","",IF('Budget du don'!D41&lt;&gt;"",'Budget du don'!D41,IF('Budget du don'!E41&lt;&gt;"",'Budget du don'!E41/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E41" s="32" t="str">
+      <c r="E41" s="18" t="str">
+        <f aca="false">IF(D41="","",D41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F41" s="33" t="str">
         <f aca="false">IF('Budget du don'!F41="","",'Budget du don'!F41)</f>
         <v/>
       </c>
-      <c r="F41" s="14"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="16"/>
-      <c r="I41" s="17" t="str">
-        <f aca="false">IF(OR(F41="",AND(G41="",H41="")),"",F41*IF(G41&lt;&gt;"",G41,H41/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J41" s="32" t="str">
-        <f aca="false">IF(OR(E41="",I41=""),"",E41-I41)</f>
-        <v/>
-      </c>
-      <c r="K41" s="33" t="str">
-        <f aca="false">IF(OR(D41="",D41=0,F41="",AND(G41="",H41="")),"",(IF(G41&lt;&gt;"",G41,H41/'Budget du don'!$G$4)-D41)/D41)</f>
-        <v/>
-      </c>
-      <c r="L41" s="4"/>
+      <c r="G41" s="18" t="str">
+        <f aca="false">IF(F41="","",F41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H41" s="14"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="17" t="str">
+        <f aca="false">IF(OR(H41="",AND(I41="",J41="")),"",H41*IF(I41&lt;&gt;"",I41,J41/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L41" s="18" t="str">
+        <f aca="false">IF(K41="","",K41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M41" s="33" t="str">
+        <f aca="false">IF(OR(F41="",K41=""),"",F41-K41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="18" t="str">
+        <f aca="false">IF(M41="","",M41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O41" s="34" t="str">
+        <f aca="false">IF(OR(D41="",D41=0,H41="",AND(I41="",J41="")),"",(IF(I41&lt;&gt;"",I41,J41/'Budget du don'!$G$4)-D41)/D41)</f>
+        <v/>
+      </c>
+      <c r="P41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29" t="str">
+      <c r="A42" s="30" t="str">
         <f aca="false">IF('Budget du don'!A42="","",'Budget du don'!A42)</f>
         <v/>
       </c>
-      <c r="B42" s="30" t="str">
+      <c r="B42" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A42="",'Budget du don'!B42=""),"",'Budget du don'!B42)</f>
         <v/>
       </c>
-      <c r="C42" s="31" t="str">
+      <c r="C42" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A42="",'Budget du don'!C42=""),"",'Budget du don'!C42)</f>
         <v/>
       </c>
-      <c r="D42" s="32" t="str">
+      <c r="D42" s="33" t="str">
         <f aca="false">IF('Budget du don'!A42="","",IF('Budget du don'!D42&lt;&gt;"",'Budget du don'!D42,IF('Budget du don'!E42&lt;&gt;"",'Budget du don'!E42/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E42" s="32" t="str">
+      <c r="E42" s="18" t="str">
+        <f aca="false">IF(D42="","",D42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F42" s="33" t="str">
         <f aca="false">IF('Budget du don'!F42="","",'Budget du don'!F42)</f>
         <v/>
       </c>
-      <c r="F42" s="14"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="16"/>
-      <c r="I42" s="17" t="str">
-        <f aca="false">IF(OR(F42="",AND(G42="",H42="")),"",F42*IF(G42&lt;&gt;"",G42,H42/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J42" s="32" t="str">
-        <f aca="false">IF(OR(E42="",I42=""),"",E42-I42)</f>
-        <v/>
-      </c>
-      <c r="K42" s="33" t="str">
-        <f aca="false">IF(OR(D42="",D42=0,F42="",AND(G42="",H42="")),"",(IF(G42&lt;&gt;"",G42,H42/'Budget du don'!$G$4)-D42)/D42)</f>
-        <v/>
-      </c>
-      <c r="L42" s="4"/>
+      <c r="G42" s="18" t="str">
+        <f aca="false">IF(F42="","",F42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H42" s="14"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="17" t="str">
+        <f aca="false">IF(OR(H42="",AND(I42="",J42="")),"",H42*IF(I42&lt;&gt;"",I42,J42/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L42" s="18" t="str">
+        <f aca="false">IF(K42="","",K42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M42" s="33" t="str">
+        <f aca="false">IF(OR(F42="",K42=""),"",F42-K42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="18" t="str">
+        <f aca="false">IF(M42="","",M42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O42" s="34" t="str">
+        <f aca="false">IF(OR(D42="",D42=0,H42="",AND(I42="",J42="")),"",(IF(I42&lt;&gt;"",I42,J42/'Budget du don'!$G$4)-D42)/D42)</f>
+        <v/>
+      </c>
+      <c r="P42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29" t="str">
+      <c r="A43" s="30" t="str">
         <f aca="false">IF('Budget du don'!A43="","",'Budget du don'!A43)</f>
         <v/>
       </c>
-      <c r="B43" s="30" t="str">
+      <c r="B43" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A43="",'Budget du don'!B43=""),"",'Budget du don'!B43)</f>
         <v/>
       </c>
-      <c r="C43" s="31" t="str">
+      <c r="C43" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A43="",'Budget du don'!C43=""),"",'Budget du don'!C43)</f>
         <v/>
       </c>
-      <c r="D43" s="32" t="str">
+      <c r="D43" s="33" t="str">
         <f aca="false">IF('Budget du don'!A43="","",IF('Budget du don'!D43&lt;&gt;"",'Budget du don'!D43,IF('Budget du don'!E43&lt;&gt;"",'Budget du don'!E43/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E43" s="32" t="str">
+      <c r="E43" s="18" t="str">
+        <f aca="false">IF(D43="","",D43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F43" s="33" t="str">
         <f aca="false">IF('Budget du don'!F43="","",'Budget du don'!F43)</f>
         <v/>
       </c>
-      <c r="F43" s="14"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="17" t="str">
-        <f aca="false">IF(OR(F43="",AND(G43="",H43="")),"",F43*IF(G43&lt;&gt;"",G43,H43/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J43" s="32" t="str">
-        <f aca="false">IF(OR(E43="",I43=""),"",E43-I43)</f>
-        <v/>
-      </c>
-      <c r="K43" s="33" t="str">
-        <f aca="false">IF(OR(D43="",D43=0,F43="",AND(G43="",H43="")),"",(IF(G43&lt;&gt;"",G43,H43/'Budget du don'!$G$4)-D43)/D43)</f>
-        <v/>
-      </c>
-      <c r="L43" s="4"/>
+      <c r="G43" s="18" t="str">
+        <f aca="false">IF(F43="","",F43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H43" s="14"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="17" t="str">
+        <f aca="false">IF(OR(H43="",AND(I43="",J43="")),"",H43*IF(I43&lt;&gt;"",I43,J43/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L43" s="18" t="str">
+        <f aca="false">IF(K43="","",K43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M43" s="33" t="str">
+        <f aca="false">IF(OR(F43="",K43=""),"",F43-K43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="18" t="str">
+        <f aca="false">IF(M43="","",M43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O43" s="34" t="str">
+        <f aca="false">IF(OR(D43="",D43=0,H43="",AND(I43="",J43="")),"",(IF(I43&lt;&gt;"",I43,J43/'Budget du don'!$G$4)-D43)/D43)</f>
+        <v/>
+      </c>
+      <c r="P43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="29" t="str">
+      <c r="A44" s="30" t="str">
         <f aca="false">IF('Budget du don'!A44="","",'Budget du don'!A44)</f>
         <v/>
       </c>
-      <c r="B44" s="30" t="str">
+      <c r="B44" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A44="",'Budget du don'!B44=""),"",'Budget du don'!B44)</f>
         <v/>
       </c>
-      <c r="C44" s="31" t="str">
+      <c r="C44" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A44="",'Budget du don'!C44=""),"",'Budget du don'!C44)</f>
         <v/>
       </c>
-      <c r="D44" s="32" t="str">
+      <c r="D44" s="33" t="str">
         <f aca="false">IF('Budget du don'!A44="","",IF('Budget du don'!D44&lt;&gt;"",'Budget du don'!D44,IF('Budget du don'!E44&lt;&gt;"",'Budget du don'!E44/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E44" s="32" t="str">
+      <c r="E44" s="18" t="str">
+        <f aca="false">IF(D44="","",D44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F44" s="33" t="str">
         <f aca="false">IF('Budget du don'!F44="","",'Budget du don'!F44)</f>
         <v/>
       </c>
-      <c r="F44" s="14"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="16"/>
-      <c r="I44" s="17" t="str">
-        <f aca="false">IF(OR(F44="",AND(G44="",H44="")),"",F44*IF(G44&lt;&gt;"",G44,H44/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J44" s="32" t="str">
-        <f aca="false">IF(OR(E44="",I44=""),"",E44-I44)</f>
-        <v/>
-      </c>
-      <c r="K44" s="33" t="str">
-        <f aca="false">IF(OR(D44="",D44=0,F44="",AND(G44="",H44="")),"",(IF(G44&lt;&gt;"",G44,H44/'Budget du don'!$G$4)-D44)/D44)</f>
-        <v/>
-      </c>
-      <c r="L44" s="4"/>
+      <c r="G44" s="18" t="str">
+        <f aca="false">IF(F44="","",F44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H44" s="14"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="17" t="str">
+        <f aca="false">IF(OR(H44="",AND(I44="",J44="")),"",H44*IF(I44&lt;&gt;"",I44,J44/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L44" s="18" t="str">
+        <f aca="false">IF(K44="","",K44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M44" s="33" t="str">
+        <f aca="false">IF(OR(F44="",K44=""),"",F44-K44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="18" t="str">
+        <f aca="false">IF(M44="","",M44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O44" s="34" t="str">
+        <f aca="false">IF(OR(D44="",D44=0,H44="",AND(I44="",J44="")),"",(IF(I44&lt;&gt;"",I44,J44/'Budget du don'!$G$4)-D44)/D44)</f>
+        <v/>
+      </c>
+      <c r="P44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="29" t="str">
+      <c r="A45" s="30" t="str">
         <f aca="false">IF('Budget du don'!A45="","",'Budget du don'!A45)</f>
         <v/>
       </c>
-      <c r="B45" s="30" t="str">
+      <c r="B45" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A45="",'Budget du don'!B45=""),"",'Budget du don'!B45)</f>
         <v/>
       </c>
-      <c r="C45" s="31" t="str">
+      <c r="C45" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A45="",'Budget du don'!C45=""),"",'Budget du don'!C45)</f>
         <v/>
       </c>
-      <c r="D45" s="32" t="str">
+      <c r="D45" s="33" t="str">
         <f aca="false">IF('Budget du don'!A45="","",IF('Budget du don'!D45&lt;&gt;"",'Budget du don'!D45,IF('Budget du don'!E45&lt;&gt;"",'Budget du don'!E45/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E45" s="32" t="str">
+      <c r="E45" s="18" t="str">
+        <f aca="false">IF(D45="","",D45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F45" s="33" t="str">
         <f aca="false">IF('Budget du don'!F45="","",'Budget du don'!F45)</f>
         <v/>
       </c>
-      <c r="F45" s="14"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="17" t="str">
-        <f aca="false">IF(OR(F45="",AND(G45="",H45="")),"",F45*IF(G45&lt;&gt;"",G45,H45/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J45" s="32" t="str">
-        <f aca="false">IF(OR(E45="",I45=""),"",E45-I45)</f>
-        <v/>
-      </c>
-      <c r="K45" s="33" t="str">
-        <f aca="false">IF(OR(D45="",D45=0,F45="",AND(G45="",H45="")),"",(IF(G45&lt;&gt;"",G45,H45/'Budget du don'!$G$4)-D45)/D45)</f>
-        <v/>
-      </c>
-      <c r="L45" s="4"/>
+      <c r="G45" s="18" t="str">
+        <f aca="false">IF(F45="","",F45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H45" s="14"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="17" t="str">
+        <f aca="false">IF(OR(H45="",AND(I45="",J45="")),"",H45*IF(I45&lt;&gt;"",I45,J45/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L45" s="18" t="str">
+        <f aca="false">IF(K45="","",K45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M45" s="33" t="str">
+        <f aca="false">IF(OR(F45="",K45=""),"",F45-K45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="18" t="str">
+        <f aca="false">IF(M45="","",M45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O45" s="34" t="str">
+        <f aca="false">IF(OR(D45="",D45=0,H45="",AND(I45="",J45="")),"",(IF(I45&lt;&gt;"",I45,J45/'Budget du don'!$G$4)-D45)/D45)</f>
+        <v/>
+      </c>
+      <c r="P45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="29" t="str">
+      <c r="A46" s="30" t="str">
         <f aca="false">IF('Budget du don'!A46="","",'Budget du don'!A46)</f>
         <v/>
       </c>
-      <c r="B46" s="30" t="str">
+      <c r="B46" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A46="",'Budget du don'!B46=""),"",'Budget du don'!B46)</f>
         <v/>
       </c>
-      <c r="C46" s="31" t="str">
+      <c r="C46" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A46="",'Budget du don'!C46=""),"",'Budget du don'!C46)</f>
         <v/>
       </c>
-      <c r="D46" s="32" t="str">
+      <c r="D46" s="33" t="str">
         <f aca="false">IF('Budget du don'!A46="","",IF('Budget du don'!D46&lt;&gt;"",'Budget du don'!D46,IF('Budget du don'!E46&lt;&gt;"",'Budget du don'!E46/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E46" s="32" t="str">
+      <c r="E46" s="18" t="str">
+        <f aca="false">IF(D46="","",D46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F46" s="33" t="str">
         <f aca="false">IF('Budget du don'!F46="","",'Budget du don'!F46)</f>
         <v/>
       </c>
-      <c r="F46" s="14"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="17" t="str">
-        <f aca="false">IF(OR(F46="",AND(G46="",H46="")),"",F46*IF(G46&lt;&gt;"",G46,H46/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J46" s="32" t="str">
-        <f aca="false">IF(OR(E46="",I46=""),"",E46-I46)</f>
-        <v/>
-      </c>
-      <c r="K46" s="33" t="str">
-        <f aca="false">IF(OR(D46="",D46=0,F46="",AND(G46="",H46="")),"",(IF(G46&lt;&gt;"",G46,H46/'Budget du don'!$G$4)-D46)/D46)</f>
-        <v/>
-      </c>
-      <c r="L46" s="4"/>
+      <c r="G46" s="18" t="str">
+        <f aca="false">IF(F46="","",F46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H46" s="14"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="17" t="str">
+        <f aca="false">IF(OR(H46="",AND(I46="",J46="")),"",H46*IF(I46&lt;&gt;"",I46,J46/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L46" s="18" t="str">
+        <f aca="false">IF(K46="","",K46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M46" s="33" t="str">
+        <f aca="false">IF(OR(F46="",K46=""),"",F46-K46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="18" t="str">
+        <f aca="false">IF(M46="","",M46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O46" s="34" t="str">
+        <f aca="false">IF(OR(D46="",D46=0,H46="",AND(I46="",J46="")),"",(IF(I46&lt;&gt;"",I46,J46/'Budget du don'!$G$4)-D46)/D46)</f>
+        <v/>
+      </c>
+      <c r="P46" s="4"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="29" t="str">
+      <c r="A47" s="30" t="str">
         <f aca="false">IF('Budget du don'!A47="","",'Budget du don'!A47)</f>
         <v/>
       </c>
-      <c r="B47" s="30" t="str">
+      <c r="B47" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A47="",'Budget du don'!B47=""),"",'Budget du don'!B47)</f>
         <v/>
       </c>
-      <c r="C47" s="31" t="str">
+      <c r="C47" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A47="",'Budget du don'!C47=""),"",'Budget du don'!C47)</f>
         <v/>
       </c>
-      <c r="D47" s="32" t="str">
+      <c r="D47" s="33" t="str">
         <f aca="false">IF('Budget du don'!A47="","",IF('Budget du don'!D47&lt;&gt;"",'Budget du don'!D47,IF('Budget du don'!E47&lt;&gt;"",'Budget du don'!E47/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E47" s="32" t="str">
+      <c r="E47" s="18" t="str">
+        <f aca="false">IF(D47="","",D47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F47" s="33" t="str">
         <f aca="false">IF('Budget du don'!F47="","",'Budget du don'!F47)</f>
         <v/>
       </c>
-      <c r="F47" s="14"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="16"/>
-      <c r="I47" s="17" t="str">
-        <f aca="false">IF(OR(F47="",AND(G47="",H47="")),"",F47*IF(G47&lt;&gt;"",G47,H47/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J47" s="32" t="str">
-        <f aca="false">IF(OR(E47="",I47=""),"",E47-I47)</f>
-        <v/>
-      </c>
-      <c r="K47" s="33" t="str">
-        <f aca="false">IF(OR(D47="",D47=0,F47="",AND(G47="",H47="")),"",(IF(G47&lt;&gt;"",G47,H47/'Budget du don'!$G$4)-D47)/D47)</f>
-        <v/>
-      </c>
-      <c r="L47" s="4"/>
+      <c r="G47" s="18" t="str">
+        <f aca="false">IF(F47="","",F47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H47" s="14"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="17" t="str">
+        <f aca="false">IF(OR(H47="",AND(I47="",J47="")),"",H47*IF(I47&lt;&gt;"",I47,J47/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L47" s="18" t="str">
+        <f aca="false">IF(K47="","",K47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M47" s="33" t="str">
+        <f aca="false">IF(OR(F47="",K47=""),"",F47-K47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="18" t="str">
+        <f aca="false">IF(M47="","",M47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O47" s="34" t="str">
+        <f aca="false">IF(OR(D47="",D47=0,H47="",AND(I47="",J47="")),"",(IF(I47&lt;&gt;"",I47,J47/'Budget du don'!$G$4)-D47)/D47)</f>
+        <v/>
+      </c>
+      <c r="P47" s="4"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="29" t="str">
+      <c r="A48" s="30" t="str">
         <f aca="false">IF('Budget du don'!A48="","",'Budget du don'!A48)</f>
         <v/>
       </c>
-      <c r="B48" s="30" t="str">
+      <c r="B48" s="31" t="str">
         <f aca="false">IF(OR('Budget du don'!A48="",'Budget du don'!B48=""),"",'Budget du don'!B48)</f>
         <v/>
       </c>
-      <c r="C48" s="31" t="str">
+      <c r="C48" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A48="",'Budget du don'!C48=""),"",'Budget du don'!C48)</f>
         <v/>
       </c>
-      <c r="D48" s="32" t="str">
+      <c r="D48" s="33" t="str">
         <f aca="false">IF('Budget du don'!A48="","",IF('Budget du don'!D48&lt;&gt;"",'Budget du don'!D48,IF('Budget du don'!E48&lt;&gt;"",'Budget du don'!E48/'Budget du don'!$G$4,"")))</f>
         <v/>
       </c>
-      <c r="E48" s="32" t="str">
+      <c r="E48" s="18" t="str">
+        <f aca="false">IF(D48="","",D48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F48" s="33" t="str">
         <f aca="false">IF('Budget du don'!F48="","",'Budget du don'!F48)</f>
         <v/>
       </c>
-      <c r="F48" s="14"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="16"/>
-      <c r="I48" s="17" t="str">
-        <f aca="false">IF(OR(F48="",AND(G48="",H48="")),"",F48*IF(G48&lt;&gt;"",G48,H48/'Budget du don'!$G$4))</f>
-        <v/>
-      </c>
-      <c r="J48" s="32" t="str">
-        <f aca="false">IF(OR(E48="",I48=""),"",E48-I48)</f>
-        <v/>
-      </c>
-      <c r="K48" s="33" t="str">
-        <f aca="false">IF(OR(D48="",D48=0,F48="",AND(G48="",H48="")),"",(IF(G48&lt;&gt;"",G48,H48/'Budget du don'!$G$4)-D48)/D48)</f>
-        <v/>
-      </c>
-      <c r="L48" s="4"/>
+      <c r="G48" s="18" t="str">
+        <f aca="false">IF(F48="","",F48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H48" s="14"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="16"/>
+      <c r="K48" s="17" t="str">
+        <f aca="false">IF(OR(H48="",AND(I48="",J48="")),"",H48*IF(I48&lt;&gt;"",I48,J48/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="L48" s="18" t="str">
+        <f aca="false">IF(K48="","",K48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="M48" s="33" t="str">
+        <f aca="false">IF(OR(F48="",K48=""),"",F48-K48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="18" t="str">
+        <f aca="false">IF(M48="","",M48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="O48" s="34" t="str">
+        <f aca="false">IF(OR(D48="",D48=0,H48="",AND(I48="",J48="")),"",(IF(I48&lt;&gt;"",I48,J48/'Budget du don'!$G$4)-D48)/D48)</f>
+        <v/>
+      </c>
+      <c r="P48" s="4"/>
     </row>
     <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="B49" s="35"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="36" t="n">
-        <f aca="false">SUM(E9:E48)</f>
+      <c r="A49" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" s="36"/>
+      <c r="C49" s="36"/>
+      <c r="D49" s="36"/>
+      <c r="E49" s="36"/>
+      <c r="F49" s="37" t="n">
+        <f aca="false">SUM(F9:F48)</f>
         <v>182.938820684892</v>
       </c>
-      <c r="F49" s="35"/>
-      <c r="G49" s="35"/>
-      <c r="H49" s="35"/>
-      <c r="I49" s="36" t="n">
-        <f aca="false">SUM(I9:I48)</f>
+      <c r="G49" s="38" t="n">
+        <f aca="false">SUM(G9:G48)</f>
+        <v>120000</v>
+      </c>
+      <c r="H49" s="36"/>
+      <c r="I49" s="36"/>
+      <c r="J49" s="36"/>
+      <c r="K49" s="37" t="n">
+        <f aca="false">SUM(K9:K48)</f>
         <v>195.134742063885</v>
       </c>
-      <c r="J49" s="36" t="n">
-        <f aca="false">SUM(J9:J48)</f>
+      <c r="L49" s="38" t="n">
+        <f aca="false">SUM(L9:L48)</f>
+        <v>128000</v>
+      </c>
+      <c r="M49" s="37" t="n">
+        <f aca="false">SUM(M9:M48)</f>
         <v>-12.1959213789929</v>
       </c>
-      <c r="K49" s="37" t="n">
-        <f aca="false">IF(SUM(E9:E48)=0,"",(SUM(I9:I48)-SUM(E9:E48))/SUM(E9:E48))</f>
+      <c r="N49" s="38" t="n">
+        <f aca="false">SUM(N9:N48)</f>
+        <v>-8000.00000000002</v>
+      </c>
+      <c r="O49" s="39" t="n">
+        <f aca="false">IF(SUM(F9:F48)=0,"",(SUM(K9:K48)-SUM(F9:F48))/SUM(F9:F48))</f>
         <v>0.0666666666666669</v>
       </c>
-      <c r="L49" s="35"/>
+      <c r="P49" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
+  <mergeCells count="17">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="M7:P7"/>
   </mergeCells>
-  <conditionalFormatting sqref="J9:J48">
+  <conditionalFormatting sqref="M9:M48">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3350,11 +4077,19 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K9:K48">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="N9:N48">
+    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O9:O48">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Budget du don : conversion €/FCFA automatique sur le prix unitaire
Le prix unitaire se saisit en € ou en FCFA ; deux colonnes affichent
la conversion dans les deux monnaies, plus les montants € et FCFA.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/budget-par-don-les-petits-enfants-de-marie.xlsx
+++ b/budget-par-don-les-petits-enfants-de-marie.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
   <si>
     <t xml:space="preserve">BUDGET PAR DON — LISTE D'ACHATS</t>
   </si>
   <si>
-    <t xml:space="preserve">Préparez ici le budget d'un don : les articles à acheter, l'unité, la quantité et le prix unitaire (en € OU en FCFA, une seule des deux colonnes). Le montant total en bas vous donne l'enveloppe à envoyer à la logistique. La ligne 9 est un exemple.</t>
+    <t xml:space="preserve">Préparez ici le budget d'un don : les articles à acheter, l'unité, la quantité et le prix unitaire saisi en € OU en FCFA (une seule des deux colonnes jaunes) — la conversion s'affiche automatiquement dans les deux monnaies. Le montant total en bas vous donne l'enveloppe à envoyer à la logistique. La ligne 9 est un exemple.</t>
   </si>
   <si>
     <t xml:space="preserve">Campagne / don :</t>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t xml:space="preserve">Quantité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PU saisi (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PU saisi (FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">Prix unitaire (€)</t>
@@ -492,11 +498,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -554,10 +564,6 @@
     </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -852,16 +858,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -874,6 +882,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -885,6 +895,8 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -932,12 +944,12 @@
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="n">
-        <f aca="false">SUM(F9:F48)</f>
+        <f aca="false">SUM(H9:H48)</f>
         <v>182.938820684892</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="n">
-        <f aca="false">SUM(G9:G48)</f>
+        <f aca="false">SUM(I9:I48)</f>
         <v>120000</v>
       </c>
       <c r="D7" s="10"/>
@@ -969,13 +981,19 @@
       <c r="G8" s="12" t="s">
         <v>17</v>
       </c>
+      <c r="H8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>10</v>
@@ -985,144 +1003,208 @@
         <v>12000</v>
       </c>
       <c r="F9" s="17" t="n">
-        <f aca="false">IF(OR(A9="",C9="",AND(D9="",E9="")),"",C9*IF(D9&lt;&gt;"",D9,E9/'Budget du don'!$G$4))</f>
-        <v>182.938820684892</v>
+        <f aca="false">IF(AND(D9="",E9=""),"",IF(D9&lt;&gt;"",D9,E9/'Budget du don'!$G$4))</f>
+        <v>18.2938820684892</v>
       </c>
       <c r="G9" s="18" t="n">
         <f aca="false">IF(F9="","",F9*'Budget du don'!$G$4)</f>
+        <v>12000</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <f aca="false">IF(OR(A9="",C9="",F9=""),"",C9*F9)</f>
+        <v>182.938820684892</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <f aca="false">IF(H9="","",H9*'Budget du don'!$G$4)</f>
         <v>120000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="15"/>
       <c r="E10" s="16"/>
       <c r="F10" s="17" t="str">
-        <f aca="false">IF(OR(A10="",C10="",AND(D10="",E10="")),"",C10*IF(D10&lt;&gt;"",D10,E10/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D10="",E10=""),"",IF(D10&lt;&gt;"",D10,E10/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G10" s="18" t="str">
         <f aca="false">IF(F10="","",F10*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H10" s="19" t="str">
+        <f aca="false">IF(OR(A10="",C10="",F10=""),"",C10*F10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="18" t="str">
+        <f aca="false">IF(H10="","",H10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="15"/>
       <c r="E11" s="16"/>
       <c r="F11" s="17" t="str">
-        <f aca="false">IF(OR(A11="",C11="",AND(D11="",E11="")),"",C11*IF(D11&lt;&gt;"",D11,E11/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D11="",E11=""),"",IF(D11&lt;&gt;"",D11,E11/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G11" s="18" t="str">
         <f aca="false">IF(F11="","",F11*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H11" s="19" t="str">
+        <f aca="false">IF(OR(A11="",C11="",F11=""),"",C11*F11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="18" t="str">
+        <f aca="false">IF(H11="","",H11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>23</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>21</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="15"/>
       <c r="E12" s="16"/>
       <c r="F12" s="17" t="str">
-        <f aca="false">IF(OR(A12="",C12="",AND(D12="",E12="")),"",C12*IF(D12&lt;&gt;"",D12,E12/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D12="",E12=""),"",IF(D12&lt;&gt;"",D12,E12/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G12" s="18" t="str">
         <f aca="false">IF(F12="","",F12*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H12" s="19" t="str">
+        <f aca="false">IF(OR(A12="",C12="",F12=""),"",C12*F12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="18" t="str">
+        <f aca="false">IF(H12="","",H12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="15"/>
       <c r="E13" s="16"/>
       <c r="F13" s="17" t="str">
-        <f aca="false">IF(OR(A13="",C13="",AND(D13="",E13="")),"",C13*IF(D13&lt;&gt;"",D13,E13/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D13="",E13=""),"",IF(D13&lt;&gt;"",D13,E13/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G13" s="18" t="str">
         <f aca="false">IF(F13="","",F13*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H13" s="19" t="str">
+        <f aca="false">IF(OR(A13="",C13="",F13=""),"",C13*F13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="18" t="str">
+        <f aca="false">IF(H13="","",H13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="15"/>
       <c r="E14" s="16"/>
       <c r="F14" s="17" t="str">
-        <f aca="false">IF(OR(A14="",C14="",AND(D14="",E14="")),"",C14*IF(D14&lt;&gt;"",D14,E14/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D14="",E14=""),"",IF(D14&lt;&gt;"",D14,E14/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G14" s="18" t="str">
         <f aca="false">IF(F14="","",F14*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H14" s="19" t="str">
+        <f aca="false">IF(OR(A14="",C14="",F14=""),"",C14*F14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="18" t="str">
+        <f aca="false">IF(H14="","",H14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15"/>
       <c r="E15" s="16"/>
       <c r="F15" s="17" t="str">
-        <f aca="false">IF(OR(A15="",C15="",AND(D15="",E15="")),"",C15*IF(D15&lt;&gt;"",D15,E15/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D15="",E15=""),"",IF(D15&lt;&gt;"",D15,E15/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G15" s="18" t="str">
         <f aca="false">IF(F15="","",F15*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H15" s="19" t="str">
+        <f aca="false">IF(OR(A15="",C15="",F15=""),"",C15*F15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="18" t="str">
+        <f aca="false">IF(H15="","",H15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15"/>
       <c r="E16" s="16"/>
       <c r="F16" s="17" t="str">
-        <f aca="false">IF(OR(A16="",C16="",AND(D16="",E16="")),"",C16*IF(D16&lt;&gt;"",D16,E16/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D16="",E16=""),"",IF(D16&lt;&gt;"",D16,E16/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G16" s="18" t="str">
         <f aca="false">IF(F16="","",F16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H16" s="19" t="str">
+        <f aca="false">IF(OR(A16="",C16="",F16=""),"",C16*F16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="18" t="str">
+        <f aca="false">IF(H16="","",H16*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1133,11 +1215,19 @@
       <c r="D17" s="15"/>
       <c r="E17" s="16"/>
       <c r="F17" s="17" t="str">
-        <f aca="false">IF(OR(A17="",C17="",AND(D17="",E17="")),"",C17*IF(D17&lt;&gt;"",D17,E17/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D17="",E17=""),"",IF(D17&lt;&gt;"",D17,E17/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G17" s="18" t="str">
         <f aca="false">IF(F17="","",F17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H17" s="19" t="str">
+        <f aca="false">IF(OR(A17="",C17="",F17=""),"",C17*F17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="18" t="str">
+        <f aca="false">IF(H17="","",H17*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1148,11 +1238,19 @@
       <c r="D18" s="15"/>
       <c r="E18" s="16"/>
       <c r="F18" s="17" t="str">
-        <f aca="false">IF(OR(A18="",C18="",AND(D18="",E18="")),"",C18*IF(D18&lt;&gt;"",D18,E18/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D18="",E18=""),"",IF(D18&lt;&gt;"",D18,E18/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G18" s="18" t="str">
         <f aca="false">IF(F18="","",F18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H18" s="19" t="str">
+        <f aca="false">IF(OR(A18="",C18="",F18=""),"",C18*F18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="18" t="str">
+        <f aca="false">IF(H18="","",H18*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1163,11 +1261,19 @@
       <c r="D19" s="15"/>
       <c r="E19" s="16"/>
       <c r="F19" s="17" t="str">
-        <f aca="false">IF(OR(A19="",C19="",AND(D19="",E19="")),"",C19*IF(D19&lt;&gt;"",D19,E19/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D19="",E19=""),"",IF(D19&lt;&gt;"",D19,E19/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G19" s="18" t="str">
         <f aca="false">IF(F19="","",F19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H19" s="19" t="str">
+        <f aca="false">IF(OR(A19="",C19="",F19=""),"",C19*F19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="18" t="str">
+        <f aca="false">IF(H19="","",H19*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1178,11 +1284,19 @@
       <c r="D20" s="15"/>
       <c r="E20" s="16"/>
       <c r="F20" s="17" t="str">
-        <f aca="false">IF(OR(A20="",C20="",AND(D20="",E20="")),"",C20*IF(D20&lt;&gt;"",D20,E20/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D20="",E20=""),"",IF(D20&lt;&gt;"",D20,E20/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G20" s="18" t="str">
         <f aca="false">IF(F20="","",F20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H20" s="19" t="str">
+        <f aca="false">IF(OR(A20="",C20="",F20=""),"",C20*F20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="18" t="str">
+        <f aca="false">IF(H20="","",H20*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1193,11 +1307,19 @@
       <c r="D21" s="15"/>
       <c r="E21" s="16"/>
       <c r="F21" s="17" t="str">
-        <f aca="false">IF(OR(A21="",C21="",AND(D21="",E21="")),"",C21*IF(D21&lt;&gt;"",D21,E21/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D21="",E21=""),"",IF(D21&lt;&gt;"",D21,E21/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G21" s="18" t="str">
         <f aca="false">IF(F21="","",F21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H21" s="19" t="str">
+        <f aca="false">IF(OR(A21="",C21="",F21=""),"",C21*F21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="18" t="str">
+        <f aca="false">IF(H21="","",H21*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1208,11 +1330,19 @@
       <c r="D22" s="15"/>
       <c r="E22" s="16"/>
       <c r="F22" s="17" t="str">
-        <f aca="false">IF(OR(A22="",C22="",AND(D22="",E22="")),"",C22*IF(D22&lt;&gt;"",D22,E22/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D22="",E22=""),"",IF(D22&lt;&gt;"",D22,E22/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G22" s="18" t="str">
         <f aca="false">IF(F22="","",F22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H22" s="19" t="str">
+        <f aca="false">IF(OR(A22="",C22="",F22=""),"",C22*F22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="18" t="str">
+        <f aca="false">IF(H22="","",H22*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1223,11 +1353,19 @@
       <c r="D23" s="15"/>
       <c r="E23" s="16"/>
       <c r="F23" s="17" t="str">
-        <f aca="false">IF(OR(A23="",C23="",AND(D23="",E23="")),"",C23*IF(D23&lt;&gt;"",D23,E23/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D23="",E23=""),"",IF(D23&lt;&gt;"",D23,E23/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G23" s="18" t="str">
         <f aca="false">IF(F23="","",F23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H23" s="19" t="str">
+        <f aca="false">IF(OR(A23="",C23="",F23=""),"",C23*F23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="18" t="str">
+        <f aca="false">IF(H23="","",H23*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1238,11 +1376,19 @@
       <c r="D24" s="15"/>
       <c r="E24" s="16"/>
       <c r="F24" s="17" t="str">
-        <f aca="false">IF(OR(A24="",C24="",AND(D24="",E24="")),"",C24*IF(D24&lt;&gt;"",D24,E24/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D24="",E24=""),"",IF(D24&lt;&gt;"",D24,E24/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G24" s="18" t="str">
         <f aca="false">IF(F24="","",F24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H24" s="19" t="str">
+        <f aca="false">IF(OR(A24="",C24="",F24=""),"",C24*F24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="18" t="str">
+        <f aca="false">IF(H24="","",H24*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1253,11 +1399,19 @@
       <c r="D25" s="15"/>
       <c r="E25" s="16"/>
       <c r="F25" s="17" t="str">
-        <f aca="false">IF(OR(A25="",C25="",AND(D25="",E25="")),"",C25*IF(D25&lt;&gt;"",D25,E25/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D25="",E25=""),"",IF(D25&lt;&gt;"",D25,E25/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G25" s="18" t="str">
         <f aca="false">IF(F25="","",F25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H25" s="19" t="str">
+        <f aca="false">IF(OR(A25="",C25="",F25=""),"",C25*F25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="18" t="str">
+        <f aca="false">IF(H25="","",H25*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1268,11 +1422,19 @@
       <c r="D26" s="15"/>
       <c r="E26" s="16"/>
       <c r="F26" s="17" t="str">
-        <f aca="false">IF(OR(A26="",C26="",AND(D26="",E26="")),"",C26*IF(D26&lt;&gt;"",D26,E26/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D26="",E26=""),"",IF(D26&lt;&gt;"",D26,E26/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G26" s="18" t="str">
         <f aca="false">IF(F26="","",F26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H26" s="19" t="str">
+        <f aca="false">IF(OR(A26="",C26="",F26=""),"",C26*F26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="18" t="str">
+        <f aca="false">IF(H26="","",H26*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1283,11 +1445,19 @@
       <c r="D27" s="15"/>
       <c r="E27" s="16"/>
       <c r="F27" s="17" t="str">
-        <f aca="false">IF(OR(A27="",C27="",AND(D27="",E27="")),"",C27*IF(D27&lt;&gt;"",D27,E27/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D27="",E27=""),"",IF(D27&lt;&gt;"",D27,E27/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G27" s="18" t="str">
         <f aca="false">IF(F27="","",F27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H27" s="19" t="str">
+        <f aca="false">IF(OR(A27="",C27="",F27=""),"",C27*F27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="18" t="str">
+        <f aca="false">IF(H27="","",H27*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1298,11 +1468,19 @@
       <c r="D28" s="15"/>
       <c r="E28" s="16"/>
       <c r="F28" s="17" t="str">
-        <f aca="false">IF(OR(A28="",C28="",AND(D28="",E28="")),"",C28*IF(D28&lt;&gt;"",D28,E28/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D28="",E28=""),"",IF(D28&lt;&gt;"",D28,E28/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G28" s="18" t="str">
         <f aca="false">IF(F28="","",F28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H28" s="19" t="str">
+        <f aca="false">IF(OR(A28="",C28="",F28=""),"",C28*F28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="18" t="str">
+        <f aca="false">IF(H28="","",H28*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1313,11 +1491,19 @@
       <c r="D29" s="15"/>
       <c r="E29" s="16"/>
       <c r="F29" s="17" t="str">
-        <f aca="false">IF(OR(A29="",C29="",AND(D29="",E29="")),"",C29*IF(D29&lt;&gt;"",D29,E29/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D29="",E29=""),"",IF(D29&lt;&gt;"",D29,E29/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G29" s="18" t="str">
         <f aca="false">IF(F29="","",F29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H29" s="19" t="str">
+        <f aca="false">IF(OR(A29="",C29="",F29=""),"",C29*F29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="18" t="str">
+        <f aca="false">IF(H29="","",H29*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1328,11 +1514,19 @@
       <c r="D30" s="15"/>
       <c r="E30" s="16"/>
       <c r="F30" s="17" t="str">
-        <f aca="false">IF(OR(A30="",C30="",AND(D30="",E30="")),"",C30*IF(D30&lt;&gt;"",D30,E30/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D30="",E30=""),"",IF(D30&lt;&gt;"",D30,E30/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G30" s="18" t="str">
         <f aca="false">IF(F30="","",F30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H30" s="19" t="str">
+        <f aca="false">IF(OR(A30="",C30="",F30=""),"",C30*F30)</f>
+        <v/>
+      </c>
+      <c r="I30" s="18" t="str">
+        <f aca="false">IF(H30="","",H30*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1343,11 +1537,19 @@
       <c r="D31" s="15"/>
       <c r="E31" s="16"/>
       <c r="F31" s="17" t="str">
-        <f aca="false">IF(OR(A31="",C31="",AND(D31="",E31="")),"",C31*IF(D31&lt;&gt;"",D31,E31/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D31="",E31=""),"",IF(D31&lt;&gt;"",D31,E31/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G31" s="18" t="str">
         <f aca="false">IF(F31="","",F31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H31" s="19" t="str">
+        <f aca="false">IF(OR(A31="",C31="",F31=""),"",C31*F31)</f>
+        <v/>
+      </c>
+      <c r="I31" s="18" t="str">
+        <f aca="false">IF(H31="","",H31*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1358,11 +1560,19 @@
       <c r="D32" s="15"/>
       <c r="E32" s="16"/>
       <c r="F32" s="17" t="str">
-        <f aca="false">IF(OR(A32="",C32="",AND(D32="",E32="")),"",C32*IF(D32&lt;&gt;"",D32,E32/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D32="",E32=""),"",IF(D32&lt;&gt;"",D32,E32/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G32" s="18" t="str">
         <f aca="false">IF(F32="","",F32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H32" s="19" t="str">
+        <f aca="false">IF(OR(A32="",C32="",F32=""),"",C32*F32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="18" t="str">
+        <f aca="false">IF(H32="","",H32*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1373,11 +1583,19 @@
       <c r="D33" s="15"/>
       <c r="E33" s="16"/>
       <c r="F33" s="17" t="str">
-        <f aca="false">IF(OR(A33="",C33="",AND(D33="",E33="")),"",C33*IF(D33&lt;&gt;"",D33,E33/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D33="",E33=""),"",IF(D33&lt;&gt;"",D33,E33/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G33" s="18" t="str">
         <f aca="false">IF(F33="","",F33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H33" s="19" t="str">
+        <f aca="false">IF(OR(A33="",C33="",F33=""),"",C33*F33)</f>
+        <v/>
+      </c>
+      <c r="I33" s="18" t="str">
+        <f aca="false">IF(H33="","",H33*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1388,11 +1606,19 @@
       <c r="D34" s="15"/>
       <c r="E34" s="16"/>
       <c r="F34" s="17" t="str">
-        <f aca="false">IF(OR(A34="",C34="",AND(D34="",E34="")),"",C34*IF(D34&lt;&gt;"",D34,E34/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D34="",E34=""),"",IF(D34&lt;&gt;"",D34,E34/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G34" s="18" t="str">
         <f aca="false">IF(F34="","",F34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H34" s="19" t="str">
+        <f aca="false">IF(OR(A34="",C34="",F34=""),"",C34*F34)</f>
+        <v/>
+      </c>
+      <c r="I34" s="18" t="str">
+        <f aca="false">IF(H34="","",H34*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1403,11 +1629,19 @@
       <c r="D35" s="15"/>
       <c r="E35" s="16"/>
       <c r="F35" s="17" t="str">
-        <f aca="false">IF(OR(A35="",C35="",AND(D35="",E35="")),"",C35*IF(D35&lt;&gt;"",D35,E35/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D35="",E35=""),"",IF(D35&lt;&gt;"",D35,E35/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G35" s="18" t="str">
         <f aca="false">IF(F35="","",F35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H35" s="19" t="str">
+        <f aca="false">IF(OR(A35="",C35="",F35=""),"",C35*F35)</f>
+        <v/>
+      </c>
+      <c r="I35" s="18" t="str">
+        <f aca="false">IF(H35="","",H35*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1418,11 +1652,19 @@
       <c r="D36" s="15"/>
       <c r="E36" s="16"/>
       <c r="F36" s="17" t="str">
-        <f aca="false">IF(OR(A36="",C36="",AND(D36="",E36="")),"",C36*IF(D36&lt;&gt;"",D36,E36/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D36="",E36=""),"",IF(D36&lt;&gt;"",D36,E36/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G36" s="18" t="str">
         <f aca="false">IF(F36="","",F36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H36" s="19" t="str">
+        <f aca="false">IF(OR(A36="",C36="",F36=""),"",C36*F36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="18" t="str">
+        <f aca="false">IF(H36="","",H36*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1433,11 +1675,19 @@
       <c r="D37" s="15"/>
       <c r="E37" s="16"/>
       <c r="F37" s="17" t="str">
-        <f aca="false">IF(OR(A37="",C37="",AND(D37="",E37="")),"",C37*IF(D37&lt;&gt;"",D37,E37/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D37="",E37=""),"",IF(D37&lt;&gt;"",D37,E37/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G37" s="18" t="str">
         <f aca="false">IF(F37="","",F37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H37" s="19" t="str">
+        <f aca="false">IF(OR(A37="",C37="",F37=""),"",C37*F37)</f>
+        <v/>
+      </c>
+      <c r="I37" s="18" t="str">
+        <f aca="false">IF(H37="","",H37*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1448,11 +1698,19 @@
       <c r="D38" s="15"/>
       <c r="E38" s="16"/>
       <c r="F38" s="17" t="str">
-        <f aca="false">IF(OR(A38="",C38="",AND(D38="",E38="")),"",C38*IF(D38&lt;&gt;"",D38,E38/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D38="",E38=""),"",IF(D38&lt;&gt;"",D38,E38/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G38" s="18" t="str">
         <f aca="false">IF(F38="","",F38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H38" s="19" t="str">
+        <f aca="false">IF(OR(A38="",C38="",F38=""),"",C38*F38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="18" t="str">
+        <f aca="false">IF(H38="","",H38*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1463,11 +1721,19 @@
       <c r="D39" s="15"/>
       <c r="E39" s="16"/>
       <c r="F39" s="17" t="str">
-        <f aca="false">IF(OR(A39="",C39="",AND(D39="",E39="")),"",C39*IF(D39&lt;&gt;"",D39,E39/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D39="",E39=""),"",IF(D39&lt;&gt;"",D39,E39/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G39" s="18" t="str">
         <f aca="false">IF(F39="","",F39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H39" s="19" t="str">
+        <f aca="false">IF(OR(A39="",C39="",F39=""),"",C39*F39)</f>
+        <v/>
+      </c>
+      <c r="I39" s="18" t="str">
+        <f aca="false">IF(H39="","",H39*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1478,11 +1744,19 @@
       <c r="D40" s="15"/>
       <c r="E40" s="16"/>
       <c r="F40" s="17" t="str">
-        <f aca="false">IF(OR(A40="",C40="",AND(D40="",E40="")),"",C40*IF(D40&lt;&gt;"",D40,E40/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D40="",E40=""),"",IF(D40&lt;&gt;"",D40,E40/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G40" s="18" t="str">
         <f aca="false">IF(F40="","",F40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H40" s="19" t="str">
+        <f aca="false">IF(OR(A40="",C40="",F40=""),"",C40*F40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="18" t="str">
+        <f aca="false">IF(H40="","",H40*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1493,11 +1767,19 @@
       <c r="D41" s="15"/>
       <c r="E41" s="16"/>
       <c r="F41" s="17" t="str">
-        <f aca="false">IF(OR(A41="",C41="",AND(D41="",E41="")),"",C41*IF(D41&lt;&gt;"",D41,E41/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D41="",E41=""),"",IF(D41&lt;&gt;"",D41,E41/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G41" s="18" t="str">
         <f aca="false">IF(F41="","",F41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H41" s="19" t="str">
+        <f aca="false">IF(OR(A41="",C41="",F41=""),"",C41*F41)</f>
+        <v/>
+      </c>
+      <c r="I41" s="18" t="str">
+        <f aca="false">IF(H41="","",H41*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1508,11 +1790,19 @@
       <c r="D42" s="15"/>
       <c r="E42" s="16"/>
       <c r="F42" s="17" t="str">
-        <f aca="false">IF(OR(A42="",C42="",AND(D42="",E42="")),"",C42*IF(D42&lt;&gt;"",D42,E42/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D42="",E42=""),"",IF(D42&lt;&gt;"",D42,E42/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G42" s="18" t="str">
         <f aca="false">IF(F42="","",F42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H42" s="19" t="str">
+        <f aca="false">IF(OR(A42="",C42="",F42=""),"",C42*F42)</f>
+        <v/>
+      </c>
+      <c r="I42" s="18" t="str">
+        <f aca="false">IF(H42="","",H42*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1523,11 +1813,19 @@
       <c r="D43" s="15"/>
       <c r="E43" s="16"/>
       <c r="F43" s="17" t="str">
-        <f aca="false">IF(OR(A43="",C43="",AND(D43="",E43="")),"",C43*IF(D43&lt;&gt;"",D43,E43/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D43="",E43=""),"",IF(D43&lt;&gt;"",D43,E43/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G43" s="18" t="str">
         <f aca="false">IF(F43="","",F43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H43" s="19" t="str">
+        <f aca="false">IF(OR(A43="",C43="",F43=""),"",C43*F43)</f>
+        <v/>
+      </c>
+      <c r="I43" s="18" t="str">
+        <f aca="false">IF(H43="","",H43*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1538,11 +1836,19 @@
       <c r="D44" s="15"/>
       <c r="E44" s="16"/>
       <c r="F44" s="17" t="str">
-        <f aca="false">IF(OR(A44="",C44="",AND(D44="",E44="")),"",C44*IF(D44&lt;&gt;"",D44,E44/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D44="",E44=""),"",IF(D44&lt;&gt;"",D44,E44/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G44" s="18" t="str">
         <f aca="false">IF(F44="","",F44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H44" s="19" t="str">
+        <f aca="false">IF(OR(A44="",C44="",F44=""),"",C44*F44)</f>
+        <v/>
+      </c>
+      <c r="I44" s="18" t="str">
+        <f aca="false">IF(H44="","",H44*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1553,11 +1859,19 @@
       <c r="D45" s="15"/>
       <c r="E45" s="16"/>
       <c r="F45" s="17" t="str">
-        <f aca="false">IF(OR(A45="",C45="",AND(D45="",E45="")),"",C45*IF(D45&lt;&gt;"",D45,E45/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D45="",E45=""),"",IF(D45&lt;&gt;"",D45,E45/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G45" s="18" t="str">
         <f aca="false">IF(F45="","",F45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H45" s="19" t="str">
+        <f aca="false">IF(OR(A45="",C45="",F45=""),"",C45*F45)</f>
+        <v/>
+      </c>
+      <c r="I45" s="18" t="str">
+        <f aca="false">IF(H45="","",H45*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1568,11 +1882,19 @@
       <c r="D46" s="15"/>
       <c r="E46" s="16"/>
       <c r="F46" s="17" t="str">
-        <f aca="false">IF(OR(A46="",C46="",AND(D46="",E46="")),"",C46*IF(D46&lt;&gt;"",D46,E46/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D46="",E46=""),"",IF(D46&lt;&gt;"",D46,E46/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G46" s="18" t="str">
         <f aca="false">IF(F46="","",F46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H46" s="19" t="str">
+        <f aca="false">IF(OR(A46="",C46="",F46=""),"",C46*F46)</f>
+        <v/>
+      </c>
+      <c r="I46" s="18" t="str">
+        <f aca="false">IF(H46="","",H46*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1583,11 +1905,19 @@
       <c r="D47" s="15"/>
       <c r="E47" s="16"/>
       <c r="F47" s="17" t="str">
-        <f aca="false">IF(OR(A47="",C47="",AND(D47="",E47="")),"",C47*IF(D47&lt;&gt;"",D47,E47/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D47="",E47=""),"",IF(D47&lt;&gt;"",D47,E47/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G47" s="18" t="str">
         <f aca="false">IF(F47="","",F47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H47" s="19" t="str">
+        <f aca="false">IF(OR(A47="",C47="",F47=""),"",C47*F47)</f>
+        <v/>
+      </c>
+      <c r="I47" s="18" t="str">
+        <f aca="false">IF(H47="","",H47*'Budget du don'!$G$4)</f>
         <v/>
       </c>
     </row>
@@ -1598,35 +1928,45 @@
       <c r="D48" s="15"/>
       <c r="E48" s="16"/>
       <c r="F48" s="17" t="str">
-        <f aca="false">IF(OR(A48="",C48="",AND(D48="",E48="")),"",C48*IF(D48&lt;&gt;"",D48,E48/'Budget du don'!$G$4))</f>
+        <f aca="false">IF(AND(D48="",E48=""),"",IF(D48&lt;&gt;"",D48,E48/'Budget du don'!$G$4))</f>
         <v/>
       </c>
       <c r="G48" s="18" t="str">
         <f aca="false">IF(F48="","",F48*'Budget du don'!$G$4)</f>
         <v/>
       </c>
+      <c r="H48" s="19" t="str">
+        <f aca="false">IF(OR(A48="",C48="",F48=""),"",C48*F48)</f>
+        <v/>
+      </c>
+      <c r="I48" s="18" t="str">
+        <f aca="false">IF(H48="","",H48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="21" t="n">
-        <f aca="false">SUM(F9:F48)</f>
+      <c r="A49" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B49" s="21"/>
+      <c r="C49" s="21"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="22" t="n">
+        <f aca="false">SUM(H9:H48)</f>
         <v>182.938820684892</v>
       </c>
-      <c r="G49" s="22" t="n">
-        <f aca="false">SUM(G9:G48)</f>
+      <c r="I49" s="23" t="n">
+        <f aca="false">SUM(I9:I48)</f>
         <v>120000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A6:B6"/>
@@ -1672,7 +2012,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1692,7 +2032,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1712,46 +2052,46 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="24" t="n">
         <f aca="false">SUM(F9:F48)</f>
         <v>182.938820684892</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="24" t="n">
+      <c r="B5" s="24"/>
+      <c r="C5" s="25" t="n">
         <f aca="false">SUM(F9:F48)*'Budget du don'!$G$4</f>
         <v>120000</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25" t="n">
+      <c r="D5" s="25"/>
+      <c r="E5" s="26" t="n">
         <f aca="false">SUM(K9:K48)</f>
         <v>195.134742063885</v>
       </c>
-      <c r="F5" s="25"/>
+      <c r="F5" s="26"/>
       <c r="G5" s="10" t="n">
         <f aca="false">SUM(K9:K48)*'Budget du don'!$G$4</f>
         <v>128000</v>
@@ -1762,109 +2102,109 @@
         <v>-12.1959213789929</v>
       </c>
       <c r="J5" s="9"/>
-      <c r="K5" s="26" t="n">
+      <c r="K5" s="27" t="n">
         <f aca="false">IF(SUM(F9:F48)=0,"",SUM(K9:K48)/SUM(F9:F48))</f>
         <v>1.06666666666667</v>
       </c>
-      <c r="L5" s="26"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="28"/>
-      <c r="L7" s="28"/>
-      <c r="M7" s="29" t="s">
+      <c r="A7" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="N7" s="29"/>
-      <c r="O7" s="29"/>
-      <c r="P7" s="29"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+      <c r="L7" s="29"/>
+      <c r="M7" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="30"/>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="30" t="str">
+      <c r="A9" s="31" t="str">
         <f aca="false">IF('Budget du don'!A9="","",'Budget du don'!A9)</f>
         <v>Sac de riz 25 kg</v>
       </c>
-      <c r="B9" s="31" t="str">
+      <c r="B9" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A9="",'Budget du don'!B9=""),"",'Budget du don'!B9)</f>
         <v>sac</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <f aca="false">IF(OR('Budget du don'!A9="",'Budget du don'!C9=""),"",'Budget du don'!C9)</f>
         <v>10</v>
       </c>
-      <c r="D9" s="33" t="n">
-        <f aca="false">IF('Budget du don'!A9="","",IF('Budget du don'!D9&lt;&gt;"",'Budget du don'!D9,IF('Budget du don'!E9&lt;&gt;"",'Budget du don'!E9/'Budget du don'!$G$4,"")))</f>
+      <c r="D9" s="17" t="n">
+        <f aca="false">IF(OR('Budget du don'!A9="",'Budget du don'!F9=""),"",'Budget du don'!F9)</f>
         <v>18.2938820684892</v>
       </c>
       <c r="E9" s="18" t="n">
         <f aca="false">IF(D9="","",D9*'Budget du don'!$G$4)</f>
         <v>12000</v>
       </c>
-      <c r="F9" s="33" t="n">
-        <f aca="false">IF('Budget du don'!F9="","",'Budget du don'!F9)</f>
+      <c r="F9" s="17" t="n">
+        <f aca="false">IF('Budget du don'!H9="","",'Budget du don'!H9)</f>
         <v>182.938820684892</v>
       </c>
       <c r="G9" s="18" t="n">
@@ -1878,7 +2218,7 @@
       <c r="J9" s="16" t="n">
         <v>12800</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="19" t="n">
         <f aca="false">IF(OR(H9="",AND(I9="",J9="")),"",H9*IF(I9&lt;&gt;"",I9,J9/'Budget du don'!$G$4))</f>
         <v>195.134742063885</v>
       </c>
@@ -1886,7 +2226,7 @@
         <f aca="false">IF(K9="","",K9*'Budget du don'!$G$4)</f>
         <v>128000</v>
       </c>
-      <c r="M9" s="33" t="n">
+      <c r="M9" s="17" t="n">
         <f aca="false">IF(OR(F9="",K9=""),"",F9-K9)</f>
         <v>-12.1959213789929</v>
       </c>
@@ -1899,32 +2239,32 @@
         <v>0.0666666666666667</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="str">
+      <c r="A10" s="31" t="str">
         <f aca="false">IF('Budget du don'!A10="","",'Budget du don'!A10)</f>
         <v>Cahier 96 pages</v>
       </c>
-      <c r="B10" s="31" t="str">
+      <c r="B10" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A10="",'Budget du don'!B10=""),"",'Budget du don'!B10)</f>
         <v>pièce</v>
       </c>
-      <c r="C10" s="32" t="str">
+      <c r="C10" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A10="",'Budget du don'!C10=""),"",'Budget du don'!C10)</f>
         <v/>
       </c>
-      <c r="D10" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A10="","",IF('Budget du don'!D10&lt;&gt;"",'Budget du don'!D10,IF('Budget du don'!E10&lt;&gt;"",'Budget du don'!E10/'Budget du don'!$G$4,"")))</f>
+      <c r="D10" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A10="",'Budget du don'!F10=""),"",'Budget du don'!F10)</f>
         <v/>
       </c>
       <c r="E10" s="18" t="str">
         <f aca="false">IF(D10="","",D10*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F10" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F10="","",'Budget du don'!F10)</f>
+      <c r="F10" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H10="","",'Budget du don'!H10)</f>
         <v/>
       </c>
       <c r="G10" s="18" t="str">
@@ -1934,7 +2274,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="15"/>
       <c r="J10" s="16"/>
-      <c r="K10" s="17" t="str">
+      <c r="K10" s="19" t="str">
         <f aca="false">IF(OR(H10="",AND(I10="",J10="")),"",H10*IF(I10&lt;&gt;"",I10,J10/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -1942,7 +2282,7 @@
         <f aca="false">IF(K10="","",K10*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M10" s="33" t="str">
+      <c r="M10" s="17" t="str">
         <f aca="false">IF(OR(F10="",K10=""),"",F10-K10)</f>
         <v/>
       </c>
@@ -1957,28 +2297,28 @@
       <c r="P10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="30" t="str">
+      <c r="A11" s="31" t="str">
         <f aca="false">IF('Budget du don'!A11="","",'Budget du don'!A11)</f>
         <v>Stylo bleu</v>
       </c>
-      <c r="B11" s="31" t="str">
+      <c r="B11" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A11="",'Budget du don'!B11=""),"",'Budget du don'!B11)</f>
         <v>pièce</v>
       </c>
-      <c r="C11" s="32" t="str">
+      <c r="C11" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A11="",'Budget du don'!C11=""),"",'Budget du don'!C11)</f>
         <v/>
       </c>
-      <c r="D11" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A11="","",IF('Budget du don'!D11&lt;&gt;"",'Budget du don'!D11,IF('Budget du don'!E11&lt;&gt;"",'Budget du don'!E11/'Budget du don'!$G$4,"")))</f>
+      <c r="D11" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A11="",'Budget du don'!F11=""),"",'Budget du don'!F11)</f>
         <v/>
       </c>
       <c r="E11" s="18" t="str">
         <f aca="false">IF(D11="","",D11*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F11" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F11="","",'Budget du don'!F11)</f>
+      <c r="F11" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H11="","",'Budget du don'!H11)</f>
         <v/>
       </c>
       <c r="G11" s="18" t="str">
@@ -1988,7 +2328,7 @@
       <c r="H11" s="14"/>
       <c r="I11" s="15"/>
       <c r="J11" s="16"/>
-      <c r="K11" s="17" t="str">
+      <c r="K11" s="19" t="str">
         <f aca="false">IF(OR(H11="",AND(I11="",J11="")),"",H11*IF(I11&lt;&gt;"",I11,J11/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -1996,7 +2336,7 @@
         <f aca="false">IF(K11="","",K11*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M11" s="33" t="str">
+      <c r="M11" s="17" t="str">
         <f aca="false">IF(OR(F11="",K11=""),"",F11-K11)</f>
         <v/>
       </c>
@@ -2011,28 +2351,28 @@
       <c r="P11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="30" t="str">
+      <c r="A12" s="31" t="str">
         <f aca="false">IF('Budget du don'!A12="","",'Budget du don'!A12)</f>
         <v>Cartable</v>
       </c>
-      <c r="B12" s="31" t="str">
+      <c r="B12" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A12="",'Budget du don'!B12=""),"",'Budget du don'!B12)</f>
         <v>pièce</v>
       </c>
-      <c r="C12" s="32" t="str">
+      <c r="C12" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A12="",'Budget du don'!C12=""),"",'Budget du don'!C12)</f>
         <v/>
       </c>
-      <c r="D12" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A12="","",IF('Budget du don'!D12&lt;&gt;"",'Budget du don'!D12,IF('Budget du don'!E12&lt;&gt;"",'Budget du don'!E12/'Budget du don'!$G$4,"")))</f>
+      <c r="D12" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A12="",'Budget du don'!F12=""),"",'Budget du don'!F12)</f>
         <v/>
       </c>
       <c r="E12" s="18" t="str">
         <f aca="false">IF(D12="","",D12*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F12" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F12="","",'Budget du don'!F12)</f>
+      <c r="F12" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H12="","",'Budget du don'!H12)</f>
         <v/>
       </c>
       <c r="G12" s="18" t="str">
@@ -2042,7 +2382,7 @@
       <c r="H12" s="14"/>
       <c r="I12" s="15"/>
       <c r="J12" s="16"/>
-      <c r="K12" s="17" t="str">
+      <c r="K12" s="19" t="str">
         <f aca="false">IF(OR(H12="",AND(I12="",J12="")),"",H12*IF(I12&lt;&gt;"",I12,J12/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2050,7 +2390,7 @@
         <f aca="false">IF(K12="","",K12*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M12" s="33" t="str">
+      <c r="M12" s="17" t="str">
         <f aca="false">IF(OR(F12="",K12=""),"",F12-K12)</f>
         <v/>
       </c>
@@ -2065,28 +2405,28 @@
       <c r="P12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="30" t="str">
+      <c r="A13" s="31" t="str">
         <f aca="false">IF('Budget du don'!A13="","",'Budget du don'!A13)</f>
         <v>Craie blanche</v>
       </c>
-      <c r="B13" s="31" t="str">
+      <c r="B13" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A13="",'Budget du don'!B13=""),"",'Budget du don'!B13)</f>
         <v>boîte de 100</v>
       </c>
-      <c r="C13" s="32" t="str">
+      <c r="C13" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A13="",'Budget du don'!C13=""),"",'Budget du don'!C13)</f>
         <v/>
       </c>
-      <c r="D13" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A13="","",IF('Budget du don'!D13&lt;&gt;"",'Budget du don'!D13,IF('Budget du don'!E13&lt;&gt;"",'Budget du don'!E13/'Budget du don'!$G$4,"")))</f>
+      <c r="D13" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A13="",'Budget du don'!F13=""),"",'Budget du don'!F13)</f>
         <v/>
       </c>
       <c r="E13" s="18" t="str">
         <f aca="false">IF(D13="","",D13*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F13" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F13="","",'Budget du don'!F13)</f>
+      <c r="F13" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H13="","",'Budget du don'!H13)</f>
         <v/>
       </c>
       <c r="G13" s="18" t="str">
@@ -2096,7 +2436,7 @@
       <c r="H13" s="14"/>
       <c r="I13" s="15"/>
       <c r="J13" s="16"/>
-      <c r="K13" s="17" t="str">
+      <c r="K13" s="19" t="str">
         <f aca="false">IF(OR(H13="",AND(I13="",J13="")),"",H13*IF(I13&lt;&gt;"",I13,J13/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2104,7 +2444,7 @@
         <f aca="false">IF(K13="","",K13*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M13" s="33" t="str">
+      <c r="M13" s="17" t="str">
         <f aca="false">IF(OR(F13="",K13=""),"",F13-K13)</f>
         <v/>
       </c>
@@ -2119,28 +2459,28 @@
       <c r="P13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="str">
+      <c r="A14" s="31" t="str">
         <f aca="false">IF('Budget du don'!A14="","",'Budget du don'!A14)</f>
         <v>Huile végétale</v>
       </c>
-      <c r="B14" s="31" t="str">
+      <c r="B14" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A14="",'Budget du don'!B14=""),"",'Budget du don'!B14)</f>
         <v>bidon 1 L</v>
       </c>
-      <c r="C14" s="32" t="str">
+      <c r="C14" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A14="",'Budget du don'!C14=""),"",'Budget du don'!C14)</f>
         <v/>
       </c>
-      <c r="D14" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A14="","",IF('Budget du don'!D14&lt;&gt;"",'Budget du don'!D14,IF('Budget du don'!E14&lt;&gt;"",'Budget du don'!E14/'Budget du don'!$G$4,"")))</f>
+      <c r="D14" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A14="",'Budget du don'!F14=""),"",'Budget du don'!F14)</f>
         <v/>
       </c>
       <c r="E14" s="18" t="str">
         <f aca="false">IF(D14="","",D14*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F14" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F14="","",'Budget du don'!F14)</f>
+      <c r="F14" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H14="","",'Budget du don'!H14)</f>
         <v/>
       </c>
       <c r="G14" s="18" t="str">
@@ -2150,7 +2490,7 @@
       <c r="H14" s="14"/>
       <c r="I14" s="15"/>
       <c r="J14" s="16"/>
-      <c r="K14" s="17" t="str">
+      <c r="K14" s="19" t="str">
         <f aca="false">IF(OR(H14="",AND(I14="",J14="")),"",H14*IF(I14&lt;&gt;"",I14,J14/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2158,7 +2498,7 @@
         <f aca="false">IF(K14="","",K14*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M14" s="33" t="str">
+      <c r="M14" s="17" t="str">
         <f aca="false">IF(OR(F14="",K14=""),"",F14-K14)</f>
         <v/>
       </c>
@@ -2173,28 +2513,28 @@
       <c r="P14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30" t="str">
+      <c r="A15" s="31" t="str">
         <f aca="false">IF('Budget du don'!A15="","",'Budget du don'!A15)</f>
         <v>Savon</v>
       </c>
-      <c r="B15" s="31" t="str">
+      <c r="B15" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A15="",'Budget du don'!B15=""),"",'Budget du don'!B15)</f>
         <v>pièce</v>
       </c>
-      <c r="C15" s="32" t="str">
+      <c r="C15" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A15="",'Budget du don'!C15=""),"",'Budget du don'!C15)</f>
         <v/>
       </c>
-      <c r="D15" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A15="","",IF('Budget du don'!D15&lt;&gt;"",'Budget du don'!D15,IF('Budget du don'!E15&lt;&gt;"",'Budget du don'!E15/'Budget du don'!$G$4,"")))</f>
+      <c r="D15" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A15="",'Budget du don'!F15=""),"",'Budget du don'!F15)</f>
         <v/>
       </c>
       <c r="E15" s="18" t="str">
         <f aca="false">IF(D15="","",D15*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F15" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F15="","",'Budget du don'!F15)</f>
+      <c r="F15" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H15="","",'Budget du don'!H15)</f>
         <v/>
       </c>
       <c r="G15" s="18" t="str">
@@ -2204,7 +2544,7 @@
       <c r="H15" s="14"/>
       <c r="I15" s="15"/>
       <c r="J15" s="16"/>
-      <c r="K15" s="17" t="str">
+      <c r="K15" s="19" t="str">
         <f aca="false">IF(OR(H15="",AND(I15="",J15="")),"",H15*IF(I15&lt;&gt;"",I15,J15/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2212,7 +2552,7 @@
         <f aca="false">IF(K15="","",K15*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M15" s="33" t="str">
+      <c r="M15" s="17" t="str">
         <f aca="false">IF(OR(F15="",K15=""),"",F15-K15)</f>
         <v/>
       </c>
@@ -2227,28 +2567,28 @@
       <c r="P15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30" t="str">
+      <c r="A16" s="31" t="str">
         <f aca="false">IF('Budget du don'!A16="","",'Budget du don'!A16)</f>
         <v>Vêtements enfant</v>
       </c>
-      <c r="B16" s="31" t="str">
+      <c r="B16" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A16="",'Budget du don'!B16=""),"",'Budget du don'!B16)</f>
         <v>lot</v>
       </c>
-      <c r="C16" s="32" t="str">
+      <c r="C16" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A16="",'Budget du don'!C16=""),"",'Budget du don'!C16)</f>
         <v/>
       </c>
-      <c r="D16" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A16="","",IF('Budget du don'!D16&lt;&gt;"",'Budget du don'!D16,IF('Budget du don'!E16&lt;&gt;"",'Budget du don'!E16/'Budget du don'!$G$4,"")))</f>
+      <c r="D16" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A16="",'Budget du don'!F16=""),"",'Budget du don'!F16)</f>
         <v/>
       </c>
       <c r="E16" s="18" t="str">
         <f aca="false">IF(D16="","",D16*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F16" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F16="","",'Budget du don'!F16)</f>
+      <c r="F16" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H16="","",'Budget du don'!H16)</f>
         <v/>
       </c>
       <c r="G16" s="18" t="str">
@@ -2258,7 +2598,7 @@
       <c r="H16" s="14"/>
       <c r="I16" s="15"/>
       <c r="J16" s="16"/>
-      <c r="K16" s="17" t="str">
+      <c r="K16" s="19" t="str">
         <f aca="false">IF(OR(H16="",AND(I16="",J16="")),"",H16*IF(I16&lt;&gt;"",I16,J16/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2266,7 +2606,7 @@
         <f aca="false">IF(K16="","",K16*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M16" s="33" t="str">
+      <c r="M16" s="17" t="str">
         <f aca="false">IF(OR(F16="",K16=""),"",F16-K16)</f>
         <v/>
       </c>
@@ -2281,28 +2621,28 @@
       <c r="P16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="30" t="str">
+      <c r="A17" s="31" t="str">
         <f aca="false">IF('Budget du don'!A17="","",'Budget du don'!A17)</f>
         <v/>
       </c>
-      <c r="B17" s="31" t="str">
+      <c r="B17" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A17="",'Budget du don'!B17=""),"",'Budget du don'!B17)</f>
         <v/>
       </c>
-      <c r="C17" s="32" t="str">
+      <c r="C17" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A17="",'Budget du don'!C17=""),"",'Budget du don'!C17)</f>
         <v/>
       </c>
-      <c r="D17" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A17="","",IF('Budget du don'!D17&lt;&gt;"",'Budget du don'!D17,IF('Budget du don'!E17&lt;&gt;"",'Budget du don'!E17/'Budget du don'!$G$4,"")))</f>
+      <c r="D17" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A17="",'Budget du don'!F17=""),"",'Budget du don'!F17)</f>
         <v/>
       </c>
       <c r="E17" s="18" t="str">
         <f aca="false">IF(D17="","",D17*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F17" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F17="","",'Budget du don'!F17)</f>
+      <c r="F17" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H17="","",'Budget du don'!H17)</f>
         <v/>
       </c>
       <c r="G17" s="18" t="str">
@@ -2312,7 +2652,7 @@
       <c r="H17" s="14"/>
       <c r="I17" s="15"/>
       <c r="J17" s="16"/>
-      <c r="K17" s="17" t="str">
+      <c r="K17" s="19" t="str">
         <f aca="false">IF(OR(H17="",AND(I17="",J17="")),"",H17*IF(I17&lt;&gt;"",I17,J17/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2320,7 +2660,7 @@
         <f aca="false">IF(K17="","",K17*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M17" s="33" t="str">
+      <c r="M17" s="17" t="str">
         <f aca="false">IF(OR(F17="",K17=""),"",F17-K17)</f>
         <v/>
       </c>
@@ -2335,28 +2675,28 @@
       <c r="P17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="30" t="str">
+      <c r="A18" s="31" t="str">
         <f aca="false">IF('Budget du don'!A18="","",'Budget du don'!A18)</f>
         <v/>
       </c>
-      <c r="B18" s="31" t="str">
+      <c r="B18" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A18="",'Budget du don'!B18=""),"",'Budget du don'!B18)</f>
         <v/>
       </c>
-      <c r="C18" s="32" t="str">
+      <c r="C18" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A18="",'Budget du don'!C18=""),"",'Budget du don'!C18)</f>
         <v/>
       </c>
-      <c r="D18" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A18="","",IF('Budget du don'!D18&lt;&gt;"",'Budget du don'!D18,IF('Budget du don'!E18&lt;&gt;"",'Budget du don'!E18/'Budget du don'!$G$4,"")))</f>
+      <c r="D18" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A18="",'Budget du don'!F18=""),"",'Budget du don'!F18)</f>
         <v/>
       </c>
       <c r="E18" s="18" t="str">
         <f aca="false">IF(D18="","",D18*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F18" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F18="","",'Budget du don'!F18)</f>
+      <c r="F18" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H18="","",'Budget du don'!H18)</f>
         <v/>
       </c>
       <c r="G18" s="18" t="str">
@@ -2366,7 +2706,7 @@
       <c r="H18" s="14"/>
       <c r="I18" s="15"/>
       <c r="J18" s="16"/>
-      <c r="K18" s="17" t="str">
+      <c r="K18" s="19" t="str">
         <f aca="false">IF(OR(H18="",AND(I18="",J18="")),"",H18*IF(I18&lt;&gt;"",I18,J18/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2374,7 +2714,7 @@
         <f aca="false">IF(K18="","",K18*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M18" s="33" t="str">
+      <c r="M18" s="17" t="str">
         <f aca="false">IF(OR(F18="",K18=""),"",F18-K18)</f>
         <v/>
       </c>
@@ -2389,28 +2729,28 @@
       <c r="P18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="str">
+      <c r="A19" s="31" t="str">
         <f aca="false">IF('Budget du don'!A19="","",'Budget du don'!A19)</f>
         <v/>
       </c>
-      <c r="B19" s="31" t="str">
+      <c r="B19" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A19="",'Budget du don'!B19=""),"",'Budget du don'!B19)</f>
         <v/>
       </c>
-      <c r="C19" s="32" t="str">
+      <c r="C19" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A19="",'Budget du don'!C19=""),"",'Budget du don'!C19)</f>
         <v/>
       </c>
-      <c r="D19" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A19="","",IF('Budget du don'!D19&lt;&gt;"",'Budget du don'!D19,IF('Budget du don'!E19&lt;&gt;"",'Budget du don'!E19/'Budget du don'!$G$4,"")))</f>
+      <c r="D19" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A19="",'Budget du don'!F19=""),"",'Budget du don'!F19)</f>
         <v/>
       </c>
       <c r="E19" s="18" t="str">
         <f aca="false">IF(D19="","",D19*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F19" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F19="","",'Budget du don'!F19)</f>
+      <c r="F19" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H19="","",'Budget du don'!H19)</f>
         <v/>
       </c>
       <c r="G19" s="18" t="str">
@@ -2420,7 +2760,7 @@
       <c r="H19" s="14"/>
       <c r="I19" s="15"/>
       <c r="J19" s="16"/>
-      <c r="K19" s="17" t="str">
+      <c r="K19" s="19" t="str">
         <f aca="false">IF(OR(H19="",AND(I19="",J19="")),"",H19*IF(I19&lt;&gt;"",I19,J19/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2428,7 +2768,7 @@
         <f aca="false">IF(K19="","",K19*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M19" s="33" t="str">
+      <c r="M19" s="17" t="str">
         <f aca="false">IF(OR(F19="",K19=""),"",F19-K19)</f>
         <v/>
       </c>
@@ -2443,28 +2783,28 @@
       <c r="P19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="str">
+      <c r="A20" s="31" t="str">
         <f aca="false">IF('Budget du don'!A20="","",'Budget du don'!A20)</f>
         <v/>
       </c>
-      <c r="B20" s="31" t="str">
+      <c r="B20" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A20="",'Budget du don'!B20=""),"",'Budget du don'!B20)</f>
         <v/>
       </c>
-      <c r="C20" s="32" t="str">
+      <c r="C20" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A20="",'Budget du don'!C20=""),"",'Budget du don'!C20)</f>
         <v/>
       </c>
-      <c r="D20" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A20="","",IF('Budget du don'!D20&lt;&gt;"",'Budget du don'!D20,IF('Budget du don'!E20&lt;&gt;"",'Budget du don'!E20/'Budget du don'!$G$4,"")))</f>
+      <c r="D20" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A20="",'Budget du don'!F20=""),"",'Budget du don'!F20)</f>
         <v/>
       </c>
       <c r="E20" s="18" t="str">
         <f aca="false">IF(D20="","",D20*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F20" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F20="","",'Budget du don'!F20)</f>
+      <c r="F20" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H20="","",'Budget du don'!H20)</f>
         <v/>
       </c>
       <c r="G20" s="18" t="str">
@@ -2474,7 +2814,7 @@
       <c r="H20" s="14"/>
       <c r="I20" s="15"/>
       <c r="J20" s="16"/>
-      <c r="K20" s="17" t="str">
+      <c r="K20" s="19" t="str">
         <f aca="false">IF(OR(H20="",AND(I20="",J20="")),"",H20*IF(I20&lt;&gt;"",I20,J20/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2482,7 +2822,7 @@
         <f aca="false">IF(K20="","",K20*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M20" s="33" t="str">
+      <c r="M20" s="17" t="str">
         <f aca="false">IF(OR(F20="",K20=""),"",F20-K20)</f>
         <v/>
       </c>
@@ -2497,28 +2837,28 @@
       <c r="P20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="str">
+      <c r="A21" s="31" t="str">
         <f aca="false">IF('Budget du don'!A21="","",'Budget du don'!A21)</f>
         <v/>
       </c>
-      <c r="B21" s="31" t="str">
+      <c r="B21" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A21="",'Budget du don'!B21=""),"",'Budget du don'!B21)</f>
         <v/>
       </c>
-      <c r="C21" s="32" t="str">
+      <c r="C21" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A21="",'Budget du don'!C21=""),"",'Budget du don'!C21)</f>
         <v/>
       </c>
-      <c r="D21" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A21="","",IF('Budget du don'!D21&lt;&gt;"",'Budget du don'!D21,IF('Budget du don'!E21&lt;&gt;"",'Budget du don'!E21/'Budget du don'!$G$4,"")))</f>
+      <c r="D21" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A21="",'Budget du don'!F21=""),"",'Budget du don'!F21)</f>
         <v/>
       </c>
       <c r="E21" s="18" t="str">
         <f aca="false">IF(D21="","",D21*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F21" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F21="","",'Budget du don'!F21)</f>
+      <c r="F21" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H21="","",'Budget du don'!H21)</f>
         <v/>
       </c>
       <c r="G21" s="18" t="str">
@@ -2528,7 +2868,7 @@
       <c r="H21" s="14"/>
       <c r="I21" s="15"/>
       <c r="J21" s="16"/>
-      <c r="K21" s="17" t="str">
+      <c r="K21" s="19" t="str">
         <f aca="false">IF(OR(H21="",AND(I21="",J21="")),"",H21*IF(I21&lt;&gt;"",I21,J21/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2536,7 +2876,7 @@
         <f aca="false">IF(K21="","",K21*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M21" s="33" t="str">
+      <c r="M21" s="17" t="str">
         <f aca="false">IF(OR(F21="",K21=""),"",F21-K21)</f>
         <v/>
       </c>
@@ -2551,28 +2891,28 @@
       <c r="P21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="str">
+      <c r="A22" s="31" t="str">
         <f aca="false">IF('Budget du don'!A22="","",'Budget du don'!A22)</f>
         <v/>
       </c>
-      <c r="B22" s="31" t="str">
+      <c r="B22" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A22="",'Budget du don'!B22=""),"",'Budget du don'!B22)</f>
         <v/>
       </c>
-      <c r="C22" s="32" t="str">
+      <c r="C22" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A22="",'Budget du don'!C22=""),"",'Budget du don'!C22)</f>
         <v/>
       </c>
-      <c r="D22" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A22="","",IF('Budget du don'!D22&lt;&gt;"",'Budget du don'!D22,IF('Budget du don'!E22&lt;&gt;"",'Budget du don'!E22/'Budget du don'!$G$4,"")))</f>
+      <c r="D22" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A22="",'Budget du don'!F22=""),"",'Budget du don'!F22)</f>
         <v/>
       </c>
       <c r="E22" s="18" t="str">
         <f aca="false">IF(D22="","",D22*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F22" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F22="","",'Budget du don'!F22)</f>
+      <c r="F22" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H22="","",'Budget du don'!H22)</f>
         <v/>
       </c>
       <c r="G22" s="18" t="str">
@@ -2582,7 +2922,7 @@
       <c r="H22" s="14"/>
       <c r="I22" s="15"/>
       <c r="J22" s="16"/>
-      <c r="K22" s="17" t="str">
+      <c r="K22" s="19" t="str">
         <f aca="false">IF(OR(H22="",AND(I22="",J22="")),"",H22*IF(I22&lt;&gt;"",I22,J22/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2590,7 +2930,7 @@
         <f aca="false">IF(K22="","",K22*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M22" s="33" t="str">
+      <c r="M22" s="17" t="str">
         <f aca="false">IF(OR(F22="",K22=""),"",F22-K22)</f>
         <v/>
       </c>
@@ -2605,28 +2945,28 @@
       <c r="P22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30" t="str">
+      <c r="A23" s="31" t="str">
         <f aca="false">IF('Budget du don'!A23="","",'Budget du don'!A23)</f>
         <v/>
       </c>
-      <c r="B23" s="31" t="str">
+      <c r="B23" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A23="",'Budget du don'!B23=""),"",'Budget du don'!B23)</f>
         <v/>
       </c>
-      <c r="C23" s="32" t="str">
+      <c r="C23" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A23="",'Budget du don'!C23=""),"",'Budget du don'!C23)</f>
         <v/>
       </c>
-      <c r="D23" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A23="","",IF('Budget du don'!D23&lt;&gt;"",'Budget du don'!D23,IF('Budget du don'!E23&lt;&gt;"",'Budget du don'!E23/'Budget du don'!$G$4,"")))</f>
+      <c r="D23" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A23="",'Budget du don'!F23=""),"",'Budget du don'!F23)</f>
         <v/>
       </c>
       <c r="E23" s="18" t="str">
         <f aca="false">IF(D23="","",D23*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F23" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F23="","",'Budget du don'!F23)</f>
+      <c r="F23" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H23="","",'Budget du don'!H23)</f>
         <v/>
       </c>
       <c r="G23" s="18" t="str">
@@ -2636,7 +2976,7 @@
       <c r="H23" s="14"/>
       <c r="I23" s="15"/>
       <c r="J23" s="16"/>
-      <c r="K23" s="17" t="str">
+      <c r="K23" s="19" t="str">
         <f aca="false">IF(OR(H23="",AND(I23="",J23="")),"",H23*IF(I23&lt;&gt;"",I23,J23/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2644,7 +2984,7 @@
         <f aca="false">IF(K23="","",K23*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M23" s="33" t="str">
+      <c r="M23" s="17" t="str">
         <f aca="false">IF(OR(F23="",K23=""),"",F23-K23)</f>
         <v/>
       </c>
@@ -2659,28 +2999,28 @@
       <c r="P23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="30" t="str">
+      <c r="A24" s="31" t="str">
         <f aca="false">IF('Budget du don'!A24="","",'Budget du don'!A24)</f>
         <v/>
       </c>
-      <c r="B24" s="31" t="str">
+      <c r="B24" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A24="",'Budget du don'!B24=""),"",'Budget du don'!B24)</f>
         <v/>
       </c>
-      <c r="C24" s="32" t="str">
+      <c r="C24" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A24="",'Budget du don'!C24=""),"",'Budget du don'!C24)</f>
         <v/>
       </c>
-      <c r="D24" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A24="","",IF('Budget du don'!D24&lt;&gt;"",'Budget du don'!D24,IF('Budget du don'!E24&lt;&gt;"",'Budget du don'!E24/'Budget du don'!$G$4,"")))</f>
+      <c r="D24" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A24="",'Budget du don'!F24=""),"",'Budget du don'!F24)</f>
         <v/>
       </c>
       <c r="E24" s="18" t="str">
         <f aca="false">IF(D24="","",D24*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F24" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F24="","",'Budget du don'!F24)</f>
+      <c r="F24" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H24="","",'Budget du don'!H24)</f>
         <v/>
       </c>
       <c r="G24" s="18" t="str">
@@ -2690,7 +3030,7 @@
       <c r="H24" s="14"/>
       <c r="I24" s="15"/>
       <c r="J24" s="16"/>
-      <c r="K24" s="17" t="str">
+      <c r="K24" s="19" t="str">
         <f aca="false">IF(OR(H24="",AND(I24="",J24="")),"",H24*IF(I24&lt;&gt;"",I24,J24/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2698,7 +3038,7 @@
         <f aca="false">IF(K24="","",K24*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M24" s="33" t="str">
+      <c r="M24" s="17" t="str">
         <f aca="false">IF(OR(F24="",K24=""),"",F24-K24)</f>
         <v/>
       </c>
@@ -2713,28 +3053,28 @@
       <c r="P24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="30" t="str">
+      <c r="A25" s="31" t="str">
         <f aca="false">IF('Budget du don'!A25="","",'Budget du don'!A25)</f>
         <v/>
       </c>
-      <c r="B25" s="31" t="str">
+      <c r="B25" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A25="",'Budget du don'!B25=""),"",'Budget du don'!B25)</f>
         <v/>
       </c>
-      <c r="C25" s="32" t="str">
+      <c r="C25" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A25="",'Budget du don'!C25=""),"",'Budget du don'!C25)</f>
         <v/>
       </c>
-      <c r="D25" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A25="","",IF('Budget du don'!D25&lt;&gt;"",'Budget du don'!D25,IF('Budget du don'!E25&lt;&gt;"",'Budget du don'!E25/'Budget du don'!$G$4,"")))</f>
+      <c r="D25" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A25="",'Budget du don'!F25=""),"",'Budget du don'!F25)</f>
         <v/>
       </c>
       <c r="E25" s="18" t="str">
         <f aca="false">IF(D25="","",D25*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F25" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F25="","",'Budget du don'!F25)</f>
+      <c r="F25" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H25="","",'Budget du don'!H25)</f>
         <v/>
       </c>
       <c r="G25" s="18" t="str">
@@ -2744,7 +3084,7 @@
       <c r="H25" s="14"/>
       <c r="I25" s="15"/>
       <c r="J25" s="16"/>
-      <c r="K25" s="17" t="str">
+      <c r="K25" s="19" t="str">
         <f aca="false">IF(OR(H25="",AND(I25="",J25="")),"",H25*IF(I25&lt;&gt;"",I25,J25/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2752,7 +3092,7 @@
         <f aca="false">IF(K25="","",K25*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M25" s="33" t="str">
+      <c r="M25" s="17" t="str">
         <f aca="false">IF(OR(F25="",K25=""),"",F25-K25)</f>
         <v/>
       </c>
@@ -2767,28 +3107,28 @@
       <c r="P25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="30" t="str">
+      <c r="A26" s="31" t="str">
         <f aca="false">IF('Budget du don'!A26="","",'Budget du don'!A26)</f>
         <v/>
       </c>
-      <c r="B26" s="31" t="str">
+      <c r="B26" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A26="",'Budget du don'!B26=""),"",'Budget du don'!B26)</f>
         <v/>
       </c>
-      <c r="C26" s="32" t="str">
+      <c r="C26" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A26="",'Budget du don'!C26=""),"",'Budget du don'!C26)</f>
         <v/>
       </c>
-      <c r="D26" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A26="","",IF('Budget du don'!D26&lt;&gt;"",'Budget du don'!D26,IF('Budget du don'!E26&lt;&gt;"",'Budget du don'!E26/'Budget du don'!$G$4,"")))</f>
+      <c r="D26" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A26="",'Budget du don'!F26=""),"",'Budget du don'!F26)</f>
         <v/>
       </c>
       <c r="E26" s="18" t="str">
         <f aca="false">IF(D26="","",D26*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F26" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F26="","",'Budget du don'!F26)</f>
+      <c r="F26" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H26="","",'Budget du don'!H26)</f>
         <v/>
       </c>
       <c r="G26" s="18" t="str">
@@ -2798,7 +3138,7 @@
       <c r="H26" s="14"/>
       <c r="I26" s="15"/>
       <c r="J26" s="16"/>
-      <c r="K26" s="17" t="str">
+      <c r="K26" s="19" t="str">
         <f aca="false">IF(OR(H26="",AND(I26="",J26="")),"",H26*IF(I26&lt;&gt;"",I26,J26/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2806,7 +3146,7 @@
         <f aca="false">IF(K26="","",K26*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M26" s="33" t="str">
+      <c r="M26" s="17" t="str">
         <f aca="false">IF(OR(F26="",K26=""),"",F26-K26)</f>
         <v/>
       </c>
@@ -2821,28 +3161,28 @@
       <c r="P26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="30" t="str">
+      <c r="A27" s="31" t="str">
         <f aca="false">IF('Budget du don'!A27="","",'Budget du don'!A27)</f>
         <v/>
       </c>
-      <c r="B27" s="31" t="str">
+      <c r="B27" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A27="",'Budget du don'!B27=""),"",'Budget du don'!B27)</f>
         <v/>
       </c>
-      <c r="C27" s="32" t="str">
+      <c r="C27" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A27="",'Budget du don'!C27=""),"",'Budget du don'!C27)</f>
         <v/>
       </c>
-      <c r="D27" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A27="","",IF('Budget du don'!D27&lt;&gt;"",'Budget du don'!D27,IF('Budget du don'!E27&lt;&gt;"",'Budget du don'!E27/'Budget du don'!$G$4,"")))</f>
+      <c r="D27" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A27="",'Budget du don'!F27=""),"",'Budget du don'!F27)</f>
         <v/>
       </c>
       <c r="E27" s="18" t="str">
         <f aca="false">IF(D27="","",D27*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F27" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F27="","",'Budget du don'!F27)</f>
+      <c r="F27" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H27="","",'Budget du don'!H27)</f>
         <v/>
       </c>
       <c r="G27" s="18" t="str">
@@ -2852,7 +3192,7 @@
       <c r="H27" s="14"/>
       <c r="I27" s="15"/>
       <c r="J27" s="16"/>
-      <c r="K27" s="17" t="str">
+      <c r="K27" s="19" t="str">
         <f aca="false">IF(OR(H27="",AND(I27="",J27="")),"",H27*IF(I27&lt;&gt;"",I27,J27/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2860,7 +3200,7 @@
         <f aca="false">IF(K27="","",K27*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M27" s="33" t="str">
+      <c r="M27" s="17" t="str">
         <f aca="false">IF(OR(F27="",K27=""),"",F27-K27)</f>
         <v/>
       </c>
@@ -2875,28 +3215,28 @@
       <c r="P27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="30" t="str">
+      <c r="A28" s="31" t="str">
         <f aca="false">IF('Budget du don'!A28="","",'Budget du don'!A28)</f>
         <v/>
       </c>
-      <c r="B28" s="31" t="str">
+      <c r="B28" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A28="",'Budget du don'!B28=""),"",'Budget du don'!B28)</f>
         <v/>
       </c>
-      <c r="C28" s="32" t="str">
+      <c r="C28" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A28="",'Budget du don'!C28=""),"",'Budget du don'!C28)</f>
         <v/>
       </c>
-      <c r="D28" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A28="","",IF('Budget du don'!D28&lt;&gt;"",'Budget du don'!D28,IF('Budget du don'!E28&lt;&gt;"",'Budget du don'!E28/'Budget du don'!$G$4,"")))</f>
+      <c r="D28" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A28="",'Budget du don'!F28=""),"",'Budget du don'!F28)</f>
         <v/>
       </c>
       <c r="E28" s="18" t="str">
         <f aca="false">IF(D28="","",D28*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F28" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F28="","",'Budget du don'!F28)</f>
+      <c r="F28" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H28="","",'Budget du don'!H28)</f>
         <v/>
       </c>
       <c r="G28" s="18" t="str">
@@ -2906,7 +3246,7 @@
       <c r="H28" s="14"/>
       <c r="I28" s="15"/>
       <c r="J28" s="16"/>
-      <c r="K28" s="17" t="str">
+      <c r="K28" s="19" t="str">
         <f aca="false">IF(OR(H28="",AND(I28="",J28="")),"",H28*IF(I28&lt;&gt;"",I28,J28/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2914,7 +3254,7 @@
         <f aca="false">IF(K28="","",K28*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M28" s="33" t="str">
+      <c r="M28" s="17" t="str">
         <f aca="false">IF(OR(F28="",K28=""),"",F28-K28)</f>
         <v/>
       </c>
@@ -2929,28 +3269,28 @@
       <c r="P28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30" t="str">
+      <c r="A29" s="31" t="str">
         <f aca="false">IF('Budget du don'!A29="","",'Budget du don'!A29)</f>
         <v/>
       </c>
-      <c r="B29" s="31" t="str">
+      <c r="B29" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A29="",'Budget du don'!B29=""),"",'Budget du don'!B29)</f>
         <v/>
       </c>
-      <c r="C29" s="32" t="str">
+      <c r="C29" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A29="",'Budget du don'!C29=""),"",'Budget du don'!C29)</f>
         <v/>
       </c>
-      <c r="D29" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A29="","",IF('Budget du don'!D29&lt;&gt;"",'Budget du don'!D29,IF('Budget du don'!E29&lt;&gt;"",'Budget du don'!E29/'Budget du don'!$G$4,"")))</f>
+      <c r="D29" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A29="",'Budget du don'!F29=""),"",'Budget du don'!F29)</f>
         <v/>
       </c>
       <c r="E29" s="18" t="str">
         <f aca="false">IF(D29="","",D29*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F29" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F29="","",'Budget du don'!F29)</f>
+      <c r="F29" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H29="","",'Budget du don'!H29)</f>
         <v/>
       </c>
       <c r="G29" s="18" t="str">
@@ -2960,7 +3300,7 @@
       <c r="H29" s="14"/>
       <c r="I29" s="15"/>
       <c r="J29" s="16"/>
-      <c r="K29" s="17" t="str">
+      <c r="K29" s="19" t="str">
         <f aca="false">IF(OR(H29="",AND(I29="",J29="")),"",H29*IF(I29&lt;&gt;"",I29,J29/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -2968,7 +3308,7 @@
         <f aca="false">IF(K29="","",K29*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M29" s="33" t="str">
+      <c r="M29" s="17" t="str">
         <f aca="false">IF(OR(F29="",K29=""),"",F29-K29)</f>
         <v/>
       </c>
@@ -2983,28 +3323,28 @@
       <c r="P29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="30" t="str">
+      <c r="A30" s="31" t="str">
         <f aca="false">IF('Budget du don'!A30="","",'Budget du don'!A30)</f>
         <v/>
       </c>
-      <c r="B30" s="31" t="str">
+      <c r="B30" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A30="",'Budget du don'!B30=""),"",'Budget du don'!B30)</f>
         <v/>
       </c>
-      <c r="C30" s="32" t="str">
+      <c r="C30" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A30="",'Budget du don'!C30=""),"",'Budget du don'!C30)</f>
         <v/>
       </c>
-      <c r="D30" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A30="","",IF('Budget du don'!D30&lt;&gt;"",'Budget du don'!D30,IF('Budget du don'!E30&lt;&gt;"",'Budget du don'!E30/'Budget du don'!$G$4,"")))</f>
+      <c r="D30" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A30="",'Budget du don'!F30=""),"",'Budget du don'!F30)</f>
         <v/>
       </c>
       <c r="E30" s="18" t="str">
         <f aca="false">IF(D30="","",D30*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F30" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F30="","",'Budget du don'!F30)</f>
+      <c r="F30" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H30="","",'Budget du don'!H30)</f>
         <v/>
       </c>
       <c r="G30" s="18" t="str">
@@ -3014,7 +3354,7 @@
       <c r="H30" s="14"/>
       <c r="I30" s="15"/>
       <c r="J30" s="16"/>
-      <c r="K30" s="17" t="str">
+      <c r="K30" s="19" t="str">
         <f aca="false">IF(OR(H30="",AND(I30="",J30="")),"",H30*IF(I30&lt;&gt;"",I30,J30/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3022,7 +3362,7 @@
         <f aca="false">IF(K30="","",K30*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M30" s="33" t="str">
+      <c r="M30" s="17" t="str">
         <f aca="false">IF(OR(F30="",K30=""),"",F30-K30)</f>
         <v/>
       </c>
@@ -3037,28 +3377,28 @@
       <c r="P30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="str">
+      <c r="A31" s="31" t="str">
         <f aca="false">IF('Budget du don'!A31="","",'Budget du don'!A31)</f>
         <v/>
       </c>
-      <c r="B31" s="31" t="str">
+      <c r="B31" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A31="",'Budget du don'!B31=""),"",'Budget du don'!B31)</f>
         <v/>
       </c>
-      <c r="C31" s="32" t="str">
+      <c r="C31" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A31="",'Budget du don'!C31=""),"",'Budget du don'!C31)</f>
         <v/>
       </c>
-      <c r="D31" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A31="","",IF('Budget du don'!D31&lt;&gt;"",'Budget du don'!D31,IF('Budget du don'!E31&lt;&gt;"",'Budget du don'!E31/'Budget du don'!$G$4,"")))</f>
+      <c r="D31" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A31="",'Budget du don'!F31=""),"",'Budget du don'!F31)</f>
         <v/>
       </c>
       <c r="E31" s="18" t="str">
         <f aca="false">IF(D31="","",D31*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F31" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F31="","",'Budget du don'!F31)</f>
+      <c r="F31" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H31="","",'Budget du don'!H31)</f>
         <v/>
       </c>
       <c r="G31" s="18" t="str">
@@ -3068,7 +3408,7 @@
       <c r="H31" s="14"/>
       <c r="I31" s="15"/>
       <c r="J31" s="16"/>
-      <c r="K31" s="17" t="str">
+      <c r="K31" s="19" t="str">
         <f aca="false">IF(OR(H31="",AND(I31="",J31="")),"",H31*IF(I31&lt;&gt;"",I31,J31/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3076,7 +3416,7 @@
         <f aca="false">IF(K31="","",K31*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M31" s="33" t="str">
+      <c r="M31" s="17" t="str">
         <f aca="false">IF(OR(F31="",K31=""),"",F31-K31)</f>
         <v/>
       </c>
@@ -3091,28 +3431,28 @@
       <c r="P31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="30" t="str">
+      <c r="A32" s="31" t="str">
         <f aca="false">IF('Budget du don'!A32="","",'Budget du don'!A32)</f>
         <v/>
       </c>
-      <c r="B32" s="31" t="str">
+      <c r="B32" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A32="",'Budget du don'!B32=""),"",'Budget du don'!B32)</f>
         <v/>
       </c>
-      <c r="C32" s="32" t="str">
+      <c r="C32" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A32="",'Budget du don'!C32=""),"",'Budget du don'!C32)</f>
         <v/>
       </c>
-      <c r="D32" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A32="","",IF('Budget du don'!D32&lt;&gt;"",'Budget du don'!D32,IF('Budget du don'!E32&lt;&gt;"",'Budget du don'!E32/'Budget du don'!$G$4,"")))</f>
+      <c r="D32" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A32="",'Budget du don'!F32=""),"",'Budget du don'!F32)</f>
         <v/>
       </c>
       <c r="E32" s="18" t="str">
         <f aca="false">IF(D32="","",D32*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F32" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F32="","",'Budget du don'!F32)</f>
+      <c r="F32" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H32="","",'Budget du don'!H32)</f>
         <v/>
       </c>
       <c r="G32" s="18" t="str">
@@ -3122,7 +3462,7 @@
       <c r="H32" s="14"/>
       <c r="I32" s="15"/>
       <c r="J32" s="16"/>
-      <c r="K32" s="17" t="str">
+      <c r="K32" s="19" t="str">
         <f aca="false">IF(OR(H32="",AND(I32="",J32="")),"",H32*IF(I32&lt;&gt;"",I32,J32/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3130,7 +3470,7 @@
         <f aca="false">IF(K32="","",K32*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M32" s="33" t="str">
+      <c r="M32" s="17" t="str">
         <f aca="false">IF(OR(F32="",K32=""),"",F32-K32)</f>
         <v/>
       </c>
@@ -3145,28 +3485,28 @@
       <c r="P32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="30" t="str">
+      <c r="A33" s="31" t="str">
         <f aca="false">IF('Budget du don'!A33="","",'Budget du don'!A33)</f>
         <v/>
       </c>
-      <c r="B33" s="31" t="str">
+      <c r="B33" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A33="",'Budget du don'!B33=""),"",'Budget du don'!B33)</f>
         <v/>
       </c>
-      <c r="C33" s="32" t="str">
+      <c r="C33" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A33="",'Budget du don'!C33=""),"",'Budget du don'!C33)</f>
         <v/>
       </c>
-      <c r="D33" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A33="","",IF('Budget du don'!D33&lt;&gt;"",'Budget du don'!D33,IF('Budget du don'!E33&lt;&gt;"",'Budget du don'!E33/'Budget du don'!$G$4,"")))</f>
+      <c r="D33" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A33="",'Budget du don'!F33=""),"",'Budget du don'!F33)</f>
         <v/>
       </c>
       <c r="E33" s="18" t="str">
         <f aca="false">IF(D33="","",D33*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F33" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F33="","",'Budget du don'!F33)</f>
+      <c r="F33" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H33="","",'Budget du don'!H33)</f>
         <v/>
       </c>
       <c r="G33" s="18" t="str">
@@ -3176,7 +3516,7 @@
       <c r="H33" s="14"/>
       <c r="I33" s="15"/>
       <c r="J33" s="16"/>
-      <c r="K33" s="17" t="str">
+      <c r="K33" s="19" t="str">
         <f aca="false">IF(OR(H33="",AND(I33="",J33="")),"",H33*IF(I33&lt;&gt;"",I33,J33/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3184,7 +3524,7 @@
         <f aca="false">IF(K33="","",K33*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M33" s="33" t="str">
+      <c r="M33" s="17" t="str">
         <f aca="false">IF(OR(F33="",K33=""),"",F33-K33)</f>
         <v/>
       </c>
@@ -3199,28 +3539,28 @@
       <c r="P33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="str">
+      <c r="A34" s="31" t="str">
         <f aca="false">IF('Budget du don'!A34="","",'Budget du don'!A34)</f>
         <v/>
       </c>
-      <c r="B34" s="31" t="str">
+      <c r="B34" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A34="",'Budget du don'!B34=""),"",'Budget du don'!B34)</f>
         <v/>
       </c>
-      <c r="C34" s="32" t="str">
+      <c r="C34" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A34="",'Budget du don'!C34=""),"",'Budget du don'!C34)</f>
         <v/>
       </c>
-      <c r="D34" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A34="","",IF('Budget du don'!D34&lt;&gt;"",'Budget du don'!D34,IF('Budget du don'!E34&lt;&gt;"",'Budget du don'!E34/'Budget du don'!$G$4,"")))</f>
+      <c r="D34" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A34="",'Budget du don'!F34=""),"",'Budget du don'!F34)</f>
         <v/>
       </c>
       <c r="E34" s="18" t="str">
         <f aca="false">IF(D34="","",D34*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F34" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F34="","",'Budget du don'!F34)</f>
+      <c r="F34" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H34="","",'Budget du don'!H34)</f>
         <v/>
       </c>
       <c r="G34" s="18" t="str">
@@ -3230,7 +3570,7 @@
       <c r="H34" s="14"/>
       <c r="I34" s="15"/>
       <c r="J34" s="16"/>
-      <c r="K34" s="17" t="str">
+      <c r="K34" s="19" t="str">
         <f aca="false">IF(OR(H34="",AND(I34="",J34="")),"",H34*IF(I34&lt;&gt;"",I34,J34/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3238,7 +3578,7 @@
         <f aca="false">IF(K34="","",K34*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M34" s="33" t="str">
+      <c r="M34" s="17" t="str">
         <f aca="false">IF(OR(F34="",K34=""),"",F34-K34)</f>
         <v/>
       </c>
@@ -3253,28 +3593,28 @@
       <c r="P34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="30" t="str">
+      <c r="A35" s="31" t="str">
         <f aca="false">IF('Budget du don'!A35="","",'Budget du don'!A35)</f>
         <v/>
       </c>
-      <c r="B35" s="31" t="str">
+      <c r="B35" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A35="",'Budget du don'!B35=""),"",'Budget du don'!B35)</f>
         <v/>
       </c>
-      <c r="C35" s="32" t="str">
+      <c r="C35" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A35="",'Budget du don'!C35=""),"",'Budget du don'!C35)</f>
         <v/>
       </c>
-      <c r="D35" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A35="","",IF('Budget du don'!D35&lt;&gt;"",'Budget du don'!D35,IF('Budget du don'!E35&lt;&gt;"",'Budget du don'!E35/'Budget du don'!$G$4,"")))</f>
+      <c r="D35" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A35="",'Budget du don'!F35=""),"",'Budget du don'!F35)</f>
         <v/>
       </c>
       <c r="E35" s="18" t="str">
         <f aca="false">IF(D35="","",D35*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F35" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F35="","",'Budget du don'!F35)</f>
+      <c r="F35" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H35="","",'Budget du don'!H35)</f>
         <v/>
       </c>
       <c r="G35" s="18" t="str">
@@ -3284,7 +3624,7 @@
       <c r="H35" s="14"/>
       <c r="I35" s="15"/>
       <c r="J35" s="16"/>
-      <c r="K35" s="17" t="str">
+      <c r="K35" s="19" t="str">
         <f aca="false">IF(OR(H35="",AND(I35="",J35="")),"",H35*IF(I35&lt;&gt;"",I35,J35/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3292,7 +3632,7 @@
         <f aca="false">IF(K35="","",K35*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M35" s="33" t="str">
+      <c r="M35" s="17" t="str">
         <f aca="false">IF(OR(F35="",K35=""),"",F35-K35)</f>
         <v/>
       </c>
@@ -3307,28 +3647,28 @@
       <c r="P35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="30" t="str">
+      <c r="A36" s="31" t="str">
         <f aca="false">IF('Budget du don'!A36="","",'Budget du don'!A36)</f>
         <v/>
       </c>
-      <c r="B36" s="31" t="str">
+      <c r="B36" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A36="",'Budget du don'!B36=""),"",'Budget du don'!B36)</f>
         <v/>
       </c>
-      <c r="C36" s="32" t="str">
+      <c r="C36" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A36="",'Budget du don'!C36=""),"",'Budget du don'!C36)</f>
         <v/>
       </c>
-      <c r="D36" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A36="","",IF('Budget du don'!D36&lt;&gt;"",'Budget du don'!D36,IF('Budget du don'!E36&lt;&gt;"",'Budget du don'!E36/'Budget du don'!$G$4,"")))</f>
+      <c r="D36" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A36="",'Budget du don'!F36=""),"",'Budget du don'!F36)</f>
         <v/>
       </c>
       <c r="E36" s="18" t="str">
         <f aca="false">IF(D36="","",D36*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F36" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F36="","",'Budget du don'!F36)</f>
+      <c r="F36" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H36="","",'Budget du don'!H36)</f>
         <v/>
       </c>
       <c r="G36" s="18" t="str">
@@ -3338,7 +3678,7 @@
       <c r="H36" s="14"/>
       <c r="I36" s="15"/>
       <c r="J36" s="16"/>
-      <c r="K36" s="17" t="str">
+      <c r="K36" s="19" t="str">
         <f aca="false">IF(OR(H36="",AND(I36="",J36="")),"",H36*IF(I36&lt;&gt;"",I36,J36/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3346,7 +3686,7 @@
         <f aca="false">IF(K36="","",K36*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M36" s="33" t="str">
+      <c r="M36" s="17" t="str">
         <f aca="false">IF(OR(F36="",K36=""),"",F36-K36)</f>
         <v/>
       </c>
@@ -3361,28 +3701,28 @@
       <c r="P36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30" t="str">
+      <c r="A37" s="31" t="str">
         <f aca="false">IF('Budget du don'!A37="","",'Budget du don'!A37)</f>
         <v/>
       </c>
-      <c r="B37" s="31" t="str">
+      <c r="B37" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A37="",'Budget du don'!B37=""),"",'Budget du don'!B37)</f>
         <v/>
       </c>
-      <c r="C37" s="32" t="str">
+      <c r="C37" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A37="",'Budget du don'!C37=""),"",'Budget du don'!C37)</f>
         <v/>
       </c>
-      <c r="D37" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A37="","",IF('Budget du don'!D37&lt;&gt;"",'Budget du don'!D37,IF('Budget du don'!E37&lt;&gt;"",'Budget du don'!E37/'Budget du don'!$G$4,"")))</f>
+      <c r="D37" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A37="",'Budget du don'!F37=""),"",'Budget du don'!F37)</f>
         <v/>
       </c>
       <c r="E37" s="18" t="str">
         <f aca="false">IF(D37="","",D37*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F37" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F37="","",'Budget du don'!F37)</f>
+      <c r="F37" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H37="","",'Budget du don'!H37)</f>
         <v/>
       </c>
       <c r="G37" s="18" t="str">
@@ -3392,7 +3732,7 @@
       <c r="H37" s="14"/>
       <c r="I37" s="15"/>
       <c r="J37" s="16"/>
-      <c r="K37" s="17" t="str">
+      <c r="K37" s="19" t="str">
         <f aca="false">IF(OR(H37="",AND(I37="",J37="")),"",H37*IF(I37&lt;&gt;"",I37,J37/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3400,7 +3740,7 @@
         <f aca="false">IF(K37="","",K37*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M37" s="33" t="str">
+      <c r="M37" s="17" t="str">
         <f aca="false">IF(OR(F37="",K37=""),"",F37-K37)</f>
         <v/>
       </c>
@@ -3415,28 +3755,28 @@
       <c r="P37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="30" t="str">
+      <c r="A38" s="31" t="str">
         <f aca="false">IF('Budget du don'!A38="","",'Budget du don'!A38)</f>
         <v/>
       </c>
-      <c r="B38" s="31" t="str">
+      <c r="B38" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A38="",'Budget du don'!B38=""),"",'Budget du don'!B38)</f>
         <v/>
       </c>
-      <c r="C38" s="32" t="str">
+      <c r="C38" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A38="",'Budget du don'!C38=""),"",'Budget du don'!C38)</f>
         <v/>
       </c>
-      <c r="D38" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A38="","",IF('Budget du don'!D38&lt;&gt;"",'Budget du don'!D38,IF('Budget du don'!E38&lt;&gt;"",'Budget du don'!E38/'Budget du don'!$G$4,"")))</f>
+      <c r="D38" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A38="",'Budget du don'!F38=""),"",'Budget du don'!F38)</f>
         <v/>
       </c>
       <c r="E38" s="18" t="str">
         <f aca="false">IF(D38="","",D38*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F38" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F38="","",'Budget du don'!F38)</f>
+      <c r="F38" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H38="","",'Budget du don'!H38)</f>
         <v/>
       </c>
       <c r="G38" s="18" t="str">
@@ -3446,7 +3786,7 @@
       <c r="H38" s="14"/>
       <c r="I38" s="15"/>
       <c r="J38" s="16"/>
-      <c r="K38" s="17" t="str">
+      <c r="K38" s="19" t="str">
         <f aca="false">IF(OR(H38="",AND(I38="",J38="")),"",H38*IF(I38&lt;&gt;"",I38,J38/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3454,7 +3794,7 @@
         <f aca="false">IF(K38="","",K38*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M38" s="33" t="str">
+      <c r="M38" s="17" t="str">
         <f aca="false">IF(OR(F38="",K38=""),"",F38-K38)</f>
         <v/>
       </c>
@@ -3469,28 +3809,28 @@
       <c r="P38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="30" t="str">
+      <c r="A39" s="31" t="str">
         <f aca="false">IF('Budget du don'!A39="","",'Budget du don'!A39)</f>
         <v/>
       </c>
-      <c r="B39" s="31" t="str">
+      <c r="B39" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A39="",'Budget du don'!B39=""),"",'Budget du don'!B39)</f>
         <v/>
       </c>
-      <c r="C39" s="32" t="str">
+      <c r="C39" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A39="",'Budget du don'!C39=""),"",'Budget du don'!C39)</f>
         <v/>
       </c>
-      <c r="D39" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A39="","",IF('Budget du don'!D39&lt;&gt;"",'Budget du don'!D39,IF('Budget du don'!E39&lt;&gt;"",'Budget du don'!E39/'Budget du don'!$G$4,"")))</f>
+      <c r="D39" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A39="",'Budget du don'!F39=""),"",'Budget du don'!F39)</f>
         <v/>
       </c>
       <c r="E39" s="18" t="str">
         <f aca="false">IF(D39="","",D39*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F39" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F39="","",'Budget du don'!F39)</f>
+      <c r="F39" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H39="","",'Budget du don'!H39)</f>
         <v/>
       </c>
       <c r="G39" s="18" t="str">
@@ -3500,7 +3840,7 @@
       <c r="H39" s="14"/>
       <c r="I39" s="15"/>
       <c r="J39" s="16"/>
-      <c r="K39" s="17" t="str">
+      <c r="K39" s="19" t="str">
         <f aca="false">IF(OR(H39="",AND(I39="",J39="")),"",H39*IF(I39&lt;&gt;"",I39,J39/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3508,7 +3848,7 @@
         <f aca="false">IF(K39="","",K39*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M39" s="33" t="str">
+      <c r="M39" s="17" t="str">
         <f aca="false">IF(OR(F39="",K39=""),"",F39-K39)</f>
         <v/>
       </c>
@@ -3523,28 +3863,28 @@
       <c r="P39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="30" t="str">
+      <c r="A40" s="31" t="str">
         <f aca="false">IF('Budget du don'!A40="","",'Budget du don'!A40)</f>
         <v/>
       </c>
-      <c r="B40" s="31" t="str">
+      <c r="B40" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A40="",'Budget du don'!B40=""),"",'Budget du don'!B40)</f>
         <v/>
       </c>
-      <c r="C40" s="32" t="str">
+      <c r="C40" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A40="",'Budget du don'!C40=""),"",'Budget du don'!C40)</f>
         <v/>
       </c>
-      <c r="D40" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A40="","",IF('Budget du don'!D40&lt;&gt;"",'Budget du don'!D40,IF('Budget du don'!E40&lt;&gt;"",'Budget du don'!E40/'Budget du don'!$G$4,"")))</f>
+      <c r="D40" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A40="",'Budget du don'!F40=""),"",'Budget du don'!F40)</f>
         <v/>
       </c>
       <c r="E40" s="18" t="str">
         <f aca="false">IF(D40="","",D40*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F40" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F40="","",'Budget du don'!F40)</f>
+      <c r="F40" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H40="","",'Budget du don'!H40)</f>
         <v/>
       </c>
       <c r="G40" s="18" t="str">
@@ -3554,7 +3894,7 @@
       <c r="H40" s="14"/>
       <c r="I40" s="15"/>
       <c r="J40" s="16"/>
-      <c r="K40" s="17" t="str">
+      <c r="K40" s="19" t="str">
         <f aca="false">IF(OR(H40="",AND(I40="",J40="")),"",H40*IF(I40&lt;&gt;"",I40,J40/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3562,7 +3902,7 @@
         <f aca="false">IF(K40="","",K40*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M40" s="33" t="str">
+      <c r="M40" s="17" t="str">
         <f aca="false">IF(OR(F40="",K40=""),"",F40-K40)</f>
         <v/>
       </c>
@@ -3577,28 +3917,28 @@
       <c r="P40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="30" t="str">
+      <c r="A41" s="31" t="str">
         <f aca="false">IF('Budget du don'!A41="","",'Budget du don'!A41)</f>
         <v/>
       </c>
-      <c r="B41" s="31" t="str">
+      <c r="B41" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A41="",'Budget du don'!B41=""),"",'Budget du don'!B41)</f>
         <v/>
       </c>
-      <c r="C41" s="32" t="str">
+      <c r="C41" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A41="",'Budget du don'!C41=""),"",'Budget du don'!C41)</f>
         <v/>
       </c>
-      <c r="D41" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A41="","",IF('Budget du don'!D41&lt;&gt;"",'Budget du don'!D41,IF('Budget du don'!E41&lt;&gt;"",'Budget du don'!E41/'Budget du don'!$G$4,"")))</f>
+      <c r="D41" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A41="",'Budget du don'!F41=""),"",'Budget du don'!F41)</f>
         <v/>
       </c>
       <c r="E41" s="18" t="str">
         <f aca="false">IF(D41="","",D41*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F41" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F41="","",'Budget du don'!F41)</f>
+      <c r="F41" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H41="","",'Budget du don'!H41)</f>
         <v/>
       </c>
       <c r="G41" s="18" t="str">
@@ -3608,7 +3948,7 @@
       <c r="H41" s="14"/>
       <c r="I41" s="15"/>
       <c r="J41" s="16"/>
-      <c r="K41" s="17" t="str">
+      <c r="K41" s="19" t="str">
         <f aca="false">IF(OR(H41="",AND(I41="",J41="")),"",H41*IF(I41&lt;&gt;"",I41,J41/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3616,7 +3956,7 @@
         <f aca="false">IF(K41="","",K41*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M41" s="33" t="str">
+      <c r="M41" s="17" t="str">
         <f aca="false">IF(OR(F41="",K41=""),"",F41-K41)</f>
         <v/>
       </c>
@@ -3631,28 +3971,28 @@
       <c r="P41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="30" t="str">
+      <c r="A42" s="31" t="str">
         <f aca="false">IF('Budget du don'!A42="","",'Budget du don'!A42)</f>
         <v/>
       </c>
-      <c r="B42" s="31" t="str">
+      <c r="B42" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A42="",'Budget du don'!B42=""),"",'Budget du don'!B42)</f>
         <v/>
       </c>
-      <c r="C42" s="32" t="str">
+      <c r="C42" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A42="",'Budget du don'!C42=""),"",'Budget du don'!C42)</f>
         <v/>
       </c>
-      <c r="D42" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A42="","",IF('Budget du don'!D42&lt;&gt;"",'Budget du don'!D42,IF('Budget du don'!E42&lt;&gt;"",'Budget du don'!E42/'Budget du don'!$G$4,"")))</f>
+      <c r="D42" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A42="",'Budget du don'!F42=""),"",'Budget du don'!F42)</f>
         <v/>
       </c>
       <c r="E42" s="18" t="str">
         <f aca="false">IF(D42="","",D42*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F42" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F42="","",'Budget du don'!F42)</f>
+      <c r="F42" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H42="","",'Budget du don'!H42)</f>
         <v/>
       </c>
       <c r="G42" s="18" t="str">
@@ -3662,7 +4002,7 @@
       <c r="H42" s="14"/>
       <c r="I42" s="15"/>
       <c r="J42" s="16"/>
-      <c r="K42" s="17" t="str">
+      <c r="K42" s="19" t="str">
         <f aca="false">IF(OR(H42="",AND(I42="",J42="")),"",H42*IF(I42&lt;&gt;"",I42,J42/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3670,7 +4010,7 @@
         <f aca="false">IF(K42="","",K42*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M42" s="33" t="str">
+      <c r="M42" s="17" t="str">
         <f aca="false">IF(OR(F42="",K42=""),"",F42-K42)</f>
         <v/>
       </c>
@@ -3685,28 +4025,28 @@
       <c r="P42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="30" t="str">
+      <c r="A43" s="31" t="str">
         <f aca="false">IF('Budget du don'!A43="","",'Budget du don'!A43)</f>
         <v/>
       </c>
-      <c r="B43" s="31" t="str">
+      <c r="B43" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A43="",'Budget du don'!B43=""),"",'Budget du don'!B43)</f>
         <v/>
       </c>
-      <c r="C43" s="32" t="str">
+      <c r="C43" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A43="",'Budget du don'!C43=""),"",'Budget du don'!C43)</f>
         <v/>
       </c>
-      <c r="D43" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A43="","",IF('Budget du don'!D43&lt;&gt;"",'Budget du don'!D43,IF('Budget du don'!E43&lt;&gt;"",'Budget du don'!E43/'Budget du don'!$G$4,"")))</f>
+      <c r="D43" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A43="",'Budget du don'!F43=""),"",'Budget du don'!F43)</f>
         <v/>
       </c>
       <c r="E43" s="18" t="str">
         <f aca="false">IF(D43="","",D43*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F43" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F43="","",'Budget du don'!F43)</f>
+      <c r="F43" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H43="","",'Budget du don'!H43)</f>
         <v/>
       </c>
       <c r="G43" s="18" t="str">
@@ -3716,7 +4056,7 @@
       <c r="H43" s="14"/>
       <c r="I43" s="15"/>
       <c r="J43" s="16"/>
-      <c r="K43" s="17" t="str">
+      <c r="K43" s="19" t="str">
         <f aca="false">IF(OR(H43="",AND(I43="",J43="")),"",H43*IF(I43&lt;&gt;"",I43,J43/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3724,7 +4064,7 @@
         <f aca="false">IF(K43="","",K43*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M43" s="33" t="str">
+      <c r="M43" s="17" t="str">
         <f aca="false">IF(OR(F43="",K43=""),"",F43-K43)</f>
         <v/>
       </c>
@@ -3739,28 +4079,28 @@
       <c r="P43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="30" t="str">
+      <c r="A44" s="31" t="str">
         <f aca="false">IF('Budget du don'!A44="","",'Budget du don'!A44)</f>
         <v/>
       </c>
-      <c r="B44" s="31" t="str">
+      <c r="B44" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A44="",'Budget du don'!B44=""),"",'Budget du don'!B44)</f>
         <v/>
       </c>
-      <c r="C44" s="32" t="str">
+      <c r="C44" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A44="",'Budget du don'!C44=""),"",'Budget du don'!C44)</f>
         <v/>
       </c>
-      <c r="D44" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A44="","",IF('Budget du don'!D44&lt;&gt;"",'Budget du don'!D44,IF('Budget du don'!E44&lt;&gt;"",'Budget du don'!E44/'Budget du don'!$G$4,"")))</f>
+      <c r="D44" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A44="",'Budget du don'!F44=""),"",'Budget du don'!F44)</f>
         <v/>
       </c>
       <c r="E44" s="18" t="str">
         <f aca="false">IF(D44="","",D44*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F44" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F44="","",'Budget du don'!F44)</f>
+      <c r="F44" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H44="","",'Budget du don'!H44)</f>
         <v/>
       </c>
       <c r="G44" s="18" t="str">
@@ -3770,7 +4110,7 @@
       <c r="H44" s="14"/>
       <c r="I44" s="15"/>
       <c r="J44" s="16"/>
-      <c r="K44" s="17" t="str">
+      <c r="K44" s="19" t="str">
         <f aca="false">IF(OR(H44="",AND(I44="",J44="")),"",H44*IF(I44&lt;&gt;"",I44,J44/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3778,7 +4118,7 @@
         <f aca="false">IF(K44="","",K44*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M44" s="33" t="str">
+      <c r="M44" s="17" t="str">
         <f aca="false">IF(OR(F44="",K44=""),"",F44-K44)</f>
         <v/>
       </c>
@@ -3793,28 +4133,28 @@
       <c r="P44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="30" t="str">
+      <c r="A45" s="31" t="str">
         <f aca="false">IF('Budget du don'!A45="","",'Budget du don'!A45)</f>
         <v/>
       </c>
-      <c r="B45" s="31" t="str">
+      <c r="B45" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A45="",'Budget du don'!B45=""),"",'Budget du don'!B45)</f>
         <v/>
       </c>
-      <c r="C45" s="32" t="str">
+      <c r="C45" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A45="",'Budget du don'!C45=""),"",'Budget du don'!C45)</f>
         <v/>
       </c>
-      <c r="D45" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A45="","",IF('Budget du don'!D45&lt;&gt;"",'Budget du don'!D45,IF('Budget du don'!E45&lt;&gt;"",'Budget du don'!E45/'Budget du don'!$G$4,"")))</f>
+      <c r="D45" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A45="",'Budget du don'!F45=""),"",'Budget du don'!F45)</f>
         <v/>
       </c>
       <c r="E45" s="18" t="str">
         <f aca="false">IF(D45="","",D45*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F45" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F45="","",'Budget du don'!F45)</f>
+      <c r="F45" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H45="","",'Budget du don'!H45)</f>
         <v/>
       </c>
       <c r="G45" s="18" t="str">
@@ -3824,7 +4164,7 @@
       <c r="H45" s="14"/>
       <c r="I45" s="15"/>
       <c r="J45" s="16"/>
-      <c r="K45" s="17" t="str">
+      <c r="K45" s="19" t="str">
         <f aca="false">IF(OR(H45="",AND(I45="",J45="")),"",H45*IF(I45&lt;&gt;"",I45,J45/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3832,7 +4172,7 @@
         <f aca="false">IF(K45="","",K45*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M45" s="33" t="str">
+      <c r="M45" s="17" t="str">
         <f aca="false">IF(OR(F45="",K45=""),"",F45-K45)</f>
         <v/>
       </c>
@@ -3847,28 +4187,28 @@
       <c r="P45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="30" t="str">
+      <c r="A46" s="31" t="str">
         <f aca="false">IF('Budget du don'!A46="","",'Budget du don'!A46)</f>
         <v/>
       </c>
-      <c r="B46" s="31" t="str">
+      <c r="B46" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A46="",'Budget du don'!B46=""),"",'Budget du don'!B46)</f>
         <v/>
       </c>
-      <c r="C46" s="32" t="str">
+      <c r="C46" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A46="",'Budget du don'!C46=""),"",'Budget du don'!C46)</f>
         <v/>
       </c>
-      <c r="D46" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A46="","",IF('Budget du don'!D46&lt;&gt;"",'Budget du don'!D46,IF('Budget du don'!E46&lt;&gt;"",'Budget du don'!E46/'Budget du don'!$G$4,"")))</f>
+      <c r="D46" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A46="",'Budget du don'!F46=""),"",'Budget du don'!F46)</f>
         <v/>
       </c>
       <c r="E46" s="18" t="str">
         <f aca="false">IF(D46="","",D46*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F46" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F46="","",'Budget du don'!F46)</f>
+      <c r="F46" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H46="","",'Budget du don'!H46)</f>
         <v/>
       </c>
       <c r="G46" s="18" t="str">
@@ -3878,7 +4218,7 @@
       <c r="H46" s="14"/>
       <c r="I46" s="15"/>
       <c r="J46" s="16"/>
-      <c r="K46" s="17" t="str">
+      <c r="K46" s="19" t="str">
         <f aca="false">IF(OR(H46="",AND(I46="",J46="")),"",H46*IF(I46&lt;&gt;"",I46,J46/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3886,7 +4226,7 @@
         <f aca="false">IF(K46="","",K46*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M46" s="33" t="str">
+      <c r="M46" s="17" t="str">
         <f aca="false">IF(OR(F46="",K46=""),"",F46-K46)</f>
         <v/>
       </c>
@@ -3901,28 +4241,28 @@
       <c r="P46" s="4"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="30" t="str">
+      <c r="A47" s="31" t="str">
         <f aca="false">IF('Budget du don'!A47="","",'Budget du don'!A47)</f>
         <v/>
       </c>
-      <c r="B47" s="31" t="str">
+      <c r="B47" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A47="",'Budget du don'!B47=""),"",'Budget du don'!B47)</f>
         <v/>
       </c>
-      <c r="C47" s="32" t="str">
+      <c r="C47" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A47="",'Budget du don'!C47=""),"",'Budget du don'!C47)</f>
         <v/>
       </c>
-      <c r="D47" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A47="","",IF('Budget du don'!D47&lt;&gt;"",'Budget du don'!D47,IF('Budget du don'!E47&lt;&gt;"",'Budget du don'!E47/'Budget du don'!$G$4,"")))</f>
+      <c r="D47" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A47="",'Budget du don'!F47=""),"",'Budget du don'!F47)</f>
         <v/>
       </c>
       <c r="E47" s="18" t="str">
         <f aca="false">IF(D47="","",D47*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F47" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F47="","",'Budget du don'!F47)</f>
+      <c r="F47" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H47="","",'Budget du don'!H47)</f>
         <v/>
       </c>
       <c r="G47" s="18" t="str">
@@ -3932,7 +4272,7 @@
       <c r="H47" s="14"/>
       <c r="I47" s="15"/>
       <c r="J47" s="16"/>
-      <c r="K47" s="17" t="str">
+      <c r="K47" s="19" t="str">
         <f aca="false">IF(OR(H47="",AND(I47="",J47="")),"",H47*IF(I47&lt;&gt;"",I47,J47/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3940,7 +4280,7 @@
         <f aca="false">IF(K47="","",K47*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M47" s="33" t="str">
+      <c r="M47" s="17" t="str">
         <f aca="false">IF(OR(F47="",K47=""),"",F47-K47)</f>
         <v/>
       </c>
@@ -3955,28 +4295,28 @@
       <c r="P47" s="4"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="30" t="str">
+      <c r="A48" s="31" t="str">
         <f aca="false">IF('Budget du don'!A48="","",'Budget du don'!A48)</f>
         <v/>
       </c>
-      <c r="B48" s="31" t="str">
+      <c r="B48" s="32" t="str">
         <f aca="false">IF(OR('Budget du don'!A48="",'Budget du don'!B48=""),"",'Budget du don'!B48)</f>
         <v/>
       </c>
-      <c r="C48" s="32" t="str">
+      <c r="C48" s="33" t="str">
         <f aca="false">IF(OR('Budget du don'!A48="",'Budget du don'!C48=""),"",'Budget du don'!C48)</f>
         <v/>
       </c>
-      <c r="D48" s="33" t="str">
-        <f aca="false">IF('Budget du don'!A48="","",IF('Budget du don'!D48&lt;&gt;"",'Budget du don'!D48,IF('Budget du don'!E48&lt;&gt;"",'Budget du don'!E48/'Budget du don'!$G$4,"")))</f>
+      <c r="D48" s="17" t="str">
+        <f aca="false">IF(OR('Budget du don'!A48="",'Budget du don'!F48=""),"",'Budget du don'!F48)</f>
         <v/>
       </c>
       <c r="E48" s="18" t="str">
         <f aca="false">IF(D48="","",D48*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="F48" s="33" t="str">
-        <f aca="false">IF('Budget du don'!F48="","",'Budget du don'!F48)</f>
+      <c r="F48" s="17" t="str">
+        <f aca="false">IF('Budget du don'!H48="","",'Budget du don'!H48)</f>
         <v/>
       </c>
       <c r="G48" s="18" t="str">
@@ -3986,7 +4326,7 @@
       <c r="H48" s="14"/>
       <c r="I48" s="15"/>
       <c r="J48" s="16"/>
-      <c r="K48" s="17" t="str">
+      <c r="K48" s="19" t="str">
         <f aca="false">IF(OR(H48="",AND(I48="",J48="")),"",H48*IF(I48&lt;&gt;"",I48,J48/'Budget du don'!$G$4))</f>
         <v/>
       </c>
@@ -3994,7 +4334,7 @@
         <f aca="false">IF(K48="","",K48*'Budget du don'!$G$4)</f>
         <v/>
       </c>
-      <c r="M48" s="33" t="str">
+      <c r="M48" s="17" t="str">
         <f aca="false">IF(OR(F48="",K48=""),"",F48-K48)</f>
         <v/>
       </c>
@@ -4010,7 +4350,7 @@
     </row>
     <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="35" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B49" s="36"/>
       <c r="C49" s="36"/>

</xml_diff>

<commit_message>
Ajout des onglets Budget annuel, Prix et Détails des dons
Le classeur budget par don devient complet : budget annuel par poste
(écart et % consommé automatiques), comparatif de l'évolution des prix
des articles par campagne, et détail des dons par orphelinat avec
double monnaie €/FCFA.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/budget-par-don-les-petits-enfants-de-marie.xlsx
+++ b/budget-par-don-les-petits-enfants-de-marie.xlsx
@@ -10,6 +10,9 @@
   <sheets>
     <sheet name="Budget du don" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Comparatif" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Budget annuel" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Prix" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Détails des dons" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="91">
   <si>
     <t xml:space="preserve">BUDGET PAR DON — LISTE D'ACHATS</t>
   </si>
@@ -207,13 +210,100 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUDGET ANNUEL PAR POSTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Votre budget global de l'année, par poste de dépense — modifiable à tout moment (cellules jaunes). Notez le dépensé réel au fil des campagnes : l'écart et le % consommé se calculent automatiquement (rouge = budget dépassé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poste / Catégorie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget prévu (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dépensé réel (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% consommé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achats articles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logistique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frais divers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPARATIF DES PRIX DES ARTICLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notez le prix unitaire de chaque article à chaque campagne (colonnes C à F : les en-têtes jaunes sont modifiables), en € ou en FCFA — gardez la même monnaie sur toute la ligne. L'évolution compare automatiquement le premier prix saisi au dernier. La ligne 6 est un exemple en FCFA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pâques 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentrée 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noël 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Évolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÉTAILS DES DONS PAR CAMPAGNE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Une ligne par article donné : campagne, orphelinat bénéficiaire, article, quantité et valeur. Saisissez le prix unitaire en € OU en FCFA (une seule des deux colonnes) : les valeurs totales se calculent dans les deux monnaies. Les lignes 7 à 9 sont des exemples à remplacer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALEUR TOTALE DES DONS (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALEUR TOTALE (FCFA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLES DONNÉS (QUANTITÉ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bénéficiaire (orphelinat…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article donné</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur totale (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeur totale (FCFA)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
@@ -222,6 +312,8 @@
     <numFmt numFmtId="169" formatCode="#,##0"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
     <numFmt numFmtId="171" formatCode="\+0.0%;\-0.0%"/>
+    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="173" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -429,7 +521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -587,6 +679,38 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4441,4 +4565,4429 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="40" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="17" t="n">
+        <f aca="false">IF(OR(A6="",B6=""),"",B6-IF(C6="",0,C6))</f>
+        <v>1500</v>
+      </c>
+      <c r="E6" s="41" t="n">
+        <f aca="false">IF(OR(A6="",B6="",B6=0),"",IF(C6="",0,C6)/B6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17" t="n">
+        <f aca="false">IF(OR(A7="",B7=""),"",B7-IF(C7="",0,C7))</f>
+        <v>300</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <f aca="false">IF(OR(A7="",B7="",B7=0),"",IF(C7="",0,C7)/B7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="17" t="n">
+        <f aca="false">IF(OR(A8="",B8=""),"",B8-IF(C8="",0,C8))</f>
+        <v>200</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <f aca="false">IF(OR(A8="",B8="",B8=0),"",IF(C8="",0,C8)/B8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="17" t="n">
+        <f aca="false">IF(OR(A9="",B9=""),"",B9-IF(C9="",0,C9))</f>
+        <v>100</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <f aca="false">IF(OR(A9="",B9="",B9=0),"",IF(C9="",0,C9)/B9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="17" t="str">
+        <f aca="false">IF(OR(A10="",B10=""),"",B10-IF(C10="",0,C10))</f>
+        <v/>
+      </c>
+      <c r="E10" s="41" t="str">
+        <f aca="false">IF(OR(A10="",B10="",B10=0),"",IF(C10="",0,C10)/B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="17" t="str">
+        <f aca="false">IF(OR(A11="",B11=""),"",B11-IF(C11="",0,C11))</f>
+        <v/>
+      </c>
+      <c r="E11" s="41" t="str">
+        <f aca="false">IF(OR(A11="",B11="",B11=0),"",IF(C11="",0,C11)/B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="17" t="str">
+        <f aca="false">IF(OR(A12="",B12=""),"",B12-IF(C12="",0,C12))</f>
+        <v/>
+      </c>
+      <c r="E12" s="41" t="str">
+        <f aca="false">IF(OR(A12="",B12="",B12=0),"",IF(C12="",0,C12)/B12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="17" t="str">
+        <f aca="false">IF(OR(A13="",B13=""),"",B13-IF(C13="",0,C13))</f>
+        <v/>
+      </c>
+      <c r="E13" s="41" t="str">
+        <f aca="false">IF(OR(A13="",B13="",B13=0),"",IF(C13="",0,C13)/B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="17" t="str">
+        <f aca="false">IF(OR(A14="",B14=""),"",B14-IF(C14="",0,C14))</f>
+        <v/>
+      </c>
+      <c r="E14" s="41" t="str">
+        <f aca="false">IF(OR(A14="",B14="",B14=0),"",IF(C14="",0,C14)/B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="17" t="str">
+        <f aca="false">IF(OR(A15="",B15=""),"",B15-IF(C15="",0,C15))</f>
+        <v/>
+      </c>
+      <c r="E15" s="41" t="str">
+        <f aca="false">IF(OR(A15="",B15="",B15=0),"",IF(C15="",0,C15)/B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="22" t="n">
+        <f aca="false">SUM(B6:B15)</f>
+        <v>2100</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <f aca="false">SUM(C6:C15)</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <f aca="false">SUM(D6:D15)</f>
+        <v>2100</v>
+      </c>
+      <c r="E16" s="42" t="n">
+        <f aca="false">IF(B16=0,"",C16/B16)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E6:E15">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="dataBar" priority="3">
+      <dataBar showValue="1" minLength="10" maxLength="90">
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FF45B84B"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{731796C0-BDAD-4AB7-879C-AA86E83BF181}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{731796C0-BDAD-4AB7-879C-AA86E83BF181}">
+            <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FF45B84B"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E6:E15</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="44" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D6" s="44" t="n">
+        <v>12800</v>
+      </c>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="45" t="n">
+        <f aca="false">IF(C6="","",IF(F6&lt;&gt;"",(F6-C6)/C6,IF(E6&lt;&gt;"",(E6-C6)/C6,IF(D6&lt;&gt;"",(D6-C6)/C6,""))))</f>
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="45" t="str">
+        <f aca="false">IF(C7="","",IF(F7&lt;&gt;"",(F7-C7)/C7,IF(E7&lt;&gt;"",(E7-C7)/C7,IF(D7&lt;&gt;"",(D7-C7)/C7,""))))</f>
+        <v/>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="45" t="str">
+        <f aca="false">IF(C8="","",IF(F8&lt;&gt;"",(F8-C8)/C8,IF(E8&lt;&gt;"",(E8-C8)/C8,IF(D8&lt;&gt;"",(D8-C8)/C8,""))))</f>
+        <v/>
+      </c>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="45" t="str">
+        <f aca="false">IF(C9="","",IF(F9&lt;&gt;"",(F9-C9)/C9,IF(E9&lt;&gt;"",(E9-C9)/C9,IF(D9&lt;&gt;"",(D9-C9)/C9,""))))</f>
+        <v/>
+      </c>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="45" t="str">
+        <f aca="false">IF(C10="","",IF(F10&lt;&gt;"",(F10-C10)/C10,IF(E10&lt;&gt;"",(E10-C10)/C10,IF(D10&lt;&gt;"",(D10-C10)/C10,""))))</f>
+        <v/>
+      </c>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="45" t="str">
+        <f aca="false">IF(C11="","",IF(F11&lt;&gt;"",(F11-C11)/C11,IF(E11&lt;&gt;"",(E11-C11)/C11,IF(D11&lt;&gt;"",(D11-C11)/C11,""))))</f>
+        <v/>
+      </c>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="45" t="str">
+        <f aca="false">IF(C12="","",IF(F12&lt;&gt;"",(F12-C12)/C12,IF(E12&lt;&gt;"",(E12-C12)/C12,IF(D12&lt;&gt;"",(D12-C12)/C12,""))))</f>
+        <v/>
+      </c>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="45" t="str">
+        <f aca="false">IF(C13="","",IF(F13&lt;&gt;"",(F13-C13)/C13,IF(E13&lt;&gt;"",(E13-C13)/C13,IF(D13&lt;&gt;"",(D13-C13)/C13,""))))</f>
+        <v/>
+      </c>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="45" t="str">
+        <f aca="false">IF(C14="","",IF(F14&lt;&gt;"",(F14-C14)/C14,IF(E14&lt;&gt;"",(E14-C14)/C14,IF(D14&lt;&gt;"",(D14-C14)/C14,""))))</f>
+        <v/>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="45" t="str">
+        <f aca="false">IF(C15="","",IF(F15&lt;&gt;"",(F15-C15)/C15,IF(E15&lt;&gt;"",(E15-C15)/C15,IF(D15&lt;&gt;"",(D15-C15)/C15,""))))</f>
+        <v/>
+      </c>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="45" t="str">
+        <f aca="false">IF(C16="","",IF(F16&lt;&gt;"",(F16-C16)/C16,IF(E16&lt;&gt;"",(E16-C16)/C16,IF(D16&lt;&gt;"",(D16-C16)/C16,""))))</f>
+        <v/>
+      </c>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45" t="str">
+        <f aca="false">IF(C17="","",IF(F17&lt;&gt;"",(F17-C17)/C17,IF(E17&lt;&gt;"",(E17-C17)/C17,IF(D17&lt;&gt;"",(D17-C17)/C17,""))))</f>
+        <v/>
+      </c>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="45" t="str">
+        <f aca="false">IF(C18="","",IF(F18&lt;&gt;"",(F18-C18)/C18,IF(E18&lt;&gt;"",(E18-C18)/C18,IF(D18&lt;&gt;"",(D18-C18)/C18,""))))</f>
+        <v/>
+      </c>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="45" t="str">
+        <f aca="false">IF(C19="","",IF(F19&lt;&gt;"",(F19-C19)/C19,IF(E19&lt;&gt;"",(E19-C19)/C19,IF(D19&lt;&gt;"",(D19-C19)/C19,""))))</f>
+        <v/>
+      </c>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="45" t="str">
+        <f aca="false">IF(C20="","",IF(F20&lt;&gt;"",(F20-C20)/C20,IF(E20&lt;&gt;"",(E20-C20)/C20,IF(D20&lt;&gt;"",(D20-C20)/C20,""))))</f>
+        <v/>
+      </c>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="45" t="str">
+        <f aca="false">IF(C21="","",IF(F21&lt;&gt;"",(F21-C21)/C21,IF(E21&lt;&gt;"",(E21-C21)/C21,IF(D21&lt;&gt;"",(D21-C21)/C21,""))))</f>
+        <v/>
+      </c>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="45" t="str">
+        <f aca="false">IF(C22="","",IF(F22&lt;&gt;"",(F22-C22)/C22,IF(E22&lt;&gt;"",(E22-C22)/C22,IF(D22&lt;&gt;"",(D22-C22)/C22,""))))</f>
+        <v/>
+      </c>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="45" t="str">
+        <f aca="false">IF(C23="","",IF(F23&lt;&gt;"",(F23-C23)/C23,IF(E23&lt;&gt;"",(E23-C23)/C23,IF(D23&lt;&gt;"",(D23-C23)/C23,""))))</f>
+        <v/>
+      </c>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="45" t="str">
+        <f aca="false">IF(C24="","",IF(F24&lt;&gt;"",(F24-C24)/C24,IF(E24&lt;&gt;"",(E24-C24)/C24,IF(D24&lt;&gt;"",(D24-C24)/C24,""))))</f>
+        <v/>
+      </c>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="45" t="str">
+        <f aca="false">IF(C25="","",IF(F25&lt;&gt;"",(F25-C25)/C25,IF(E25&lt;&gt;"",(E25-C25)/C25,IF(D25&lt;&gt;"",(D25-C25)/C25,""))))</f>
+        <v/>
+      </c>
+      <c r="H25" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G6:G25">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:J206"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="n">
+        <f aca="false">SUM(H7:H206)</f>
+        <v>205.218409133526</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="46" t="n">
+        <f aca="false">SUM(H7:H206)*'Budget du don'!$G$4</f>
+        <v>134614.452</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="47" t="n">
+        <f aca="false">SUM(E7:E206)</f>
+        <v>122</v>
+      </c>
+      <c r="F5" s="47"/>
+    </row>
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="15"/>
+      <c r="G7" s="16" t="n">
+        <v>330</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <f aca="false">IF(OR(E7="",AND(F7="",G7="")),"",E7*IF(F7&lt;&gt;"",F7,G7/'Budget du don'!$G$4))</f>
+        <v>50.3081756883454</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <f aca="false">IF(H7="","",H7*'Budget du don'!$G$4)</f>
+        <v>33000</v>
+      </c>
+      <c r="J7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="G8" s="16"/>
+      <c r="H8" s="19" t="n">
+        <f aca="false">IF(OR(E8="",AND(F8="",G8="")),"",E8*IF(F8&lt;&gt;"",F8,G8/'Budget du don'!$G$4))</f>
+        <v>36</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <f aca="false">IF(H8="","",H8*'Budget du don'!$G$4)</f>
+        <v>23614.452</v>
+      </c>
+      <c r="J8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="16" t="n">
+        <v>3900</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <f aca="false">IF(OR(E9="",AND(F9="",G9="")),"",E9*IF(F9&lt;&gt;"",F9,G9/'Budget du don'!$G$4))</f>
+        <v>118.91023344518</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <f aca="false">IF(H9="","",H9*'Budget du don'!$G$4)</f>
+        <v>78000</v>
+      </c>
+      <c r="J9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="19" t="str">
+        <f aca="false">IF(OR(E10="",AND(F10="",G10="")),"",E10*IF(F10&lt;&gt;"",F10,G10/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I10" s="18" t="str">
+        <f aca="false">IF(H10="","",H10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="19" t="str">
+        <f aca="false">IF(OR(E11="",AND(F11="",G11="")),"",E11*IF(F11&lt;&gt;"",F11,G11/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I11" s="18" t="str">
+        <f aca="false">IF(H11="","",H11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="19" t="str">
+        <f aca="false">IF(OR(E12="",AND(F12="",G12="")),"",E12*IF(F12&lt;&gt;"",F12,G12/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I12" s="18" t="str">
+        <f aca="false">IF(H12="","",H12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="19" t="str">
+        <f aca="false">IF(OR(E13="",AND(F13="",G13="")),"",E13*IF(F13&lt;&gt;"",F13,G13/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I13" s="18" t="str">
+        <f aca="false">IF(H13="","",H13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="19" t="str">
+        <f aca="false">IF(OR(E14="",AND(F14="",G14="")),"",E14*IF(F14&lt;&gt;"",F14,G14/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I14" s="18" t="str">
+        <f aca="false">IF(H14="","",H14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="19" t="str">
+        <f aca="false">IF(OR(E15="",AND(F15="",G15="")),"",E15*IF(F15&lt;&gt;"",F15,G15/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I15" s="18" t="str">
+        <f aca="false">IF(H15="","",H15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="19" t="str">
+        <f aca="false">IF(OR(E16="",AND(F16="",G16="")),"",E16*IF(F16&lt;&gt;"",F16,G16/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I16" s="18" t="str">
+        <f aca="false">IF(H16="","",H16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="19" t="str">
+        <f aca="false">IF(OR(E17="",AND(F17="",G17="")),"",E17*IF(F17&lt;&gt;"",F17,G17/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I17" s="18" t="str">
+        <f aca="false">IF(H17="","",H17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="19" t="str">
+        <f aca="false">IF(OR(E18="",AND(F18="",G18="")),"",E18*IF(F18&lt;&gt;"",F18,G18/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I18" s="18" t="str">
+        <f aca="false">IF(H18="","",H18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="19" t="str">
+        <f aca="false">IF(OR(E19="",AND(F19="",G19="")),"",E19*IF(F19&lt;&gt;"",F19,G19/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I19" s="18" t="str">
+        <f aca="false">IF(H19="","",H19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="19" t="str">
+        <f aca="false">IF(OR(E20="",AND(F20="",G20="")),"",E20*IF(F20&lt;&gt;"",F20,G20/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I20" s="18" t="str">
+        <f aca="false">IF(H20="","",H20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="19" t="str">
+        <f aca="false">IF(OR(E21="",AND(F21="",G21="")),"",E21*IF(F21&lt;&gt;"",F21,G21/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I21" s="18" t="str">
+        <f aca="false">IF(H21="","",H21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="19" t="str">
+        <f aca="false">IF(OR(E22="",AND(F22="",G22="")),"",E22*IF(F22&lt;&gt;"",F22,G22/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I22" s="18" t="str">
+        <f aca="false">IF(H22="","",H22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="19" t="str">
+        <f aca="false">IF(OR(E23="",AND(F23="",G23="")),"",E23*IF(F23&lt;&gt;"",F23,G23/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I23" s="18" t="str">
+        <f aca="false">IF(H23="","",H23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="19" t="str">
+        <f aca="false">IF(OR(E24="",AND(F24="",G24="")),"",E24*IF(F24&lt;&gt;"",F24,G24/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I24" s="18" t="str">
+        <f aca="false">IF(H24="","",H24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="19" t="str">
+        <f aca="false">IF(OR(E25="",AND(F25="",G25="")),"",E25*IF(F25&lt;&gt;"",F25,G25/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I25" s="18" t="str">
+        <f aca="false">IF(H25="","",H25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="19" t="str">
+        <f aca="false">IF(OR(E26="",AND(F26="",G26="")),"",E26*IF(F26&lt;&gt;"",F26,G26/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I26" s="18" t="str">
+        <f aca="false">IF(H26="","",H26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="19" t="str">
+        <f aca="false">IF(OR(E27="",AND(F27="",G27="")),"",E27*IF(F27&lt;&gt;"",F27,G27/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I27" s="18" t="str">
+        <f aca="false">IF(H27="","",H27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="19" t="str">
+        <f aca="false">IF(OR(E28="",AND(F28="",G28="")),"",E28*IF(F28&lt;&gt;"",F28,G28/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I28" s="18" t="str">
+        <f aca="false">IF(H28="","",H28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="19" t="str">
+        <f aca="false">IF(OR(E29="",AND(F29="",G29="")),"",E29*IF(F29&lt;&gt;"",F29,G29/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I29" s="18" t="str">
+        <f aca="false">IF(H29="","",H29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="19" t="str">
+        <f aca="false">IF(OR(E30="",AND(F30="",G30="")),"",E30*IF(F30&lt;&gt;"",F30,G30/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I30" s="18" t="str">
+        <f aca="false">IF(H30="","",H30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="19" t="str">
+        <f aca="false">IF(OR(E31="",AND(F31="",G31="")),"",E31*IF(F31&lt;&gt;"",F31,G31/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I31" s="18" t="str">
+        <f aca="false">IF(H31="","",H31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="19" t="str">
+        <f aca="false">IF(OR(E32="",AND(F32="",G32="")),"",E32*IF(F32&lt;&gt;"",F32,G32/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I32" s="18" t="str">
+        <f aca="false">IF(H32="","",H32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="19" t="str">
+        <f aca="false">IF(OR(E33="",AND(F33="",G33="")),"",E33*IF(F33&lt;&gt;"",F33,G33/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I33" s="18" t="str">
+        <f aca="false">IF(H33="","",H33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J33" s="4"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="19" t="str">
+        <f aca="false">IF(OR(E34="",AND(F34="",G34="")),"",E34*IF(F34&lt;&gt;"",F34,G34/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I34" s="18" t="str">
+        <f aca="false">IF(H34="","",H34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="19" t="str">
+        <f aca="false">IF(OR(E35="",AND(F35="",G35="")),"",E35*IF(F35&lt;&gt;"",F35,G35/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I35" s="18" t="str">
+        <f aca="false">IF(H35="","",H35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="19" t="str">
+        <f aca="false">IF(OR(E36="",AND(F36="",G36="")),"",E36*IF(F36&lt;&gt;"",F36,G36/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I36" s="18" t="str">
+        <f aca="false">IF(H36="","",H36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="19" t="str">
+        <f aca="false">IF(OR(E37="",AND(F37="",G37="")),"",E37*IF(F37&lt;&gt;"",F37,G37/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I37" s="18" t="str">
+        <f aca="false">IF(H37="","",H37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="19" t="str">
+        <f aca="false">IF(OR(E38="",AND(F38="",G38="")),"",E38*IF(F38&lt;&gt;"",F38,G38/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I38" s="18" t="str">
+        <f aca="false">IF(H38="","",H38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="19" t="str">
+        <f aca="false">IF(OR(E39="",AND(F39="",G39="")),"",E39*IF(F39&lt;&gt;"",F39,G39/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I39" s="18" t="str">
+        <f aca="false">IF(H39="","",H39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="19" t="str">
+        <f aca="false">IF(OR(E40="",AND(F40="",G40="")),"",E40*IF(F40&lt;&gt;"",F40,G40/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I40" s="18" t="str">
+        <f aca="false">IF(H40="","",H40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="16"/>
+      <c r="H41" s="19" t="str">
+        <f aca="false">IF(OR(E41="",AND(F41="",G41="")),"",E41*IF(F41&lt;&gt;"",F41,G41/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I41" s="18" t="str">
+        <f aca="false">IF(H41="","",H41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J41" s="4"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="16"/>
+      <c r="H42" s="19" t="str">
+        <f aca="false">IF(OR(E42="",AND(F42="",G42="")),"",E42*IF(F42&lt;&gt;"",F42,G42/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I42" s="18" t="str">
+        <f aca="false">IF(H42="","",H42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J42" s="4"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="19" t="str">
+        <f aca="false">IF(OR(E43="",AND(F43="",G43="")),"",E43*IF(F43&lt;&gt;"",F43,G43/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I43" s="18" t="str">
+        <f aca="false">IF(H43="","",H43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="16"/>
+      <c r="H44" s="19" t="str">
+        <f aca="false">IF(OR(E44="",AND(F44="",G44="")),"",E44*IF(F44&lt;&gt;"",F44,G44/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I44" s="18" t="str">
+        <f aca="false">IF(H44="","",H44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J44" s="4"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="19" t="str">
+        <f aca="false">IF(OR(E45="",AND(F45="",G45="")),"",E45*IF(F45&lt;&gt;"",F45,G45/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I45" s="18" t="str">
+        <f aca="false">IF(H45="","",H45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J45" s="4"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="19" t="str">
+        <f aca="false">IF(OR(E46="",AND(F46="",G46="")),"",E46*IF(F46&lt;&gt;"",F46,G46/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I46" s="18" t="str">
+        <f aca="false">IF(H46="","",H46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J46" s="4"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="19" t="str">
+        <f aca="false">IF(OR(E47="",AND(F47="",G47="")),"",E47*IF(F47&lt;&gt;"",F47,G47/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I47" s="18" t="str">
+        <f aca="false">IF(H47="","",H47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J47" s="4"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="16"/>
+      <c r="H48" s="19" t="str">
+        <f aca="false">IF(OR(E48="",AND(F48="",G48="")),"",E48*IF(F48&lt;&gt;"",F48,G48/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I48" s="18" t="str">
+        <f aca="false">IF(H48="","",H48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="16"/>
+      <c r="H49" s="19" t="str">
+        <f aca="false">IF(OR(E49="",AND(F49="",G49="")),"",E49*IF(F49&lt;&gt;"",F49,G49/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I49" s="18" t="str">
+        <f aca="false">IF(H49="","",H49*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="14"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="16"/>
+      <c r="H50" s="19" t="str">
+        <f aca="false">IF(OR(E50="",AND(F50="",G50="")),"",E50*IF(F50&lt;&gt;"",F50,G50/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I50" s="18" t="str">
+        <f aca="false">IF(H50="","",H50*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J50" s="4"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="19" t="str">
+        <f aca="false">IF(OR(E51="",AND(F51="",G51="")),"",E51*IF(F51&lt;&gt;"",F51,G51/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I51" s="18" t="str">
+        <f aca="false">IF(H51="","",H51*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="19" t="str">
+        <f aca="false">IF(OR(E52="",AND(F52="",G52="")),"",E52*IF(F52&lt;&gt;"",F52,G52/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I52" s="18" t="str">
+        <f aca="false">IF(H52="","",H52*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="16"/>
+      <c r="H53" s="19" t="str">
+        <f aca="false">IF(OR(E53="",AND(F53="",G53="")),"",E53*IF(F53&lt;&gt;"",F53,G53/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I53" s="18" t="str">
+        <f aca="false">IF(H53="","",H53*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J53" s="4"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="16"/>
+      <c r="H54" s="19" t="str">
+        <f aca="false">IF(OR(E54="",AND(F54="",G54="")),"",E54*IF(F54&lt;&gt;"",F54,G54/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I54" s="18" t="str">
+        <f aca="false">IF(H54="","",H54*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="19" t="str">
+        <f aca="false">IF(OR(E55="",AND(F55="",G55="")),"",E55*IF(F55&lt;&gt;"",F55,G55/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I55" s="18" t="str">
+        <f aca="false">IF(H55="","",H55*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J55" s="4"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="16"/>
+      <c r="H56" s="19" t="str">
+        <f aca="false">IF(OR(E56="",AND(F56="",G56="")),"",E56*IF(F56&lt;&gt;"",F56,G56/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I56" s="18" t="str">
+        <f aca="false">IF(H56="","",H56*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="19" t="str">
+        <f aca="false">IF(OR(E57="",AND(F57="",G57="")),"",E57*IF(F57&lt;&gt;"",F57,G57/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I57" s="18" t="str">
+        <f aca="false">IF(H57="","",H57*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J57" s="4"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="19" t="str">
+        <f aca="false">IF(OR(E58="",AND(F58="",G58="")),"",E58*IF(F58&lt;&gt;"",F58,G58/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I58" s="18" t="str">
+        <f aca="false">IF(H58="","",H58*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="19" t="str">
+        <f aca="false">IF(OR(E59="",AND(F59="",G59="")),"",E59*IF(F59&lt;&gt;"",F59,G59/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I59" s="18" t="str">
+        <f aca="false">IF(H59="","",H59*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J59" s="4"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="19" t="str">
+        <f aca="false">IF(OR(E60="",AND(F60="",G60="")),"",E60*IF(F60&lt;&gt;"",F60,G60/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I60" s="18" t="str">
+        <f aca="false">IF(H60="","",H60*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J60" s="4"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="19" t="str">
+        <f aca="false">IF(OR(E61="",AND(F61="",G61="")),"",E61*IF(F61&lt;&gt;"",F61,G61/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I61" s="18" t="str">
+        <f aca="false">IF(H61="","",H61*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="19" t="str">
+        <f aca="false">IF(OR(E62="",AND(F62="",G62="")),"",E62*IF(F62&lt;&gt;"",F62,G62/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I62" s="18" t="str">
+        <f aca="false">IF(H62="","",H62*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J62" s="4"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="16"/>
+      <c r="H63" s="19" t="str">
+        <f aca="false">IF(OR(E63="",AND(F63="",G63="")),"",E63*IF(F63&lt;&gt;"",F63,G63/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I63" s="18" t="str">
+        <f aca="false">IF(H63="","",H63*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J63" s="4"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4"/>
+      <c r="B64" s="5"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="19" t="str">
+        <f aca="false">IF(OR(E64="",AND(F64="",G64="")),"",E64*IF(F64&lt;&gt;"",F64,G64/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I64" s="18" t="str">
+        <f aca="false">IF(H64="","",H64*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J64" s="4"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="19" t="str">
+        <f aca="false">IF(OR(E65="",AND(F65="",G65="")),"",E65*IF(F65&lt;&gt;"",F65,G65/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I65" s="18" t="str">
+        <f aca="false">IF(H65="","",H65*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J65" s="4"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="16"/>
+      <c r="H66" s="19" t="str">
+        <f aca="false">IF(OR(E66="",AND(F66="",G66="")),"",E66*IF(F66&lt;&gt;"",F66,G66/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I66" s="18" t="str">
+        <f aca="false">IF(H66="","",H66*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J66" s="4"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="19" t="str">
+        <f aca="false">IF(OR(E67="",AND(F67="",G67="")),"",E67*IF(F67&lt;&gt;"",F67,G67/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I67" s="18" t="str">
+        <f aca="false">IF(H67="","",H67*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J67" s="4"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="14"/>
+      <c r="F68" s="15"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="19" t="str">
+        <f aca="false">IF(OR(E68="",AND(F68="",G68="")),"",E68*IF(F68&lt;&gt;"",F68,G68/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I68" s="18" t="str">
+        <f aca="false">IF(H68="","",H68*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J68" s="4"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="14"/>
+      <c r="F69" s="15"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="19" t="str">
+        <f aca="false">IF(OR(E69="",AND(F69="",G69="")),"",E69*IF(F69&lt;&gt;"",F69,G69/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I69" s="18" t="str">
+        <f aca="false">IF(H69="","",H69*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J69" s="4"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="14"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="19" t="str">
+        <f aca="false">IF(OR(E70="",AND(F70="",G70="")),"",E70*IF(F70&lt;&gt;"",F70,G70/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I70" s="18" t="str">
+        <f aca="false">IF(H70="","",H70*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J70" s="4"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4"/>
+      <c r="B71" s="5"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="14"/>
+      <c r="F71" s="15"/>
+      <c r="G71" s="16"/>
+      <c r="H71" s="19" t="str">
+        <f aca="false">IF(OR(E71="",AND(F71="",G71="")),"",E71*IF(F71&lt;&gt;"",F71,G71/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I71" s="18" t="str">
+        <f aca="false">IF(H71="","",H71*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J71" s="4"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4"/>
+      <c r="B72" s="5"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="14"/>
+      <c r="F72" s="15"/>
+      <c r="G72" s="16"/>
+      <c r="H72" s="19" t="str">
+        <f aca="false">IF(OR(E72="",AND(F72="",G72="")),"",E72*IF(F72&lt;&gt;"",F72,G72/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I72" s="18" t="str">
+        <f aca="false">IF(H72="","",H72*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J72" s="4"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="15"/>
+      <c r="G73" s="16"/>
+      <c r="H73" s="19" t="str">
+        <f aca="false">IF(OR(E73="",AND(F73="",G73="")),"",E73*IF(F73&lt;&gt;"",F73,G73/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I73" s="18" t="str">
+        <f aca="false">IF(H73="","",H73*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J73" s="4"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="4"/>
+      <c r="B74" s="5"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="15"/>
+      <c r="G74" s="16"/>
+      <c r="H74" s="19" t="str">
+        <f aca="false">IF(OR(E74="",AND(F74="",G74="")),"",E74*IF(F74&lt;&gt;"",F74,G74/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I74" s="18" t="str">
+        <f aca="false">IF(H74="","",H74*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J74" s="4"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="4"/>
+      <c r="B75" s="5"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="15"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="19" t="str">
+        <f aca="false">IF(OR(E75="",AND(F75="",G75="")),"",E75*IF(F75&lt;&gt;"",F75,G75/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I75" s="18" t="str">
+        <f aca="false">IF(H75="","",H75*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J75" s="4"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="4"/>
+      <c r="B76" s="5"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="15"/>
+      <c r="G76" s="16"/>
+      <c r="H76" s="19" t="str">
+        <f aca="false">IF(OR(E76="",AND(F76="",G76="")),"",E76*IF(F76&lt;&gt;"",F76,G76/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I76" s="18" t="str">
+        <f aca="false">IF(H76="","",H76*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J76" s="4"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="15"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="19" t="str">
+        <f aca="false">IF(OR(E77="",AND(F77="",G77="")),"",E77*IF(F77&lt;&gt;"",F77,G77/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I77" s="18" t="str">
+        <f aca="false">IF(H77="","",H77*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J77" s="4"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4"/>
+      <c r="B78" s="5"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="14"/>
+      <c r="F78" s="15"/>
+      <c r="G78" s="16"/>
+      <c r="H78" s="19" t="str">
+        <f aca="false">IF(OR(E78="",AND(F78="",G78="")),"",E78*IF(F78&lt;&gt;"",F78,G78/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I78" s="18" t="str">
+        <f aca="false">IF(H78="","",H78*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J78" s="4"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4"/>
+      <c r="B79" s="5"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="15"/>
+      <c r="G79" s="16"/>
+      <c r="H79" s="19" t="str">
+        <f aca="false">IF(OR(E79="",AND(F79="",G79="")),"",E79*IF(F79&lt;&gt;"",F79,G79/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I79" s="18" t="str">
+        <f aca="false">IF(H79="","",H79*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J79" s="4"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4"/>
+      <c r="B80" s="5"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="14"/>
+      <c r="F80" s="15"/>
+      <c r="G80" s="16"/>
+      <c r="H80" s="19" t="str">
+        <f aca="false">IF(OR(E80="",AND(F80="",G80="")),"",E80*IF(F80&lt;&gt;"",F80,G80/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I80" s="18" t="str">
+        <f aca="false">IF(H80="","",H80*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J80" s="4"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="15"/>
+      <c r="G81" s="16"/>
+      <c r="H81" s="19" t="str">
+        <f aca="false">IF(OR(E81="",AND(F81="",G81="")),"",E81*IF(F81&lt;&gt;"",F81,G81/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I81" s="18" t="str">
+        <f aca="false">IF(H81="","",H81*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J81" s="4"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="4"/>
+      <c r="B82" s="5"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="4"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="15"/>
+      <c r="G82" s="16"/>
+      <c r="H82" s="19" t="str">
+        <f aca="false">IF(OR(E82="",AND(F82="",G82="")),"",E82*IF(F82&lt;&gt;"",F82,G82/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I82" s="18" t="str">
+        <f aca="false">IF(H82="","",H82*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J82" s="4"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="4"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="15"/>
+      <c r="G83" s="16"/>
+      <c r="H83" s="19" t="str">
+        <f aca="false">IF(OR(E83="",AND(F83="",G83="")),"",E83*IF(F83&lt;&gt;"",F83,G83/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I83" s="18" t="str">
+        <f aca="false">IF(H83="","",H83*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J83" s="4"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="4"/>
+      <c r="B84" s="5"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="14"/>
+      <c r="F84" s="15"/>
+      <c r="G84" s="16"/>
+      <c r="H84" s="19" t="str">
+        <f aca="false">IF(OR(E84="",AND(F84="",G84="")),"",E84*IF(F84&lt;&gt;"",F84,G84/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I84" s="18" t="str">
+        <f aca="false">IF(H84="","",H84*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J84" s="4"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="4"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="15"/>
+      <c r="G85" s="16"/>
+      <c r="H85" s="19" t="str">
+        <f aca="false">IF(OR(E85="",AND(F85="",G85="")),"",E85*IF(F85&lt;&gt;"",F85,G85/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I85" s="18" t="str">
+        <f aca="false">IF(H85="","",H85*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J85" s="4"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="4"/>
+      <c r="B86" s="5"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="15"/>
+      <c r="G86" s="16"/>
+      <c r="H86" s="19" t="str">
+        <f aca="false">IF(OR(E86="",AND(F86="",G86="")),"",E86*IF(F86&lt;&gt;"",F86,G86/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I86" s="18" t="str">
+        <f aca="false">IF(H86="","",H86*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J86" s="4"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="4"/>
+      <c r="B87" s="5"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="15"/>
+      <c r="G87" s="16"/>
+      <c r="H87" s="19" t="str">
+        <f aca="false">IF(OR(E87="",AND(F87="",G87="")),"",E87*IF(F87&lt;&gt;"",F87,G87/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I87" s="18" t="str">
+        <f aca="false">IF(H87="","",H87*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J87" s="4"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="4"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="15"/>
+      <c r="G88" s="16"/>
+      <c r="H88" s="19" t="str">
+        <f aca="false">IF(OR(E88="",AND(F88="",G88="")),"",E88*IF(F88&lt;&gt;"",F88,G88/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I88" s="18" t="str">
+        <f aca="false">IF(H88="","",H88*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J88" s="4"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="4"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="15"/>
+      <c r="G89" s="16"/>
+      <c r="H89" s="19" t="str">
+        <f aca="false">IF(OR(E89="",AND(F89="",G89="")),"",E89*IF(F89&lt;&gt;"",F89,G89/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I89" s="18" t="str">
+        <f aca="false">IF(H89="","",H89*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="4"/>
+      <c r="B90" s="5"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="14"/>
+      <c r="F90" s="15"/>
+      <c r="G90" s="16"/>
+      <c r="H90" s="19" t="str">
+        <f aca="false">IF(OR(E90="",AND(F90="",G90="")),"",E90*IF(F90&lt;&gt;"",F90,G90/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I90" s="18" t="str">
+        <f aca="false">IF(H90="","",H90*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="4"/>
+      <c r="B91" s="5"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="15"/>
+      <c r="G91" s="16"/>
+      <c r="H91" s="19" t="str">
+        <f aca="false">IF(OR(E91="",AND(F91="",G91="")),"",E91*IF(F91&lt;&gt;"",F91,G91/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I91" s="18" t="str">
+        <f aca="false">IF(H91="","",H91*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="4"/>
+      <c r="B92" s="5"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="14"/>
+      <c r="F92" s="15"/>
+      <c r="G92" s="16"/>
+      <c r="H92" s="19" t="str">
+        <f aca="false">IF(OR(E92="",AND(F92="",G92="")),"",E92*IF(F92&lt;&gt;"",F92,G92/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I92" s="18" t="str">
+        <f aca="false">IF(H92="","",H92*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J92" s="4"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="4"/>
+      <c r="B93" s="5"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="15"/>
+      <c r="G93" s="16"/>
+      <c r="H93" s="19" t="str">
+        <f aca="false">IF(OR(E93="",AND(F93="",G93="")),"",E93*IF(F93&lt;&gt;"",F93,G93/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I93" s="18" t="str">
+        <f aca="false">IF(H93="","",H93*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J93" s="4"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="4"/>
+      <c r="B94" s="5"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="14"/>
+      <c r="F94" s="15"/>
+      <c r="G94" s="16"/>
+      <c r="H94" s="19" t="str">
+        <f aca="false">IF(OR(E94="",AND(F94="",G94="")),"",E94*IF(F94&lt;&gt;"",F94,G94/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I94" s="18" t="str">
+        <f aca="false">IF(H94="","",H94*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J94" s="4"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="4"/>
+      <c r="B95" s="5"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="15"/>
+      <c r="G95" s="16"/>
+      <c r="H95" s="19" t="str">
+        <f aca="false">IF(OR(E95="",AND(F95="",G95="")),"",E95*IF(F95&lt;&gt;"",F95,G95/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I95" s="18" t="str">
+        <f aca="false">IF(H95="","",H95*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J95" s="4"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="4"/>
+      <c r="B96" s="5"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="4"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="15"/>
+      <c r="G96" s="16"/>
+      <c r="H96" s="19" t="str">
+        <f aca="false">IF(OR(E96="",AND(F96="",G96="")),"",E96*IF(F96&lt;&gt;"",F96,G96/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I96" s="18" t="str">
+        <f aca="false">IF(H96="","",H96*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J96" s="4"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="4"/>
+      <c r="B97" s="5"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="15"/>
+      <c r="G97" s="16"/>
+      <c r="H97" s="19" t="str">
+        <f aca="false">IF(OR(E97="",AND(F97="",G97="")),"",E97*IF(F97&lt;&gt;"",F97,G97/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I97" s="18" t="str">
+        <f aca="false">IF(H97="","",H97*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J97" s="4"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="4"/>
+      <c r="B98" s="5"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="14"/>
+      <c r="F98" s="15"/>
+      <c r="G98" s="16"/>
+      <c r="H98" s="19" t="str">
+        <f aca="false">IF(OR(E98="",AND(F98="",G98="")),"",E98*IF(F98&lt;&gt;"",F98,G98/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I98" s="18" t="str">
+        <f aca="false">IF(H98="","",H98*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J98" s="4"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="4"/>
+      <c r="B99" s="5"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="15"/>
+      <c r="G99" s="16"/>
+      <c r="H99" s="19" t="str">
+        <f aca="false">IF(OR(E99="",AND(F99="",G99="")),"",E99*IF(F99&lt;&gt;"",F99,G99/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I99" s="18" t="str">
+        <f aca="false">IF(H99="","",H99*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J99" s="4"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="4"/>
+      <c r="B100" s="5"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="15"/>
+      <c r="G100" s="16"/>
+      <c r="H100" s="19" t="str">
+        <f aca="false">IF(OR(E100="",AND(F100="",G100="")),"",E100*IF(F100&lt;&gt;"",F100,G100/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I100" s="18" t="str">
+        <f aca="false">IF(H100="","",H100*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J100" s="4"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="4"/>
+      <c r="B101" s="5"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="15"/>
+      <c r="G101" s="16"/>
+      <c r="H101" s="19" t="str">
+        <f aca="false">IF(OR(E101="",AND(F101="",G101="")),"",E101*IF(F101&lt;&gt;"",F101,G101/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I101" s="18" t="str">
+        <f aca="false">IF(H101="","",H101*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J101" s="4"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="4"/>
+      <c r="B102" s="5"/>
+      <c r="C102" s="4"/>
+      <c r="D102" s="4"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="15"/>
+      <c r="G102" s="16"/>
+      <c r="H102" s="19" t="str">
+        <f aca="false">IF(OR(E102="",AND(F102="",G102="")),"",E102*IF(F102&lt;&gt;"",F102,G102/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I102" s="18" t="str">
+        <f aca="false">IF(H102="","",H102*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J102" s="4"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="4"/>
+      <c r="B103" s="5"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="4"/>
+      <c r="E103" s="14"/>
+      <c r="F103" s="15"/>
+      <c r="G103" s="16"/>
+      <c r="H103" s="19" t="str">
+        <f aca="false">IF(OR(E103="",AND(F103="",G103="")),"",E103*IF(F103&lt;&gt;"",F103,G103/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I103" s="18" t="str">
+        <f aca="false">IF(H103="","",H103*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J103" s="4"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="4"/>
+      <c r="B104" s="5"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="14"/>
+      <c r="F104" s="15"/>
+      <c r="G104" s="16"/>
+      <c r="H104" s="19" t="str">
+        <f aca="false">IF(OR(E104="",AND(F104="",G104="")),"",E104*IF(F104&lt;&gt;"",F104,G104/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I104" s="18" t="str">
+        <f aca="false">IF(H104="","",H104*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J104" s="4"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="4"/>
+      <c r="B105" s="5"/>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="14"/>
+      <c r="F105" s="15"/>
+      <c r="G105" s="16"/>
+      <c r="H105" s="19" t="str">
+        <f aca="false">IF(OR(E105="",AND(F105="",G105="")),"",E105*IF(F105&lt;&gt;"",F105,G105/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I105" s="18" t="str">
+        <f aca="false">IF(H105="","",H105*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J105" s="4"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="4"/>
+      <c r="B106" s="5"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="4"/>
+      <c r="E106" s="14"/>
+      <c r="F106" s="15"/>
+      <c r="G106" s="16"/>
+      <c r="H106" s="19" t="str">
+        <f aca="false">IF(OR(E106="",AND(F106="",G106="")),"",E106*IF(F106&lt;&gt;"",F106,G106/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I106" s="18" t="str">
+        <f aca="false">IF(H106="","",H106*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J106" s="4"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="4"/>
+      <c r="B107" s="5"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="14"/>
+      <c r="F107" s="15"/>
+      <c r="G107" s="16"/>
+      <c r="H107" s="19" t="str">
+        <f aca="false">IF(OR(E107="",AND(F107="",G107="")),"",E107*IF(F107&lt;&gt;"",F107,G107/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I107" s="18" t="str">
+        <f aca="false">IF(H107="","",H107*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J107" s="4"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="4"/>
+      <c r="B108" s="5"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="4"/>
+      <c r="E108" s="14"/>
+      <c r="F108" s="15"/>
+      <c r="G108" s="16"/>
+      <c r="H108" s="19" t="str">
+        <f aca="false">IF(OR(E108="",AND(F108="",G108="")),"",E108*IF(F108&lt;&gt;"",F108,G108/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I108" s="18" t="str">
+        <f aca="false">IF(H108="","",H108*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J108" s="4"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="4"/>
+      <c r="B109" s="5"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="4"/>
+      <c r="E109" s="14"/>
+      <c r="F109" s="15"/>
+      <c r="G109" s="16"/>
+      <c r="H109" s="19" t="str">
+        <f aca="false">IF(OR(E109="",AND(F109="",G109="")),"",E109*IF(F109&lt;&gt;"",F109,G109/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I109" s="18" t="str">
+        <f aca="false">IF(H109="","",H109*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J109" s="4"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="4"/>
+      <c r="B110" s="5"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="4"/>
+      <c r="E110" s="14"/>
+      <c r="F110" s="15"/>
+      <c r="G110" s="16"/>
+      <c r="H110" s="19" t="str">
+        <f aca="false">IF(OR(E110="",AND(F110="",G110="")),"",E110*IF(F110&lt;&gt;"",F110,G110/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I110" s="18" t="str">
+        <f aca="false">IF(H110="","",H110*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J110" s="4"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="4"/>
+      <c r="B111" s="5"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="14"/>
+      <c r="F111" s="15"/>
+      <c r="G111" s="16"/>
+      <c r="H111" s="19" t="str">
+        <f aca="false">IF(OR(E111="",AND(F111="",G111="")),"",E111*IF(F111&lt;&gt;"",F111,G111/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I111" s="18" t="str">
+        <f aca="false">IF(H111="","",H111*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J111" s="4"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="4"/>
+      <c r="B112" s="5"/>
+      <c r="C112" s="4"/>
+      <c r="D112" s="4"/>
+      <c r="E112" s="14"/>
+      <c r="F112" s="15"/>
+      <c r="G112" s="16"/>
+      <c r="H112" s="19" t="str">
+        <f aca="false">IF(OR(E112="",AND(F112="",G112="")),"",E112*IF(F112&lt;&gt;"",F112,G112/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I112" s="18" t="str">
+        <f aca="false">IF(H112="","",H112*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J112" s="4"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="4"/>
+      <c r="B113" s="5"/>
+      <c r="C113" s="4"/>
+      <c r="D113" s="4"/>
+      <c r="E113" s="14"/>
+      <c r="F113" s="15"/>
+      <c r="G113" s="16"/>
+      <c r="H113" s="19" t="str">
+        <f aca="false">IF(OR(E113="",AND(F113="",G113="")),"",E113*IF(F113&lt;&gt;"",F113,G113/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I113" s="18" t="str">
+        <f aca="false">IF(H113="","",H113*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J113" s="4"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="4"/>
+      <c r="B114" s="5"/>
+      <c r="C114" s="4"/>
+      <c r="D114" s="4"/>
+      <c r="E114" s="14"/>
+      <c r="F114" s="15"/>
+      <c r="G114" s="16"/>
+      <c r="H114" s="19" t="str">
+        <f aca="false">IF(OR(E114="",AND(F114="",G114="")),"",E114*IF(F114&lt;&gt;"",F114,G114/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I114" s="18" t="str">
+        <f aca="false">IF(H114="","",H114*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J114" s="4"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="4"/>
+      <c r="B115" s="5"/>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="14"/>
+      <c r="F115" s="15"/>
+      <c r="G115" s="16"/>
+      <c r="H115" s="19" t="str">
+        <f aca="false">IF(OR(E115="",AND(F115="",G115="")),"",E115*IF(F115&lt;&gt;"",F115,G115/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I115" s="18" t="str">
+        <f aca="false">IF(H115="","",H115*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J115" s="4"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="4"/>
+      <c r="B116" s="5"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="4"/>
+      <c r="E116" s="14"/>
+      <c r="F116" s="15"/>
+      <c r="G116" s="16"/>
+      <c r="H116" s="19" t="str">
+        <f aca="false">IF(OR(E116="",AND(F116="",G116="")),"",E116*IF(F116&lt;&gt;"",F116,G116/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I116" s="18" t="str">
+        <f aca="false">IF(H116="","",H116*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J116" s="4"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="4"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="4"/>
+      <c r="D117" s="4"/>
+      <c r="E117" s="14"/>
+      <c r="F117" s="15"/>
+      <c r="G117" s="16"/>
+      <c r="H117" s="19" t="str">
+        <f aca="false">IF(OR(E117="",AND(F117="",G117="")),"",E117*IF(F117&lt;&gt;"",F117,G117/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I117" s="18" t="str">
+        <f aca="false">IF(H117="","",H117*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J117" s="4"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="4"/>
+      <c r="B118" s="5"/>
+      <c r="C118" s="4"/>
+      <c r="D118" s="4"/>
+      <c r="E118" s="14"/>
+      <c r="F118" s="15"/>
+      <c r="G118" s="16"/>
+      <c r="H118" s="19" t="str">
+        <f aca="false">IF(OR(E118="",AND(F118="",G118="")),"",E118*IF(F118&lt;&gt;"",F118,G118/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I118" s="18" t="str">
+        <f aca="false">IF(H118="","",H118*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J118" s="4"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="4"/>
+      <c r="B119" s="5"/>
+      <c r="C119" s="4"/>
+      <c r="D119" s="4"/>
+      <c r="E119" s="14"/>
+      <c r="F119" s="15"/>
+      <c r="G119" s="16"/>
+      <c r="H119" s="19" t="str">
+        <f aca="false">IF(OR(E119="",AND(F119="",G119="")),"",E119*IF(F119&lt;&gt;"",F119,G119/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I119" s="18" t="str">
+        <f aca="false">IF(H119="","",H119*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J119" s="4"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="4"/>
+      <c r="B120" s="5"/>
+      <c r="C120" s="4"/>
+      <c r="D120" s="4"/>
+      <c r="E120" s="14"/>
+      <c r="F120" s="15"/>
+      <c r="G120" s="16"/>
+      <c r="H120" s="19" t="str">
+        <f aca="false">IF(OR(E120="",AND(F120="",G120="")),"",E120*IF(F120&lt;&gt;"",F120,G120/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I120" s="18" t="str">
+        <f aca="false">IF(H120="","",H120*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J120" s="4"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="4"/>
+      <c r="B121" s="5"/>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4"/>
+      <c r="E121" s="14"/>
+      <c r="F121" s="15"/>
+      <c r="G121" s="16"/>
+      <c r="H121" s="19" t="str">
+        <f aca="false">IF(OR(E121="",AND(F121="",G121="")),"",E121*IF(F121&lt;&gt;"",F121,G121/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I121" s="18" t="str">
+        <f aca="false">IF(H121="","",H121*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J121" s="4"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="4"/>
+      <c r="B122" s="5"/>
+      <c r="C122" s="4"/>
+      <c r="D122" s="4"/>
+      <c r="E122" s="14"/>
+      <c r="F122" s="15"/>
+      <c r="G122" s="16"/>
+      <c r="H122" s="19" t="str">
+        <f aca="false">IF(OR(E122="",AND(F122="",G122="")),"",E122*IF(F122&lt;&gt;"",F122,G122/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I122" s="18" t="str">
+        <f aca="false">IF(H122="","",H122*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J122" s="4"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="4"/>
+      <c r="B123" s="5"/>
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="14"/>
+      <c r="F123" s="15"/>
+      <c r="G123" s="16"/>
+      <c r="H123" s="19" t="str">
+        <f aca="false">IF(OR(E123="",AND(F123="",G123="")),"",E123*IF(F123&lt;&gt;"",F123,G123/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I123" s="18" t="str">
+        <f aca="false">IF(H123="","",H123*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J123" s="4"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="4"/>
+      <c r="B124" s="5"/>
+      <c r="C124" s="4"/>
+      <c r="D124" s="4"/>
+      <c r="E124" s="14"/>
+      <c r="F124" s="15"/>
+      <c r="G124" s="16"/>
+      <c r="H124" s="19" t="str">
+        <f aca="false">IF(OR(E124="",AND(F124="",G124="")),"",E124*IF(F124&lt;&gt;"",F124,G124/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I124" s="18" t="str">
+        <f aca="false">IF(H124="","",H124*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J124" s="4"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="4"/>
+      <c r="B125" s="5"/>
+      <c r="C125" s="4"/>
+      <c r="D125" s="4"/>
+      <c r="E125" s="14"/>
+      <c r="F125" s="15"/>
+      <c r="G125" s="16"/>
+      <c r="H125" s="19" t="str">
+        <f aca="false">IF(OR(E125="",AND(F125="",G125="")),"",E125*IF(F125&lt;&gt;"",F125,G125/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I125" s="18" t="str">
+        <f aca="false">IF(H125="","",H125*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J125" s="4"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="4"/>
+      <c r="B126" s="5"/>
+      <c r="C126" s="4"/>
+      <c r="D126" s="4"/>
+      <c r="E126" s="14"/>
+      <c r="F126" s="15"/>
+      <c r="G126" s="16"/>
+      <c r="H126" s="19" t="str">
+        <f aca="false">IF(OR(E126="",AND(F126="",G126="")),"",E126*IF(F126&lt;&gt;"",F126,G126/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I126" s="18" t="str">
+        <f aca="false">IF(H126="","",H126*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J126" s="4"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="4"/>
+      <c r="B127" s="5"/>
+      <c r="C127" s="4"/>
+      <c r="D127" s="4"/>
+      <c r="E127" s="14"/>
+      <c r="F127" s="15"/>
+      <c r="G127" s="16"/>
+      <c r="H127" s="19" t="str">
+        <f aca="false">IF(OR(E127="",AND(F127="",G127="")),"",E127*IF(F127&lt;&gt;"",F127,G127/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I127" s="18" t="str">
+        <f aca="false">IF(H127="","",H127*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J127" s="4"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="4"/>
+      <c r="B128" s="5"/>
+      <c r="C128" s="4"/>
+      <c r="D128" s="4"/>
+      <c r="E128" s="14"/>
+      <c r="F128" s="15"/>
+      <c r="G128" s="16"/>
+      <c r="H128" s="19" t="str">
+        <f aca="false">IF(OR(E128="",AND(F128="",G128="")),"",E128*IF(F128&lt;&gt;"",F128,G128/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I128" s="18" t="str">
+        <f aca="false">IF(H128="","",H128*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J128" s="4"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="4"/>
+      <c r="B129" s="5"/>
+      <c r="C129" s="4"/>
+      <c r="D129" s="4"/>
+      <c r="E129" s="14"/>
+      <c r="F129" s="15"/>
+      <c r="G129" s="16"/>
+      <c r="H129" s="19" t="str">
+        <f aca="false">IF(OR(E129="",AND(F129="",G129="")),"",E129*IF(F129&lt;&gt;"",F129,G129/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I129" s="18" t="str">
+        <f aca="false">IF(H129="","",H129*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J129" s="4"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="4"/>
+      <c r="B130" s="5"/>
+      <c r="C130" s="4"/>
+      <c r="D130" s="4"/>
+      <c r="E130" s="14"/>
+      <c r="F130" s="15"/>
+      <c r="G130" s="16"/>
+      <c r="H130" s="19" t="str">
+        <f aca="false">IF(OR(E130="",AND(F130="",G130="")),"",E130*IF(F130&lt;&gt;"",F130,G130/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I130" s="18" t="str">
+        <f aca="false">IF(H130="","",H130*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J130" s="4"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="4"/>
+      <c r="B131" s="5"/>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="14"/>
+      <c r="F131" s="15"/>
+      <c r="G131" s="16"/>
+      <c r="H131" s="19" t="str">
+        <f aca="false">IF(OR(E131="",AND(F131="",G131="")),"",E131*IF(F131&lt;&gt;"",F131,G131/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I131" s="18" t="str">
+        <f aca="false">IF(H131="","",H131*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J131" s="4"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="4"/>
+      <c r="B132" s="5"/>
+      <c r="C132" s="4"/>
+      <c r="D132" s="4"/>
+      <c r="E132" s="14"/>
+      <c r="F132" s="15"/>
+      <c r="G132" s="16"/>
+      <c r="H132" s="19" t="str">
+        <f aca="false">IF(OR(E132="",AND(F132="",G132="")),"",E132*IF(F132&lt;&gt;"",F132,G132/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I132" s="18" t="str">
+        <f aca="false">IF(H132="","",H132*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J132" s="4"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="4"/>
+      <c r="B133" s="5"/>
+      <c r="C133" s="4"/>
+      <c r="D133" s="4"/>
+      <c r="E133" s="14"/>
+      <c r="F133" s="15"/>
+      <c r="G133" s="16"/>
+      <c r="H133" s="19" t="str">
+        <f aca="false">IF(OR(E133="",AND(F133="",G133="")),"",E133*IF(F133&lt;&gt;"",F133,G133/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I133" s="18" t="str">
+        <f aca="false">IF(H133="","",H133*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J133" s="4"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="4"/>
+      <c r="B134" s="5"/>
+      <c r="C134" s="4"/>
+      <c r="D134" s="4"/>
+      <c r="E134" s="14"/>
+      <c r="F134" s="15"/>
+      <c r="G134" s="16"/>
+      <c r="H134" s="19" t="str">
+        <f aca="false">IF(OR(E134="",AND(F134="",G134="")),"",E134*IF(F134&lt;&gt;"",F134,G134/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I134" s="18" t="str">
+        <f aca="false">IF(H134="","",H134*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J134" s="4"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="4"/>
+      <c r="B135" s="5"/>
+      <c r="C135" s="4"/>
+      <c r="D135" s="4"/>
+      <c r="E135" s="14"/>
+      <c r="F135" s="15"/>
+      <c r="G135" s="16"/>
+      <c r="H135" s="19" t="str">
+        <f aca="false">IF(OR(E135="",AND(F135="",G135="")),"",E135*IF(F135&lt;&gt;"",F135,G135/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I135" s="18" t="str">
+        <f aca="false">IF(H135="","",H135*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J135" s="4"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="4"/>
+      <c r="B136" s="5"/>
+      <c r="C136" s="4"/>
+      <c r="D136" s="4"/>
+      <c r="E136" s="14"/>
+      <c r="F136" s="15"/>
+      <c r="G136" s="16"/>
+      <c r="H136" s="19" t="str">
+        <f aca="false">IF(OR(E136="",AND(F136="",G136="")),"",E136*IF(F136&lt;&gt;"",F136,G136/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I136" s="18" t="str">
+        <f aca="false">IF(H136="","",H136*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J136" s="4"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="4"/>
+      <c r="B137" s="5"/>
+      <c r="C137" s="4"/>
+      <c r="D137" s="4"/>
+      <c r="E137" s="14"/>
+      <c r="F137" s="15"/>
+      <c r="G137" s="16"/>
+      <c r="H137" s="19" t="str">
+        <f aca="false">IF(OR(E137="",AND(F137="",G137="")),"",E137*IF(F137&lt;&gt;"",F137,G137/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I137" s="18" t="str">
+        <f aca="false">IF(H137="","",H137*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J137" s="4"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="4"/>
+      <c r="B138" s="5"/>
+      <c r="C138" s="4"/>
+      <c r="D138" s="4"/>
+      <c r="E138" s="14"/>
+      <c r="F138" s="15"/>
+      <c r="G138" s="16"/>
+      <c r="H138" s="19" t="str">
+        <f aca="false">IF(OR(E138="",AND(F138="",G138="")),"",E138*IF(F138&lt;&gt;"",F138,G138/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I138" s="18" t="str">
+        <f aca="false">IF(H138="","",H138*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J138" s="4"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="4"/>
+      <c r="B139" s="5"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="14"/>
+      <c r="F139" s="15"/>
+      <c r="G139" s="16"/>
+      <c r="H139" s="19" t="str">
+        <f aca="false">IF(OR(E139="",AND(F139="",G139="")),"",E139*IF(F139&lt;&gt;"",F139,G139/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I139" s="18" t="str">
+        <f aca="false">IF(H139="","",H139*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J139" s="4"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="4"/>
+      <c r="B140" s="5"/>
+      <c r="C140" s="4"/>
+      <c r="D140" s="4"/>
+      <c r="E140" s="14"/>
+      <c r="F140" s="15"/>
+      <c r="G140" s="16"/>
+      <c r="H140" s="19" t="str">
+        <f aca="false">IF(OR(E140="",AND(F140="",G140="")),"",E140*IF(F140&lt;&gt;"",F140,G140/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I140" s="18" t="str">
+        <f aca="false">IF(H140="","",H140*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J140" s="4"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="4"/>
+      <c r="B141" s="5"/>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="14"/>
+      <c r="F141" s="15"/>
+      <c r="G141" s="16"/>
+      <c r="H141" s="19" t="str">
+        <f aca="false">IF(OR(E141="",AND(F141="",G141="")),"",E141*IF(F141&lt;&gt;"",F141,G141/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I141" s="18" t="str">
+        <f aca="false">IF(H141="","",H141*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J141" s="4"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="4"/>
+      <c r="B142" s="5"/>
+      <c r="C142" s="4"/>
+      <c r="D142" s="4"/>
+      <c r="E142" s="14"/>
+      <c r="F142" s="15"/>
+      <c r="G142" s="16"/>
+      <c r="H142" s="19" t="str">
+        <f aca="false">IF(OR(E142="",AND(F142="",G142="")),"",E142*IF(F142&lt;&gt;"",F142,G142/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I142" s="18" t="str">
+        <f aca="false">IF(H142="","",H142*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J142" s="4"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="4"/>
+      <c r="B143" s="5"/>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="14"/>
+      <c r="F143" s="15"/>
+      <c r="G143" s="16"/>
+      <c r="H143" s="19" t="str">
+        <f aca="false">IF(OR(E143="",AND(F143="",G143="")),"",E143*IF(F143&lt;&gt;"",F143,G143/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I143" s="18" t="str">
+        <f aca="false">IF(H143="","",H143*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J143" s="4"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="4"/>
+      <c r="B144" s="5"/>
+      <c r="C144" s="4"/>
+      <c r="D144" s="4"/>
+      <c r="E144" s="14"/>
+      <c r="F144" s="15"/>
+      <c r="G144" s="16"/>
+      <c r="H144" s="19" t="str">
+        <f aca="false">IF(OR(E144="",AND(F144="",G144="")),"",E144*IF(F144&lt;&gt;"",F144,G144/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I144" s="18" t="str">
+        <f aca="false">IF(H144="","",H144*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J144" s="4"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="4"/>
+      <c r="B145" s="5"/>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="14"/>
+      <c r="F145" s="15"/>
+      <c r="G145" s="16"/>
+      <c r="H145" s="19" t="str">
+        <f aca="false">IF(OR(E145="",AND(F145="",G145="")),"",E145*IF(F145&lt;&gt;"",F145,G145/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I145" s="18" t="str">
+        <f aca="false">IF(H145="","",H145*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J145" s="4"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="4"/>
+      <c r="B146" s="5"/>
+      <c r="C146" s="4"/>
+      <c r="D146" s="4"/>
+      <c r="E146" s="14"/>
+      <c r="F146" s="15"/>
+      <c r="G146" s="16"/>
+      <c r="H146" s="19" t="str">
+        <f aca="false">IF(OR(E146="",AND(F146="",G146="")),"",E146*IF(F146&lt;&gt;"",F146,G146/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I146" s="18" t="str">
+        <f aca="false">IF(H146="","",H146*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J146" s="4"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="4"/>
+      <c r="B147" s="5"/>
+      <c r="C147" s="4"/>
+      <c r="D147" s="4"/>
+      <c r="E147" s="14"/>
+      <c r="F147" s="15"/>
+      <c r="G147" s="16"/>
+      <c r="H147" s="19" t="str">
+        <f aca="false">IF(OR(E147="",AND(F147="",G147="")),"",E147*IF(F147&lt;&gt;"",F147,G147/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I147" s="18" t="str">
+        <f aca="false">IF(H147="","",H147*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J147" s="4"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="4"/>
+      <c r="B148" s="5"/>
+      <c r="C148" s="4"/>
+      <c r="D148" s="4"/>
+      <c r="E148" s="14"/>
+      <c r="F148" s="15"/>
+      <c r="G148" s="16"/>
+      <c r="H148" s="19" t="str">
+        <f aca="false">IF(OR(E148="",AND(F148="",G148="")),"",E148*IF(F148&lt;&gt;"",F148,G148/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I148" s="18" t="str">
+        <f aca="false">IF(H148="","",H148*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J148" s="4"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="4"/>
+      <c r="B149" s="5"/>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="14"/>
+      <c r="F149" s="15"/>
+      <c r="G149" s="16"/>
+      <c r="H149" s="19" t="str">
+        <f aca="false">IF(OR(E149="",AND(F149="",G149="")),"",E149*IF(F149&lt;&gt;"",F149,G149/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I149" s="18" t="str">
+        <f aca="false">IF(H149="","",H149*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J149" s="4"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="4"/>
+      <c r="B150" s="5"/>
+      <c r="C150" s="4"/>
+      <c r="D150" s="4"/>
+      <c r="E150" s="14"/>
+      <c r="F150" s="15"/>
+      <c r="G150" s="16"/>
+      <c r="H150" s="19" t="str">
+        <f aca="false">IF(OR(E150="",AND(F150="",G150="")),"",E150*IF(F150&lt;&gt;"",F150,G150/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I150" s="18" t="str">
+        <f aca="false">IF(H150="","",H150*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J150" s="4"/>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="4"/>
+      <c r="B151" s="5"/>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="14"/>
+      <c r="F151" s="15"/>
+      <c r="G151" s="16"/>
+      <c r="H151" s="19" t="str">
+        <f aca="false">IF(OR(E151="",AND(F151="",G151="")),"",E151*IF(F151&lt;&gt;"",F151,G151/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I151" s="18" t="str">
+        <f aca="false">IF(H151="","",H151*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J151" s="4"/>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="4"/>
+      <c r="B152" s="5"/>
+      <c r="C152" s="4"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="14"/>
+      <c r="F152" s="15"/>
+      <c r="G152" s="16"/>
+      <c r="H152" s="19" t="str">
+        <f aca="false">IF(OR(E152="",AND(F152="",G152="")),"",E152*IF(F152&lt;&gt;"",F152,G152/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I152" s="18" t="str">
+        <f aca="false">IF(H152="","",H152*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J152" s="4"/>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="4"/>
+      <c r="B153" s="5"/>
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="14"/>
+      <c r="F153" s="15"/>
+      <c r="G153" s="16"/>
+      <c r="H153" s="19" t="str">
+        <f aca="false">IF(OR(E153="",AND(F153="",G153="")),"",E153*IF(F153&lt;&gt;"",F153,G153/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I153" s="18" t="str">
+        <f aca="false">IF(H153="","",H153*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J153" s="4"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="4"/>
+      <c r="B154" s="5"/>
+      <c r="C154" s="4"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="14"/>
+      <c r="F154" s="15"/>
+      <c r="G154" s="16"/>
+      <c r="H154" s="19" t="str">
+        <f aca="false">IF(OR(E154="",AND(F154="",G154="")),"",E154*IF(F154&lt;&gt;"",F154,G154/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I154" s="18" t="str">
+        <f aca="false">IF(H154="","",H154*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J154" s="4"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="4"/>
+      <c r="B155" s="5"/>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="14"/>
+      <c r="F155" s="15"/>
+      <c r="G155" s="16"/>
+      <c r="H155" s="19" t="str">
+        <f aca="false">IF(OR(E155="",AND(F155="",G155="")),"",E155*IF(F155&lt;&gt;"",F155,G155/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I155" s="18" t="str">
+        <f aca="false">IF(H155="","",H155*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J155" s="4"/>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="4"/>
+      <c r="B156" s="5"/>
+      <c r="C156" s="4"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="14"/>
+      <c r="F156" s="15"/>
+      <c r="G156" s="16"/>
+      <c r="H156" s="19" t="str">
+        <f aca="false">IF(OR(E156="",AND(F156="",G156="")),"",E156*IF(F156&lt;&gt;"",F156,G156/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I156" s="18" t="str">
+        <f aca="false">IF(H156="","",H156*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J156" s="4"/>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="4"/>
+      <c r="B157" s="5"/>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="14"/>
+      <c r="F157" s="15"/>
+      <c r="G157" s="16"/>
+      <c r="H157" s="19" t="str">
+        <f aca="false">IF(OR(E157="",AND(F157="",G157="")),"",E157*IF(F157&lt;&gt;"",F157,G157/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I157" s="18" t="str">
+        <f aca="false">IF(H157="","",H157*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J157" s="4"/>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="4"/>
+      <c r="B158" s="5"/>
+      <c r="C158" s="4"/>
+      <c r="D158" s="4"/>
+      <c r="E158" s="14"/>
+      <c r="F158" s="15"/>
+      <c r="G158" s="16"/>
+      <c r="H158" s="19" t="str">
+        <f aca="false">IF(OR(E158="",AND(F158="",G158="")),"",E158*IF(F158&lt;&gt;"",F158,G158/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I158" s="18" t="str">
+        <f aca="false">IF(H158="","",H158*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J158" s="4"/>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="4"/>
+      <c r="B159" s="5"/>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="14"/>
+      <c r="F159" s="15"/>
+      <c r="G159" s="16"/>
+      <c r="H159" s="19" t="str">
+        <f aca="false">IF(OR(E159="",AND(F159="",G159="")),"",E159*IF(F159&lt;&gt;"",F159,G159/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I159" s="18" t="str">
+        <f aca="false">IF(H159="","",H159*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J159" s="4"/>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="4"/>
+      <c r="B160" s="5"/>
+      <c r="C160" s="4"/>
+      <c r="D160" s="4"/>
+      <c r="E160" s="14"/>
+      <c r="F160" s="15"/>
+      <c r="G160" s="16"/>
+      <c r="H160" s="19" t="str">
+        <f aca="false">IF(OR(E160="",AND(F160="",G160="")),"",E160*IF(F160&lt;&gt;"",F160,G160/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I160" s="18" t="str">
+        <f aca="false">IF(H160="","",H160*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J160" s="4"/>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="4"/>
+      <c r="B161" s="5"/>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="14"/>
+      <c r="F161" s="15"/>
+      <c r="G161" s="16"/>
+      <c r="H161" s="19" t="str">
+        <f aca="false">IF(OR(E161="",AND(F161="",G161="")),"",E161*IF(F161&lt;&gt;"",F161,G161/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I161" s="18" t="str">
+        <f aca="false">IF(H161="","",H161*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J161" s="4"/>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="4"/>
+      <c r="B162" s="5"/>
+      <c r="C162" s="4"/>
+      <c r="D162" s="4"/>
+      <c r="E162" s="14"/>
+      <c r="F162" s="15"/>
+      <c r="G162" s="16"/>
+      <c r="H162" s="19" t="str">
+        <f aca="false">IF(OR(E162="",AND(F162="",G162="")),"",E162*IF(F162&lt;&gt;"",F162,G162/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I162" s="18" t="str">
+        <f aca="false">IF(H162="","",H162*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J162" s="4"/>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="4"/>
+      <c r="B163" s="5"/>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="14"/>
+      <c r="F163" s="15"/>
+      <c r="G163" s="16"/>
+      <c r="H163" s="19" t="str">
+        <f aca="false">IF(OR(E163="",AND(F163="",G163="")),"",E163*IF(F163&lt;&gt;"",F163,G163/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I163" s="18" t="str">
+        <f aca="false">IF(H163="","",H163*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J163" s="4"/>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="4"/>
+      <c r="B164" s="5"/>
+      <c r="C164" s="4"/>
+      <c r="D164" s="4"/>
+      <c r="E164" s="14"/>
+      <c r="F164" s="15"/>
+      <c r="G164" s="16"/>
+      <c r="H164" s="19" t="str">
+        <f aca="false">IF(OR(E164="",AND(F164="",G164="")),"",E164*IF(F164&lt;&gt;"",F164,G164/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I164" s="18" t="str">
+        <f aca="false">IF(H164="","",H164*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J164" s="4"/>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="4"/>
+      <c r="B165" s="5"/>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="14"/>
+      <c r="F165" s="15"/>
+      <c r="G165" s="16"/>
+      <c r="H165" s="19" t="str">
+        <f aca="false">IF(OR(E165="",AND(F165="",G165="")),"",E165*IF(F165&lt;&gt;"",F165,G165/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I165" s="18" t="str">
+        <f aca="false">IF(H165="","",H165*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J165" s="4"/>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="4"/>
+      <c r="B166" s="5"/>
+      <c r="C166" s="4"/>
+      <c r="D166" s="4"/>
+      <c r="E166" s="14"/>
+      <c r="F166" s="15"/>
+      <c r="G166" s="16"/>
+      <c r="H166" s="19" t="str">
+        <f aca="false">IF(OR(E166="",AND(F166="",G166="")),"",E166*IF(F166&lt;&gt;"",F166,G166/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I166" s="18" t="str">
+        <f aca="false">IF(H166="","",H166*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J166" s="4"/>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="4"/>
+      <c r="B167" s="5"/>
+      <c r="C167" s="4"/>
+      <c r="D167" s="4"/>
+      <c r="E167" s="14"/>
+      <c r="F167" s="15"/>
+      <c r="G167" s="16"/>
+      <c r="H167" s="19" t="str">
+        <f aca="false">IF(OR(E167="",AND(F167="",G167="")),"",E167*IF(F167&lt;&gt;"",F167,G167/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I167" s="18" t="str">
+        <f aca="false">IF(H167="","",H167*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J167" s="4"/>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="4"/>
+      <c r="B168" s="5"/>
+      <c r="C168" s="4"/>
+      <c r="D168" s="4"/>
+      <c r="E168" s="14"/>
+      <c r="F168" s="15"/>
+      <c r="G168" s="16"/>
+      <c r="H168" s="19" t="str">
+        <f aca="false">IF(OR(E168="",AND(F168="",G168="")),"",E168*IF(F168&lt;&gt;"",F168,G168/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I168" s="18" t="str">
+        <f aca="false">IF(H168="","",H168*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J168" s="4"/>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="4"/>
+      <c r="B169" s="5"/>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="14"/>
+      <c r="F169" s="15"/>
+      <c r="G169" s="16"/>
+      <c r="H169" s="19" t="str">
+        <f aca="false">IF(OR(E169="",AND(F169="",G169="")),"",E169*IF(F169&lt;&gt;"",F169,G169/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I169" s="18" t="str">
+        <f aca="false">IF(H169="","",H169*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J169" s="4"/>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="4"/>
+      <c r="B170" s="5"/>
+      <c r="C170" s="4"/>
+      <c r="D170" s="4"/>
+      <c r="E170" s="14"/>
+      <c r="F170" s="15"/>
+      <c r="G170" s="16"/>
+      <c r="H170" s="19" t="str">
+        <f aca="false">IF(OR(E170="",AND(F170="",G170="")),"",E170*IF(F170&lt;&gt;"",F170,G170/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I170" s="18" t="str">
+        <f aca="false">IF(H170="","",H170*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J170" s="4"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="4"/>
+      <c r="B171" s="5"/>
+      <c r="C171" s="4"/>
+      <c r="D171" s="4"/>
+      <c r="E171" s="14"/>
+      <c r="F171" s="15"/>
+      <c r="G171" s="16"/>
+      <c r="H171" s="19" t="str">
+        <f aca="false">IF(OR(E171="",AND(F171="",G171="")),"",E171*IF(F171&lt;&gt;"",F171,G171/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I171" s="18" t="str">
+        <f aca="false">IF(H171="","",H171*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J171" s="4"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="4"/>
+      <c r="B172" s="5"/>
+      <c r="C172" s="4"/>
+      <c r="D172" s="4"/>
+      <c r="E172" s="14"/>
+      <c r="F172" s="15"/>
+      <c r="G172" s="16"/>
+      <c r="H172" s="19" t="str">
+        <f aca="false">IF(OR(E172="",AND(F172="",G172="")),"",E172*IF(F172&lt;&gt;"",F172,G172/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I172" s="18" t="str">
+        <f aca="false">IF(H172="","",H172*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J172" s="4"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="4"/>
+      <c r="B173" s="5"/>
+      <c r="C173" s="4"/>
+      <c r="D173" s="4"/>
+      <c r="E173" s="14"/>
+      <c r="F173" s="15"/>
+      <c r="G173" s="16"/>
+      <c r="H173" s="19" t="str">
+        <f aca="false">IF(OR(E173="",AND(F173="",G173="")),"",E173*IF(F173&lt;&gt;"",F173,G173/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I173" s="18" t="str">
+        <f aca="false">IF(H173="","",H173*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J173" s="4"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="4"/>
+      <c r="B174" s="5"/>
+      <c r="C174" s="4"/>
+      <c r="D174" s="4"/>
+      <c r="E174" s="14"/>
+      <c r="F174" s="15"/>
+      <c r="G174" s="16"/>
+      <c r="H174" s="19" t="str">
+        <f aca="false">IF(OR(E174="",AND(F174="",G174="")),"",E174*IF(F174&lt;&gt;"",F174,G174/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I174" s="18" t="str">
+        <f aca="false">IF(H174="","",H174*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J174" s="4"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="4"/>
+      <c r="B175" s="5"/>
+      <c r="C175" s="4"/>
+      <c r="D175" s="4"/>
+      <c r="E175" s="14"/>
+      <c r="F175" s="15"/>
+      <c r="G175" s="16"/>
+      <c r="H175" s="19" t="str">
+        <f aca="false">IF(OR(E175="",AND(F175="",G175="")),"",E175*IF(F175&lt;&gt;"",F175,G175/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I175" s="18" t="str">
+        <f aca="false">IF(H175="","",H175*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J175" s="4"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="4"/>
+      <c r="B176" s="5"/>
+      <c r="C176" s="4"/>
+      <c r="D176" s="4"/>
+      <c r="E176" s="14"/>
+      <c r="F176" s="15"/>
+      <c r="G176" s="16"/>
+      <c r="H176" s="19" t="str">
+        <f aca="false">IF(OR(E176="",AND(F176="",G176="")),"",E176*IF(F176&lt;&gt;"",F176,G176/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I176" s="18" t="str">
+        <f aca="false">IF(H176="","",H176*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J176" s="4"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="4"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="4"/>
+      <c r="D177" s="4"/>
+      <c r="E177" s="14"/>
+      <c r="F177" s="15"/>
+      <c r="G177" s="16"/>
+      <c r="H177" s="19" t="str">
+        <f aca="false">IF(OR(E177="",AND(F177="",G177="")),"",E177*IF(F177&lt;&gt;"",F177,G177/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I177" s="18" t="str">
+        <f aca="false">IF(H177="","",H177*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J177" s="4"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="4"/>
+      <c r="B178" s="5"/>
+      <c r="C178" s="4"/>
+      <c r="D178" s="4"/>
+      <c r="E178" s="14"/>
+      <c r="F178" s="15"/>
+      <c r="G178" s="16"/>
+      <c r="H178" s="19" t="str">
+        <f aca="false">IF(OR(E178="",AND(F178="",G178="")),"",E178*IF(F178&lt;&gt;"",F178,G178/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I178" s="18" t="str">
+        <f aca="false">IF(H178="","",H178*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J178" s="4"/>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="4"/>
+      <c r="B179" s="5"/>
+      <c r="C179" s="4"/>
+      <c r="D179" s="4"/>
+      <c r="E179" s="14"/>
+      <c r="F179" s="15"/>
+      <c r="G179" s="16"/>
+      <c r="H179" s="19" t="str">
+        <f aca="false">IF(OR(E179="",AND(F179="",G179="")),"",E179*IF(F179&lt;&gt;"",F179,G179/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I179" s="18" t="str">
+        <f aca="false">IF(H179="","",H179*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J179" s="4"/>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="4"/>
+      <c r="B180" s="5"/>
+      <c r="C180" s="4"/>
+      <c r="D180" s="4"/>
+      <c r="E180" s="14"/>
+      <c r="F180" s="15"/>
+      <c r="G180" s="16"/>
+      <c r="H180" s="19" t="str">
+        <f aca="false">IF(OR(E180="",AND(F180="",G180="")),"",E180*IF(F180&lt;&gt;"",F180,G180/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I180" s="18" t="str">
+        <f aca="false">IF(H180="","",H180*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J180" s="4"/>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="4"/>
+      <c r="B181" s="5"/>
+      <c r="C181" s="4"/>
+      <c r="D181" s="4"/>
+      <c r="E181" s="14"/>
+      <c r="F181" s="15"/>
+      <c r="G181" s="16"/>
+      <c r="H181" s="19" t="str">
+        <f aca="false">IF(OR(E181="",AND(F181="",G181="")),"",E181*IF(F181&lt;&gt;"",F181,G181/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I181" s="18" t="str">
+        <f aca="false">IF(H181="","",H181*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J181" s="4"/>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="4"/>
+      <c r="B182" s="5"/>
+      <c r="C182" s="4"/>
+      <c r="D182" s="4"/>
+      <c r="E182" s="14"/>
+      <c r="F182" s="15"/>
+      <c r="G182" s="16"/>
+      <c r="H182" s="19" t="str">
+        <f aca="false">IF(OR(E182="",AND(F182="",G182="")),"",E182*IF(F182&lt;&gt;"",F182,G182/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I182" s="18" t="str">
+        <f aca="false">IF(H182="","",H182*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J182" s="4"/>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="4"/>
+      <c r="B183" s="5"/>
+      <c r="C183" s="4"/>
+      <c r="D183" s="4"/>
+      <c r="E183" s="14"/>
+      <c r="F183" s="15"/>
+      <c r="G183" s="16"/>
+      <c r="H183" s="19" t="str">
+        <f aca="false">IF(OR(E183="",AND(F183="",G183="")),"",E183*IF(F183&lt;&gt;"",F183,G183/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I183" s="18" t="str">
+        <f aca="false">IF(H183="","",H183*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J183" s="4"/>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="4"/>
+      <c r="B184" s="5"/>
+      <c r="C184" s="4"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="14"/>
+      <c r="F184" s="15"/>
+      <c r="G184" s="16"/>
+      <c r="H184" s="19" t="str">
+        <f aca="false">IF(OR(E184="",AND(F184="",G184="")),"",E184*IF(F184&lt;&gt;"",F184,G184/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I184" s="18" t="str">
+        <f aca="false">IF(H184="","",H184*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J184" s="4"/>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="4"/>
+      <c r="B185" s="5"/>
+      <c r="C185" s="4"/>
+      <c r="D185" s="4"/>
+      <c r="E185" s="14"/>
+      <c r="F185" s="15"/>
+      <c r="G185" s="16"/>
+      <c r="H185" s="19" t="str">
+        <f aca="false">IF(OR(E185="",AND(F185="",G185="")),"",E185*IF(F185&lt;&gt;"",F185,G185/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I185" s="18" t="str">
+        <f aca="false">IF(H185="","",H185*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J185" s="4"/>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="4"/>
+      <c r="B186" s="5"/>
+      <c r="C186" s="4"/>
+      <c r="D186" s="4"/>
+      <c r="E186" s="14"/>
+      <c r="F186" s="15"/>
+      <c r="G186" s="16"/>
+      <c r="H186" s="19" t="str">
+        <f aca="false">IF(OR(E186="",AND(F186="",G186="")),"",E186*IF(F186&lt;&gt;"",F186,G186/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I186" s="18" t="str">
+        <f aca="false">IF(H186="","",H186*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J186" s="4"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="4"/>
+      <c r="B187" s="5"/>
+      <c r="C187" s="4"/>
+      <c r="D187" s="4"/>
+      <c r="E187" s="14"/>
+      <c r="F187" s="15"/>
+      <c r="G187" s="16"/>
+      <c r="H187" s="19" t="str">
+        <f aca="false">IF(OR(E187="",AND(F187="",G187="")),"",E187*IF(F187&lt;&gt;"",F187,G187/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I187" s="18" t="str">
+        <f aca="false">IF(H187="","",H187*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J187" s="4"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="4"/>
+      <c r="B188" s="5"/>
+      <c r="C188" s="4"/>
+      <c r="D188" s="4"/>
+      <c r="E188" s="14"/>
+      <c r="F188" s="15"/>
+      <c r="G188" s="16"/>
+      <c r="H188" s="19" t="str">
+        <f aca="false">IF(OR(E188="",AND(F188="",G188="")),"",E188*IF(F188&lt;&gt;"",F188,G188/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I188" s="18" t="str">
+        <f aca="false">IF(H188="","",H188*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J188" s="4"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="4"/>
+      <c r="B189" s="5"/>
+      <c r="C189" s="4"/>
+      <c r="D189" s="4"/>
+      <c r="E189" s="14"/>
+      <c r="F189" s="15"/>
+      <c r="G189" s="16"/>
+      <c r="H189" s="19" t="str">
+        <f aca="false">IF(OR(E189="",AND(F189="",G189="")),"",E189*IF(F189&lt;&gt;"",F189,G189/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I189" s="18" t="str">
+        <f aca="false">IF(H189="","",H189*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J189" s="4"/>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="4"/>
+      <c r="B190" s="5"/>
+      <c r="C190" s="4"/>
+      <c r="D190" s="4"/>
+      <c r="E190" s="14"/>
+      <c r="F190" s="15"/>
+      <c r="G190" s="16"/>
+      <c r="H190" s="19" t="str">
+        <f aca="false">IF(OR(E190="",AND(F190="",G190="")),"",E190*IF(F190&lt;&gt;"",F190,G190/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I190" s="18" t="str">
+        <f aca="false">IF(H190="","",H190*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J190" s="4"/>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="4"/>
+      <c r="B191" s="5"/>
+      <c r="C191" s="4"/>
+      <c r="D191" s="4"/>
+      <c r="E191" s="14"/>
+      <c r="F191" s="15"/>
+      <c r="G191" s="16"/>
+      <c r="H191" s="19" t="str">
+        <f aca="false">IF(OR(E191="",AND(F191="",G191="")),"",E191*IF(F191&lt;&gt;"",F191,G191/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I191" s="18" t="str">
+        <f aca="false">IF(H191="","",H191*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J191" s="4"/>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="4"/>
+      <c r="B192" s="5"/>
+      <c r="C192" s="4"/>
+      <c r="D192" s="4"/>
+      <c r="E192" s="14"/>
+      <c r="F192" s="15"/>
+      <c r="G192" s="16"/>
+      <c r="H192" s="19" t="str">
+        <f aca="false">IF(OR(E192="",AND(F192="",G192="")),"",E192*IF(F192&lt;&gt;"",F192,G192/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I192" s="18" t="str">
+        <f aca="false">IF(H192="","",H192*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J192" s="4"/>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="4"/>
+      <c r="B193" s="5"/>
+      <c r="C193" s="4"/>
+      <c r="D193" s="4"/>
+      <c r="E193" s="14"/>
+      <c r="F193" s="15"/>
+      <c r="G193" s="16"/>
+      <c r="H193" s="19" t="str">
+        <f aca="false">IF(OR(E193="",AND(F193="",G193="")),"",E193*IF(F193&lt;&gt;"",F193,G193/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I193" s="18" t="str">
+        <f aca="false">IF(H193="","",H193*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J193" s="4"/>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="4"/>
+      <c r="B194" s="5"/>
+      <c r="C194" s="4"/>
+      <c r="D194" s="4"/>
+      <c r="E194" s="14"/>
+      <c r="F194" s="15"/>
+      <c r="G194" s="16"/>
+      <c r="H194" s="19" t="str">
+        <f aca="false">IF(OR(E194="",AND(F194="",G194="")),"",E194*IF(F194&lt;&gt;"",F194,G194/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I194" s="18" t="str">
+        <f aca="false">IF(H194="","",H194*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J194" s="4"/>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="4"/>
+      <c r="B195" s="5"/>
+      <c r="C195" s="4"/>
+      <c r="D195" s="4"/>
+      <c r="E195" s="14"/>
+      <c r="F195" s="15"/>
+      <c r="G195" s="16"/>
+      <c r="H195" s="19" t="str">
+        <f aca="false">IF(OR(E195="",AND(F195="",G195="")),"",E195*IF(F195&lt;&gt;"",F195,G195/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I195" s="18" t="str">
+        <f aca="false">IF(H195="","",H195*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J195" s="4"/>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="4"/>
+      <c r="B196" s="5"/>
+      <c r="C196" s="4"/>
+      <c r="D196" s="4"/>
+      <c r="E196" s="14"/>
+      <c r="F196" s="15"/>
+      <c r="G196" s="16"/>
+      <c r="H196" s="19" t="str">
+        <f aca="false">IF(OR(E196="",AND(F196="",G196="")),"",E196*IF(F196&lt;&gt;"",F196,G196/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I196" s="18" t="str">
+        <f aca="false">IF(H196="","",H196*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J196" s="4"/>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="4"/>
+      <c r="B197" s="5"/>
+      <c r="C197" s="4"/>
+      <c r="D197" s="4"/>
+      <c r="E197" s="14"/>
+      <c r="F197" s="15"/>
+      <c r="G197" s="16"/>
+      <c r="H197" s="19" t="str">
+        <f aca="false">IF(OR(E197="",AND(F197="",G197="")),"",E197*IF(F197&lt;&gt;"",F197,G197/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I197" s="18" t="str">
+        <f aca="false">IF(H197="","",H197*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J197" s="4"/>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="4"/>
+      <c r="B198" s="5"/>
+      <c r="C198" s="4"/>
+      <c r="D198" s="4"/>
+      <c r="E198" s="14"/>
+      <c r="F198" s="15"/>
+      <c r="G198" s="16"/>
+      <c r="H198" s="19" t="str">
+        <f aca="false">IF(OR(E198="",AND(F198="",G198="")),"",E198*IF(F198&lt;&gt;"",F198,G198/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I198" s="18" t="str">
+        <f aca="false">IF(H198="","",H198*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J198" s="4"/>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="4"/>
+      <c r="B199" s="5"/>
+      <c r="C199" s="4"/>
+      <c r="D199" s="4"/>
+      <c r="E199" s="14"/>
+      <c r="F199" s="15"/>
+      <c r="G199" s="16"/>
+      <c r="H199" s="19" t="str">
+        <f aca="false">IF(OR(E199="",AND(F199="",G199="")),"",E199*IF(F199&lt;&gt;"",F199,G199/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I199" s="18" t="str">
+        <f aca="false">IF(H199="","",H199*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J199" s="4"/>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="4"/>
+      <c r="B200" s="5"/>
+      <c r="C200" s="4"/>
+      <c r="D200" s="4"/>
+      <c r="E200" s="14"/>
+      <c r="F200" s="15"/>
+      <c r="G200" s="16"/>
+      <c r="H200" s="19" t="str">
+        <f aca="false">IF(OR(E200="",AND(F200="",G200="")),"",E200*IF(F200&lt;&gt;"",F200,G200/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I200" s="18" t="str">
+        <f aca="false">IF(H200="","",H200*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J200" s="4"/>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="4"/>
+      <c r="B201" s="5"/>
+      <c r="C201" s="4"/>
+      <c r="D201" s="4"/>
+      <c r="E201" s="14"/>
+      <c r="F201" s="15"/>
+      <c r="G201" s="16"/>
+      <c r="H201" s="19" t="str">
+        <f aca="false">IF(OR(E201="",AND(F201="",G201="")),"",E201*IF(F201&lt;&gt;"",F201,G201/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I201" s="18" t="str">
+        <f aca="false">IF(H201="","",H201*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J201" s="4"/>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="4"/>
+      <c r="B202" s="5"/>
+      <c r="C202" s="4"/>
+      <c r="D202" s="4"/>
+      <c r="E202" s="14"/>
+      <c r="F202" s="15"/>
+      <c r="G202" s="16"/>
+      <c r="H202" s="19" t="str">
+        <f aca="false">IF(OR(E202="",AND(F202="",G202="")),"",E202*IF(F202&lt;&gt;"",F202,G202/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I202" s="18" t="str">
+        <f aca="false">IF(H202="","",H202*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J202" s="4"/>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="4"/>
+      <c r="B203" s="5"/>
+      <c r="C203" s="4"/>
+      <c r="D203" s="4"/>
+      <c r="E203" s="14"/>
+      <c r="F203" s="15"/>
+      <c r="G203" s="16"/>
+      <c r="H203" s="19" t="str">
+        <f aca="false">IF(OR(E203="",AND(F203="",G203="")),"",E203*IF(F203&lt;&gt;"",F203,G203/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I203" s="18" t="str">
+        <f aca="false">IF(H203="","",H203*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J203" s="4"/>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="4"/>
+      <c r="B204" s="5"/>
+      <c r="C204" s="4"/>
+      <c r="D204" s="4"/>
+      <c r="E204" s="14"/>
+      <c r="F204" s="15"/>
+      <c r="G204" s="16"/>
+      <c r="H204" s="19" t="str">
+        <f aca="false">IF(OR(E204="",AND(F204="",G204="")),"",E204*IF(F204&lt;&gt;"",F204,G204/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I204" s="18" t="str">
+        <f aca="false">IF(H204="","",H204*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J204" s="4"/>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="4"/>
+      <c r="B205" s="5"/>
+      <c r="C205" s="4"/>
+      <c r="D205" s="4"/>
+      <c r="E205" s="14"/>
+      <c r="F205" s="15"/>
+      <c r="G205" s="16"/>
+      <c r="H205" s="19" t="str">
+        <f aca="false">IF(OR(E205="",AND(F205="",G205="")),"",E205*IF(F205&lt;&gt;"",F205,G205/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I205" s="18" t="str">
+        <f aca="false">IF(H205="","",H205*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J205" s="4"/>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="4"/>
+      <c r="B206" s="5"/>
+      <c r="C206" s="4"/>
+      <c r="D206" s="4"/>
+      <c r="E206" s="14"/>
+      <c r="F206" s="15"/>
+      <c r="G206" s="16"/>
+      <c r="H206" s="19" t="str">
+        <f aca="false">IF(OR(E206="",AND(F206="",G206="")),"",E206*IF(F206&lt;&gt;"",F206,G206/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I206" s="18" t="str">
+        <f aca="false">IF(H206="","",H206*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J206" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Budget annuel : colonnes de conversion €/FCFA dans les deux sens
Le budget prévu et le dépensé réel se saisissent en € ou en FCFA ;
les montants convertis, l'écart et le % consommé s'affichent
automatiquement dans les deux monnaies.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/budget-par-don-les-petits-enfants-de-marie.xlsx
+++ b/budget-par-don-les-petits-enfants-de-marie.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="98">
   <si>
     <t xml:space="preserve">BUDGET PAR DON — LISTE D'ACHATS</t>
   </si>
@@ -215,19 +215,40 @@
     <t xml:space="preserve">BUDGET ANNUEL PAR POSTE</t>
   </si>
   <si>
-    <t xml:space="preserve">Votre budget global de l'année, par poste de dépense — modifiable à tout moment (cellules jaunes). Notez le dépensé réel au fil des campagnes : l'écart et le % consommé se calculent automatiquement (rouge = budget dépassé).</t>
+    <t xml:space="preserve">Votre budget global de l'année, par poste de dépense — modifiable à tout moment. Saisissez le budget prévu et le dépensé réel en € OU en FCFA (une seule des deux colonnes jaunes) : la conversion s'affiche dans les deux monnaies, et l'écart et le % consommé se calculent automatiquement (rouge = budget dépassé).</t>
   </si>
   <si>
     <t xml:space="preserve">Année :</t>
   </si>
   <si>
+    <t xml:space="preserve">BUDGET PRÉVU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÉPENSÉ RÉEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALYSE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Poste / Catégorie</t>
   </si>
   <si>
+    <t xml:space="preserve">Saisi (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisi (FCFA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Budget prévu (€)</t>
   </si>
   <si>
+    <t xml:space="preserve">Budget prévu (FCFA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dépensé réel (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dépensé réel (FCFA)</t>
   </si>
   <si>
     <t xml:space="preserve">% consommé</t>
@@ -4572,13 +4593,19 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4589,6 +4616,13 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -4598,6 +4632,13 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -4607,196 +4648,475 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+    <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="17" t="n">
-        <f aca="false">IF(OR(A6="",B6=""),"",B6-IF(C6="",0,C6))</f>
-        <v>1500</v>
-      </c>
-      <c r="E6" s="41" t="n">
-        <f aca="false">IF(OR(A6="",B6="",B6=0),"",IF(C6="",0,C6)/B6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>300</v>
-      </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="17" t="n">
-        <f aca="false">IF(OR(A7="",B7=""),"",B7-IF(C7="",0,C7))</f>
-        <v>300</v>
-      </c>
-      <c r="E7" s="41" t="n">
-        <f aca="false">IF(OR(A7="",B7="",B7=0),"",IF(C7="",0,C7)/B7)</f>
-        <v>0</v>
+      <c r="K7" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" s="15" t="n">
-        <v>200</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="17" t="n">
-        <f aca="false">IF(OR(A8="",B8=""),"",B8-IF(C8="",0,C8))</f>
-        <v>200</v>
-      </c>
-      <c r="E8" s="41" t="n">
-        <f aca="false">IF(OR(A8="",B8="",B8=0),"",IF(C8="",0,C8)/B8)</f>
+        <v>1500</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="19" t="n">
+        <f aca="false">IF(AND(B8="",C8=""),"",IF(B8&lt;&gt;"",B8,C8/'Budget du don'!$G$4))</f>
+        <v>1500</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <f aca="false">IF(D8="","",D8*'Budget du don'!$G$4)</f>
+        <v>983935.5</v>
+      </c>
+      <c r="F8" s="15"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="19" t="str">
+        <f aca="false">IF(AND(F8="",G8=""),"",IF(F8&lt;&gt;"",F8,G8/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I8" s="18" t="str">
+        <f aca="false">IF(H8="","",H8*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J8" s="17" t="n">
+        <f aca="false">IF(OR(A8="",D8=""),"",D8-IF(H8="",0,H8))</f>
+        <v>1500</v>
+      </c>
+      <c r="K8" s="18" t="n">
+        <f aca="false">IF(J8="","",J8*'Budget du don'!$G$4)</f>
+        <v>983935.5</v>
+      </c>
+      <c r="L8" s="41" t="n">
+        <f aca="false">IF(OR(A8="",D8="",D8=0),"",IF(H8="",0,H8)/D8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B9" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="19" t="n">
+        <f aca="false">IF(AND(B9="",C9=""),"",IF(B9&lt;&gt;"",B9,C9/'Budget du don'!$G$4))</f>
+        <v>300</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <f aca="false">IF(D9="","",D9*'Budget du don'!$G$4)</f>
+        <v>196787.1</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="19" t="str">
+        <f aca="false">IF(AND(F9="",G9=""),"",IF(F9&lt;&gt;"",F9,G9/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I9" s="18" t="str">
+        <f aca="false">IF(H9="","",H9*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J9" s="17" t="n">
+        <f aca="false">IF(OR(A9="",D9=""),"",D9-IF(H9="",0,H9))</f>
+        <v>300</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <f aca="false">IF(J9="","",J9*'Budget du don'!$G$4)</f>
+        <v>196787.1</v>
+      </c>
+      <c r="L9" s="41" t="n">
+        <f aca="false">IF(OR(A9="",D9="",D9=0),"",IF(H9="",0,H9)/D9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="C10" s="16"/>
+      <c r="D10" s="19" t="n">
+        <f aca="false">IF(AND(B10="",C10=""),"",IF(B10&lt;&gt;"",B10,C10/'Budget du don'!$G$4))</f>
+        <v>200</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <f aca="false">IF(D10="","",D10*'Budget du don'!$G$4)</f>
+        <v>131191.4</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="19" t="str">
+        <f aca="false">IF(AND(F10="",G10=""),"",IF(F10&lt;&gt;"",F10,G10/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I10" s="18" t="str">
+        <f aca="false">IF(H10="","",H10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J10" s="17" t="n">
+        <f aca="false">IF(OR(A10="",D10=""),"",D10-IF(H10="",0,H10))</f>
+        <v>200</v>
+      </c>
+      <c r="K10" s="18" t="n">
+        <f aca="false">IF(J10="","",J10*'Budget du don'!$G$4)</f>
+        <v>131191.4</v>
+      </c>
+      <c r="L10" s="41" t="n">
+        <f aca="false">IF(OR(A10="",D10="",D10=0),"",IF(H10="",0,H10)/D10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="17" t="n">
-        <f aca="false">IF(OR(A9="",B9=""),"",B9-IF(C9="",0,C9))</f>
+      <c r="C11" s="16"/>
+      <c r="D11" s="19" t="n">
+        <f aca="false">IF(AND(B11="",C11=""),"",IF(B11&lt;&gt;"",B11,C11/'Budget du don'!$G$4))</f>
         <v>100</v>
       </c>
-      <c r="E9" s="41" t="n">
-        <f aca="false">IF(OR(A9="",B9="",B9=0),"",IF(C9="",0,C9)/B9)</f>
+      <c r="E11" s="18" t="n">
+        <f aca="false">IF(D11="","",D11*'Budget du don'!$G$4)</f>
+        <v>65595.7</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="19" t="str">
+        <f aca="false">IF(AND(F11="",G11=""),"",IF(F11&lt;&gt;"",F11,G11/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I11" s="18" t="str">
+        <f aca="false">IF(H11="","",H11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J11" s="17" t="n">
+        <f aca="false">IF(OR(A11="",D11=""),"",D11-IF(H11="",0,H11))</f>
+        <v>100</v>
+      </c>
+      <c r="K11" s="18" t="n">
+        <f aca="false">IF(J11="","",J11*'Budget du don'!$G$4)</f>
+        <v>65595.7</v>
+      </c>
+      <c r="L11" s="41" t="n">
+        <f aca="false">IF(OR(A11="",D11="",D11=0),"",IF(H11="",0,H11)/D11)</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="17" t="str">
-        <f aca="false">IF(OR(A10="",B10=""),"",B10-IF(C10="",0,C10))</f>
-        <v/>
-      </c>
-      <c r="E10" s="41" t="str">
-        <f aca="false">IF(OR(A10="",B10="",B10=0),"",IF(C10="",0,C10)/B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="17" t="str">
-        <f aca="false">IF(OR(A11="",B11=""),"",B11-IF(C11="",0,C11))</f>
-        <v/>
-      </c>
-      <c r="E11" s="41" t="str">
-        <f aca="false">IF(OR(A11="",B11="",B11=0),"",IF(C11="",0,C11)/B11)</f>
-        <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4"/>
       <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="17" t="str">
-        <f aca="false">IF(OR(A12="",B12=""),"",B12-IF(C12="",0,C12))</f>
-        <v/>
-      </c>
-      <c r="E12" s="41" t="str">
-        <f aca="false">IF(OR(A12="",B12="",B12=0),"",IF(C12="",0,C12)/B12)</f>
+      <c r="C12" s="16"/>
+      <c r="D12" s="19" t="str">
+        <f aca="false">IF(AND(B12="",C12=""),"",IF(B12&lt;&gt;"",B12,C12/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E12" s="18" t="str">
+        <f aca="false">IF(D12="","",D12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="19" t="str">
+        <f aca="false">IF(AND(F12="",G12=""),"",IF(F12&lt;&gt;"",F12,G12/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I12" s="18" t="str">
+        <f aca="false">IF(H12="","",H12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J12" s="17" t="str">
+        <f aca="false">IF(OR(A12="",D12=""),"",D12-IF(H12="",0,H12))</f>
+        <v/>
+      </c>
+      <c r="K12" s="18" t="str">
+        <f aca="false">IF(J12="","",J12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L12" s="41" t="str">
+        <f aca="false">IF(OR(A12="",D12="",D12=0),"",IF(H12="",0,H12)/D12)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4"/>
       <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="17" t="str">
-        <f aca="false">IF(OR(A13="",B13=""),"",B13-IF(C13="",0,C13))</f>
-        <v/>
-      </c>
-      <c r="E13" s="41" t="str">
-        <f aca="false">IF(OR(A13="",B13="",B13=0),"",IF(C13="",0,C13)/B13)</f>
+      <c r="C13" s="16"/>
+      <c r="D13" s="19" t="str">
+        <f aca="false">IF(AND(B13="",C13=""),"",IF(B13&lt;&gt;"",B13,C13/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E13" s="18" t="str">
+        <f aca="false">IF(D13="","",D13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="19" t="str">
+        <f aca="false">IF(AND(F13="",G13=""),"",IF(F13&lt;&gt;"",F13,G13/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I13" s="18" t="str">
+        <f aca="false">IF(H13="","",H13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J13" s="17" t="str">
+        <f aca="false">IF(OR(A13="",D13=""),"",D13-IF(H13="",0,H13))</f>
+        <v/>
+      </c>
+      <c r="K13" s="18" t="str">
+        <f aca="false">IF(J13="","",J13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L13" s="41" t="str">
+        <f aca="false">IF(OR(A13="",D13="",D13=0),"",IF(H13="",0,H13)/D13)</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4"/>
       <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="17" t="str">
-        <f aca="false">IF(OR(A14="",B14=""),"",B14-IF(C14="",0,C14))</f>
-        <v/>
-      </c>
-      <c r="E14" s="41" t="str">
-        <f aca="false">IF(OR(A14="",B14="",B14=0),"",IF(C14="",0,C14)/B14)</f>
+      <c r="C14" s="16"/>
+      <c r="D14" s="19" t="str">
+        <f aca="false">IF(AND(B14="",C14=""),"",IF(B14&lt;&gt;"",B14,C14/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E14" s="18" t="str">
+        <f aca="false">IF(D14="","",D14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F14" s="15"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="19" t="str">
+        <f aca="false">IF(AND(F14="",G14=""),"",IF(F14&lt;&gt;"",F14,G14/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I14" s="18" t="str">
+        <f aca="false">IF(H14="","",H14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J14" s="17" t="str">
+        <f aca="false">IF(OR(A14="",D14=""),"",D14-IF(H14="",0,H14))</f>
+        <v/>
+      </c>
+      <c r="K14" s="18" t="str">
+        <f aca="false">IF(J14="","",J14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L14" s="41" t="str">
+        <f aca="false">IF(OR(A14="",D14="",D14=0),"",IF(H14="",0,H14)/D14)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4"/>
       <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="17" t="str">
-        <f aca="false">IF(OR(A15="",B15=""),"",B15-IF(C15="",0,C15))</f>
-        <v/>
-      </c>
-      <c r="E15" s="41" t="str">
-        <f aca="false">IF(OR(A15="",B15="",B15=0),"",IF(C15="",0,C15)/B15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+      <c r="C15" s="16"/>
+      <c r="D15" s="19" t="str">
+        <f aca="false">IF(AND(B15="",C15=""),"",IF(B15&lt;&gt;"",B15,C15/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E15" s="18" t="str">
+        <f aca="false">IF(D15="","",D15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="19" t="str">
+        <f aca="false">IF(AND(F15="",G15=""),"",IF(F15&lt;&gt;"",F15,G15/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I15" s="18" t="str">
+        <f aca="false">IF(H15="","",H15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J15" s="17" t="str">
+        <f aca="false">IF(OR(A15="",D15=""),"",D15-IF(H15="",0,H15))</f>
+        <v/>
+      </c>
+      <c r="K15" s="18" t="str">
+        <f aca="false">IF(J15="","",J15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L15" s="41" t="str">
+        <f aca="false">IF(OR(A15="",D15="",D15=0),"",IF(H15="",0,H15)/D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="19" t="str">
+        <f aca="false">IF(AND(B16="",C16=""),"",IF(B16&lt;&gt;"",B16,C16/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E16" s="18" t="str">
+        <f aca="false">IF(D16="","",D16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="19" t="str">
+        <f aca="false">IF(AND(F16="",G16=""),"",IF(F16&lt;&gt;"",F16,G16/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I16" s="18" t="str">
+        <f aca="false">IF(H16="","",H16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J16" s="17" t="str">
+        <f aca="false">IF(OR(A16="",D16=""),"",D16-IF(H16="",0,H16))</f>
+        <v/>
+      </c>
+      <c r="K16" s="18" t="str">
+        <f aca="false">IF(J16="","",J16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L16" s="41" t="str">
+        <f aca="false">IF(OR(A16="",D16="",D16=0),"",IF(H16="",0,H16)/D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="19" t="str">
+        <f aca="false">IF(AND(B17="",C17=""),"",IF(B17&lt;&gt;"",B17,C17/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="E17" s="18" t="str">
+        <f aca="false">IF(D17="","",D17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="19" t="str">
+        <f aca="false">IF(AND(F17="",G17=""),"",IF(F17&lt;&gt;"",F17,G17/'Budget du don'!$G$4))</f>
+        <v/>
+      </c>
+      <c r="I17" s="18" t="str">
+        <f aca="false">IF(H17="","",H17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="J17" s="17" t="str">
+        <f aca="false">IF(OR(A17="",D17=""),"",D17-IF(H17="",0,H17))</f>
+        <v/>
+      </c>
+      <c r="K17" s="18" t="str">
+        <f aca="false">IF(J17="","",J17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="L17" s="41" t="str">
+        <f aca="false">IF(OR(A17="",D17="",D17=0),"",IF(H17="",0,H17)/D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="22" t="n">
-        <f aca="false">SUM(B6:B15)</f>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="22" t="n">
+        <f aca="false">SUM(D8:D17)</f>
         <v>2100</v>
       </c>
-      <c r="C16" s="22" t="n">
-        <f aca="false">SUM(C6:C15)</f>
+      <c r="E18" s="23" t="n">
+        <f aca="false">SUM(E8:E17)</f>
+        <v>1377509.7</v>
+      </c>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="22" t="n">
+        <f aca="false">SUM(H8:H17)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22" t="n">
-        <f aca="false">SUM(D6:D15)</f>
+      <c r="I18" s="23" t="n">
+        <f aca="false">SUM(I8:I17)</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="22" t="n">
+        <f aca="false">SUM(J8:J17)</f>
         <v>2100</v>
       </c>
-      <c r="E16" s="42" t="n">
-        <f aca="false">IF(B16=0,"",C16/B16)</f>
+      <c r="K18" s="23" t="n">
+        <f aca="false">SUM(K8:K17)</f>
+        <v>1377509.7</v>
+      </c>
+      <c r="L18" s="42" t="n">
+        <f aca="false">IF(D18=0,"",H18/D18)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="J5:L5"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E15">
+  <conditionalFormatting sqref="L8:L17">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>1</formula>
     </cfRule>
@@ -4808,9 +5128,14 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{731796C0-BDAD-4AB7-879C-AA86E83BF181}</x14:id>
+          <x14:id>{A09BB63F-9A53-4485-88A4-14EA103E1FB4}</x14:id>
         </ext>
       </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J8:J17">
+    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4824,7 +5149,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{731796C0-BDAD-4AB7-879C-AA86E83BF181}">
+          <x14:cfRule type="dataBar" id="{A09BB63F-9A53-4485-88A4-14EA103E1FB4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -4836,7 +5161,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E6:E15</xm:sqref>
+          <xm:sqref>L8:L17</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4861,7 +5186,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4873,7 +5198,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4894,19 +5219,19 @@
         <v>3</v>
       </c>
       <c r="D5" s="43" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5246,7 +5571,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5260,7 +5585,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5274,15 +5599,15 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F4" s="8"/>
     </row>
@@ -5305,16 +5630,16 @@
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>13</v>
@@ -5326,13 +5651,13 @@
         <v>17</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Dons sans prix : valeurs totales conservées, seuls les prix unitaires retirés
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/budget-par-don-les-petits-enfants-de-marie.xlsx
+++ b/budget-par-don-les-petits-enfants-de-marie.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="107">
   <si>
     <t xml:space="preserve">BUDGET PAR DON — LISTE D'ACHATS</t>
   </si>
@@ -322,10 +322,10 @@
     <t xml:space="preserve">Valeur totale (FCFA)</t>
   </si>
   <si>
-    <t xml:space="preserve">DÉTAILS DES DONS — VERSION SANS PRIX</t>
+    <t xml:space="preserve">DÉTAILS DES DONS — SANS LES PRIX UNITAIRES</t>
   </si>
   <si>
-    <t xml:space="preserve">Cet onglet se remplit tout seul depuis l'onglet « Détails des dons » : mêmes informations, sans les prix. Rien à saisir ici — idéal à imprimer ou partager sans montrer les montants.</t>
+    <t xml:space="preserve">Cet onglet se remplit tout seul depuis l'onglet « Détails des dons » : mêmes informations avec les valeurs totales, mais sans les prix unitaires. Rien à saisir ici.</t>
   </si>
   <si>
     <t xml:space="preserve">FICHE DE DON — À REMPLIR PAR LE BÉNÉFICIAIRE</t>
@@ -5173,7 +5173,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E2A9CFE-463F-42EF-AAA0-104B8EC1649F}</x14:id>
+          <x14:id>{F989D778-C6EC-4860-B211-56207034E11B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5194,7 +5194,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E2A9CFE-463F-42EF-AAA0-104B8EC1649F}">
+          <x14:cfRule type="dataBar" id="{F989D778-C6EC-4860-B211-56207034E11B}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -9367,15 +9367,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F206"/>
+  <dimension ref="A1:H206"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9387,6 +9389,8 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -9397,19 +9401,39 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47" t="n">
+      <c r="A5" s="9" t="n">
+        <f aca="false">SUM(F7:F206)</f>
+        <v>205.218409133526</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="46" t="n">
+        <f aca="false">SUM(F7:F206)*'Budget du don'!$G$4</f>
+        <v>134614.452</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="47" t="n">
         <f aca="false">SUM(E7:E206)</f>
         <v>122</v>
       </c>
-      <c r="B5" s="47"/>
+      <c r="F5" s="47"/>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
@@ -9428,6 +9452,12 @@
         <v>13</v>
       </c>
       <c r="F6" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" s="12" t="s">
         <v>86</v>
       </c>
     </row>
@@ -9452,7 +9482,15 @@
         <f aca="false">IF(OR('Détails des dons'!A7="",'Détails des dons'!E7=""),"",'Détails des dons'!E7)</f>
         <v>100</v>
       </c>
-      <c r="F7" s="48" t="str">
+      <c r="F7" s="19" t="n">
+        <f aca="false">IF(OR('Détails des dons'!A7="",'Détails des dons'!H7=""),"",'Détails des dons'!H7)</f>
+        <v>50.3081756883454</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <f aca="false">IF(F7="","",F7*'Budget du don'!$G$4)</f>
+        <v>33000</v>
+      </c>
+      <c r="H7" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A7="",'Détails des dons'!J7=""),"",'Détails des dons'!J7)</f>
         <v/>
       </c>
@@ -9478,7 +9516,15 @@
         <f aca="false">IF(OR('Détails des dons'!A8="",'Détails des dons'!E8=""),"",'Détails des dons'!E8)</f>
         <v>2</v>
       </c>
-      <c r="F8" s="48" t="str">
+      <c r="F8" s="19" t="n">
+        <f aca="false">IF(OR('Détails des dons'!A8="",'Détails des dons'!H8=""),"",'Détails des dons'!H8)</f>
+        <v>36</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <f aca="false">IF(F8="","",F8*'Budget du don'!$G$4)</f>
+        <v>23614.452</v>
+      </c>
+      <c r="H8" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A8="",'Détails des dons'!J8=""),"",'Détails des dons'!J8)</f>
         <v/>
       </c>
@@ -9504,7 +9550,15 @@
         <f aca="false">IF(OR('Détails des dons'!A9="",'Détails des dons'!E9=""),"",'Détails des dons'!E9)</f>
         <v>20</v>
       </c>
-      <c r="F9" s="48" t="str">
+      <c r="F9" s="19" t="n">
+        <f aca="false">IF(OR('Détails des dons'!A9="",'Détails des dons'!H9=""),"",'Détails des dons'!H9)</f>
+        <v>118.91023344518</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <f aca="false">IF(F9="","",F9*'Budget du don'!$G$4)</f>
+        <v>78000</v>
+      </c>
+      <c r="H9" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A9="",'Détails des dons'!J9=""),"",'Détails des dons'!J9)</f>
         <v/>
       </c>
@@ -9530,7 +9584,15 @@
         <f aca="false">IF(OR('Détails des dons'!A10="",'Détails des dons'!E10=""),"",'Détails des dons'!E10)</f>
         <v/>
       </c>
-      <c r="F10" s="48" t="str">
+      <c r="F10" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A10="",'Détails des dons'!H10=""),"",'Détails des dons'!H10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="18" t="str">
+        <f aca="false">IF(F10="","",F10*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H10" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A10="",'Détails des dons'!J10=""),"",'Détails des dons'!J10)</f>
         <v/>
       </c>
@@ -9556,7 +9618,15 @@
         <f aca="false">IF(OR('Détails des dons'!A11="",'Détails des dons'!E11=""),"",'Détails des dons'!E11)</f>
         <v/>
       </c>
-      <c r="F11" s="48" t="str">
+      <c r="F11" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A11="",'Détails des dons'!H11=""),"",'Détails des dons'!H11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="18" t="str">
+        <f aca="false">IF(F11="","",F11*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H11" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A11="",'Détails des dons'!J11=""),"",'Détails des dons'!J11)</f>
         <v/>
       </c>
@@ -9582,7 +9652,15 @@
         <f aca="false">IF(OR('Détails des dons'!A12="",'Détails des dons'!E12=""),"",'Détails des dons'!E12)</f>
         <v/>
       </c>
-      <c r="F12" s="48" t="str">
+      <c r="F12" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A12="",'Détails des dons'!H12=""),"",'Détails des dons'!H12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="18" t="str">
+        <f aca="false">IF(F12="","",F12*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H12" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A12="",'Détails des dons'!J12=""),"",'Détails des dons'!J12)</f>
         <v/>
       </c>
@@ -9608,7 +9686,15 @@
         <f aca="false">IF(OR('Détails des dons'!A13="",'Détails des dons'!E13=""),"",'Détails des dons'!E13)</f>
         <v/>
       </c>
-      <c r="F13" s="48" t="str">
+      <c r="F13" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A13="",'Détails des dons'!H13=""),"",'Détails des dons'!H13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="18" t="str">
+        <f aca="false">IF(F13="","",F13*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H13" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A13="",'Détails des dons'!J13=""),"",'Détails des dons'!J13)</f>
         <v/>
       </c>
@@ -9634,7 +9720,15 @@
         <f aca="false">IF(OR('Détails des dons'!A14="",'Détails des dons'!E14=""),"",'Détails des dons'!E14)</f>
         <v/>
       </c>
-      <c r="F14" s="48" t="str">
+      <c r="F14" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A14="",'Détails des dons'!H14=""),"",'Détails des dons'!H14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="18" t="str">
+        <f aca="false">IF(F14="","",F14*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H14" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A14="",'Détails des dons'!J14=""),"",'Détails des dons'!J14)</f>
         <v/>
       </c>
@@ -9660,7 +9754,15 @@
         <f aca="false">IF(OR('Détails des dons'!A15="",'Détails des dons'!E15=""),"",'Détails des dons'!E15)</f>
         <v/>
       </c>
-      <c r="F15" s="48" t="str">
+      <c r="F15" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A15="",'Détails des dons'!H15=""),"",'Détails des dons'!H15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="18" t="str">
+        <f aca="false">IF(F15="","",F15*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H15" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A15="",'Détails des dons'!J15=""),"",'Détails des dons'!J15)</f>
         <v/>
       </c>
@@ -9686,7 +9788,15 @@
         <f aca="false">IF(OR('Détails des dons'!A16="",'Détails des dons'!E16=""),"",'Détails des dons'!E16)</f>
         <v/>
       </c>
-      <c r="F16" s="48" t="str">
+      <c r="F16" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A16="",'Détails des dons'!H16=""),"",'Détails des dons'!H16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="18" t="str">
+        <f aca="false">IF(F16="","",F16*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H16" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A16="",'Détails des dons'!J16=""),"",'Détails des dons'!J16)</f>
         <v/>
       </c>
@@ -9712,7 +9822,15 @@
         <f aca="false">IF(OR('Détails des dons'!A17="",'Détails des dons'!E17=""),"",'Détails des dons'!E17)</f>
         <v/>
       </c>
-      <c r="F17" s="48" t="str">
+      <c r="F17" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A17="",'Détails des dons'!H17=""),"",'Détails des dons'!H17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="18" t="str">
+        <f aca="false">IF(F17="","",F17*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H17" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A17="",'Détails des dons'!J17=""),"",'Détails des dons'!J17)</f>
         <v/>
       </c>
@@ -9738,7 +9856,15 @@
         <f aca="false">IF(OR('Détails des dons'!A18="",'Détails des dons'!E18=""),"",'Détails des dons'!E18)</f>
         <v/>
       </c>
-      <c r="F18" s="48" t="str">
+      <c r="F18" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A18="",'Détails des dons'!H18=""),"",'Détails des dons'!H18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="18" t="str">
+        <f aca="false">IF(F18="","",F18*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H18" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A18="",'Détails des dons'!J18=""),"",'Détails des dons'!J18)</f>
         <v/>
       </c>
@@ -9764,7 +9890,15 @@
         <f aca="false">IF(OR('Détails des dons'!A19="",'Détails des dons'!E19=""),"",'Détails des dons'!E19)</f>
         <v/>
       </c>
-      <c r="F19" s="48" t="str">
+      <c r="F19" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A19="",'Détails des dons'!H19=""),"",'Détails des dons'!H19)</f>
+        <v/>
+      </c>
+      <c r="G19" s="18" t="str">
+        <f aca="false">IF(F19="","",F19*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H19" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A19="",'Détails des dons'!J19=""),"",'Détails des dons'!J19)</f>
         <v/>
       </c>
@@ -9790,7 +9924,15 @@
         <f aca="false">IF(OR('Détails des dons'!A20="",'Détails des dons'!E20=""),"",'Détails des dons'!E20)</f>
         <v/>
       </c>
-      <c r="F20" s="48" t="str">
+      <c r="F20" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A20="",'Détails des dons'!H20=""),"",'Détails des dons'!H20)</f>
+        <v/>
+      </c>
+      <c r="G20" s="18" t="str">
+        <f aca="false">IF(F20="","",F20*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H20" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A20="",'Détails des dons'!J20=""),"",'Détails des dons'!J20)</f>
         <v/>
       </c>
@@ -9816,7 +9958,15 @@
         <f aca="false">IF(OR('Détails des dons'!A21="",'Détails des dons'!E21=""),"",'Détails des dons'!E21)</f>
         <v/>
       </c>
-      <c r="F21" s="48" t="str">
+      <c r="F21" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A21="",'Détails des dons'!H21=""),"",'Détails des dons'!H21)</f>
+        <v/>
+      </c>
+      <c r="G21" s="18" t="str">
+        <f aca="false">IF(F21="","",F21*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H21" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A21="",'Détails des dons'!J21=""),"",'Détails des dons'!J21)</f>
         <v/>
       </c>
@@ -9842,7 +9992,15 @@
         <f aca="false">IF(OR('Détails des dons'!A22="",'Détails des dons'!E22=""),"",'Détails des dons'!E22)</f>
         <v/>
       </c>
-      <c r="F22" s="48" t="str">
+      <c r="F22" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A22="",'Détails des dons'!H22=""),"",'Détails des dons'!H22)</f>
+        <v/>
+      </c>
+      <c r="G22" s="18" t="str">
+        <f aca="false">IF(F22="","",F22*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H22" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A22="",'Détails des dons'!J22=""),"",'Détails des dons'!J22)</f>
         <v/>
       </c>
@@ -9868,7 +10026,15 @@
         <f aca="false">IF(OR('Détails des dons'!A23="",'Détails des dons'!E23=""),"",'Détails des dons'!E23)</f>
         <v/>
       </c>
-      <c r="F23" s="48" t="str">
+      <c r="F23" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A23="",'Détails des dons'!H23=""),"",'Détails des dons'!H23)</f>
+        <v/>
+      </c>
+      <c r="G23" s="18" t="str">
+        <f aca="false">IF(F23="","",F23*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H23" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A23="",'Détails des dons'!J23=""),"",'Détails des dons'!J23)</f>
         <v/>
       </c>
@@ -9894,7 +10060,15 @@
         <f aca="false">IF(OR('Détails des dons'!A24="",'Détails des dons'!E24=""),"",'Détails des dons'!E24)</f>
         <v/>
       </c>
-      <c r="F24" s="48" t="str">
+      <c r="F24" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A24="",'Détails des dons'!H24=""),"",'Détails des dons'!H24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="18" t="str">
+        <f aca="false">IF(F24="","",F24*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H24" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A24="",'Détails des dons'!J24=""),"",'Détails des dons'!J24)</f>
         <v/>
       </c>
@@ -9920,7 +10094,15 @@
         <f aca="false">IF(OR('Détails des dons'!A25="",'Détails des dons'!E25=""),"",'Détails des dons'!E25)</f>
         <v/>
       </c>
-      <c r="F25" s="48" t="str">
+      <c r="F25" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A25="",'Détails des dons'!H25=""),"",'Détails des dons'!H25)</f>
+        <v/>
+      </c>
+      <c r="G25" s="18" t="str">
+        <f aca="false">IF(F25="","",F25*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H25" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A25="",'Détails des dons'!J25=""),"",'Détails des dons'!J25)</f>
         <v/>
       </c>
@@ -9946,7 +10128,15 @@
         <f aca="false">IF(OR('Détails des dons'!A26="",'Détails des dons'!E26=""),"",'Détails des dons'!E26)</f>
         <v/>
       </c>
-      <c r="F26" s="48" t="str">
+      <c r="F26" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A26="",'Détails des dons'!H26=""),"",'Détails des dons'!H26)</f>
+        <v/>
+      </c>
+      <c r="G26" s="18" t="str">
+        <f aca="false">IF(F26="","",F26*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H26" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A26="",'Détails des dons'!J26=""),"",'Détails des dons'!J26)</f>
         <v/>
       </c>
@@ -9972,7 +10162,15 @@
         <f aca="false">IF(OR('Détails des dons'!A27="",'Détails des dons'!E27=""),"",'Détails des dons'!E27)</f>
         <v/>
       </c>
-      <c r="F27" s="48" t="str">
+      <c r="F27" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A27="",'Détails des dons'!H27=""),"",'Détails des dons'!H27)</f>
+        <v/>
+      </c>
+      <c r="G27" s="18" t="str">
+        <f aca="false">IF(F27="","",F27*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H27" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A27="",'Détails des dons'!J27=""),"",'Détails des dons'!J27)</f>
         <v/>
       </c>
@@ -9998,7 +10196,15 @@
         <f aca="false">IF(OR('Détails des dons'!A28="",'Détails des dons'!E28=""),"",'Détails des dons'!E28)</f>
         <v/>
       </c>
-      <c r="F28" s="48" t="str">
+      <c r="F28" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A28="",'Détails des dons'!H28=""),"",'Détails des dons'!H28)</f>
+        <v/>
+      </c>
+      <c r="G28" s="18" t="str">
+        <f aca="false">IF(F28="","",F28*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H28" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A28="",'Détails des dons'!J28=""),"",'Détails des dons'!J28)</f>
         <v/>
       </c>
@@ -10024,7 +10230,15 @@
         <f aca="false">IF(OR('Détails des dons'!A29="",'Détails des dons'!E29=""),"",'Détails des dons'!E29)</f>
         <v/>
       </c>
-      <c r="F29" s="48" t="str">
+      <c r="F29" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A29="",'Détails des dons'!H29=""),"",'Détails des dons'!H29)</f>
+        <v/>
+      </c>
+      <c r="G29" s="18" t="str">
+        <f aca="false">IF(F29="","",F29*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H29" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A29="",'Détails des dons'!J29=""),"",'Détails des dons'!J29)</f>
         <v/>
       </c>
@@ -10050,7 +10264,15 @@
         <f aca="false">IF(OR('Détails des dons'!A30="",'Détails des dons'!E30=""),"",'Détails des dons'!E30)</f>
         <v/>
       </c>
-      <c r="F30" s="48" t="str">
+      <c r="F30" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A30="",'Détails des dons'!H30=""),"",'Détails des dons'!H30)</f>
+        <v/>
+      </c>
+      <c r="G30" s="18" t="str">
+        <f aca="false">IF(F30="","",F30*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H30" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A30="",'Détails des dons'!J30=""),"",'Détails des dons'!J30)</f>
         <v/>
       </c>
@@ -10076,7 +10298,15 @@
         <f aca="false">IF(OR('Détails des dons'!A31="",'Détails des dons'!E31=""),"",'Détails des dons'!E31)</f>
         <v/>
       </c>
-      <c r="F31" s="48" t="str">
+      <c r="F31" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A31="",'Détails des dons'!H31=""),"",'Détails des dons'!H31)</f>
+        <v/>
+      </c>
+      <c r="G31" s="18" t="str">
+        <f aca="false">IF(F31="","",F31*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H31" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A31="",'Détails des dons'!J31=""),"",'Détails des dons'!J31)</f>
         <v/>
       </c>
@@ -10102,7 +10332,15 @@
         <f aca="false">IF(OR('Détails des dons'!A32="",'Détails des dons'!E32=""),"",'Détails des dons'!E32)</f>
         <v/>
       </c>
-      <c r="F32" s="48" t="str">
+      <c r="F32" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A32="",'Détails des dons'!H32=""),"",'Détails des dons'!H32)</f>
+        <v/>
+      </c>
+      <c r="G32" s="18" t="str">
+        <f aca="false">IF(F32="","",F32*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H32" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A32="",'Détails des dons'!J32=""),"",'Détails des dons'!J32)</f>
         <v/>
       </c>
@@ -10128,7 +10366,15 @@
         <f aca="false">IF(OR('Détails des dons'!A33="",'Détails des dons'!E33=""),"",'Détails des dons'!E33)</f>
         <v/>
       </c>
-      <c r="F33" s="48" t="str">
+      <c r="F33" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A33="",'Détails des dons'!H33=""),"",'Détails des dons'!H33)</f>
+        <v/>
+      </c>
+      <c r="G33" s="18" t="str">
+        <f aca="false">IF(F33="","",F33*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H33" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A33="",'Détails des dons'!J33=""),"",'Détails des dons'!J33)</f>
         <v/>
       </c>
@@ -10154,7 +10400,15 @@
         <f aca="false">IF(OR('Détails des dons'!A34="",'Détails des dons'!E34=""),"",'Détails des dons'!E34)</f>
         <v/>
       </c>
-      <c r="F34" s="48" t="str">
+      <c r="F34" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A34="",'Détails des dons'!H34=""),"",'Détails des dons'!H34)</f>
+        <v/>
+      </c>
+      <c r="G34" s="18" t="str">
+        <f aca="false">IF(F34="","",F34*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H34" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A34="",'Détails des dons'!J34=""),"",'Détails des dons'!J34)</f>
         <v/>
       </c>
@@ -10180,7 +10434,15 @@
         <f aca="false">IF(OR('Détails des dons'!A35="",'Détails des dons'!E35=""),"",'Détails des dons'!E35)</f>
         <v/>
       </c>
-      <c r="F35" s="48" t="str">
+      <c r="F35" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A35="",'Détails des dons'!H35=""),"",'Détails des dons'!H35)</f>
+        <v/>
+      </c>
+      <c r="G35" s="18" t="str">
+        <f aca="false">IF(F35="","",F35*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H35" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A35="",'Détails des dons'!J35=""),"",'Détails des dons'!J35)</f>
         <v/>
       </c>
@@ -10206,7 +10468,15 @@
         <f aca="false">IF(OR('Détails des dons'!A36="",'Détails des dons'!E36=""),"",'Détails des dons'!E36)</f>
         <v/>
       </c>
-      <c r="F36" s="48" t="str">
+      <c r="F36" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A36="",'Détails des dons'!H36=""),"",'Détails des dons'!H36)</f>
+        <v/>
+      </c>
+      <c r="G36" s="18" t="str">
+        <f aca="false">IF(F36="","",F36*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H36" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A36="",'Détails des dons'!J36=""),"",'Détails des dons'!J36)</f>
         <v/>
       </c>
@@ -10232,7 +10502,15 @@
         <f aca="false">IF(OR('Détails des dons'!A37="",'Détails des dons'!E37=""),"",'Détails des dons'!E37)</f>
         <v/>
       </c>
-      <c r="F37" s="48" t="str">
+      <c r="F37" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A37="",'Détails des dons'!H37=""),"",'Détails des dons'!H37)</f>
+        <v/>
+      </c>
+      <c r="G37" s="18" t="str">
+        <f aca="false">IF(F37="","",F37*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H37" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A37="",'Détails des dons'!J37=""),"",'Détails des dons'!J37)</f>
         <v/>
       </c>
@@ -10258,7 +10536,15 @@
         <f aca="false">IF(OR('Détails des dons'!A38="",'Détails des dons'!E38=""),"",'Détails des dons'!E38)</f>
         <v/>
       </c>
-      <c r="F38" s="48" t="str">
+      <c r="F38" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A38="",'Détails des dons'!H38=""),"",'Détails des dons'!H38)</f>
+        <v/>
+      </c>
+      <c r="G38" s="18" t="str">
+        <f aca="false">IF(F38="","",F38*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H38" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A38="",'Détails des dons'!J38=""),"",'Détails des dons'!J38)</f>
         <v/>
       </c>
@@ -10284,7 +10570,15 @@
         <f aca="false">IF(OR('Détails des dons'!A39="",'Détails des dons'!E39=""),"",'Détails des dons'!E39)</f>
         <v/>
       </c>
-      <c r="F39" s="48" t="str">
+      <c r="F39" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A39="",'Détails des dons'!H39=""),"",'Détails des dons'!H39)</f>
+        <v/>
+      </c>
+      <c r="G39" s="18" t="str">
+        <f aca="false">IF(F39="","",F39*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H39" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A39="",'Détails des dons'!J39=""),"",'Détails des dons'!J39)</f>
         <v/>
       </c>
@@ -10310,7 +10604,15 @@
         <f aca="false">IF(OR('Détails des dons'!A40="",'Détails des dons'!E40=""),"",'Détails des dons'!E40)</f>
         <v/>
       </c>
-      <c r="F40" s="48" t="str">
+      <c r="F40" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A40="",'Détails des dons'!H40=""),"",'Détails des dons'!H40)</f>
+        <v/>
+      </c>
+      <c r="G40" s="18" t="str">
+        <f aca="false">IF(F40="","",F40*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H40" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A40="",'Détails des dons'!J40=""),"",'Détails des dons'!J40)</f>
         <v/>
       </c>
@@ -10336,7 +10638,15 @@
         <f aca="false">IF(OR('Détails des dons'!A41="",'Détails des dons'!E41=""),"",'Détails des dons'!E41)</f>
         <v/>
       </c>
-      <c r="F41" s="48" t="str">
+      <c r="F41" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A41="",'Détails des dons'!H41=""),"",'Détails des dons'!H41)</f>
+        <v/>
+      </c>
+      <c r="G41" s="18" t="str">
+        <f aca="false">IF(F41="","",F41*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H41" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A41="",'Détails des dons'!J41=""),"",'Détails des dons'!J41)</f>
         <v/>
       </c>
@@ -10362,7 +10672,15 @@
         <f aca="false">IF(OR('Détails des dons'!A42="",'Détails des dons'!E42=""),"",'Détails des dons'!E42)</f>
         <v/>
       </c>
-      <c r="F42" s="48" t="str">
+      <c r="F42" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A42="",'Détails des dons'!H42=""),"",'Détails des dons'!H42)</f>
+        <v/>
+      </c>
+      <c r="G42" s="18" t="str">
+        <f aca="false">IF(F42="","",F42*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H42" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A42="",'Détails des dons'!J42=""),"",'Détails des dons'!J42)</f>
         <v/>
       </c>
@@ -10388,7 +10706,15 @@
         <f aca="false">IF(OR('Détails des dons'!A43="",'Détails des dons'!E43=""),"",'Détails des dons'!E43)</f>
         <v/>
       </c>
-      <c r="F43" s="48" t="str">
+      <c r="F43" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A43="",'Détails des dons'!H43=""),"",'Détails des dons'!H43)</f>
+        <v/>
+      </c>
+      <c r="G43" s="18" t="str">
+        <f aca="false">IF(F43="","",F43*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H43" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A43="",'Détails des dons'!J43=""),"",'Détails des dons'!J43)</f>
         <v/>
       </c>
@@ -10414,7 +10740,15 @@
         <f aca="false">IF(OR('Détails des dons'!A44="",'Détails des dons'!E44=""),"",'Détails des dons'!E44)</f>
         <v/>
       </c>
-      <c r="F44" s="48" t="str">
+      <c r="F44" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A44="",'Détails des dons'!H44=""),"",'Détails des dons'!H44)</f>
+        <v/>
+      </c>
+      <c r="G44" s="18" t="str">
+        <f aca="false">IF(F44="","",F44*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H44" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A44="",'Détails des dons'!J44=""),"",'Détails des dons'!J44)</f>
         <v/>
       </c>
@@ -10440,7 +10774,15 @@
         <f aca="false">IF(OR('Détails des dons'!A45="",'Détails des dons'!E45=""),"",'Détails des dons'!E45)</f>
         <v/>
       </c>
-      <c r="F45" s="48" t="str">
+      <c r="F45" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A45="",'Détails des dons'!H45=""),"",'Détails des dons'!H45)</f>
+        <v/>
+      </c>
+      <c r="G45" s="18" t="str">
+        <f aca="false">IF(F45="","",F45*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H45" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A45="",'Détails des dons'!J45=""),"",'Détails des dons'!J45)</f>
         <v/>
       </c>
@@ -10466,7 +10808,15 @@
         <f aca="false">IF(OR('Détails des dons'!A46="",'Détails des dons'!E46=""),"",'Détails des dons'!E46)</f>
         <v/>
       </c>
-      <c r="F46" s="48" t="str">
+      <c r="F46" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A46="",'Détails des dons'!H46=""),"",'Détails des dons'!H46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="18" t="str">
+        <f aca="false">IF(F46="","",F46*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H46" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A46="",'Détails des dons'!J46=""),"",'Détails des dons'!J46)</f>
         <v/>
       </c>
@@ -10492,7 +10842,15 @@
         <f aca="false">IF(OR('Détails des dons'!A47="",'Détails des dons'!E47=""),"",'Détails des dons'!E47)</f>
         <v/>
       </c>
-      <c r="F47" s="48" t="str">
+      <c r="F47" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A47="",'Détails des dons'!H47=""),"",'Détails des dons'!H47)</f>
+        <v/>
+      </c>
+      <c r="G47" s="18" t="str">
+        <f aca="false">IF(F47="","",F47*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H47" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A47="",'Détails des dons'!J47=""),"",'Détails des dons'!J47)</f>
         <v/>
       </c>
@@ -10518,7 +10876,15 @@
         <f aca="false">IF(OR('Détails des dons'!A48="",'Détails des dons'!E48=""),"",'Détails des dons'!E48)</f>
         <v/>
       </c>
-      <c r="F48" s="48" t="str">
+      <c r="F48" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A48="",'Détails des dons'!H48=""),"",'Détails des dons'!H48)</f>
+        <v/>
+      </c>
+      <c r="G48" s="18" t="str">
+        <f aca="false">IF(F48="","",F48*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H48" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A48="",'Détails des dons'!J48=""),"",'Détails des dons'!J48)</f>
         <v/>
       </c>
@@ -10544,7 +10910,15 @@
         <f aca="false">IF(OR('Détails des dons'!A49="",'Détails des dons'!E49=""),"",'Détails des dons'!E49)</f>
         <v/>
       </c>
-      <c r="F49" s="48" t="str">
+      <c r="F49" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A49="",'Détails des dons'!H49=""),"",'Détails des dons'!H49)</f>
+        <v/>
+      </c>
+      <c r="G49" s="18" t="str">
+        <f aca="false">IF(F49="","",F49*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H49" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A49="",'Détails des dons'!J49=""),"",'Détails des dons'!J49)</f>
         <v/>
       </c>
@@ -10570,7 +10944,15 @@
         <f aca="false">IF(OR('Détails des dons'!A50="",'Détails des dons'!E50=""),"",'Détails des dons'!E50)</f>
         <v/>
       </c>
-      <c r="F50" s="48" t="str">
+      <c r="F50" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A50="",'Détails des dons'!H50=""),"",'Détails des dons'!H50)</f>
+        <v/>
+      </c>
+      <c r="G50" s="18" t="str">
+        <f aca="false">IF(F50="","",F50*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H50" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A50="",'Détails des dons'!J50=""),"",'Détails des dons'!J50)</f>
         <v/>
       </c>
@@ -10596,7 +10978,15 @@
         <f aca="false">IF(OR('Détails des dons'!A51="",'Détails des dons'!E51=""),"",'Détails des dons'!E51)</f>
         <v/>
       </c>
-      <c r="F51" s="48" t="str">
+      <c r="F51" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A51="",'Détails des dons'!H51=""),"",'Détails des dons'!H51)</f>
+        <v/>
+      </c>
+      <c r="G51" s="18" t="str">
+        <f aca="false">IF(F51="","",F51*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H51" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A51="",'Détails des dons'!J51=""),"",'Détails des dons'!J51)</f>
         <v/>
       </c>
@@ -10622,7 +11012,15 @@
         <f aca="false">IF(OR('Détails des dons'!A52="",'Détails des dons'!E52=""),"",'Détails des dons'!E52)</f>
         <v/>
       </c>
-      <c r="F52" s="48" t="str">
+      <c r="F52" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A52="",'Détails des dons'!H52=""),"",'Détails des dons'!H52)</f>
+        <v/>
+      </c>
+      <c r="G52" s="18" t="str">
+        <f aca="false">IF(F52="","",F52*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H52" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A52="",'Détails des dons'!J52=""),"",'Détails des dons'!J52)</f>
         <v/>
       </c>
@@ -10648,7 +11046,15 @@
         <f aca="false">IF(OR('Détails des dons'!A53="",'Détails des dons'!E53=""),"",'Détails des dons'!E53)</f>
         <v/>
       </c>
-      <c r="F53" s="48" t="str">
+      <c r="F53" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A53="",'Détails des dons'!H53=""),"",'Détails des dons'!H53)</f>
+        <v/>
+      </c>
+      <c r="G53" s="18" t="str">
+        <f aca="false">IF(F53="","",F53*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H53" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A53="",'Détails des dons'!J53=""),"",'Détails des dons'!J53)</f>
         <v/>
       </c>
@@ -10674,7 +11080,15 @@
         <f aca="false">IF(OR('Détails des dons'!A54="",'Détails des dons'!E54=""),"",'Détails des dons'!E54)</f>
         <v/>
       </c>
-      <c r="F54" s="48" t="str">
+      <c r="F54" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A54="",'Détails des dons'!H54=""),"",'Détails des dons'!H54)</f>
+        <v/>
+      </c>
+      <c r="G54" s="18" t="str">
+        <f aca="false">IF(F54="","",F54*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H54" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A54="",'Détails des dons'!J54=""),"",'Détails des dons'!J54)</f>
         <v/>
       </c>
@@ -10700,7 +11114,15 @@
         <f aca="false">IF(OR('Détails des dons'!A55="",'Détails des dons'!E55=""),"",'Détails des dons'!E55)</f>
         <v/>
       </c>
-      <c r="F55" s="48" t="str">
+      <c r="F55" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A55="",'Détails des dons'!H55=""),"",'Détails des dons'!H55)</f>
+        <v/>
+      </c>
+      <c r="G55" s="18" t="str">
+        <f aca="false">IF(F55="","",F55*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H55" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A55="",'Détails des dons'!J55=""),"",'Détails des dons'!J55)</f>
         <v/>
       </c>
@@ -10726,7 +11148,15 @@
         <f aca="false">IF(OR('Détails des dons'!A56="",'Détails des dons'!E56=""),"",'Détails des dons'!E56)</f>
         <v/>
       </c>
-      <c r="F56" s="48" t="str">
+      <c r="F56" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A56="",'Détails des dons'!H56=""),"",'Détails des dons'!H56)</f>
+        <v/>
+      </c>
+      <c r="G56" s="18" t="str">
+        <f aca="false">IF(F56="","",F56*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H56" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A56="",'Détails des dons'!J56=""),"",'Détails des dons'!J56)</f>
         <v/>
       </c>
@@ -10752,7 +11182,15 @@
         <f aca="false">IF(OR('Détails des dons'!A57="",'Détails des dons'!E57=""),"",'Détails des dons'!E57)</f>
         <v/>
       </c>
-      <c r="F57" s="48" t="str">
+      <c r="F57" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A57="",'Détails des dons'!H57=""),"",'Détails des dons'!H57)</f>
+        <v/>
+      </c>
+      <c r="G57" s="18" t="str">
+        <f aca="false">IF(F57="","",F57*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H57" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A57="",'Détails des dons'!J57=""),"",'Détails des dons'!J57)</f>
         <v/>
       </c>
@@ -10778,7 +11216,15 @@
         <f aca="false">IF(OR('Détails des dons'!A58="",'Détails des dons'!E58=""),"",'Détails des dons'!E58)</f>
         <v/>
       </c>
-      <c r="F58" s="48" t="str">
+      <c r="F58" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A58="",'Détails des dons'!H58=""),"",'Détails des dons'!H58)</f>
+        <v/>
+      </c>
+      <c r="G58" s="18" t="str">
+        <f aca="false">IF(F58="","",F58*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H58" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A58="",'Détails des dons'!J58=""),"",'Détails des dons'!J58)</f>
         <v/>
       </c>
@@ -10804,7 +11250,15 @@
         <f aca="false">IF(OR('Détails des dons'!A59="",'Détails des dons'!E59=""),"",'Détails des dons'!E59)</f>
         <v/>
       </c>
-      <c r="F59" s="48" t="str">
+      <c r="F59" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A59="",'Détails des dons'!H59=""),"",'Détails des dons'!H59)</f>
+        <v/>
+      </c>
+      <c r="G59" s="18" t="str">
+        <f aca="false">IF(F59="","",F59*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H59" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A59="",'Détails des dons'!J59=""),"",'Détails des dons'!J59)</f>
         <v/>
       </c>
@@ -10830,7 +11284,15 @@
         <f aca="false">IF(OR('Détails des dons'!A60="",'Détails des dons'!E60=""),"",'Détails des dons'!E60)</f>
         <v/>
       </c>
-      <c r="F60" s="48" t="str">
+      <c r="F60" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A60="",'Détails des dons'!H60=""),"",'Détails des dons'!H60)</f>
+        <v/>
+      </c>
+      <c r="G60" s="18" t="str">
+        <f aca="false">IF(F60="","",F60*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H60" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A60="",'Détails des dons'!J60=""),"",'Détails des dons'!J60)</f>
         <v/>
       </c>
@@ -10856,7 +11318,15 @@
         <f aca="false">IF(OR('Détails des dons'!A61="",'Détails des dons'!E61=""),"",'Détails des dons'!E61)</f>
         <v/>
       </c>
-      <c r="F61" s="48" t="str">
+      <c r="F61" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A61="",'Détails des dons'!H61=""),"",'Détails des dons'!H61)</f>
+        <v/>
+      </c>
+      <c r="G61" s="18" t="str">
+        <f aca="false">IF(F61="","",F61*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H61" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A61="",'Détails des dons'!J61=""),"",'Détails des dons'!J61)</f>
         <v/>
       </c>
@@ -10882,7 +11352,15 @@
         <f aca="false">IF(OR('Détails des dons'!A62="",'Détails des dons'!E62=""),"",'Détails des dons'!E62)</f>
         <v/>
       </c>
-      <c r="F62" s="48" t="str">
+      <c r="F62" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A62="",'Détails des dons'!H62=""),"",'Détails des dons'!H62)</f>
+        <v/>
+      </c>
+      <c r="G62" s="18" t="str">
+        <f aca="false">IF(F62="","",F62*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H62" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A62="",'Détails des dons'!J62=""),"",'Détails des dons'!J62)</f>
         <v/>
       </c>
@@ -10908,7 +11386,15 @@
         <f aca="false">IF(OR('Détails des dons'!A63="",'Détails des dons'!E63=""),"",'Détails des dons'!E63)</f>
         <v/>
       </c>
-      <c r="F63" s="48" t="str">
+      <c r="F63" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A63="",'Détails des dons'!H63=""),"",'Détails des dons'!H63)</f>
+        <v/>
+      </c>
+      <c r="G63" s="18" t="str">
+        <f aca="false">IF(F63="","",F63*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H63" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A63="",'Détails des dons'!J63=""),"",'Détails des dons'!J63)</f>
         <v/>
       </c>
@@ -10934,7 +11420,15 @@
         <f aca="false">IF(OR('Détails des dons'!A64="",'Détails des dons'!E64=""),"",'Détails des dons'!E64)</f>
         <v/>
       </c>
-      <c r="F64" s="48" t="str">
+      <c r="F64" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A64="",'Détails des dons'!H64=""),"",'Détails des dons'!H64)</f>
+        <v/>
+      </c>
+      <c r="G64" s="18" t="str">
+        <f aca="false">IF(F64="","",F64*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H64" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A64="",'Détails des dons'!J64=""),"",'Détails des dons'!J64)</f>
         <v/>
       </c>
@@ -10960,7 +11454,15 @@
         <f aca="false">IF(OR('Détails des dons'!A65="",'Détails des dons'!E65=""),"",'Détails des dons'!E65)</f>
         <v/>
       </c>
-      <c r="F65" s="48" t="str">
+      <c r="F65" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A65="",'Détails des dons'!H65=""),"",'Détails des dons'!H65)</f>
+        <v/>
+      </c>
+      <c r="G65" s="18" t="str">
+        <f aca="false">IF(F65="","",F65*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H65" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A65="",'Détails des dons'!J65=""),"",'Détails des dons'!J65)</f>
         <v/>
       </c>
@@ -10986,7 +11488,15 @@
         <f aca="false">IF(OR('Détails des dons'!A66="",'Détails des dons'!E66=""),"",'Détails des dons'!E66)</f>
         <v/>
       </c>
-      <c r="F66" s="48" t="str">
+      <c r="F66" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A66="",'Détails des dons'!H66=""),"",'Détails des dons'!H66)</f>
+        <v/>
+      </c>
+      <c r="G66" s="18" t="str">
+        <f aca="false">IF(F66="","",F66*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H66" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A66="",'Détails des dons'!J66=""),"",'Détails des dons'!J66)</f>
         <v/>
       </c>
@@ -11012,7 +11522,15 @@
         <f aca="false">IF(OR('Détails des dons'!A67="",'Détails des dons'!E67=""),"",'Détails des dons'!E67)</f>
         <v/>
       </c>
-      <c r="F67" s="48" t="str">
+      <c r="F67" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A67="",'Détails des dons'!H67=""),"",'Détails des dons'!H67)</f>
+        <v/>
+      </c>
+      <c r="G67" s="18" t="str">
+        <f aca="false">IF(F67="","",F67*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H67" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A67="",'Détails des dons'!J67=""),"",'Détails des dons'!J67)</f>
         <v/>
       </c>
@@ -11038,7 +11556,15 @@
         <f aca="false">IF(OR('Détails des dons'!A68="",'Détails des dons'!E68=""),"",'Détails des dons'!E68)</f>
         <v/>
       </c>
-      <c r="F68" s="48" t="str">
+      <c r="F68" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A68="",'Détails des dons'!H68=""),"",'Détails des dons'!H68)</f>
+        <v/>
+      </c>
+      <c r="G68" s="18" t="str">
+        <f aca="false">IF(F68="","",F68*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H68" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A68="",'Détails des dons'!J68=""),"",'Détails des dons'!J68)</f>
         <v/>
       </c>
@@ -11064,7 +11590,15 @@
         <f aca="false">IF(OR('Détails des dons'!A69="",'Détails des dons'!E69=""),"",'Détails des dons'!E69)</f>
         <v/>
       </c>
-      <c r="F69" s="48" t="str">
+      <c r="F69" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A69="",'Détails des dons'!H69=""),"",'Détails des dons'!H69)</f>
+        <v/>
+      </c>
+      <c r="G69" s="18" t="str">
+        <f aca="false">IF(F69="","",F69*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H69" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A69="",'Détails des dons'!J69=""),"",'Détails des dons'!J69)</f>
         <v/>
       </c>
@@ -11090,7 +11624,15 @@
         <f aca="false">IF(OR('Détails des dons'!A70="",'Détails des dons'!E70=""),"",'Détails des dons'!E70)</f>
         <v/>
       </c>
-      <c r="F70" s="48" t="str">
+      <c r="F70" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A70="",'Détails des dons'!H70=""),"",'Détails des dons'!H70)</f>
+        <v/>
+      </c>
+      <c r="G70" s="18" t="str">
+        <f aca="false">IF(F70="","",F70*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H70" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A70="",'Détails des dons'!J70=""),"",'Détails des dons'!J70)</f>
         <v/>
       </c>
@@ -11116,7 +11658,15 @@
         <f aca="false">IF(OR('Détails des dons'!A71="",'Détails des dons'!E71=""),"",'Détails des dons'!E71)</f>
         <v/>
       </c>
-      <c r="F71" s="48" t="str">
+      <c r="F71" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A71="",'Détails des dons'!H71=""),"",'Détails des dons'!H71)</f>
+        <v/>
+      </c>
+      <c r="G71" s="18" t="str">
+        <f aca="false">IF(F71="","",F71*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H71" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A71="",'Détails des dons'!J71=""),"",'Détails des dons'!J71)</f>
         <v/>
       </c>
@@ -11142,7 +11692,15 @@
         <f aca="false">IF(OR('Détails des dons'!A72="",'Détails des dons'!E72=""),"",'Détails des dons'!E72)</f>
         <v/>
       </c>
-      <c r="F72" s="48" t="str">
+      <c r="F72" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A72="",'Détails des dons'!H72=""),"",'Détails des dons'!H72)</f>
+        <v/>
+      </c>
+      <c r="G72" s="18" t="str">
+        <f aca="false">IF(F72="","",F72*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H72" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A72="",'Détails des dons'!J72=""),"",'Détails des dons'!J72)</f>
         <v/>
       </c>
@@ -11168,7 +11726,15 @@
         <f aca="false">IF(OR('Détails des dons'!A73="",'Détails des dons'!E73=""),"",'Détails des dons'!E73)</f>
         <v/>
       </c>
-      <c r="F73" s="48" t="str">
+      <c r="F73" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A73="",'Détails des dons'!H73=""),"",'Détails des dons'!H73)</f>
+        <v/>
+      </c>
+      <c r="G73" s="18" t="str">
+        <f aca="false">IF(F73="","",F73*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H73" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A73="",'Détails des dons'!J73=""),"",'Détails des dons'!J73)</f>
         <v/>
       </c>
@@ -11194,7 +11760,15 @@
         <f aca="false">IF(OR('Détails des dons'!A74="",'Détails des dons'!E74=""),"",'Détails des dons'!E74)</f>
         <v/>
       </c>
-      <c r="F74" s="48" t="str">
+      <c r="F74" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A74="",'Détails des dons'!H74=""),"",'Détails des dons'!H74)</f>
+        <v/>
+      </c>
+      <c r="G74" s="18" t="str">
+        <f aca="false">IF(F74="","",F74*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H74" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A74="",'Détails des dons'!J74=""),"",'Détails des dons'!J74)</f>
         <v/>
       </c>
@@ -11220,7 +11794,15 @@
         <f aca="false">IF(OR('Détails des dons'!A75="",'Détails des dons'!E75=""),"",'Détails des dons'!E75)</f>
         <v/>
       </c>
-      <c r="F75" s="48" t="str">
+      <c r="F75" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A75="",'Détails des dons'!H75=""),"",'Détails des dons'!H75)</f>
+        <v/>
+      </c>
+      <c r="G75" s="18" t="str">
+        <f aca="false">IF(F75="","",F75*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H75" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A75="",'Détails des dons'!J75=""),"",'Détails des dons'!J75)</f>
         <v/>
       </c>
@@ -11246,7 +11828,15 @@
         <f aca="false">IF(OR('Détails des dons'!A76="",'Détails des dons'!E76=""),"",'Détails des dons'!E76)</f>
         <v/>
       </c>
-      <c r="F76" s="48" t="str">
+      <c r="F76" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A76="",'Détails des dons'!H76=""),"",'Détails des dons'!H76)</f>
+        <v/>
+      </c>
+      <c r="G76" s="18" t="str">
+        <f aca="false">IF(F76="","",F76*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H76" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A76="",'Détails des dons'!J76=""),"",'Détails des dons'!J76)</f>
         <v/>
       </c>
@@ -11272,7 +11862,15 @@
         <f aca="false">IF(OR('Détails des dons'!A77="",'Détails des dons'!E77=""),"",'Détails des dons'!E77)</f>
         <v/>
       </c>
-      <c r="F77" s="48" t="str">
+      <c r="F77" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A77="",'Détails des dons'!H77=""),"",'Détails des dons'!H77)</f>
+        <v/>
+      </c>
+      <c r="G77" s="18" t="str">
+        <f aca="false">IF(F77="","",F77*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H77" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A77="",'Détails des dons'!J77=""),"",'Détails des dons'!J77)</f>
         <v/>
       </c>
@@ -11298,7 +11896,15 @@
         <f aca="false">IF(OR('Détails des dons'!A78="",'Détails des dons'!E78=""),"",'Détails des dons'!E78)</f>
         <v/>
       </c>
-      <c r="F78" s="48" t="str">
+      <c r="F78" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A78="",'Détails des dons'!H78=""),"",'Détails des dons'!H78)</f>
+        <v/>
+      </c>
+      <c r="G78" s="18" t="str">
+        <f aca="false">IF(F78="","",F78*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H78" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A78="",'Détails des dons'!J78=""),"",'Détails des dons'!J78)</f>
         <v/>
       </c>
@@ -11324,7 +11930,15 @@
         <f aca="false">IF(OR('Détails des dons'!A79="",'Détails des dons'!E79=""),"",'Détails des dons'!E79)</f>
         <v/>
       </c>
-      <c r="F79" s="48" t="str">
+      <c r="F79" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A79="",'Détails des dons'!H79=""),"",'Détails des dons'!H79)</f>
+        <v/>
+      </c>
+      <c r="G79" s="18" t="str">
+        <f aca="false">IF(F79="","",F79*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H79" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A79="",'Détails des dons'!J79=""),"",'Détails des dons'!J79)</f>
         <v/>
       </c>
@@ -11350,7 +11964,15 @@
         <f aca="false">IF(OR('Détails des dons'!A80="",'Détails des dons'!E80=""),"",'Détails des dons'!E80)</f>
         <v/>
       </c>
-      <c r="F80" s="48" t="str">
+      <c r="F80" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A80="",'Détails des dons'!H80=""),"",'Détails des dons'!H80)</f>
+        <v/>
+      </c>
+      <c r="G80" s="18" t="str">
+        <f aca="false">IF(F80="","",F80*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H80" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A80="",'Détails des dons'!J80=""),"",'Détails des dons'!J80)</f>
         <v/>
       </c>
@@ -11376,7 +11998,15 @@
         <f aca="false">IF(OR('Détails des dons'!A81="",'Détails des dons'!E81=""),"",'Détails des dons'!E81)</f>
         <v/>
       </c>
-      <c r="F81" s="48" t="str">
+      <c r="F81" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A81="",'Détails des dons'!H81=""),"",'Détails des dons'!H81)</f>
+        <v/>
+      </c>
+      <c r="G81" s="18" t="str">
+        <f aca="false">IF(F81="","",F81*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H81" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A81="",'Détails des dons'!J81=""),"",'Détails des dons'!J81)</f>
         <v/>
       </c>
@@ -11402,7 +12032,15 @@
         <f aca="false">IF(OR('Détails des dons'!A82="",'Détails des dons'!E82=""),"",'Détails des dons'!E82)</f>
         <v/>
       </c>
-      <c r="F82" s="48" t="str">
+      <c r="F82" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A82="",'Détails des dons'!H82=""),"",'Détails des dons'!H82)</f>
+        <v/>
+      </c>
+      <c r="G82" s="18" t="str">
+        <f aca="false">IF(F82="","",F82*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H82" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A82="",'Détails des dons'!J82=""),"",'Détails des dons'!J82)</f>
         <v/>
       </c>
@@ -11428,7 +12066,15 @@
         <f aca="false">IF(OR('Détails des dons'!A83="",'Détails des dons'!E83=""),"",'Détails des dons'!E83)</f>
         <v/>
       </c>
-      <c r="F83" s="48" t="str">
+      <c r="F83" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A83="",'Détails des dons'!H83=""),"",'Détails des dons'!H83)</f>
+        <v/>
+      </c>
+      <c r="G83" s="18" t="str">
+        <f aca="false">IF(F83="","",F83*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H83" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A83="",'Détails des dons'!J83=""),"",'Détails des dons'!J83)</f>
         <v/>
       </c>
@@ -11454,7 +12100,15 @@
         <f aca="false">IF(OR('Détails des dons'!A84="",'Détails des dons'!E84=""),"",'Détails des dons'!E84)</f>
         <v/>
       </c>
-      <c r="F84" s="48" t="str">
+      <c r="F84" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A84="",'Détails des dons'!H84=""),"",'Détails des dons'!H84)</f>
+        <v/>
+      </c>
+      <c r="G84" s="18" t="str">
+        <f aca="false">IF(F84="","",F84*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H84" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A84="",'Détails des dons'!J84=""),"",'Détails des dons'!J84)</f>
         <v/>
       </c>
@@ -11480,7 +12134,15 @@
         <f aca="false">IF(OR('Détails des dons'!A85="",'Détails des dons'!E85=""),"",'Détails des dons'!E85)</f>
         <v/>
       </c>
-      <c r="F85" s="48" t="str">
+      <c r="F85" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A85="",'Détails des dons'!H85=""),"",'Détails des dons'!H85)</f>
+        <v/>
+      </c>
+      <c r="G85" s="18" t="str">
+        <f aca="false">IF(F85="","",F85*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H85" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A85="",'Détails des dons'!J85=""),"",'Détails des dons'!J85)</f>
         <v/>
       </c>
@@ -11506,7 +12168,15 @@
         <f aca="false">IF(OR('Détails des dons'!A86="",'Détails des dons'!E86=""),"",'Détails des dons'!E86)</f>
         <v/>
       </c>
-      <c r="F86" s="48" t="str">
+      <c r="F86" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A86="",'Détails des dons'!H86=""),"",'Détails des dons'!H86)</f>
+        <v/>
+      </c>
+      <c r="G86" s="18" t="str">
+        <f aca="false">IF(F86="","",F86*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H86" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A86="",'Détails des dons'!J86=""),"",'Détails des dons'!J86)</f>
         <v/>
       </c>
@@ -11532,7 +12202,15 @@
         <f aca="false">IF(OR('Détails des dons'!A87="",'Détails des dons'!E87=""),"",'Détails des dons'!E87)</f>
         <v/>
       </c>
-      <c r="F87" s="48" t="str">
+      <c r="F87" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A87="",'Détails des dons'!H87=""),"",'Détails des dons'!H87)</f>
+        <v/>
+      </c>
+      <c r="G87" s="18" t="str">
+        <f aca="false">IF(F87="","",F87*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H87" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A87="",'Détails des dons'!J87=""),"",'Détails des dons'!J87)</f>
         <v/>
       </c>
@@ -11558,7 +12236,15 @@
         <f aca="false">IF(OR('Détails des dons'!A88="",'Détails des dons'!E88=""),"",'Détails des dons'!E88)</f>
         <v/>
       </c>
-      <c r="F88" s="48" t="str">
+      <c r="F88" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A88="",'Détails des dons'!H88=""),"",'Détails des dons'!H88)</f>
+        <v/>
+      </c>
+      <c r="G88" s="18" t="str">
+        <f aca="false">IF(F88="","",F88*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H88" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A88="",'Détails des dons'!J88=""),"",'Détails des dons'!J88)</f>
         <v/>
       </c>
@@ -11584,7 +12270,15 @@
         <f aca="false">IF(OR('Détails des dons'!A89="",'Détails des dons'!E89=""),"",'Détails des dons'!E89)</f>
         <v/>
       </c>
-      <c r="F89" s="48" t="str">
+      <c r="F89" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A89="",'Détails des dons'!H89=""),"",'Détails des dons'!H89)</f>
+        <v/>
+      </c>
+      <c r="G89" s="18" t="str">
+        <f aca="false">IF(F89="","",F89*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H89" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A89="",'Détails des dons'!J89=""),"",'Détails des dons'!J89)</f>
         <v/>
       </c>
@@ -11610,7 +12304,15 @@
         <f aca="false">IF(OR('Détails des dons'!A90="",'Détails des dons'!E90=""),"",'Détails des dons'!E90)</f>
         <v/>
       </c>
-      <c r="F90" s="48" t="str">
+      <c r="F90" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A90="",'Détails des dons'!H90=""),"",'Détails des dons'!H90)</f>
+        <v/>
+      </c>
+      <c r="G90" s="18" t="str">
+        <f aca="false">IF(F90="","",F90*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H90" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A90="",'Détails des dons'!J90=""),"",'Détails des dons'!J90)</f>
         <v/>
       </c>
@@ -11636,7 +12338,15 @@
         <f aca="false">IF(OR('Détails des dons'!A91="",'Détails des dons'!E91=""),"",'Détails des dons'!E91)</f>
         <v/>
       </c>
-      <c r="F91" s="48" t="str">
+      <c r="F91" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A91="",'Détails des dons'!H91=""),"",'Détails des dons'!H91)</f>
+        <v/>
+      </c>
+      <c r="G91" s="18" t="str">
+        <f aca="false">IF(F91="","",F91*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H91" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A91="",'Détails des dons'!J91=""),"",'Détails des dons'!J91)</f>
         <v/>
       </c>
@@ -11662,7 +12372,15 @@
         <f aca="false">IF(OR('Détails des dons'!A92="",'Détails des dons'!E92=""),"",'Détails des dons'!E92)</f>
         <v/>
       </c>
-      <c r="F92" s="48" t="str">
+      <c r="F92" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A92="",'Détails des dons'!H92=""),"",'Détails des dons'!H92)</f>
+        <v/>
+      </c>
+      <c r="G92" s="18" t="str">
+        <f aca="false">IF(F92="","",F92*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H92" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A92="",'Détails des dons'!J92=""),"",'Détails des dons'!J92)</f>
         <v/>
       </c>
@@ -11688,7 +12406,15 @@
         <f aca="false">IF(OR('Détails des dons'!A93="",'Détails des dons'!E93=""),"",'Détails des dons'!E93)</f>
         <v/>
       </c>
-      <c r="F93" s="48" t="str">
+      <c r="F93" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A93="",'Détails des dons'!H93=""),"",'Détails des dons'!H93)</f>
+        <v/>
+      </c>
+      <c r="G93" s="18" t="str">
+        <f aca="false">IF(F93="","",F93*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H93" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A93="",'Détails des dons'!J93=""),"",'Détails des dons'!J93)</f>
         <v/>
       </c>
@@ -11714,7 +12440,15 @@
         <f aca="false">IF(OR('Détails des dons'!A94="",'Détails des dons'!E94=""),"",'Détails des dons'!E94)</f>
         <v/>
       </c>
-      <c r="F94" s="48" t="str">
+      <c r="F94" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A94="",'Détails des dons'!H94=""),"",'Détails des dons'!H94)</f>
+        <v/>
+      </c>
+      <c r="G94" s="18" t="str">
+        <f aca="false">IF(F94="","",F94*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H94" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A94="",'Détails des dons'!J94=""),"",'Détails des dons'!J94)</f>
         <v/>
       </c>
@@ -11740,7 +12474,15 @@
         <f aca="false">IF(OR('Détails des dons'!A95="",'Détails des dons'!E95=""),"",'Détails des dons'!E95)</f>
         <v/>
       </c>
-      <c r="F95" s="48" t="str">
+      <c r="F95" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A95="",'Détails des dons'!H95=""),"",'Détails des dons'!H95)</f>
+        <v/>
+      </c>
+      <c r="G95" s="18" t="str">
+        <f aca="false">IF(F95="","",F95*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H95" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A95="",'Détails des dons'!J95=""),"",'Détails des dons'!J95)</f>
         <v/>
       </c>
@@ -11766,7 +12508,15 @@
         <f aca="false">IF(OR('Détails des dons'!A96="",'Détails des dons'!E96=""),"",'Détails des dons'!E96)</f>
         <v/>
       </c>
-      <c r="F96" s="48" t="str">
+      <c r="F96" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A96="",'Détails des dons'!H96=""),"",'Détails des dons'!H96)</f>
+        <v/>
+      </c>
+      <c r="G96" s="18" t="str">
+        <f aca="false">IF(F96="","",F96*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H96" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A96="",'Détails des dons'!J96=""),"",'Détails des dons'!J96)</f>
         <v/>
       </c>
@@ -11792,7 +12542,15 @@
         <f aca="false">IF(OR('Détails des dons'!A97="",'Détails des dons'!E97=""),"",'Détails des dons'!E97)</f>
         <v/>
       </c>
-      <c r="F97" s="48" t="str">
+      <c r="F97" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A97="",'Détails des dons'!H97=""),"",'Détails des dons'!H97)</f>
+        <v/>
+      </c>
+      <c r="G97" s="18" t="str">
+        <f aca="false">IF(F97="","",F97*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H97" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A97="",'Détails des dons'!J97=""),"",'Détails des dons'!J97)</f>
         <v/>
       </c>
@@ -11818,7 +12576,15 @@
         <f aca="false">IF(OR('Détails des dons'!A98="",'Détails des dons'!E98=""),"",'Détails des dons'!E98)</f>
         <v/>
       </c>
-      <c r="F98" s="48" t="str">
+      <c r="F98" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A98="",'Détails des dons'!H98=""),"",'Détails des dons'!H98)</f>
+        <v/>
+      </c>
+      <c r="G98" s="18" t="str">
+        <f aca="false">IF(F98="","",F98*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H98" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A98="",'Détails des dons'!J98=""),"",'Détails des dons'!J98)</f>
         <v/>
       </c>
@@ -11844,7 +12610,15 @@
         <f aca="false">IF(OR('Détails des dons'!A99="",'Détails des dons'!E99=""),"",'Détails des dons'!E99)</f>
         <v/>
       </c>
-      <c r="F99" s="48" t="str">
+      <c r="F99" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A99="",'Détails des dons'!H99=""),"",'Détails des dons'!H99)</f>
+        <v/>
+      </c>
+      <c r="G99" s="18" t="str">
+        <f aca="false">IF(F99="","",F99*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H99" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A99="",'Détails des dons'!J99=""),"",'Détails des dons'!J99)</f>
         <v/>
       </c>
@@ -11870,7 +12644,15 @@
         <f aca="false">IF(OR('Détails des dons'!A100="",'Détails des dons'!E100=""),"",'Détails des dons'!E100)</f>
         <v/>
       </c>
-      <c r="F100" s="48" t="str">
+      <c r="F100" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A100="",'Détails des dons'!H100=""),"",'Détails des dons'!H100)</f>
+        <v/>
+      </c>
+      <c r="G100" s="18" t="str">
+        <f aca="false">IF(F100="","",F100*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H100" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A100="",'Détails des dons'!J100=""),"",'Détails des dons'!J100)</f>
         <v/>
       </c>
@@ -11896,7 +12678,15 @@
         <f aca="false">IF(OR('Détails des dons'!A101="",'Détails des dons'!E101=""),"",'Détails des dons'!E101)</f>
         <v/>
       </c>
-      <c r="F101" s="48" t="str">
+      <c r="F101" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A101="",'Détails des dons'!H101=""),"",'Détails des dons'!H101)</f>
+        <v/>
+      </c>
+      <c r="G101" s="18" t="str">
+        <f aca="false">IF(F101="","",F101*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H101" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A101="",'Détails des dons'!J101=""),"",'Détails des dons'!J101)</f>
         <v/>
       </c>
@@ -11922,7 +12712,15 @@
         <f aca="false">IF(OR('Détails des dons'!A102="",'Détails des dons'!E102=""),"",'Détails des dons'!E102)</f>
         <v/>
       </c>
-      <c r="F102" s="48" t="str">
+      <c r="F102" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A102="",'Détails des dons'!H102=""),"",'Détails des dons'!H102)</f>
+        <v/>
+      </c>
+      <c r="G102" s="18" t="str">
+        <f aca="false">IF(F102="","",F102*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H102" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A102="",'Détails des dons'!J102=""),"",'Détails des dons'!J102)</f>
         <v/>
       </c>
@@ -11948,7 +12746,15 @@
         <f aca="false">IF(OR('Détails des dons'!A103="",'Détails des dons'!E103=""),"",'Détails des dons'!E103)</f>
         <v/>
       </c>
-      <c r="F103" s="48" t="str">
+      <c r="F103" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A103="",'Détails des dons'!H103=""),"",'Détails des dons'!H103)</f>
+        <v/>
+      </c>
+      <c r="G103" s="18" t="str">
+        <f aca="false">IF(F103="","",F103*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H103" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A103="",'Détails des dons'!J103=""),"",'Détails des dons'!J103)</f>
         <v/>
       </c>
@@ -11974,7 +12780,15 @@
         <f aca="false">IF(OR('Détails des dons'!A104="",'Détails des dons'!E104=""),"",'Détails des dons'!E104)</f>
         <v/>
       </c>
-      <c r="F104" s="48" t="str">
+      <c r="F104" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A104="",'Détails des dons'!H104=""),"",'Détails des dons'!H104)</f>
+        <v/>
+      </c>
+      <c r="G104" s="18" t="str">
+        <f aca="false">IF(F104="","",F104*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H104" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A104="",'Détails des dons'!J104=""),"",'Détails des dons'!J104)</f>
         <v/>
       </c>
@@ -12000,7 +12814,15 @@
         <f aca="false">IF(OR('Détails des dons'!A105="",'Détails des dons'!E105=""),"",'Détails des dons'!E105)</f>
         <v/>
       </c>
-      <c r="F105" s="48" t="str">
+      <c r="F105" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A105="",'Détails des dons'!H105=""),"",'Détails des dons'!H105)</f>
+        <v/>
+      </c>
+      <c r="G105" s="18" t="str">
+        <f aca="false">IF(F105="","",F105*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H105" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A105="",'Détails des dons'!J105=""),"",'Détails des dons'!J105)</f>
         <v/>
       </c>
@@ -12026,7 +12848,15 @@
         <f aca="false">IF(OR('Détails des dons'!A106="",'Détails des dons'!E106=""),"",'Détails des dons'!E106)</f>
         <v/>
       </c>
-      <c r="F106" s="48" t="str">
+      <c r="F106" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A106="",'Détails des dons'!H106=""),"",'Détails des dons'!H106)</f>
+        <v/>
+      </c>
+      <c r="G106" s="18" t="str">
+        <f aca="false">IF(F106="","",F106*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H106" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A106="",'Détails des dons'!J106=""),"",'Détails des dons'!J106)</f>
         <v/>
       </c>
@@ -12052,7 +12882,15 @@
         <f aca="false">IF(OR('Détails des dons'!A107="",'Détails des dons'!E107=""),"",'Détails des dons'!E107)</f>
         <v/>
       </c>
-      <c r="F107" s="48" t="str">
+      <c r="F107" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A107="",'Détails des dons'!H107=""),"",'Détails des dons'!H107)</f>
+        <v/>
+      </c>
+      <c r="G107" s="18" t="str">
+        <f aca="false">IF(F107="","",F107*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H107" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A107="",'Détails des dons'!J107=""),"",'Détails des dons'!J107)</f>
         <v/>
       </c>
@@ -12078,7 +12916,15 @@
         <f aca="false">IF(OR('Détails des dons'!A108="",'Détails des dons'!E108=""),"",'Détails des dons'!E108)</f>
         <v/>
       </c>
-      <c r="F108" s="48" t="str">
+      <c r="F108" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A108="",'Détails des dons'!H108=""),"",'Détails des dons'!H108)</f>
+        <v/>
+      </c>
+      <c r="G108" s="18" t="str">
+        <f aca="false">IF(F108="","",F108*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H108" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A108="",'Détails des dons'!J108=""),"",'Détails des dons'!J108)</f>
         <v/>
       </c>
@@ -12104,7 +12950,15 @@
         <f aca="false">IF(OR('Détails des dons'!A109="",'Détails des dons'!E109=""),"",'Détails des dons'!E109)</f>
         <v/>
       </c>
-      <c r="F109" s="48" t="str">
+      <c r="F109" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A109="",'Détails des dons'!H109=""),"",'Détails des dons'!H109)</f>
+        <v/>
+      </c>
+      <c r="G109" s="18" t="str">
+        <f aca="false">IF(F109="","",F109*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H109" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A109="",'Détails des dons'!J109=""),"",'Détails des dons'!J109)</f>
         <v/>
       </c>
@@ -12130,7 +12984,15 @@
         <f aca="false">IF(OR('Détails des dons'!A110="",'Détails des dons'!E110=""),"",'Détails des dons'!E110)</f>
         <v/>
       </c>
-      <c r="F110" s="48" t="str">
+      <c r="F110" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A110="",'Détails des dons'!H110=""),"",'Détails des dons'!H110)</f>
+        <v/>
+      </c>
+      <c r="G110" s="18" t="str">
+        <f aca="false">IF(F110="","",F110*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H110" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A110="",'Détails des dons'!J110=""),"",'Détails des dons'!J110)</f>
         <v/>
       </c>
@@ -12156,7 +13018,15 @@
         <f aca="false">IF(OR('Détails des dons'!A111="",'Détails des dons'!E111=""),"",'Détails des dons'!E111)</f>
         <v/>
       </c>
-      <c r="F111" s="48" t="str">
+      <c r="F111" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A111="",'Détails des dons'!H111=""),"",'Détails des dons'!H111)</f>
+        <v/>
+      </c>
+      <c r="G111" s="18" t="str">
+        <f aca="false">IF(F111="","",F111*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H111" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A111="",'Détails des dons'!J111=""),"",'Détails des dons'!J111)</f>
         <v/>
       </c>
@@ -12182,7 +13052,15 @@
         <f aca="false">IF(OR('Détails des dons'!A112="",'Détails des dons'!E112=""),"",'Détails des dons'!E112)</f>
         <v/>
       </c>
-      <c r="F112" s="48" t="str">
+      <c r="F112" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A112="",'Détails des dons'!H112=""),"",'Détails des dons'!H112)</f>
+        <v/>
+      </c>
+      <c r="G112" s="18" t="str">
+        <f aca="false">IF(F112="","",F112*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H112" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A112="",'Détails des dons'!J112=""),"",'Détails des dons'!J112)</f>
         <v/>
       </c>
@@ -12208,7 +13086,15 @@
         <f aca="false">IF(OR('Détails des dons'!A113="",'Détails des dons'!E113=""),"",'Détails des dons'!E113)</f>
         <v/>
       </c>
-      <c r="F113" s="48" t="str">
+      <c r="F113" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A113="",'Détails des dons'!H113=""),"",'Détails des dons'!H113)</f>
+        <v/>
+      </c>
+      <c r="G113" s="18" t="str">
+        <f aca="false">IF(F113="","",F113*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H113" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A113="",'Détails des dons'!J113=""),"",'Détails des dons'!J113)</f>
         <v/>
       </c>
@@ -12234,7 +13120,15 @@
         <f aca="false">IF(OR('Détails des dons'!A114="",'Détails des dons'!E114=""),"",'Détails des dons'!E114)</f>
         <v/>
       </c>
-      <c r="F114" s="48" t="str">
+      <c r="F114" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A114="",'Détails des dons'!H114=""),"",'Détails des dons'!H114)</f>
+        <v/>
+      </c>
+      <c r="G114" s="18" t="str">
+        <f aca="false">IF(F114="","",F114*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H114" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A114="",'Détails des dons'!J114=""),"",'Détails des dons'!J114)</f>
         <v/>
       </c>
@@ -12260,7 +13154,15 @@
         <f aca="false">IF(OR('Détails des dons'!A115="",'Détails des dons'!E115=""),"",'Détails des dons'!E115)</f>
         <v/>
       </c>
-      <c r="F115" s="48" t="str">
+      <c r="F115" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A115="",'Détails des dons'!H115=""),"",'Détails des dons'!H115)</f>
+        <v/>
+      </c>
+      <c r="G115" s="18" t="str">
+        <f aca="false">IF(F115="","",F115*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H115" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A115="",'Détails des dons'!J115=""),"",'Détails des dons'!J115)</f>
         <v/>
       </c>
@@ -12286,7 +13188,15 @@
         <f aca="false">IF(OR('Détails des dons'!A116="",'Détails des dons'!E116=""),"",'Détails des dons'!E116)</f>
         <v/>
       </c>
-      <c r="F116" s="48" t="str">
+      <c r="F116" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A116="",'Détails des dons'!H116=""),"",'Détails des dons'!H116)</f>
+        <v/>
+      </c>
+      <c r="G116" s="18" t="str">
+        <f aca="false">IF(F116="","",F116*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H116" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A116="",'Détails des dons'!J116=""),"",'Détails des dons'!J116)</f>
         <v/>
       </c>
@@ -12312,7 +13222,15 @@
         <f aca="false">IF(OR('Détails des dons'!A117="",'Détails des dons'!E117=""),"",'Détails des dons'!E117)</f>
         <v/>
       </c>
-      <c r="F117" s="48" t="str">
+      <c r="F117" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A117="",'Détails des dons'!H117=""),"",'Détails des dons'!H117)</f>
+        <v/>
+      </c>
+      <c r="G117" s="18" t="str">
+        <f aca="false">IF(F117="","",F117*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H117" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A117="",'Détails des dons'!J117=""),"",'Détails des dons'!J117)</f>
         <v/>
       </c>
@@ -12338,7 +13256,15 @@
         <f aca="false">IF(OR('Détails des dons'!A118="",'Détails des dons'!E118=""),"",'Détails des dons'!E118)</f>
         <v/>
       </c>
-      <c r="F118" s="48" t="str">
+      <c r="F118" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A118="",'Détails des dons'!H118=""),"",'Détails des dons'!H118)</f>
+        <v/>
+      </c>
+      <c r="G118" s="18" t="str">
+        <f aca="false">IF(F118="","",F118*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H118" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A118="",'Détails des dons'!J118=""),"",'Détails des dons'!J118)</f>
         <v/>
       </c>
@@ -12364,7 +13290,15 @@
         <f aca="false">IF(OR('Détails des dons'!A119="",'Détails des dons'!E119=""),"",'Détails des dons'!E119)</f>
         <v/>
       </c>
-      <c r="F119" s="48" t="str">
+      <c r="F119" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A119="",'Détails des dons'!H119=""),"",'Détails des dons'!H119)</f>
+        <v/>
+      </c>
+      <c r="G119" s="18" t="str">
+        <f aca="false">IF(F119="","",F119*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H119" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A119="",'Détails des dons'!J119=""),"",'Détails des dons'!J119)</f>
         <v/>
       </c>
@@ -12390,7 +13324,15 @@
         <f aca="false">IF(OR('Détails des dons'!A120="",'Détails des dons'!E120=""),"",'Détails des dons'!E120)</f>
         <v/>
       </c>
-      <c r="F120" s="48" t="str">
+      <c r="F120" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A120="",'Détails des dons'!H120=""),"",'Détails des dons'!H120)</f>
+        <v/>
+      </c>
+      <c r="G120" s="18" t="str">
+        <f aca="false">IF(F120="","",F120*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H120" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A120="",'Détails des dons'!J120=""),"",'Détails des dons'!J120)</f>
         <v/>
       </c>
@@ -12416,7 +13358,15 @@
         <f aca="false">IF(OR('Détails des dons'!A121="",'Détails des dons'!E121=""),"",'Détails des dons'!E121)</f>
         <v/>
       </c>
-      <c r="F121" s="48" t="str">
+      <c r="F121" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A121="",'Détails des dons'!H121=""),"",'Détails des dons'!H121)</f>
+        <v/>
+      </c>
+      <c r="G121" s="18" t="str">
+        <f aca="false">IF(F121="","",F121*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H121" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A121="",'Détails des dons'!J121=""),"",'Détails des dons'!J121)</f>
         <v/>
       </c>
@@ -12442,7 +13392,15 @@
         <f aca="false">IF(OR('Détails des dons'!A122="",'Détails des dons'!E122=""),"",'Détails des dons'!E122)</f>
         <v/>
       </c>
-      <c r="F122" s="48" t="str">
+      <c r="F122" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A122="",'Détails des dons'!H122=""),"",'Détails des dons'!H122)</f>
+        <v/>
+      </c>
+      <c r="G122" s="18" t="str">
+        <f aca="false">IF(F122="","",F122*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H122" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A122="",'Détails des dons'!J122=""),"",'Détails des dons'!J122)</f>
         <v/>
       </c>
@@ -12468,7 +13426,15 @@
         <f aca="false">IF(OR('Détails des dons'!A123="",'Détails des dons'!E123=""),"",'Détails des dons'!E123)</f>
         <v/>
       </c>
-      <c r="F123" s="48" t="str">
+      <c r="F123" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A123="",'Détails des dons'!H123=""),"",'Détails des dons'!H123)</f>
+        <v/>
+      </c>
+      <c r="G123" s="18" t="str">
+        <f aca="false">IF(F123="","",F123*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H123" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A123="",'Détails des dons'!J123=""),"",'Détails des dons'!J123)</f>
         <v/>
       </c>
@@ -12494,7 +13460,15 @@
         <f aca="false">IF(OR('Détails des dons'!A124="",'Détails des dons'!E124=""),"",'Détails des dons'!E124)</f>
         <v/>
       </c>
-      <c r="F124" s="48" t="str">
+      <c r="F124" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A124="",'Détails des dons'!H124=""),"",'Détails des dons'!H124)</f>
+        <v/>
+      </c>
+      <c r="G124" s="18" t="str">
+        <f aca="false">IF(F124="","",F124*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H124" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A124="",'Détails des dons'!J124=""),"",'Détails des dons'!J124)</f>
         <v/>
       </c>
@@ -12520,7 +13494,15 @@
         <f aca="false">IF(OR('Détails des dons'!A125="",'Détails des dons'!E125=""),"",'Détails des dons'!E125)</f>
         <v/>
       </c>
-      <c r="F125" s="48" t="str">
+      <c r="F125" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A125="",'Détails des dons'!H125=""),"",'Détails des dons'!H125)</f>
+        <v/>
+      </c>
+      <c r="G125" s="18" t="str">
+        <f aca="false">IF(F125="","",F125*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H125" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A125="",'Détails des dons'!J125=""),"",'Détails des dons'!J125)</f>
         <v/>
       </c>
@@ -12546,7 +13528,15 @@
         <f aca="false">IF(OR('Détails des dons'!A126="",'Détails des dons'!E126=""),"",'Détails des dons'!E126)</f>
         <v/>
       </c>
-      <c r="F126" s="48" t="str">
+      <c r="F126" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A126="",'Détails des dons'!H126=""),"",'Détails des dons'!H126)</f>
+        <v/>
+      </c>
+      <c r="G126" s="18" t="str">
+        <f aca="false">IF(F126="","",F126*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H126" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A126="",'Détails des dons'!J126=""),"",'Détails des dons'!J126)</f>
         <v/>
       </c>
@@ -12572,7 +13562,15 @@
         <f aca="false">IF(OR('Détails des dons'!A127="",'Détails des dons'!E127=""),"",'Détails des dons'!E127)</f>
         <v/>
       </c>
-      <c r="F127" s="48" t="str">
+      <c r="F127" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A127="",'Détails des dons'!H127=""),"",'Détails des dons'!H127)</f>
+        <v/>
+      </c>
+      <c r="G127" s="18" t="str">
+        <f aca="false">IF(F127="","",F127*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H127" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A127="",'Détails des dons'!J127=""),"",'Détails des dons'!J127)</f>
         <v/>
       </c>
@@ -12598,7 +13596,15 @@
         <f aca="false">IF(OR('Détails des dons'!A128="",'Détails des dons'!E128=""),"",'Détails des dons'!E128)</f>
         <v/>
       </c>
-      <c r="F128" s="48" t="str">
+      <c r="F128" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A128="",'Détails des dons'!H128=""),"",'Détails des dons'!H128)</f>
+        <v/>
+      </c>
+      <c r="G128" s="18" t="str">
+        <f aca="false">IF(F128="","",F128*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H128" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A128="",'Détails des dons'!J128=""),"",'Détails des dons'!J128)</f>
         <v/>
       </c>
@@ -12624,7 +13630,15 @@
         <f aca="false">IF(OR('Détails des dons'!A129="",'Détails des dons'!E129=""),"",'Détails des dons'!E129)</f>
         <v/>
       </c>
-      <c r="F129" s="48" t="str">
+      <c r="F129" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A129="",'Détails des dons'!H129=""),"",'Détails des dons'!H129)</f>
+        <v/>
+      </c>
+      <c r="G129" s="18" t="str">
+        <f aca="false">IF(F129="","",F129*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H129" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A129="",'Détails des dons'!J129=""),"",'Détails des dons'!J129)</f>
         <v/>
       </c>
@@ -12650,7 +13664,15 @@
         <f aca="false">IF(OR('Détails des dons'!A130="",'Détails des dons'!E130=""),"",'Détails des dons'!E130)</f>
         <v/>
       </c>
-      <c r="F130" s="48" t="str">
+      <c r="F130" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A130="",'Détails des dons'!H130=""),"",'Détails des dons'!H130)</f>
+        <v/>
+      </c>
+      <c r="G130" s="18" t="str">
+        <f aca="false">IF(F130="","",F130*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H130" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A130="",'Détails des dons'!J130=""),"",'Détails des dons'!J130)</f>
         <v/>
       </c>
@@ -12676,7 +13698,15 @@
         <f aca="false">IF(OR('Détails des dons'!A131="",'Détails des dons'!E131=""),"",'Détails des dons'!E131)</f>
         <v/>
       </c>
-      <c r="F131" s="48" t="str">
+      <c r="F131" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A131="",'Détails des dons'!H131=""),"",'Détails des dons'!H131)</f>
+        <v/>
+      </c>
+      <c r="G131" s="18" t="str">
+        <f aca="false">IF(F131="","",F131*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H131" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A131="",'Détails des dons'!J131=""),"",'Détails des dons'!J131)</f>
         <v/>
       </c>
@@ -12702,7 +13732,15 @@
         <f aca="false">IF(OR('Détails des dons'!A132="",'Détails des dons'!E132=""),"",'Détails des dons'!E132)</f>
         <v/>
       </c>
-      <c r="F132" s="48" t="str">
+      <c r="F132" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A132="",'Détails des dons'!H132=""),"",'Détails des dons'!H132)</f>
+        <v/>
+      </c>
+      <c r="G132" s="18" t="str">
+        <f aca="false">IF(F132="","",F132*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H132" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A132="",'Détails des dons'!J132=""),"",'Détails des dons'!J132)</f>
         <v/>
       </c>
@@ -12728,7 +13766,15 @@
         <f aca="false">IF(OR('Détails des dons'!A133="",'Détails des dons'!E133=""),"",'Détails des dons'!E133)</f>
         <v/>
       </c>
-      <c r="F133" s="48" t="str">
+      <c r="F133" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A133="",'Détails des dons'!H133=""),"",'Détails des dons'!H133)</f>
+        <v/>
+      </c>
+      <c r="G133" s="18" t="str">
+        <f aca="false">IF(F133="","",F133*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H133" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A133="",'Détails des dons'!J133=""),"",'Détails des dons'!J133)</f>
         <v/>
       </c>
@@ -12754,7 +13800,15 @@
         <f aca="false">IF(OR('Détails des dons'!A134="",'Détails des dons'!E134=""),"",'Détails des dons'!E134)</f>
         <v/>
       </c>
-      <c r="F134" s="48" t="str">
+      <c r="F134" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A134="",'Détails des dons'!H134=""),"",'Détails des dons'!H134)</f>
+        <v/>
+      </c>
+      <c r="G134" s="18" t="str">
+        <f aca="false">IF(F134="","",F134*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H134" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A134="",'Détails des dons'!J134=""),"",'Détails des dons'!J134)</f>
         <v/>
       </c>
@@ -12780,7 +13834,15 @@
         <f aca="false">IF(OR('Détails des dons'!A135="",'Détails des dons'!E135=""),"",'Détails des dons'!E135)</f>
         <v/>
       </c>
-      <c r="F135" s="48" t="str">
+      <c r="F135" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A135="",'Détails des dons'!H135=""),"",'Détails des dons'!H135)</f>
+        <v/>
+      </c>
+      <c r="G135" s="18" t="str">
+        <f aca="false">IF(F135="","",F135*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H135" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A135="",'Détails des dons'!J135=""),"",'Détails des dons'!J135)</f>
         <v/>
       </c>
@@ -12806,7 +13868,15 @@
         <f aca="false">IF(OR('Détails des dons'!A136="",'Détails des dons'!E136=""),"",'Détails des dons'!E136)</f>
         <v/>
       </c>
-      <c r="F136" s="48" t="str">
+      <c r="F136" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A136="",'Détails des dons'!H136=""),"",'Détails des dons'!H136)</f>
+        <v/>
+      </c>
+      <c r="G136" s="18" t="str">
+        <f aca="false">IF(F136="","",F136*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H136" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A136="",'Détails des dons'!J136=""),"",'Détails des dons'!J136)</f>
         <v/>
       </c>
@@ -12832,7 +13902,15 @@
         <f aca="false">IF(OR('Détails des dons'!A137="",'Détails des dons'!E137=""),"",'Détails des dons'!E137)</f>
         <v/>
       </c>
-      <c r="F137" s="48" t="str">
+      <c r="F137" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A137="",'Détails des dons'!H137=""),"",'Détails des dons'!H137)</f>
+        <v/>
+      </c>
+      <c r="G137" s="18" t="str">
+        <f aca="false">IF(F137="","",F137*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H137" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A137="",'Détails des dons'!J137=""),"",'Détails des dons'!J137)</f>
         <v/>
       </c>
@@ -12858,7 +13936,15 @@
         <f aca="false">IF(OR('Détails des dons'!A138="",'Détails des dons'!E138=""),"",'Détails des dons'!E138)</f>
         <v/>
       </c>
-      <c r="F138" s="48" t="str">
+      <c r="F138" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A138="",'Détails des dons'!H138=""),"",'Détails des dons'!H138)</f>
+        <v/>
+      </c>
+      <c r="G138" s="18" t="str">
+        <f aca="false">IF(F138="","",F138*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H138" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A138="",'Détails des dons'!J138=""),"",'Détails des dons'!J138)</f>
         <v/>
       </c>
@@ -12884,7 +13970,15 @@
         <f aca="false">IF(OR('Détails des dons'!A139="",'Détails des dons'!E139=""),"",'Détails des dons'!E139)</f>
         <v/>
       </c>
-      <c r="F139" s="48" t="str">
+      <c r="F139" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A139="",'Détails des dons'!H139=""),"",'Détails des dons'!H139)</f>
+        <v/>
+      </c>
+      <c r="G139" s="18" t="str">
+        <f aca="false">IF(F139="","",F139*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H139" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A139="",'Détails des dons'!J139=""),"",'Détails des dons'!J139)</f>
         <v/>
       </c>
@@ -12910,7 +14004,15 @@
         <f aca="false">IF(OR('Détails des dons'!A140="",'Détails des dons'!E140=""),"",'Détails des dons'!E140)</f>
         <v/>
       </c>
-      <c r="F140" s="48" t="str">
+      <c r="F140" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A140="",'Détails des dons'!H140=""),"",'Détails des dons'!H140)</f>
+        <v/>
+      </c>
+      <c r="G140" s="18" t="str">
+        <f aca="false">IF(F140="","",F140*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H140" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A140="",'Détails des dons'!J140=""),"",'Détails des dons'!J140)</f>
         <v/>
       </c>
@@ -12936,7 +14038,15 @@
         <f aca="false">IF(OR('Détails des dons'!A141="",'Détails des dons'!E141=""),"",'Détails des dons'!E141)</f>
         <v/>
       </c>
-      <c r="F141" s="48" t="str">
+      <c r="F141" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A141="",'Détails des dons'!H141=""),"",'Détails des dons'!H141)</f>
+        <v/>
+      </c>
+      <c r="G141" s="18" t="str">
+        <f aca="false">IF(F141="","",F141*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H141" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A141="",'Détails des dons'!J141=""),"",'Détails des dons'!J141)</f>
         <v/>
       </c>
@@ -12962,7 +14072,15 @@
         <f aca="false">IF(OR('Détails des dons'!A142="",'Détails des dons'!E142=""),"",'Détails des dons'!E142)</f>
         <v/>
       </c>
-      <c r="F142" s="48" t="str">
+      <c r="F142" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A142="",'Détails des dons'!H142=""),"",'Détails des dons'!H142)</f>
+        <v/>
+      </c>
+      <c r="G142" s="18" t="str">
+        <f aca="false">IF(F142="","",F142*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H142" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A142="",'Détails des dons'!J142=""),"",'Détails des dons'!J142)</f>
         <v/>
       </c>
@@ -12988,7 +14106,15 @@
         <f aca="false">IF(OR('Détails des dons'!A143="",'Détails des dons'!E143=""),"",'Détails des dons'!E143)</f>
         <v/>
       </c>
-      <c r="F143" s="48" t="str">
+      <c r="F143" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A143="",'Détails des dons'!H143=""),"",'Détails des dons'!H143)</f>
+        <v/>
+      </c>
+      <c r="G143" s="18" t="str">
+        <f aca="false">IF(F143="","",F143*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H143" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A143="",'Détails des dons'!J143=""),"",'Détails des dons'!J143)</f>
         <v/>
       </c>
@@ -13014,7 +14140,15 @@
         <f aca="false">IF(OR('Détails des dons'!A144="",'Détails des dons'!E144=""),"",'Détails des dons'!E144)</f>
         <v/>
       </c>
-      <c r="F144" s="48" t="str">
+      <c r="F144" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A144="",'Détails des dons'!H144=""),"",'Détails des dons'!H144)</f>
+        <v/>
+      </c>
+      <c r="G144" s="18" t="str">
+        <f aca="false">IF(F144="","",F144*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H144" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A144="",'Détails des dons'!J144=""),"",'Détails des dons'!J144)</f>
         <v/>
       </c>
@@ -13040,7 +14174,15 @@
         <f aca="false">IF(OR('Détails des dons'!A145="",'Détails des dons'!E145=""),"",'Détails des dons'!E145)</f>
         <v/>
       </c>
-      <c r="F145" s="48" t="str">
+      <c r="F145" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A145="",'Détails des dons'!H145=""),"",'Détails des dons'!H145)</f>
+        <v/>
+      </c>
+      <c r="G145" s="18" t="str">
+        <f aca="false">IF(F145="","",F145*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H145" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A145="",'Détails des dons'!J145=""),"",'Détails des dons'!J145)</f>
         <v/>
       </c>
@@ -13066,7 +14208,15 @@
         <f aca="false">IF(OR('Détails des dons'!A146="",'Détails des dons'!E146=""),"",'Détails des dons'!E146)</f>
         <v/>
       </c>
-      <c r="F146" s="48" t="str">
+      <c r="F146" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A146="",'Détails des dons'!H146=""),"",'Détails des dons'!H146)</f>
+        <v/>
+      </c>
+      <c r="G146" s="18" t="str">
+        <f aca="false">IF(F146="","",F146*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H146" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A146="",'Détails des dons'!J146=""),"",'Détails des dons'!J146)</f>
         <v/>
       </c>
@@ -13092,7 +14242,15 @@
         <f aca="false">IF(OR('Détails des dons'!A147="",'Détails des dons'!E147=""),"",'Détails des dons'!E147)</f>
         <v/>
       </c>
-      <c r="F147" s="48" t="str">
+      <c r="F147" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A147="",'Détails des dons'!H147=""),"",'Détails des dons'!H147)</f>
+        <v/>
+      </c>
+      <c r="G147" s="18" t="str">
+        <f aca="false">IF(F147="","",F147*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H147" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A147="",'Détails des dons'!J147=""),"",'Détails des dons'!J147)</f>
         <v/>
       </c>
@@ -13118,7 +14276,15 @@
         <f aca="false">IF(OR('Détails des dons'!A148="",'Détails des dons'!E148=""),"",'Détails des dons'!E148)</f>
         <v/>
       </c>
-      <c r="F148" s="48" t="str">
+      <c r="F148" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A148="",'Détails des dons'!H148=""),"",'Détails des dons'!H148)</f>
+        <v/>
+      </c>
+      <c r="G148" s="18" t="str">
+        <f aca="false">IF(F148="","",F148*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H148" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A148="",'Détails des dons'!J148=""),"",'Détails des dons'!J148)</f>
         <v/>
       </c>
@@ -13144,7 +14310,15 @@
         <f aca="false">IF(OR('Détails des dons'!A149="",'Détails des dons'!E149=""),"",'Détails des dons'!E149)</f>
         <v/>
       </c>
-      <c r="F149" s="48" t="str">
+      <c r="F149" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A149="",'Détails des dons'!H149=""),"",'Détails des dons'!H149)</f>
+        <v/>
+      </c>
+      <c r="G149" s="18" t="str">
+        <f aca="false">IF(F149="","",F149*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H149" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A149="",'Détails des dons'!J149=""),"",'Détails des dons'!J149)</f>
         <v/>
       </c>
@@ -13170,7 +14344,15 @@
         <f aca="false">IF(OR('Détails des dons'!A150="",'Détails des dons'!E150=""),"",'Détails des dons'!E150)</f>
         <v/>
       </c>
-      <c r="F150" s="48" t="str">
+      <c r="F150" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A150="",'Détails des dons'!H150=""),"",'Détails des dons'!H150)</f>
+        <v/>
+      </c>
+      <c r="G150" s="18" t="str">
+        <f aca="false">IF(F150="","",F150*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H150" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A150="",'Détails des dons'!J150=""),"",'Détails des dons'!J150)</f>
         <v/>
       </c>
@@ -13196,7 +14378,15 @@
         <f aca="false">IF(OR('Détails des dons'!A151="",'Détails des dons'!E151=""),"",'Détails des dons'!E151)</f>
         <v/>
       </c>
-      <c r="F151" s="48" t="str">
+      <c r="F151" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A151="",'Détails des dons'!H151=""),"",'Détails des dons'!H151)</f>
+        <v/>
+      </c>
+      <c r="G151" s="18" t="str">
+        <f aca="false">IF(F151="","",F151*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H151" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A151="",'Détails des dons'!J151=""),"",'Détails des dons'!J151)</f>
         <v/>
       </c>
@@ -13222,7 +14412,15 @@
         <f aca="false">IF(OR('Détails des dons'!A152="",'Détails des dons'!E152=""),"",'Détails des dons'!E152)</f>
         <v/>
       </c>
-      <c r="F152" s="48" t="str">
+      <c r="F152" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A152="",'Détails des dons'!H152=""),"",'Détails des dons'!H152)</f>
+        <v/>
+      </c>
+      <c r="G152" s="18" t="str">
+        <f aca="false">IF(F152="","",F152*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H152" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A152="",'Détails des dons'!J152=""),"",'Détails des dons'!J152)</f>
         <v/>
       </c>
@@ -13248,7 +14446,15 @@
         <f aca="false">IF(OR('Détails des dons'!A153="",'Détails des dons'!E153=""),"",'Détails des dons'!E153)</f>
         <v/>
       </c>
-      <c r="F153" s="48" t="str">
+      <c r="F153" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A153="",'Détails des dons'!H153=""),"",'Détails des dons'!H153)</f>
+        <v/>
+      </c>
+      <c r="G153" s="18" t="str">
+        <f aca="false">IF(F153="","",F153*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H153" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A153="",'Détails des dons'!J153=""),"",'Détails des dons'!J153)</f>
         <v/>
       </c>
@@ -13274,7 +14480,15 @@
         <f aca="false">IF(OR('Détails des dons'!A154="",'Détails des dons'!E154=""),"",'Détails des dons'!E154)</f>
         <v/>
       </c>
-      <c r="F154" s="48" t="str">
+      <c r="F154" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A154="",'Détails des dons'!H154=""),"",'Détails des dons'!H154)</f>
+        <v/>
+      </c>
+      <c r="G154" s="18" t="str">
+        <f aca="false">IF(F154="","",F154*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H154" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A154="",'Détails des dons'!J154=""),"",'Détails des dons'!J154)</f>
         <v/>
       </c>
@@ -13300,7 +14514,15 @@
         <f aca="false">IF(OR('Détails des dons'!A155="",'Détails des dons'!E155=""),"",'Détails des dons'!E155)</f>
         <v/>
       </c>
-      <c r="F155" s="48" t="str">
+      <c r="F155" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A155="",'Détails des dons'!H155=""),"",'Détails des dons'!H155)</f>
+        <v/>
+      </c>
+      <c r="G155" s="18" t="str">
+        <f aca="false">IF(F155="","",F155*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H155" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A155="",'Détails des dons'!J155=""),"",'Détails des dons'!J155)</f>
         <v/>
       </c>
@@ -13326,7 +14548,15 @@
         <f aca="false">IF(OR('Détails des dons'!A156="",'Détails des dons'!E156=""),"",'Détails des dons'!E156)</f>
         <v/>
       </c>
-      <c r="F156" s="48" t="str">
+      <c r="F156" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A156="",'Détails des dons'!H156=""),"",'Détails des dons'!H156)</f>
+        <v/>
+      </c>
+      <c r="G156" s="18" t="str">
+        <f aca="false">IF(F156="","",F156*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H156" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A156="",'Détails des dons'!J156=""),"",'Détails des dons'!J156)</f>
         <v/>
       </c>
@@ -13352,7 +14582,15 @@
         <f aca="false">IF(OR('Détails des dons'!A157="",'Détails des dons'!E157=""),"",'Détails des dons'!E157)</f>
         <v/>
       </c>
-      <c r="F157" s="48" t="str">
+      <c r="F157" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A157="",'Détails des dons'!H157=""),"",'Détails des dons'!H157)</f>
+        <v/>
+      </c>
+      <c r="G157" s="18" t="str">
+        <f aca="false">IF(F157="","",F157*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H157" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A157="",'Détails des dons'!J157=""),"",'Détails des dons'!J157)</f>
         <v/>
       </c>
@@ -13378,7 +14616,15 @@
         <f aca="false">IF(OR('Détails des dons'!A158="",'Détails des dons'!E158=""),"",'Détails des dons'!E158)</f>
         <v/>
       </c>
-      <c r="F158" s="48" t="str">
+      <c r="F158" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A158="",'Détails des dons'!H158=""),"",'Détails des dons'!H158)</f>
+        <v/>
+      </c>
+      <c r="G158" s="18" t="str">
+        <f aca="false">IF(F158="","",F158*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H158" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A158="",'Détails des dons'!J158=""),"",'Détails des dons'!J158)</f>
         <v/>
       </c>
@@ -13404,7 +14650,15 @@
         <f aca="false">IF(OR('Détails des dons'!A159="",'Détails des dons'!E159=""),"",'Détails des dons'!E159)</f>
         <v/>
       </c>
-      <c r="F159" s="48" t="str">
+      <c r="F159" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A159="",'Détails des dons'!H159=""),"",'Détails des dons'!H159)</f>
+        <v/>
+      </c>
+      <c r="G159" s="18" t="str">
+        <f aca="false">IF(F159="","",F159*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H159" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A159="",'Détails des dons'!J159=""),"",'Détails des dons'!J159)</f>
         <v/>
       </c>
@@ -13430,7 +14684,15 @@
         <f aca="false">IF(OR('Détails des dons'!A160="",'Détails des dons'!E160=""),"",'Détails des dons'!E160)</f>
         <v/>
       </c>
-      <c r="F160" s="48" t="str">
+      <c r="F160" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A160="",'Détails des dons'!H160=""),"",'Détails des dons'!H160)</f>
+        <v/>
+      </c>
+      <c r="G160" s="18" t="str">
+        <f aca="false">IF(F160="","",F160*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H160" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A160="",'Détails des dons'!J160=""),"",'Détails des dons'!J160)</f>
         <v/>
       </c>
@@ -13456,7 +14718,15 @@
         <f aca="false">IF(OR('Détails des dons'!A161="",'Détails des dons'!E161=""),"",'Détails des dons'!E161)</f>
         <v/>
       </c>
-      <c r="F161" s="48" t="str">
+      <c r="F161" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A161="",'Détails des dons'!H161=""),"",'Détails des dons'!H161)</f>
+        <v/>
+      </c>
+      <c r="G161" s="18" t="str">
+        <f aca="false">IF(F161="","",F161*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H161" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A161="",'Détails des dons'!J161=""),"",'Détails des dons'!J161)</f>
         <v/>
       </c>
@@ -13482,7 +14752,15 @@
         <f aca="false">IF(OR('Détails des dons'!A162="",'Détails des dons'!E162=""),"",'Détails des dons'!E162)</f>
         <v/>
       </c>
-      <c r="F162" s="48" t="str">
+      <c r="F162" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A162="",'Détails des dons'!H162=""),"",'Détails des dons'!H162)</f>
+        <v/>
+      </c>
+      <c r="G162" s="18" t="str">
+        <f aca="false">IF(F162="","",F162*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H162" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A162="",'Détails des dons'!J162=""),"",'Détails des dons'!J162)</f>
         <v/>
       </c>
@@ -13508,7 +14786,15 @@
         <f aca="false">IF(OR('Détails des dons'!A163="",'Détails des dons'!E163=""),"",'Détails des dons'!E163)</f>
         <v/>
       </c>
-      <c r="F163" s="48" t="str">
+      <c r="F163" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A163="",'Détails des dons'!H163=""),"",'Détails des dons'!H163)</f>
+        <v/>
+      </c>
+      <c r="G163" s="18" t="str">
+        <f aca="false">IF(F163="","",F163*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H163" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A163="",'Détails des dons'!J163=""),"",'Détails des dons'!J163)</f>
         <v/>
       </c>
@@ -13534,7 +14820,15 @@
         <f aca="false">IF(OR('Détails des dons'!A164="",'Détails des dons'!E164=""),"",'Détails des dons'!E164)</f>
         <v/>
       </c>
-      <c r="F164" s="48" t="str">
+      <c r="F164" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A164="",'Détails des dons'!H164=""),"",'Détails des dons'!H164)</f>
+        <v/>
+      </c>
+      <c r="G164" s="18" t="str">
+        <f aca="false">IF(F164="","",F164*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H164" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A164="",'Détails des dons'!J164=""),"",'Détails des dons'!J164)</f>
         <v/>
       </c>
@@ -13560,7 +14854,15 @@
         <f aca="false">IF(OR('Détails des dons'!A165="",'Détails des dons'!E165=""),"",'Détails des dons'!E165)</f>
         <v/>
       </c>
-      <c r="F165" s="48" t="str">
+      <c r="F165" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A165="",'Détails des dons'!H165=""),"",'Détails des dons'!H165)</f>
+        <v/>
+      </c>
+      <c r="G165" s="18" t="str">
+        <f aca="false">IF(F165="","",F165*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H165" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A165="",'Détails des dons'!J165=""),"",'Détails des dons'!J165)</f>
         <v/>
       </c>
@@ -13586,7 +14888,15 @@
         <f aca="false">IF(OR('Détails des dons'!A166="",'Détails des dons'!E166=""),"",'Détails des dons'!E166)</f>
         <v/>
       </c>
-      <c r="F166" s="48" t="str">
+      <c r="F166" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A166="",'Détails des dons'!H166=""),"",'Détails des dons'!H166)</f>
+        <v/>
+      </c>
+      <c r="G166" s="18" t="str">
+        <f aca="false">IF(F166="","",F166*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H166" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A166="",'Détails des dons'!J166=""),"",'Détails des dons'!J166)</f>
         <v/>
       </c>
@@ -13612,7 +14922,15 @@
         <f aca="false">IF(OR('Détails des dons'!A167="",'Détails des dons'!E167=""),"",'Détails des dons'!E167)</f>
         <v/>
       </c>
-      <c r="F167" s="48" t="str">
+      <c r="F167" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A167="",'Détails des dons'!H167=""),"",'Détails des dons'!H167)</f>
+        <v/>
+      </c>
+      <c r="G167" s="18" t="str">
+        <f aca="false">IF(F167="","",F167*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H167" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A167="",'Détails des dons'!J167=""),"",'Détails des dons'!J167)</f>
         <v/>
       </c>
@@ -13638,7 +14956,15 @@
         <f aca="false">IF(OR('Détails des dons'!A168="",'Détails des dons'!E168=""),"",'Détails des dons'!E168)</f>
         <v/>
       </c>
-      <c r="F168" s="48" t="str">
+      <c r="F168" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A168="",'Détails des dons'!H168=""),"",'Détails des dons'!H168)</f>
+        <v/>
+      </c>
+      <c r="G168" s="18" t="str">
+        <f aca="false">IF(F168="","",F168*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H168" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A168="",'Détails des dons'!J168=""),"",'Détails des dons'!J168)</f>
         <v/>
       </c>
@@ -13664,7 +14990,15 @@
         <f aca="false">IF(OR('Détails des dons'!A169="",'Détails des dons'!E169=""),"",'Détails des dons'!E169)</f>
         <v/>
       </c>
-      <c r="F169" s="48" t="str">
+      <c r="F169" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A169="",'Détails des dons'!H169=""),"",'Détails des dons'!H169)</f>
+        <v/>
+      </c>
+      <c r="G169" s="18" t="str">
+        <f aca="false">IF(F169="","",F169*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H169" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A169="",'Détails des dons'!J169=""),"",'Détails des dons'!J169)</f>
         <v/>
       </c>
@@ -13690,7 +15024,15 @@
         <f aca="false">IF(OR('Détails des dons'!A170="",'Détails des dons'!E170=""),"",'Détails des dons'!E170)</f>
         <v/>
       </c>
-      <c r="F170" s="48" t="str">
+      <c r="F170" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A170="",'Détails des dons'!H170=""),"",'Détails des dons'!H170)</f>
+        <v/>
+      </c>
+      <c r="G170" s="18" t="str">
+        <f aca="false">IF(F170="","",F170*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H170" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A170="",'Détails des dons'!J170=""),"",'Détails des dons'!J170)</f>
         <v/>
       </c>
@@ -13716,7 +15058,15 @@
         <f aca="false">IF(OR('Détails des dons'!A171="",'Détails des dons'!E171=""),"",'Détails des dons'!E171)</f>
         <v/>
       </c>
-      <c r="F171" s="48" t="str">
+      <c r="F171" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A171="",'Détails des dons'!H171=""),"",'Détails des dons'!H171)</f>
+        <v/>
+      </c>
+      <c r="G171" s="18" t="str">
+        <f aca="false">IF(F171="","",F171*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H171" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A171="",'Détails des dons'!J171=""),"",'Détails des dons'!J171)</f>
         <v/>
       </c>
@@ -13742,7 +15092,15 @@
         <f aca="false">IF(OR('Détails des dons'!A172="",'Détails des dons'!E172=""),"",'Détails des dons'!E172)</f>
         <v/>
       </c>
-      <c r="F172" s="48" t="str">
+      <c r="F172" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A172="",'Détails des dons'!H172=""),"",'Détails des dons'!H172)</f>
+        <v/>
+      </c>
+      <c r="G172" s="18" t="str">
+        <f aca="false">IF(F172="","",F172*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H172" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A172="",'Détails des dons'!J172=""),"",'Détails des dons'!J172)</f>
         <v/>
       </c>
@@ -13768,7 +15126,15 @@
         <f aca="false">IF(OR('Détails des dons'!A173="",'Détails des dons'!E173=""),"",'Détails des dons'!E173)</f>
         <v/>
       </c>
-      <c r="F173" s="48" t="str">
+      <c r="F173" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A173="",'Détails des dons'!H173=""),"",'Détails des dons'!H173)</f>
+        <v/>
+      </c>
+      <c r="G173" s="18" t="str">
+        <f aca="false">IF(F173="","",F173*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H173" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A173="",'Détails des dons'!J173=""),"",'Détails des dons'!J173)</f>
         <v/>
       </c>
@@ -13794,7 +15160,15 @@
         <f aca="false">IF(OR('Détails des dons'!A174="",'Détails des dons'!E174=""),"",'Détails des dons'!E174)</f>
         <v/>
       </c>
-      <c r="F174" s="48" t="str">
+      <c r="F174" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A174="",'Détails des dons'!H174=""),"",'Détails des dons'!H174)</f>
+        <v/>
+      </c>
+      <c r="G174" s="18" t="str">
+        <f aca="false">IF(F174="","",F174*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H174" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A174="",'Détails des dons'!J174=""),"",'Détails des dons'!J174)</f>
         <v/>
       </c>
@@ -13820,7 +15194,15 @@
         <f aca="false">IF(OR('Détails des dons'!A175="",'Détails des dons'!E175=""),"",'Détails des dons'!E175)</f>
         <v/>
       </c>
-      <c r="F175" s="48" t="str">
+      <c r="F175" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A175="",'Détails des dons'!H175=""),"",'Détails des dons'!H175)</f>
+        <v/>
+      </c>
+      <c r="G175" s="18" t="str">
+        <f aca="false">IF(F175="","",F175*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H175" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A175="",'Détails des dons'!J175=""),"",'Détails des dons'!J175)</f>
         <v/>
       </c>
@@ -13846,7 +15228,15 @@
         <f aca="false">IF(OR('Détails des dons'!A176="",'Détails des dons'!E176=""),"",'Détails des dons'!E176)</f>
         <v/>
       </c>
-      <c r="F176" s="48" t="str">
+      <c r="F176" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A176="",'Détails des dons'!H176=""),"",'Détails des dons'!H176)</f>
+        <v/>
+      </c>
+      <c r="G176" s="18" t="str">
+        <f aca="false">IF(F176="","",F176*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H176" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A176="",'Détails des dons'!J176=""),"",'Détails des dons'!J176)</f>
         <v/>
       </c>
@@ -13872,7 +15262,15 @@
         <f aca="false">IF(OR('Détails des dons'!A177="",'Détails des dons'!E177=""),"",'Détails des dons'!E177)</f>
         <v/>
       </c>
-      <c r="F177" s="48" t="str">
+      <c r="F177" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A177="",'Détails des dons'!H177=""),"",'Détails des dons'!H177)</f>
+        <v/>
+      </c>
+      <c r="G177" s="18" t="str">
+        <f aca="false">IF(F177="","",F177*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H177" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A177="",'Détails des dons'!J177=""),"",'Détails des dons'!J177)</f>
         <v/>
       </c>
@@ -13898,7 +15296,15 @@
         <f aca="false">IF(OR('Détails des dons'!A178="",'Détails des dons'!E178=""),"",'Détails des dons'!E178)</f>
         <v/>
       </c>
-      <c r="F178" s="48" t="str">
+      <c r="F178" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A178="",'Détails des dons'!H178=""),"",'Détails des dons'!H178)</f>
+        <v/>
+      </c>
+      <c r="G178" s="18" t="str">
+        <f aca="false">IF(F178="","",F178*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H178" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A178="",'Détails des dons'!J178=""),"",'Détails des dons'!J178)</f>
         <v/>
       </c>
@@ -13924,7 +15330,15 @@
         <f aca="false">IF(OR('Détails des dons'!A179="",'Détails des dons'!E179=""),"",'Détails des dons'!E179)</f>
         <v/>
       </c>
-      <c r="F179" s="48" t="str">
+      <c r="F179" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A179="",'Détails des dons'!H179=""),"",'Détails des dons'!H179)</f>
+        <v/>
+      </c>
+      <c r="G179" s="18" t="str">
+        <f aca="false">IF(F179="","",F179*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H179" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A179="",'Détails des dons'!J179=""),"",'Détails des dons'!J179)</f>
         <v/>
       </c>
@@ -13950,7 +15364,15 @@
         <f aca="false">IF(OR('Détails des dons'!A180="",'Détails des dons'!E180=""),"",'Détails des dons'!E180)</f>
         <v/>
       </c>
-      <c r="F180" s="48" t="str">
+      <c r="F180" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A180="",'Détails des dons'!H180=""),"",'Détails des dons'!H180)</f>
+        <v/>
+      </c>
+      <c r="G180" s="18" t="str">
+        <f aca="false">IF(F180="","",F180*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H180" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A180="",'Détails des dons'!J180=""),"",'Détails des dons'!J180)</f>
         <v/>
       </c>
@@ -13976,7 +15398,15 @@
         <f aca="false">IF(OR('Détails des dons'!A181="",'Détails des dons'!E181=""),"",'Détails des dons'!E181)</f>
         <v/>
       </c>
-      <c r="F181" s="48" t="str">
+      <c r="F181" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A181="",'Détails des dons'!H181=""),"",'Détails des dons'!H181)</f>
+        <v/>
+      </c>
+      <c r="G181" s="18" t="str">
+        <f aca="false">IF(F181="","",F181*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H181" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A181="",'Détails des dons'!J181=""),"",'Détails des dons'!J181)</f>
         <v/>
       </c>
@@ -14002,7 +15432,15 @@
         <f aca="false">IF(OR('Détails des dons'!A182="",'Détails des dons'!E182=""),"",'Détails des dons'!E182)</f>
         <v/>
       </c>
-      <c r="F182" s="48" t="str">
+      <c r="F182" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A182="",'Détails des dons'!H182=""),"",'Détails des dons'!H182)</f>
+        <v/>
+      </c>
+      <c r="G182" s="18" t="str">
+        <f aca="false">IF(F182="","",F182*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H182" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A182="",'Détails des dons'!J182=""),"",'Détails des dons'!J182)</f>
         <v/>
       </c>
@@ -14028,7 +15466,15 @@
         <f aca="false">IF(OR('Détails des dons'!A183="",'Détails des dons'!E183=""),"",'Détails des dons'!E183)</f>
         <v/>
       </c>
-      <c r="F183" s="48" t="str">
+      <c r="F183" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A183="",'Détails des dons'!H183=""),"",'Détails des dons'!H183)</f>
+        <v/>
+      </c>
+      <c r="G183" s="18" t="str">
+        <f aca="false">IF(F183="","",F183*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H183" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A183="",'Détails des dons'!J183=""),"",'Détails des dons'!J183)</f>
         <v/>
       </c>
@@ -14054,7 +15500,15 @@
         <f aca="false">IF(OR('Détails des dons'!A184="",'Détails des dons'!E184=""),"",'Détails des dons'!E184)</f>
         <v/>
       </c>
-      <c r="F184" s="48" t="str">
+      <c r="F184" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A184="",'Détails des dons'!H184=""),"",'Détails des dons'!H184)</f>
+        <v/>
+      </c>
+      <c r="G184" s="18" t="str">
+        <f aca="false">IF(F184="","",F184*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H184" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A184="",'Détails des dons'!J184=""),"",'Détails des dons'!J184)</f>
         <v/>
       </c>
@@ -14080,7 +15534,15 @@
         <f aca="false">IF(OR('Détails des dons'!A185="",'Détails des dons'!E185=""),"",'Détails des dons'!E185)</f>
         <v/>
       </c>
-      <c r="F185" s="48" t="str">
+      <c r="F185" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A185="",'Détails des dons'!H185=""),"",'Détails des dons'!H185)</f>
+        <v/>
+      </c>
+      <c r="G185" s="18" t="str">
+        <f aca="false">IF(F185="","",F185*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H185" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A185="",'Détails des dons'!J185=""),"",'Détails des dons'!J185)</f>
         <v/>
       </c>
@@ -14106,7 +15568,15 @@
         <f aca="false">IF(OR('Détails des dons'!A186="",'Détails des dons'!E186=""),"",'Détails des dons'!E186)</f>
         <v/>
       </c>
-      <c r="F186" s="48" t="str">
+      <c r="F186" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A186="",'Détails des dons'!H186=""),"",'Détails des dons'!H186)</f>
+        <v/>
+      </c>
+      <c r="G186" s="18" t="str">
+        <f aca="false">IF(F186="","",F186*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H186" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A186="",'Détails des dons'!J186=""),"",'Détails des dons'!J186)</f>
         <v/>
       </c>
@@ -14132,7 +15602,15 @@
         <f aca="false">IF(OR('Détails des dons'!A187="",'Détails des dons'!E187=""),"",'Détails des dons'!E187)</f>
         <v/>
       </c>
-      <c r="F187" s="48" t="str">
+      <c r="F187" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A187="",'Détails des dons'!H187=""),"",'Détails des dons'!H187)</f>
+        <v/>
+      </c>
+      <c r="G187" s="18" t="str">
+        <f aca="false">IF(F187="","",F187*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H187" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A187="",'Détails des dons'!J187=""),"",'Détails des dons'!J187)</f>
         <v/>
       </c>
@@ -14158,7 +15636,15 @@
         <f aca="false">IF(OR('Détails des dons'!A188="",'Détails des dons'!E188=""),"",'Détails des dons'!E188)</f>
         <v/>
       </c>
-      <c r="F188" s="48" t="str">
+      <c r="F188" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A188="",'Détails des dons'!H188=""),"",'Détails des dons'!H188)</f>
+        <v/>
+      </c>
+      <c r="G188" s="18" t="str">
+        <f aca="false">IF(F188="","",F188*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H188" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A188="",'Détails des dons'!J188=""),"",'Détails des dons'!J188)</f>
         <v/>
       </c>
@@ -14184,7 +15670,15 @@
         <f aca="false">IF(OR('Détails des dons'!A189="",'Détails des dons'!E189=""),"",'Détails des dons'!E189)</f>
         <v/>
       </c>
-      <c r="F189" s="48" t="str">
+      <c r="F189" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A189="",'Détails des dons'!H189=""),"",'Détails des dons'!H189)</f>
+        <v/>
+      </c>
+      <c r="G189" s="18" t="str">
+        <f aca="false">IF(F189="","",F189*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H189" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A189="",'Détails des dons'!J189=""),"",'Détails des dons'!J189)</f>
         <v/>
       </c>
@@ -14210,7 +15704,15 @@
         <f aca="false">IF(OR('Détails des dons'!A190="",'Détails des dons'!E190=""),"",'Détails des dons'!E190)</f>
         <v/>
       </c>
-      <c r="F190" s="48" t="str">
+      <c r="F190" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A190="",'Détails des dons'!H190=""),"",'Détails des dons'!H190)</f>
+        <v/>
+      </c>
+      <c r="G190" s="18" t="str">
+        <f aca="false">IF(F190="","",F190*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H190" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A190="",'Détails des dons'!J190=""),"",'Détails des dons'!J190)</f>
         <v/>
       </c>
@@ -14236,7 +15738,15 @@
         <f aca="false">IF(OR('Détails des dons'!A191="",'Détails des dons'!E191=""),"",'Détails des dons'!E191)</f>
         <v/>
       </c>
-      <c r="F191" s="48" t="str">
+      <c r="F191" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A191="",'Détails des dons'!H191=""),"",'Détails des dons'!H191)</f>
+        <v/>
+      </c>
+      <c r="G191" s="18" t="str">
+        <f aca="false">IF(F191="","",F191*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H191" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A191="",'Détails des dons'!J191=""),"",'Détails des dons'!J191)</f>
         <v/>
       </c>
@@ -14262,7 +15772,15 @@
         <f aca="false">IF(OR('Détails des dons'!A192="",'Détails des dons'!E192=""),"",'Détails des dons'!E192)</f>
         <v/>
       </c>
-      <c r="F192" s="48" t="str">
+      <c r="F192" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A192="",'Détails des dons'!H192=""),"",'Détails des dons'!H192)</f>
+        <v/>
+      </c>
+      <c r="G192" s="18" t="str">
+        <f aca="false">IF(F192="","",F192*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H192" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A192="",'Détails des dons'!J192=""),"",'Détails des dons'!J192)</f>
         <v/>
       </c>
@@ -14288,7 +15806,15 @@
         <f aca="false">IF(OR('Détails des dons'!A193="",'Détails des dons'!E193=""),"",'Détails des dons'!E193)</f>
         <v/>
       </c>
-      <c r="F193" s="48" t="str">
+      <c r="F193" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A193="",'Détails des dons'!H193=""),"",'Détails des dons'!H193)</f>
+        <v/>
+      </c>
+      <c r="G193" s="18" t="str">
+        <f aca="false">IF(F193="","",F193*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H193" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A193="",'Détails des dons'!J193=""),"",'Détails des dons'!J193)</f>
         <v/>
       </c>
@@ -14314,7 +15840,15 @@
         <f aca="false">IF(OR('Détails des dons'!A194="",'Détails des dons'!E194=""),"",'Détails des dons'!E194)</f>
         <v/>
       </c>
-      <c r="F194" s="48" t="str">
+      <c r="F194" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A194="",'Détails des dons'!H194=""),"",'Détails des dons'!H194)</f>
+        <v/>
+      </c>
+      <c r="G194" s="18" t="str">
+        <f aca="false">IF(F194="","",F194*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H194" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A194="",'Détails des dons'!J194=""),"",'Détails des dons'!J194)</f>
         <v/>
       </c>
@@ -14340,7 +15874,15 @@
         <f aca="false">IF(OR('Détails des dons'!A195="",'Détails des dons'!E195=""),"",'Détails des dons'!E195)</f>
         <v/>
       </c>
-      <c r="F195" s="48" t="str">
+      <c r="F195" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A195="",'Détails des dons'!H195=""),"",'Détails des dons'!H195)</f>
+        <v/>
+      </c>
+      <c r="G195" s="18" t="str">
+        <f aca="false">IF(F195="","",F195*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H195" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A195="",'Détails des dons'!J195=""),"",'Détails des dons'!J195)</f>
         <v/>
       </c>
@@ -14366,7 +15908,15 @@
         <f aca="false">IF(OR('Détails des dons'!A196="",'Détails des dons'!E196=""),"",'Détails des dons'!E196)</f>
         <v/>
       </c>
-      <c r="F196" s="48" t="str">
+      <c r="F196" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A196="",'Détails des dons'!H196=""),"",'Détails des dons'!H196)</f>
+        <v/>
+      </c>
+      <c r="G196" s="18" t="str">
+        <f aca="false">IF(F196="","",F196*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H196" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A196="",'Détails des dons'!J196=""),"",'Détails des dons'!J196)</f>
         <v/>
       </c>
@@ -14392,7 +15942,15 @@
         <f aca="false">IF(OR('Détails des dons'!A197="",'Détails des dons'!E197=""),"",'Détails des dons'!E197)</f>
         <v/>
       </c>
-      <c r="F197" s="48" t="str">
+      <c r="F197" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A197="",'Détails des dons'!H197=""),"",'Détails des dons'!H197)</f>
+        <v/>
+      </c>
+      <c r="G197" s="18" t="str">
+        <f aca="false">IF(F197="","",F197*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H197" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A197="",'Détails des dons'!J197=""),"",'Détails des dons'!J197)</f>
         <v/>
       </c>
@@ -14418,7 +15976,15 @@
         <f aca="false">IF(OR('Détails des dons'!A198="",'Détails des dons'!E198=""),"",'Détails des dons'!E198)</f>
         <v/>
       </c>
-      <c r="F198" s="48" t="str">
+      <c r="F198" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A198="",'Détails des dons'!H198=""),"",'Détails des dons'!H198)</f>
+        <v/>
+      </c>
+      <c r="G198" s="18" t="str">
+        <f aca="false">IF(F198="","",F198*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H198" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A198="",'Détails des dons'!J198=""),"",'Détails des dons'!J198)</f>
         <v/>
       </c>
@@ -14444,7 +16010,15 @@
         <f aca="false">IF(OR('Détails des dons'!A199="",'Détails des dons'!E199=""),"",'Détails des dons'!E199)</f>
         <v/>
       </c>
-      <c r="F199" s="48" t="str">
+      <c r="F199" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A199="",'Détails des dons'!H199=""),"",'Détails des dons'!H199)</f>
+        <v/>
+      </c>
+      <c r="G199" s="18" t="str">
+        <f aca="false">IF(F199="","",F199*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H199" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A199="",'Détails des dons'!J199=""),"",'Détails des dons'!J199)</f>
         <v/>
       </c>
@@ -14470,7 +16044,15 @@
         <f aca="false">IF(OR('Détails des dons'!A200="",'Détails des dons'!E200=""),"",'Détails des dons'!E200)</f>
         <v/>
       </c>
-      <c r="F200" s="48" t="str">
+      <c r="F200" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A200="",'Détails des dons'!H200=""),"",'Détails des dons'!H200)</f>
+        <v/>
+      </c>
+      <c r="G200" s="18" t="str">
+        <f aca="false">IF(F200="","",F200*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H200" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A200="",'Détails des dons'!J200=""),"",'Détails des dons'!J200)</f>
         <v/>
       </c>
@@ -14496,7 +16078,15 @@
         <f aca="false">IF(OR('Détails des dons'!A201="",'Détails des dons'!E201=""),"",'Détails des dons'!E201)</f>
         <v/>
       </c>
-      <c r="F201" s="48" t="str">
+      <c r="F201" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A201="",'Détails des dons'!H201=""),"",'Détails des dons'!H201)</f>
+        <v/>
+      </c>
+      <c r="G201" s="18" t="str">
+        <f aca="false">IF(F201="","",F201*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H201" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A201="",'Détails des dons'!J201=""),"",'Détails des dons'!J201)</f>
         <v/>
       </c>
@@ -14522,7 +16112,15 @@
         <f aca="false">IF(OR('Détails des dons'!A202="",'Détails des dons'!E202=""),"",'Détails des dons'!E202)</f>
         <v/>
       </c>
-      <c r="F202" s="48" t="str">
+      <c r="F202" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A202="",'Détails des dons'!H202=""),"",'Détails des dons'!H202)</f>
+        <v/>
+      </c>
+      <c r="G202" s="18" t="str">
+        <f aca="false">IF(F202="","",F202*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H202" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A202="",'Détails des dons'!J202=""),"",'Détails des dons'!J202)</f>
         <v/>
       </c>
@@ -14548,7 +16146,15 @@
         <f aca="false">IF(OR('Détails des dons'!A203="",'Détails des dons'!E203=""),"",'Détails des dons'!E203)</f>
         <v/>
       </c>
-      <c r="F203" s="48" t="str">
+      <c r="F203" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A203="",'Détails des dons'!H203=""),"",'Détails des dons'!H203)</f>
+        <v/>
+      </c>
+      <c r="G203" s="18" t="str">
+        <f aca="false">IF(F203="","",F203*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H203" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A203="",'Détails des dons'!J203=""),"",'Détails des dons'!J203)</f>
         <v/>
       </c>
@@ -14574,7 +16180,15 @@
         <f aca="false">IF(OR('Détails des dons'!A204="",'Détails des dons'!E204=""),"",'Détails des dons'!E204)</f>
         <v/>
       </c>
-      <c r="F204" s="48" t="str">
+      <c r="F204" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A204="",'Détails des dons'!H204=""),"",'Détails des dons'!H204)</f>
+        <v/>
+      </c>
+      <c r="G204" s="18" t="str">
+        <f aca="false">IF(F204="","",F204*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H204" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A204="",'Détails des dons'!J204=""),"",'Détails des dons'!J204)</f>
         <v/>
       </c>
@@ -14600,7 +16214,15 @@
         <f aca="false">IF(OR('Détails des dons'!A205="",'Détails des dons'!E205=""),"",'Détails des dons'!E205)</f>
         <v/>
       </c>
-      <c r="F205" s="48" t="str">
+      <c r="F205" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A205="",'Détails des dons'!H205=""),"",'Détails des dons'!H205)</f>
+        <v/>
+      </c>
+      <c r="G205" s="18" t="str">
+        <f aca="false">IF(F205="","",F205*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H205" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A205="",'Détails des dons'!J205=""),"",'Détails des dons'!J205)</f>
         <v/>
       </c>
@@ -14626,17 +16248,29 @@
         <f aca="false">IF(OR('Détails des dons'!A206="",'Détails des dons'!E206=""),"",'Détails des dons'!E206)</f>
         <v/>
       </c>
-      <c r="F206" s="48" t="str">
+      <c r="F206" s="19" t="str">
+        <f aca="false">IF(OR('Détails des dons'!A206="",'Détails des dons'!H206=""),"",'Détails des dons'!H206)</f>
+        <v/>
+      </c>
+      <c r="G206" s="18" t="str">
+        <f aca="false">IF(F206="","",F206*'Budget du don'!$G$4)</f>
+        <v/>
+      </c>
+      <c r="H206" s="48" t="str">
         <f aca="false">IF(OR('Détails des dons'!A206="",'Détails des dons'!J206=""),"",'Détails des dons'!J206)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>